<commit_message>
Deliver episodes 21–25 storyboards with text blocking and completed text review
</commit_message>
<xml_diff>
--- a/archive/projects/la-reina-del-bajo-mundo/deliverables/前夫黑道酵母_分镜_21-33.xlsx
+++ b/archive/projects/la-reina-del-bajo-mundo/deliverables/前夫黑道酵母_分镜_21-33.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分镜脚本" sheetId="1" r:id="R904b0a6fe5a844a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分镜脚本" sheetId="1" r:id="R3937f7487433491c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -480,268 +480,2432 @@
       </x:c>
     </x:row>
     <x:row r="2" ht="200" customHeight="1">
-      <x:c r="A2" s="2"/>
-      <x:c r="B2" s="2"/>
-      <x:c r="C2" s="2"/>
-      <x:c r="D2" s="2"/>
-      <x:c r="E2" s="2"/>
-      <x:c r="F2" s="2"/>
-      <x:c r="G2" s="2"/>
-      <x:c r="H2" s="2"/>
-      <x:c r="I2" s="2"/>
+      <x:c r="A2" s="2" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B2" s="2" t="str">
+        <x:v>21-1A</x:v>
+      </x:c>
+      <x:c r="C2" s="2" t="str">
+        <x:v>Vera常服；Emiliano常服</x:v>
+      </x:c>
+      <x:c r="D2" s="2" t="str">
+        <x:v>轿车内（文字设定·夜）</x:v>
+      </x:c>
+      <x:c r="E2" s="2" t="str">
+        <x:v>白色卡片（文字设定）</x:v>
+      </x:c>
+      <x:c r="F2" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+轿车内（文字设定·夜），9:16竖屏。车外旅馆霓虹在侧窗形成冷蓝边光，道路灯经前挡风玻璃斜侧透入；面部保留暗部。
+[音轨规则]
+远层：旅馆入口外的雨后道路车流与夜间底噪。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
+3.1s—5.6s，@Emiliano常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Un departamento corporativo. Está vacío.」
+6.6s—8.1s，@Vera常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「No acepto favores.」
+9.6s—11.1s，@Emiliano常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Entonces llámalo inversión.」
+11.3s—13.5s，@Emiliano常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Si pierdes, pierdo mi dinero.」
+[锚定列表]
+场景：轿车内（文字设定·夜）
+角色：@Vera常服；@Emiliano常服
+道具：白色卡片（文字设定）
+未带@的本段场景或物件按已授权的文字设计执行，保持下述位置、数量和状态。
+[空间布局总览]
+轿车驾驶舱，夜，停在汽车旅馆入口外；驾驶位在车辆左侧，副驾驶在车辆右侧，前排隔中央扶手，右车门朝人行道。Emiliano常服坐驾驶位，Vera常服坐副驾驶，二人均未下车。卡片起初由Emiliano常服右手夹持。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（5个硬切分镜）]
+分镜一：【景别/视角：手部近景/后排中央向前 | 运镜：从中央扶手后方向右短移，落在卡片边缘】
+【时长】3.0s
+【构图】Emiliano常服右手将空白白色卡片递至中央扶手上方；卡片无字面朝下，Vera常服双手仍在自己腿侧。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】卡片停在两人之间，尚未交接。
+【镜头结尾·站位收束】卡片停在两人之间，尚未交接。
+画面硬切到分镜二。
+分镜二：【景别/视角：Emiliano常服前侧近景 | 运镜：在后排驾驶侧固定，焦点留在Emiliano常服眼部】
+【时长】3.5s
+【构图】Emiliano常服转头看向副驾驶，右手维持卡片高度；身体仍由驾驶座承托。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Emiliano常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】他说完，视线仍停在Vera常服。
+【镜头结尾·站位收束】他说完，视线仍停在Vera常服。
+画面硬切到分镜三。
+分镜三：【景别/视角：Vera常服侧面近景 | 运镜：切至后排副驾驶侧，保持二人视线轴同侧】
+【时长】3.0s
+【构图】Vera常服靠着副驾驶椅背，看一眼卡片再看Emiliano常服；唇部自然开合，说完只轻合。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Vera常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Vera常服未接卡，也未移座。
+【镜头结尾·站位收束】Vera常服未接卡，也未移座。
+画面硬切到分镜四。
+分镜四：【景别/视角：双人中近景/后排中央 | 运镜：向中央扶手轻推后落稳】
+【时长】4.0s
+【构图】Emiliano常服唇角略松，仍举着卡片，先回应，再补充投资的代价；Vera常服保持眼神接触。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Emiliano常服的对白按本段唯一声音骨架连续发声；@Emiliano常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】双方仍坐在前排，卡片仍在Emiliano常服右手。
+【镜头结尾·站位收束】双方仍坐在前排，卡片仍在Emiliano常服右手。
+画面硬切到分镜五。
+分镜五：【景别/视角：手部特写/副驾驶斜后方 | 运镜：固定，保持双方手指和卡片均在焦内】
+【时长】3.5s
+【构图】Vera常服右手伸向卡片远端；两人各持一端，Vera常服夹稳后Emiliano常服才松指，卡片移入Vera常服右手。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】Vera常服右手收回卡片；Emiliano常服右手落向扶手。
+【镜头结尾·站位收束】Vera常服右手收回卡片；Emiliano常服右手落向扶手。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：17s</x:v>
+      </x:c>
+      <x:c r="G2" s="2" t="str">
+        <x:v>Emiliano：「Un departamento corporativo. Está vacío.」
+Vera：「No acepto favores.」
+Emiliano：「Entonces llámalo inversión.」
+Emiliano：「Si pierdes, pierdo mi dinero.」</x:v>
+      </x:c>
+      <x:c r="H2" s="2" t="str">
+        <x:v>第21集
+21-1 轿车内 夜 内
+人物：Vera、Emiliano、Emiliano
+△ 镜头特写：一张白色银行卡被两根修长的手指夹着，递向画面左侧。背景是车窗外模糊的雨夜街景。
+△ 镜头近景：Emiliano坐在驾驶位，穿着黑色西装和白衬衫，打着黑色领带。他转过头看向副驾驶位的 Vera，眼神中带着一种复杂的施舍感。
+Emiliano：Un departamento corporativo. Está vacío.
+△ 镜头反打：Vera 坐在副驾驶位，穿着米色风衣（gabardina beige），长发微乱。她靠在椅背上，转头冷冷地盯着 Emiliano，眼神中没有丝毫畏惧或感激。
+Vera（语气冷淡）：No acepto favores.
+△ 镜头切换：Emiliano 依然举着那张卡，嘴角微微上扬，露出一抹似是而非的笑意。
+Emiliano：Entonces llámalo inversión.
+△ 镜头特写：Emiliano 微微晃动了一下手中的银行卡，手指修长，骨节分明。
+Emiliano：Si pierdes, pierdo mi dinero.
+△ 镜头近景：Vera 盯着那张卡片，沉默了半秒，随后伸手接过了卡。
+△ 动作特写：两人的手指在卡片边缘交错。Vera 的动作干脆利落。</x:v>
+      </x:c>
+      <x:c r="I2" s="2" t="str">
+        <x:v>17s</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="200" customHeight="1">
-      <x:c r="A3" s="2"/>
-      <x:c r="B3" s="2"/>
-      <x:c r="C3" s="2"/>
-      <x:c r="D3" s="2"/>
-      <x:c r="E3" s="2"/>
-      <x:c r="F3" s="2"/>
-      <x:c r="G3" s="2"/>
-      <x:c r="H3" s="2"/>
-      <x:c r="I3" s="2"/>
+      <x:c r="A3" s="2" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B3" s="2" t="str">
+        <x:v>21-1B</x:v>
+      </x:c>
+      <x:c r="C3" s="2" t="str">
+        <x:v>Vera常服；Emiliano常服</x:v>
+      </x:c>
+      <x:c r="D3" s="2" t="str">
+        <x:v>汽车旅馆103房（外·夜）</x:v>
+      </x:c>
+      <x:c r="E3" s="2" t="str">
+        <x:v>白色卡片（文字设定）；轿车（文字设定）</x:v>
+      </x:c>
+      <x:c r="F3" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+汽车旅馆103房（外·夜），9:16竖屏。旅馆蓝色灯光形成侧逆光，门边实用灯照亮人行道；招牌光面不含字样。
+[音轨规则]
+远层：旅馆入口外的雨后道路车流与夜间底噪。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
+6.6s—8.4s，@Vera常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Bonitos zapatos, por cierto.」
+[锚定列表]
+场景：@汽车旅馆103房（外·夜）
+角色：@Vera常服；@Emiliano常服
+道具：白色卡片（文字设定）；轿车（文字设定）
+未带@的本段场景或物件按已授权的文字设计执行，保持下述位置、数量和状态。
+[空间布局总览]
+轿车驾驶舱，夜，停在汽车旅馆入口外；驾驶位在车辆左侧，副驾驶在车辆右侧，前排隔中央扶手，右车门朝人行道。右车门外是人行道，旅馆入口在车头前方偏右。卡片已被Vera常服收进自己右侧口袋，Emiliano常服始终留在驾驶位。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（5个硬切分镜）]
+分镜一：【景别/视角：车外右侧中景 | 运镜：从副驾驶门外向后侧让开半步】
+【时长】3.5s
+【构图】Vera常服从内部推开右车门，双脚依次落在人行道，扶门框起身离座。
+【音效】门扇与门锁随实际开合发声、鞋底接触地面声；台词期间压低动作声。
+【台词】无台词。
+【变化】Vera常服已站在车外；车门仍打开。
+【镜头结尾·站位收束】Vera常服已站在车外；车门仍打开。
+画面硬切到分镜二。
+分镜二：【景别/视角：侧后中景/人行道 | 运镜：与Vera常服同向前行，保持一步距离】
+【时长】3.0s
+【构图】Vera常服回手关好副驾驶门，沿人行道朝旅馆入口走出数步。
+【音效】门扇与门锁随实际开合发声、脚步随起停出现；台词期间压低动作声。
+【台词】无台词。
+【变化】车门关闭；Vera常服位于车头右前方。
+【镜头结尾·站位收束】车门关闭；Vera常服位于车头右前方。
+画面硬切到分镜三。
+分镜三：【景别/视角：Vera常服侧面中近景 | 运镜：在车头右外侧固定，车窗留在画面另一端】
+【时长】4.0s
+【构图】Vera常服停步，回身看向侧窗内的Emiliano常服，平静说出一句评语；身体留在人行道。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Vera常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】她说完后重心转回旅馆方向。
+【镜头结尾·站位收束】她说完后重心转回旅馆方向。
+画面硬切到分镜四。
+分镜四：【景别/视角：隔侧窗Emiliano常服近景 | 运镜：从副驾驶外侧固定观察，镜头不进入玻璃】
+【时长】3.0s
+【构图】Emiliano常服坐在左侧驾驶位，看着Vera常服继续离开，嘴角收住一丝笑意，右手回到车辆控制区。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】车内只有Emiliano常服；Vera常服已走向入口。
+【镜头结尾·站位收束】车内只有Emiliano常服；Vera常服已走向入口。
+画面硬切到分镜五。
+分镜五：【景别/视角：旅馆入口远中景 | 运镜：镜头留在人行道，从车身轻摇向入口】
+【时长】3.0s
+【构图】Vera常服跨过入口门槛，步速正常；身后的轿车发动，车辆只在门边画外发出引擎声。
+【音效】门扇与门锁随实际开合发声；台词期间压低动作声。
+【台词】无台词。
+【变化】Vera常服进入旅馆，Emiliano常服留在车内；本段以这次离场结束。
+【镜头结尾·站位收束】Vera常服进入旅馆，Emiliano常服留在车内；本段以这次离场结束。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：16.5s</x:v>
+      </x:c>
+      <x:c r="G3" s="2" t="str">
+        <x:v>Vera：「Bonitos zapatos, por cierto.」</x:v>
+      </x:c>
+      <x:c r="H3" s="2" t="str">
+        <x:v>△ 画面切到车外：Vera 推开车门走下车。背景是汽车旅馆103房（Motel Vista Pacífico）的大门，蓝色的霓虹灯牌在雨后的夜空中闪烁。
+△ 镜头跟随：Vera 穿着米色风衣，步履轻盈而坚定地走向旅馆大门。
+△ 镜头切回车内：Emiliano 坐在驾驶位，透过侧窗看着 Vera 的背影，眼神深邃。
+△ 镜头近景：Vera 停下脚步，转过身，隔着车窗看向 Emiliano。
+Vera（语气平静）：Bonitos zapatos, por cierto.
+△ 动作特写：Vera 潇洒地转身离去，留下一个倔强的背影。
+△ 镜头切到 Emiliano：他看着 Vera 离去，脸上浮现出一抹玩味的笑容，随即发动了汽车。</x:v>
+      </x:c>
+      <x:c r="I3" s="2" t="str">
+        <x:v>16.5s</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="200" customHeight="1">
-      <x:c r="A4" s="2"/>
-      <x:c r="B4" s="2"/>
-      <x:c r="C4" s="2"/>
-      <x:c r="D4" s="2"/>
-      <x:c r="E4" s="2"/>
-      <x:c r="F4" s="2"/>
-      <x:c r="G4" s="2"/>
-      <x:c r="H4" s="2"/>
-      <x:c r="I4" s="2"/>
+      <x:c r="A4" s="2" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B4" s="2" t="str">
+        <x:v>21-2A</x:v>
+      </x:c>
+      <x:c r="C4" s="2" t="str">
+        <x:v>Vera常服</x:v>
+      </x:c>
+      <x:c r="D4" s="2" t="str">
+        <x:v>高层公寓客厅（夜）</x:v>
+      </x:c>
+      <x:c r="E4" s="2" t="str">
+        <x:v>牛皮纸档案袋（文字设定）；两张便利贴（文字设定）；黑色胶卷转盘（文字设定）</x:v>
+      </x:c>
+      <x:c r="F4" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+高层公寓客厅（夜），9:16竖屏。东窗外城市散光作轮廓，客厅实际落地灯从北侧斜照茶几，暖光不正面直打脸。
+[音轨规则]
+远层：公寓外远处车流低声，室内维持安静。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段无原定对白或旁白，不新增发声。
+[锚定列表]
+场景：@高层公寓客厅（夜）
+角色：@Vera常服
+道具：牛皮纸档案袋（文字设定）；两张便利贴（文字设定）；黑色胶卷转盘（文字设定）
+未带@的本段场景或物件按已授权的文字设计执行，保持下述位置、数量和状态。
+[空间布局总览]
+公寓室内为文字确定的连续空间：入口门在西墙，向室内开启；入口向东进入客厅，茶几在中部、沙发在其北侧；东侧为临街落地窗，东北转角窄玻璃面朝相邻楼；阳台移门在南侧。本文方位为世界参照，不随反打改变。Vera常服从西侧入口进入，档案袋和两层便利贴在茶几中央；胶卷转盘起初在袋内。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（6个硬切分镜）]
+分镜一：【景别/视角：客厅远景/入口内侧 | 运镜：沿入口向东短移，展示门、茶几与落地窗的关系】
+【时长】3.0s
+【构图】Vera常服从西门走进室内，先停在茶几西侧观察房间。
+【音效】门扇与门锁随实际开合发声、脚步随起停出现；台词期间压低动作声。
+【台词】无台词。
+【变化】Vera常服在茶几西侧，档案袋在桌中央。
+【镜头结尾·站位收束】Vera常服在茶几西侧，档案袋在桌中央。
+画面硬切到分镜二。
+分镜二：【景别/视角：脚步与桌沿低位中景 | 运镜：沿茶几西沿平移半步后停止】
+【时长】3.0s
+【构图】Vera常服靠近茶几，脚步收住；衣摆只随停步自然回落。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】双脚停稳，身体面向茶几。
+【镜头结尾·站位收束】双脚停稳，身体面向茶几。
+画面硬切到分镜三。
+分镜三：【景别/视角：档案袋与右手近景 | 运镜：在桌面西南角固定，纸面浅景深】
+【时长】3.5s
+【构图】Vera常服右指触到上层便利贴边缘；纸面留为空白，视线与指尖停顿保留发现留言的节拍。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】右手触贴，袋口未开。
+【镜头结尾·站位收束】右手触贴，袋口未开。
+画面硬切到分镜四。
+分镜四：【景别/视角：Vera常服侧面与手部中近景 | 运镜：从茶几南侧向右轻移，露出两层纸片】
+【时长】3.0s
+【构图】她揭起上层空白便利贴，发现下面还有一层；看向第二层，唇部不发声。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】上层便利贴在右手，下层仍贴袋面。
+【镜头结尾·站位收束】上层便利贴在右手，下层仍贴袋面。
+画面硬切到分镜五。
+分镜五：【景别/视角：袋口与胶卷特写 | 运镜：固定在桌边，焦点覆盖袋口与落点】
+【时长】3.5s
+【构图】Vera常服把揭下的纸片放在袋旁，双手开袋，将黑色胶卷转盘滑到桌上；手掌贴近桌面控制落差。
+【音效】纸张轻擦声；台词期间压低动作声。
+【台词】无台词。
+【变化】转盘平放茶几，纸片与档案袋在其旁。
+【镜头结尾·站位收束】转盘平放茶几，纸片与档案袋在其旁。
+画面硬切到分镜六。
+分镜六：【景别/视角：Vera常服侧后近景 | 运镜：轻抬机位，由桌面摇至她望向东窗的侧脸】
+【时长】3.0s
+【构图】Vera常服看一眼转盘，再抬眼望向城市；下颌维持原有张力，不新增惊呼。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】Vera常服仍在茶几西侧，转盘留在桌面。
+【镜头结尾·站位收束】Vera常服仍在茶几西侧，转盘留在桌面。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：19s</x:v>
+      </x:c>
+      <x:c r="G4" s="2" t="str"/>
+      <x:c r="H4" s="2" t="str">
+        <x:v>21-2 高层公寓（Departamento ejecutivo, Piso 21, Reforma） 夜 内
+人物：Vera
+△ 画面全景：一间极具现代感的豪华套房。巨大的落地窗正对着改革大道璀璨的夜景，灯火辉煌。室内装修简约而奢华，木质地板在灯光下泛着温润的光泽。
+△ 动作特写：一双穿着黑色高跟短靴的脚走入画面，踩在深色的地毯上。
+△ 镜头跟随：Vera 缓缓走进客厅，米色风衣随风摆动。她环视着这个宽敞的空间。
+△ 镜头特写：在大理石纹路的茶几上，静静地躺着一个棕色的牛皮纸档案袋。袋子上贴着一张黄色的便利贴。
+△ 画面近景：Vera 走到桌边，弯腰看向便利贴上的字迹。
+【字幕：Bienvenida a casa. — E.】
+△ 动作特写：Vera 伸出右手，指尖轻触便利贴上的“E”署名。她的指甲修剪整齐，涂着浅色的甲油。
+△ 镜头切换：Vera 撕下第一张便利贴，发现下面还有第二张。
+△ 画面特写：第二张便利贴上的字迹整齐而犀利。
+【字幕：P.D. Los guardias de abajo están en mi nómina. No les des lata.】
+△ 镜头近景：Vera 读完文字，眼中闪过一丝复杂的情绪，随即她伸手将档案袋里的东西倒了出来。
+△ 动作特写：一个黑色的胶卷转盘从袋子里滑出，落在桌面上，发出沉闷的碰撞声。
+△ 镜头切到 Vera：她抬头看向窗外壮丽的夜色，眼神逐渐变得深不可测。</x:v>
+      </x:c>
+      <x:c r="I4" s="2" t="str">
+        <x:v>19s</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="200" customHeight="1">
-      <x:c r="A5" s="2"/>
-      <x:c r="B5" s="2"/>
-      <x:c r="C5" s="2"/>
-      <x:c r="D5" s="2"/>
-      <x:c r="E5" s="2"/>
-      <x:c r="F5" s="2"/>
-      <x:c r="G5" s="2"/>
-      <x:c r="H5" s="2"/>
-      <x:c r="I5" s="2"/>
+      <x:c r="A5" s="2" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B5" s="2" t="str">
+        <x:v>21-3A</x:v>
+      </x:c>
+      <x:c r="C5" s="2" t="str">
+        <x:v>Vera常服</x:v>
+      </x:c>
+      <x:c r="D5" s="2" t="str">
+        <x:v>高层公寓窗边与入口（文字设定·夜）</x:v>
+      </x:c>
+      <x:c r="E5" s="2" t="str"/>
+      <x:c r="F5" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+高层公寓窗边与入口（文字设定·夜），9:16竖屏。城市夜光从窗外勾勒肩部；楼下门灯只照入口与两位保镖。
+[音轨规则]
+远层：公寓外远处车流低声，室内维持安静。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段无原定对白或旁白，不新增发声。
+[锚定列表]
+场景：高层公寓窗边与入口（文字设定·夜）
+角色：@Vera常服
+未带@的本段场景或物件按已授权的文字设计执行，保持下述位置、数量和状态。
+[空间布局总览]
+公寓室内为文字确定的连续空间：入口门在西墙，向室内开启；入口向东进入客厅，茶几在中部、沙发在其北侧；东侧为临街落地窗，东北转角窄玻璃面朝相邻楼；阳台移门在南侧。本文方位为世界参照，不随反打改变。Vera常服在东窗内侧。楼下门卫两人为普通背景保镖，各守入口两侧，身份不与Escolta A合并。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（4个硬切分镜）]
+分镜一：【景别/视角：背面中景/客厅西侧望东 | 运镜：缓慢向东推进，落在Vera常服与窗框构成的关系画面】
+【时长】3.0s
+【构图】Vera常服站在窗内，双臂交叠；楼下道路与城市灯点处在她视线方向。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】Vera常服未移动，视线向下。
+【镜头结尾·站位收束】Vera常服未移动，视线向下。
+画面硬切到分镜二。
+分镜二：【景别/视角：极高俯拍/窗边向楼下 | 运镜：固定，沿已建立的垂直方向向下取景】
+【时长】3.0s
+【构图】两名普通背景保镖分站楼下入口两侧，各守一边；画面仅交代体量、位置和朝向，不要求读到细微表情。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】两人留在入口两侧，没有换位。
+【镜头结尾·站位收束】两人留在入口两侧，没有换位。
+画面硬切到分镜三。
+分镜三：【景别/视角：入口低位中景 | 运镜：在入口外侧固定，向上构图保留楼体方向】
+【时长】3.0s
+【构图】两名保镖先抬眼再抬头，朝高层同一个窗口略点头；动作先后自然。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】两人朝上，双脚仍在原岗位。
+【镜头结尾·站位收束】两人朝上，双脚仍在原岗位。
+画面硬切到分镜四。
+分镜四：【景别/视角：Vera常服侧面近景/室内南侧 | 运镜：固定，窗框形成画面竖向边界】
+【时长】3.0s
+【构图】Vera常服收回俯视，仍站窗内；唇部放松闭合，保持观察。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】Vera常服站位不变；楼下岗位关系已建立。
+【镜头结尾·站位收束】Vera常服站位不变；楼下岗位关系已建立。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：12s</x:v>
+      </x:c>
+      <x:c r="G5" s="2" t="str"/>
+      <x:c r="H5" s="2" t="str">
+        <x:v>21-3 高层公寓落地窗前 夜 内/外
+人物：Vera、保镖甲、保镖乙
+△ 画面全景：Vera 站在落地窗前，双臂交叠在胸前，背影在繁星般的城市灯火映照下显得格外纤细且孤寂。
+△ 镜头俯拍：公寓大楼入口处。两名穿着黑色西装、戴着皮手套的保镖像雕塑一般笔直地站在门柱旁，神情肃穆，双手交叠在身前。
+△ 镜头反打：保镖们似乎察觉到了楼上的目光，整齐划一地抬头看向高层窗户，并微微低头致意。
+△ 镜头切到 Vera：她依然站在窗前，面无表情地注视着下方的动向。</x:v>
+      </x:c>
+      <x:c r="I5" s="2" t="str">
+        <x:v>12s</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="200" customHeight="1">
-      <x:c r="A6" s="2"/>
-      <x:c r="B6" s="2"/>
-      <x:c r="C6" s="2"/>
-      <x:c r="D6" s="2"/>
-      <x:c r="E6" s="2"/>
-      <x:c r="F6" s="2"/>
-      <x:c r="G6" s="2"/>
-      <x:c r="H6" s="2"/>
-      <x:c r="I6" s="2"/>
+      <x:c r="A6" s="2" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B6" s="2" t="str">
+        <x:v>21-4A</x:v>
+      </x:c>
+      <x:c r="C6" s="2" t="str">
+        <x:v>Vera常服</x:v>
+      </x:c>
+      <x:c r="D6" s="2" t="str">
+        <x:v>高层公寓客厅（夜）</x:v>
+      </x:c>
+      <x:c r="E6" s="2" t="str">
+        <x:v>狙击镜观察画面（文字设定）</x:v>
+      </x:c>
+      <x:c r="F6" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+高层公寓客厅（夜），9:16竖屏。客厅灯已落在人物侧后；外来细红光从东北侧窄窗斜入肩背，方向与观察视线一致。
+[音轨规则]
+远层：公寓外远处车流低声，室内维持安静。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段无原定对白或旁白，不新增发声。
+[锚定列表]
+场景：@高层公寓客厅（夜）
+角色：@Vera常服
+道具：狙击镜观察画面（文字设定）
+未带@的本段场景或物件按已授权的文字设计执行，保持下述位置、数量和状态。
+[空间布局总览]
+公寓室内为文字确定的连续空间：入口门在西墙，向室内开启；入口向东进入客厅，茶几在中部、沙发在其北侧；东侧为临街落地窗，东北转角窄玻璃面朝相邻楼；阳台移门在南侧。本文方位为世界参照，不随反打改变。Vera常服位于东窗偏北，身体朝东南看夜景；东北转角玻璃使相邻楼斜后方视线能看到她肩背。观察者始终在对楼，镜头不穿玻璃。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（3个硬切分镜）]
+分镜一：【景别/视角：远距主观特写/狙击镜视角 | 运镜：微幅调整朝向，保持远距机位不平移】
+【时长】3.0s
+【构图】圆形光学视野内仅留绿色十字线，缓慢寻到窗内Vera常服肩背；不显示字母、刻度数字或界面文字。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】十字线接近肩部，Vera常服未转身。
+【镜头结尾·站位收束】十字线接近肩部，Vera常服未转身。
+画面硬切到分镜二。
+分镜二：【景别/视角：肩背近景/客厅内侧 | 运镜：固定观察侧后方，焦点落在衣料受光处】
+【时长】3.0s
+【构图】细红光沿肩背短距离移向后颈；Vera常服仍看窗外，衣料自然呼吸起伏。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】红光接近后颈，人物尚未回应。
+【镜头结尾·站位收束】红光接近后颈，人物尚未回应。
+画面硬切到分镜三。
+分镜三：【景别/视角：远距主观近景/对楼 | 运镜：随观察者一次自然呼吸产生很小起伏后落稳】
+【时长】3.0s
+【构图】十字线落在头后侧轮廓，城市散光被压在窗后；仅保留低弱画外呼吸。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】准星停住，威胁悬而未决。
+【镜头结尾·站位收束】准星停住，威胁悬而未决。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：9s</x:v>
+      </x:c>
+      <x:c r="G6" s="2" t="str"/>
+      <x:c r="H6" s="2" t="str">
+        <x:v>21-4 高层公寓/狙击视角 夜 内
+人物：Vera
+△ 画面切换：镜头突然转变为狙击镜视角。绿色的十字准星在画面中心晃动，红色的激光点在 Vera 的米色风衣背部不断游走。
+△ 镜头特写：狙击镜中的 Vera 毫无察觉。红色光点从她的肩膀移到了后颈处。
+△ 镜头切换：画面剧烈摇晃，伴随着重重的喘息声。
+△ 镜头收尾：狙击镜的十字准星死死锁定了 Vera 的头部。红光在她的发丝间闪烁。</x:v>
+      </x:c>
+      <x:c r="I6" s="2" t="str">
+        <x:v>9s</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="200" customHeight="1">
-      <x:c r="A7" s="2"/>
-      <x:c r="B7" s="2"/>
-      <x:c r="C7" s="2"/>
-      <x:c r="D7" s="2"/>
-      <x:c r="E7" s="2"/>
-      <x:c r="F7" s="2"/>
-      <x:c r="G7" s="2"/>
-      <x:c r="H7" s="2"/>
-      <x:c r="I7" s="2"/>
+      <x:c r="A7" s="2" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B7" s="2" t="str">
+        <x:v>22-1A</x:v>
+      </x:c>
+      <x:c r="C7" s="2" t="str">
+        <x:v>Vera常服</x:v>
+      </x:c>
+      <x:c r="D7" s="2" t="str">
+        <x:v>高层公寓客厅（夜）</x:v>
+      </x:c>
+      <x:c r="E7" s="2" t="str">
+        <x:v>狙击镜观察画面（文字设定）</x:v>
+      </x:c>
+      <x:c r="F7" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+高层公寓客厅（夜），9:16竖屏。东窗城市漫反光维持脸部轮廓，细红光来自东北斜后方，玻璃只给出符合角度的局部反射。
+[音轨规则]
+远层：公寓外远处车流低声，室内维持安静。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段无原定对白或旁白，不新增发声。
+[锚定列表]
+场景：@高层公寓客厅（夜）
+角色：@Vera常服
+道具：狙击镜观察画面（文字设定）
+未带@的本段场景或物件按已授权的文字设计执行，保持下述位置、数量和状态。
+[空间布局总览]
+公寓室内为文字确定的连续空间：入口门在西墙，向室内开启；入口向东进入客厅，茶几在中部、沙发在其北侧；东侧为临街落地窗，东北转角窄玻璃面朝相邻楼；阳台移门在南侧。本文方位为世界参照，不随反打改变。沿用Vera常服在东窗偏北面向东南的站位；东北侧窄窗允许对楼观察其肩背。红光先在后心附近，随她侧头调整到头后侧。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（4个硬切分镜）]
+分镜一：【景别/视角：肩背近景/东北侧斜望 | 运镜：固定，避免让玻璃同时映出不可能的完整背面】
+【时长】3.0s
+【构图】红光自后颈沿衣料滑向肩胛与背部；她仍在窗边，肩部随自然呼吸略动。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】红光留在背部，Vera常服未移动双脚。
+【镜头结尾·站位收束】红光留在背部，Vera常服未移动双脚。
+画面硬切到分镜二。
+分镜二：【景别/视角：对楼主观近景 | 运镜：缓慢摇摄，从后颈收至头后轮廓】
+【时长】3.0s
+【构图】准星移动有连续方向，Vera常服头后侧留在窗内可见区。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】准星落在头后侧。
+【镜头结尾·站位收束】准星落在头后侧。
+画面硬切到分镜三。
+分镜三：【景别/视角：Vera常服侧面近景/室内南侧 | 运镜：小幅侧移，从窗框遮挡外露出她的侧脸】
+【时长】3.5s
+【构图】Vera常服目光先稍偏，随后头部轻转；眉部略收，唇缝短暂轻合，不新增吸气或瞪眼。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】头部转出小角度，脚下位置不变。
+【镜头结尾·站位收束】头部转出小角度，脚下位置不变。
+画面硬切到分镜四。
+分镜四：【景别/视角：对楼主观近景 | 运镜：顺Vera常服转头方向轻摇后固定】
+【时长】3.0s
+【构图】准星跟随头部轮廓重新落稳；观察者仍在对楼，画面不越过墙体。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】Vera常服仍在窗内，追踪仍持续。
+【镜头结尾·站位收束】Vera常服仍在窗内，追踪仍持续。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：12.5s</x:v>
+      </x:c>
+      <x:c r="G7" s="2" t="str"/>
+      <x:c r="H7" s="2" t="str">
+        <x:v>第22集
+22-1 高层公寓落地窗前 夜 内
+人物：Vera
+△ 画面特写：窗玻璃的倒影中，Vera 的背部出现了一个清晰的红点。红点在米色风衣的布料上微微颤动，从左肩胛骨缓慢移动到后心位置。
+△ 镜头反打：Vera 依然静静地站立着，望着窗外繁华的夜景，对背后的死亡威胁毫无察觉。她的发丝随风微动，眼神深邃而沉静。
+△ 镜头切换：狙击镜的视角。绿色的电子辅助线交织，Vera 的头后部正处于十字准星的中心。红色激光点锁定了她的后脑勺，画面随着狙击手的呼吸轻微起伏。
+△ 镜头特写：Vera 似乎察觉到了什么，她微微侧过头，长长的睫毛在落地窗映出的微光中颤动。
+△ 镜头切换：狙击镜视角。准星随着 Vera 的动作迅速调整，始终死死咬住她的头部轮廓。</x:v>
+      </x:c>
+      <x:c r="I7" s="2" t="str">
+        <x:v>12.5s</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="200" customHeight="1">
-      <x:c r="A8" s="2"/>
-      <x:c r="B8" s="2"/>
-      <x:c r="C8" s="2"/>
-      <x:c r="D8" s="2"/>
-      <x:c r="E8" s="2"/>
-      <x:c r="F8" s="2"/>
-      <x:c r="G8" s="2"/>
-      <x:c r="H8" s="2"/>
-      <x:c r="I8" s="2"/>
+      <x:c r="A8" s="2" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B8" s="2" t="str">
+        <x:v>22-2A</x:v>
+      </x:c>
+      <x:c r="C8" s="2" t="str">
+        <x:v>Víctor常服；Damián常服；Escorpión常服；Escolta A常服</x:v>
+      </x:c>
+      <x:c r="D8" s="2" t="str">
+        <x:v>家主书房（夜）</x:v>
+      </x:c>
+      <x:c r="E8" s="2" t="str">
+        <x:v>黑色皮革手提箱</x:v>
+      </x:c>
+      <x:c r="F8" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+家主书房（夜），9:16竖屏。西侧台灯暖光斜切书桌，书架和门口落暗；皮箱表面只反射实际灯光。
+[音轨规则]
+远层：书房内安静的室内底噪，门外动静低于台词。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
+6.1s—7.9s，@Víctor常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Cuánto tiempo sin verlo.」
+9.1s—11.2s，@Escorpión常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Reembolso completo. Me retiro.」
+12.1s—17.0s，@Damián常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「¡Tres millones de pesos! ¡Eres el limpiador más caro del país!」
+[锚定列表]
+场景：@家主书房（夜）
+角色：@Víctor常服；@Damián常服；@Escorpión常服；@Escolta A常服
+道具：@黑色皮革手提箱
+[空间布局总览]
+书桌位于书房北部，Víctor常服在桌北侧主位面向南；Damián常服在桌东端面向西南；客位在桌南侧；门在南墙偏西，书架在西墙，通道沿桌西侧与南侧保留。Escorpión常服从南门进入后停在桌南侧，手提箱由其双手放至桌南沿；Escolta A站门内西侧。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（6个硬切分镜）]
+分镜一：【景别/视角：书房关系全景/门内东侧 | 运镜：从门侧沿南部通道向西短移】
+【时长】3.0s
+【构图】Víctor常服坐桌北，Damián常服站桌东，Escolta A守门内西侧；Escorpión常服站桌南，把手提箱放稳。
+【音效】门扇与门锁随实际开合发声、箱体或扣锁的实际接触声；台词期间压低动作声。
+【台词】无台词。
+【变化】手提箱在桌南沿；四人各处于已定位置。
+【镜头结尾·站位收束】手提箱在桌南沿；四人各处于已定位置。
+画面硬切到分镜二。
+分镜二：【景别/视角：箱扣手部特写 | 运镜：固定，箱盖与双手保持可读】
+【时长】3.0s
+【构图】Escorpión常服依次打开两侧扣锁，再向北侧掀开箱盖；手指离开夹缝。
+【音效】箱体或扣锁的实际接触声；台词期间压低动作声。
+【台词】无台词。
+【变化】两侧扣已开，箱盖向北立起。
+【镜头结尾·站位收束】两侧扣已开，箱盖向北立起。
+画面硬切到分镜三。
+分镜三：【景别/视角：Víctor常服侧面近景/桌西侧 | 运镜：沿桌西侧轻推后停住】
+【时长】3.0s
+【构图】Víctor常服手中雪茄暂时不动，抬眼看向Escorpión常服，声音低平。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Víctor常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Víctor常服仍坐桌北，目光落在来客。
+【镜头结尾·站位收束】Víctor常服仍坐桌北，目光落在来客。
+画面硬切到分镜四。
+分镜四：【景别/视角：Escorpión常服中近景/桌东南侧 | 运镜：固定，箱盖下缘留作前景】
+【时长】3.0s
+【构图】Escorpión常服看向Víctor常服，站稳后直接说明退款决定，双手已离开箱扣。
+【音效】箱体或扣锁的实际接触声；台词期间压低动作声。
+【台词】@Escorpión常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Escorpión常服站桌南，肩背保持平直。
+【镜头结尾·站位收束】Escorpión常服站桌南，肩背保持平直。
+画面硬切到分镜五。
+分镜五：【景别/视角：Damián常服侧面近景/桌南侧 | 运镜：短促向右摇到Damián常服后落稳】
+【时长】3.5s
+【构图】Damián常服原本站立在桌东，听到退款时转向箱子，指向桌面；不再安排第二次从座位起身。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Damián常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Damián常服仍站桌东，手指指向箱内。
+【镜头结尾·站位收束】Damián常服仍站桌东，手指指向箱内。
+画面硬切到分镜六。
+分镜六：【景别/视角：Escorpión常服与Víctor常服双人关系中景 | 运镜：从书桌西侧固定观察两人】
+【时长】3.0s
+【构图】Escorpión常服不回应Damián常服，目光越过箱盖停在Víctor常服脸上；Víctor常服前臂离开椅扶手少许。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Damián常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】三角视线关系清楚；Escolta A仍在门侧。
+【镜头结尾·站位收束】三角视线关系清楚；Escolta A仍在门侧。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：18.5s</x:v>
+      </x:c>
+      <x:c r="G8" s="2" t="str">
+        <x:v>Víctor：「Cuánto tiempo sin verlo.」
+Escorpión：「Reembolso completo. Me retiro.」
+Damián：「¡Tres millones de pesos! ¡Eres el limpiador más caro del país!」</x:v>
+      </x:c>
+      <x:c r="H8" s="2" t="str">
+        <x:v>22-2 家主书房（Estudio, Mansión Vargas） 夜 内
+人物：Víctor、Damián、保镖甲、Escorpión
+△ 画面特写：Víctor 穿着黑金花纹西装，坐在书桌后的皮椅上。他双眼微眯，神情阴冷，手中把玩着一支昂贵的雪茄。
+△ 镜头全景：书房内气氛压抑。书架整齐排布，灯光昏暗。Damián 站在桌旁，保镖甲守在后方。
+△ 镜头反打：书桌对面，Escorpión 站姿笔挺，穿着黑色工装外套，背着黑色双肩包，双手戴着黑色半指手套。他正将一个沉重的黑色皮革手提箱放在书桌上。
+△ 动作特写：Escorpión 伸出手，动作利落地按下手提箱两侧的锁扣。随着“咔哒”两声清脆的金属撞击声，箱盖弹开。
+Víctor（声音低沉有力）：Cuánto tiempo sin verlo.
+△ 镜头切到 Escorpión：他神情冷峻，目光在 Víctor 和旁边的 Damián 身上扫过，没有任何情感波动。
+Escorpión（语气生硬，不带感情）：Reembolso completo. Me retiro.
+△ 镜头特写：Damián 听到这话，猛地从座位上站了起来。他穿着棕紫色西装，脸色铁青，额头青筋暴起，显得极度愤怒。
+Damián（指着箱子咆哮）：¡Tres millones de pesos! ¡Eres el limpiador más caro del país!
+△ 镜头切到 Escorpión：他完全无视了 Damián 的愤怒，眼神冰冷地盯着 Víctor。他的双眼微红，透着一种决绝的疲态。
+△ 镜头反打：Víctor 依旧气定神闲地坐着，甚至没有看那箱钱，只是盯着 Escorpión 的眼睛。</x:v>
+      </x:c>
+      <x:c r="I8" s="2" t="str">
+        <x:v>18.5s</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="200" customHeight="1">
-      <x:c r="A9" s="2"/>
-      <x:c r="B9" s="2"/>
-      <x:c r="C9" s="2"/>
-      <x:c r="D9" s="2"/>
-      <x:c r="E9" s="2"/>
-      <x:c r="F9" s="2"/>
-      <x:c r="G9" s="2"/>
-      <x:c r="H9" s="2"/>
-      <x:c r="I9" s="2"/>
+      <x:c r="A9" s="2" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B9" s="2" t="str">
+        <x:v>22-2B</x:v>
+      </x:c>
+      <x:c r="C9" s="2" t="str">
+        <x:v>Víctor常服；Damián常服；Escorpión常服；Escolta A常服</x:v>
+      </x:c>
+      <x:c r="D9" s="2" t="str">
+        <x:v>家主书房（夜）</x:v>
+      </x:c>
+      <x:c r="E9" s="2" t="str">
+        <x:v>黑色皮革手提箱</x:v>
+      </x:c>
+      <x:c r="F9" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+家主书房（夜），9:16竖屏。台灯侧光随Escorpión常服离开桌区逐渐减弱，门口已有走廊散光勾出侧面。
+[音轨规则]
+远层：书房内安静的室内底噪，门外动静低于台词。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
+0.2s—4.7s，@Escorpión常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Un consejo gratis: huye esta noche. Y no mires atrás.」
+4.9s—6.4s，@Víctor常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「¿Qué es ella?」
+7.1s—10.8s，@Escorpión常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Todo lo que sé… me lo enseñó ella.」
+[锚定列表]
+场景：@家主书房（夜）
+角色：@Víctor常服；@Damián常服；@Escorpión常服；@Escolta A常服
+道具：@黑色皮革手提箱
+[空间布局总览]
+书桌位于书房北部，Víctor常服在桌北侧主位面向南；Damián常服在桌东端面向西南；客位在桌南侧；门在南墙偏西，书架在西墙，通道沿桌西侧与南侧保留。开箱留在桌南沿；Escorpión常服从桌南沿西侧通道走向南门。Víctor常服坐桌北，Damián常服站桌东，Escolta A守门西侧不挡出口。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（5个硬切分镜）]
+分镜一：【景别/视角：Escorpión常服侧面中景/桌西通道 | 运镜：向南后退伴随两步，避开桌角】
+【时长】4.0s
+【构图】Escorpión常服先背好自己的双肩包，再沿桌西侧通道朝南门走；警告声低而清楚。
+【音效】门扇与门锁随实际开合发声、脚步随起停出现；台词期间压低动作声。
+【台词】@Escorpión常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Escorpión常服离开桌沿，走向门口。
+【镜头结尾·站位收束】Escorpión常服离开桌沿，走向门口。
+画面硬切到分镜二。
+分镜二：【景别/视角：Víctor常服近景/桌西侧 | 运镜：固定，保护眼神与低声发问】
+【时长】3.0s
+【构图】Víctor常服向前倾身，视线追到门口，手中雪茄停在桌面上方。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Escorpión常服的对白按本段唯一声音骨架连续发声；@Víctor常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Víctor常服仍在桌北椅位，未追出。
+【镜头结尾·站位收束】Víctor常服仍在桌北椅位，未追出。
+画面硬切到分镜三。
+分镜三：【景别/视角：门口Escorpión常服半身近景 | 运镜：从书房东南角短弧向门侧移动后落稳】
+【时长】3.5s
+【构图】Escorpión常服右手扶门，转头看向Víctor常服；唇角短暂放松后说出回应，不安排大笑。
+【音效】门扇与门锁随实际开合发声；台词期间压低动作声。
+【台词】@Escorpión常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】右手扶门，身体已朝出口。
+【镜头结尾·站位收束】右手扶门，身体已朝出口。
+画面硬切到分镜四。
+分镜四：【景别/视角：门侧中景 | 运镜：固定，门洞边界完整入画】
+【时长】3.0s
+【构图】Escorpión常服跨过门槛后回手合门；Escolta A留在门内西侧，给出通道。
+【音效】门扇与门锁随实际开合发声；台词期间压低动作声。
+【台词】@Escorpión常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Escorpión常服在门外，门合拢。
+【镜头结尾·站位收束】Escorpión常服在门外，门合拢。
+画面硬切到分镜五。
+分镜五：【景别/视角：Víctor常服与Damián常服关系中景 | 运镜：缓慢向后拉，显出开着的箱子与两人距离】
+【时长】3.0s
+【构图】Víctor常服目光留在已关闭的南门，Damián常服手指收回；开箱仍在桌面。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】Víctor常服桌北、Damián常服桌东，门关闭，箱子未移动。
+【镜头结尾·站位收束】Víctor常服桌北、Damián常服桌东，门关闭，箱子未移动。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：16.5s</x:v>
+      </x:c>
+      <x:c r="G9" s="2" t="str">
+        <x:v>Escorpión：「Un consejo gratis: huye esta noche. Y no mires atrás.」
+Víctor：「¿Qué es ella?」
+Escorpión：「Todo lo que sé… me lo enseñó ella.」</x:v>
+      </x:c>
+      <x:c r="H9" s="2" t="str">
+        <x:v>Escorpión（缓缓背上双肩包，语气冰冷）：Un consejo gratis: huye esta noche. Y no mires atrás.
+△ 镜头特写：Víctor 听完这话，原本把玩雪茄的手停住了。他身体微微前倾，双眼死死锁住 Escorpión。
+Víctor（压低声音，语气中透着一丝不易察觉的寒意）：¿Qué es ella?
+△ 镜头切到 Escorpión：他已经走到门口，扶住沉重的木门。他转过身，脸上竟然露出了一抹充满讽刺与敬畏的笑容，笑容灿烂却令人胆寒。
+Escorpión（语气坚定且崇拜）：Todo lo que sé… me lo enseñó ella.
+△ 动作特写：Escorpión 果断转身走出房间，反手将门重重关上。“砰”的一声闷响回荡在书房内。</x:v>
+      </x:c>
+      <x:c r="I9" s="2" t="str">
+        <x:v>16.5s</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="200" customHeight="1">
-      <x:c r="A10" s="2"/>
-      <x:c r="B10" s="2"/>
-      <x:c r="C10" s="2"/>
-      <x:c r="D10" s="2"/>
-      <x:c r="E10" s="2"/>
-      <x:c r="F10" s="2"/>
-      <x:c r="G10" s="2"/>
-      <x:c r="H10" s="2"/>
-      <x:c r="I10" s="2"/>
+      <x:c r="A10" s="2" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B10" s="2" t="str">
+        <x:v>22-3A</x:v>
+      </x:c>
+      <x:c r="C10" s="2" t="str">
+        <x:v>Víctor常服；Damián常服</x:v>
+      </x:c>
+      <x:c r="D10" s="2" t="str">
+        <x:v>家主书房（夜）</x:v>
+      </x:c>
+      <x:c r="E10" s="2" t="str">
+        <x:v>旧皮箱（文字设定）；泛黄法律文件</x:v>
+      </x:c>
+      <x:c r="F10" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+家主书房（夜），9:16竖屏。台灯从桌西后方斜照纸面与手背，书架间保留暗部。
+[音轨规则]
+远层：书房内安静的室内底噪，门外动静低于台词。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段无原定对白或旁白，不新增发声。
+[锚定列表]
+场景：@家主书房（夜）
+角色：@Víctor常服；@Damián常服
+道具：旧皮箱（文字设定）；@泛黄法律文件
+未带@的本段场景或物件按已授权的文字设计执行，保持下述位置、数量和状态。
+[空间布局总览]
+书桌位于书房北部，Víctor常服在桌北侧主位面向南；Damián常服在桌东端面向西南；客位在桌南侧；门在南墙偏西，书架在西墙，通道沿桌西侧与南侧保留。黑色退款箱仍在桌南沿，旧棕色皮箱将放在桌西沿，两箱不互换。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（6个硬切分镜）]
+分镜一：【景别/视角：南门与Damián常服中景 | 运镜：从门内向东轻摇，落在Damián常服停住的手】
+【时长】3.0s
+【构图】门已经关闭；Damián常服仍在桌东，望向门口后转看父亲，呼吸自然偏重但无喘鸣。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】Damián常服站位不变。
+【镜头结尾·站位收束】Damián常服站位不变。
+画面硬切到分镜二。
+分镜二：【景别/视角：Víctor常服全身中景/书桌南侧 | 运镜：沿西侧通道伴随Víctor常服走向书架】
+【时长】3.5s
+【构图】Víctor常服由椅子起身，绕桌西沿走到西墙书架，抬手从高层后方取下棕色旧皮箱。
+【音效】脚步随起停出现、箱体或扣锁的实际接触声；台词期间压低动作声。
+【台词】无台词。
+【变化】旧皮箱由Víctor常服双手托住，双脚仍在书架前。
+【镜头结尾·站位收束】旧皮箱由Víctor常服双手托住，双脚仍在书架前。
+画面硬切到分镜三。
+分镜三：【景别/视角：旧皮箱与桌沿近景 | 运镜：顺人物回程向南短移，落在桌西沿】
+【时长】3.5s
+【构图】Víctor常服沿同一通道回桌边，双手把旧箱放在桌西沿，离退款箱保留空隙。
+【音效】箱体或扣锁的实际接触声；台词期间压低动作声。
+【台词】无台词。
+【变化】棕色旧箱桌西沿，黑色退款箱桌南沿。
+【镜头结尾·站位收束】棕色旧箱桌西沿，黑色退款箱桌南沿。
+画面硬切到分镜四。
+分镜四：【景别/视角：旧箱锁扣特写 | 运镜：固定，扣锁与手指完整在焦内】
+【时长】3.0s
+【构图】Víctor常服一手稳箱体，另一手掀开生锈扣锁，再打开箱盖，露出成叠旧文件。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】旧箱打开，文件仍在箱内。
+【镜头结尾·站位收束】旧箱打开，文件仍在箱内。
+画面硬切到分镜五。
+分镜五：【景别/视角：纸张手部近景 | 运镜：从桌西侧斜上方缓推，纸面保持背向镜头】
+【时长】3.5s
+【构图】Víctor常服取出上层烧焦边缘的旧文件，翻到签名处，镜头只看纸背与焦边；文字不入画。
+【音效】纸张轻擦声；台词期间压低动作声。
+【台词】无台词。
+【变化】文件在Víctor常服手中，旧箱留桌西沿。
+【镜头结尾·站位收束】文件在Víctor常服手中，旧箱留桌西沿。
+画面硬切到分镜六。
+分镜六：【景别/视角：Víctor常服近景/桌南侧 | 运镜：固定，焦点落在视线与停住的指尖】
+【时长】3.0s
+【构图】Víctor常服读到签名后，指尖停住，眼睑略收，随后缓慢抬眼；不新增发声。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】Víctor常服手持文件，Damián常服仍在桌东观察。
+【镜头结尾·站位收束】Víctor常服手持文件，Damián常服仍在桌东观察。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：19.5s</x:v>
+      </x:c>
+      <x:c r="G10" s="2" t="str"/>
+      <x:c r="H10" s="2" t="str">
+        <x:v>22-3 家主书房（Estudio, Mansión Vargas） 夜 内
+人物：Víctor、Damián
+△ 镜头特写：大门紧闭。Damián 依然站在桌边，神情复杂地看着关闭的房门，呼吸急促。
+△ 镜头反打：Víctor 缓缓站起身。他走到巨大的书架前，神情凝重地思考了片刻，随后伸出手，从最高的一排书架后方取出了一个磨损严重的棕色老式皮箱。
+△ 动作特写：Víctor 走回书桌，将皮箱放在桌面上。箱体上的皮革有多处划痕，金属扣已经生锈。
+△ 镜头特写：Víctor 颤抖着手，费力地拨开生锈的锁扣。
+△ 镜头俯拍：箱子被打开，里面整齐地存放着几叠泛黄的旧文件。
+△ 动作特写：Víctor 翻开其中一份文件，那是多年前的合约。
+△ 画面特写：发黄的纸张上，受托人一栏赫然签着一个巨大的手写字母“W”，笔触凌厉。
+【字幕：Parte A: W】
+△ 镜头切到 Víctor：他看着那个签名，眼神中终于流露出了深层的恐惧。</x:v>
+      </x:c>
+      <x:c r="I10" s="2" t="str">
+        <x:v>19.5s</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="200" customHeight="1">
-      <x:c r="A11" s="2"/>
-      <x:c r="B11" s="2"/>
-      <x:c r="C11" s="2"/>
-      <x:c r="D11" s="2"/>
-      <x:c r="E11" s="2"/>
-      <x:c r="F11" s="2"/>
-      <x:c r="G11" s="2"/>
-      <x:c r="H11" s="2"/>
-      <x:c r="I11" s="2"/>
+      <x:c r="A11" s="2" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="B11" s="2" t="str">
+        <x:v>23-1A</x:v>
+      </x:c>
+      <x:c r="C11" s="2" t="str">
+        <x:v>Víctor常服；Damián常服</x:v>
+      </x:c>
+      <x:c r="D11" s="2" t="str">
+        <x:v>家主书房（夜）</x:v>
+      </x:c>
+      <x:c r="E11" s="2" t="str">
+        <x:v>泛黄法律文件</x:v>
+      </x:c>
+      <x:c r="F11" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+家主书房（夜），9:16竖屏。台灯斜照两人之间的纸张边缘，主位背景书架落暗。
+[音轨规则]
+远层：书房内安静的室内底噪，门外动静低于台词。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
+2.6s—7.6s，@Damián常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Ningún miembro de ninguna familia tocará, investigará ni hará daño a W.」
+9.6s—12.9s，@Damián常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Quien lo viole… lo demás se quemó.」
+13.1s—16.9s，@Víctor常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Tu abuelo la protegió hasta el día que murió.」
+[锚定列表]
+场景：@家主书房（夜）
+角色：@Víctor常服；@Damián常服
+道具：@泛黄法律文件
+[空间布局总览]
+书桌位于书房北部，Víctor常服在桌北侧主位面向南；Damián常服在桌东端面向西南；客位在桌南侧；门在南墙偏西，书架在西墙，通道沿桌西侧与南侧保留。Damián常服站桌东，双手待接烧焦残页；Víctor常服站桌西侧近主位，面向Damián常服；两箱仍在桌上原位；烧焦残页起初在Víctor常服手中，首镜交给Damián常服。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（6个硬切分镜）]
+分镜一：【景别/视角：两人手部中景/书桌南侧 | 运镜：固定，完整看见纸张交接】
+【时长】2.5s
+【构图】Víctor常服由西侧将残页递向桌东的Damián常服，两人各持一边；Damián常服夹稳后Víctor常服松指，纸面始终不朝镜头。
+【音效】纸张轻擦声；台词期间压低动作声。
+【台词】无台词。
+【变化】残页归Damián常服双手，Víctor常服双手已离纸。
+【镜头结尾·站位收束】残页归Damián常服双手，Víctor常服双手已离纸。
+画面硬切到分镜二。
+分镜二：【景别/视角：残页与Damián常服中近景/桌南侧 | 运镜：从纸背轻摇到Damián常服的脸】
+【时长】4.0s
+【构图】Damián常服低头读残页，纸面朝自己，焦边可见，画面不出现文字；他用自然低声读条款。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Damián常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】文件由Damián常服双手持住。
+【镜头结尾·站位收束】文件由Damián常服双手持住。
+画面硬切到分镜三。
+分镜三：【景别/视角：Víctor常服听者近景/桌东南侧 | 运镜：固定，视线越过纸张边缘】
+【时长】3.0s
+【构图】Damián常服读条款的声音继续；Víctor常服看着他，手仍在自己身体一侧，不提前抢纸。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Damián常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Víctor常服仍在桌西侧。
+【镜头结尾·站位收束】Víctor常服仍在桌西侧。
+画面硬切到分镜四。
+分镜四：【景别/视角：Damián常服近景/桌西南侧 | 运镜：缓推至抬眼停顿，随后落稳】
+【时长】3.5s
+【构图】Damián常服看向残页下缘的焦口，再抬眼看向Víctor常服，读出缺失部分的说明。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Damián常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Damián常服仍持残页，目光转向父亲。
+【镜头结尾·站位收束】Damián常服仍持残页，目光转向父亲。
+画面硬切到分镜五。
+分镜五：【景别/视角：两人手部中景/桌南侧 | 运镜：轻向西平移，保留交接接触区】
+【时长】4.0s
+【构图】Víctor常服伸手夹住纸张一角，Damián常服松指后Víctor常服将文件拿回；Víctor常服接话，身体不越过桌面。
+【音效】纸张轻擦声；台词期间压低动作声。
+【台词】@Víctor常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】残页转到Víctor常服手中。
+【镜头结尾·站位收束】残页转到Víctor常服手中。
+画面硬切到分镜六。
+分镜六：【景别/视角：Víctor常服侧后中景 | 运镜：沿西侧通道短移，显出书架与桌面的关系】
+【时长】3.0s
+【构图】Víctor常服转向近处书架，将残页夹入更厚文件内；Damián常服留桌东。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】残页夹入厚文件，Víctor常服站书架前。
+【镜头结尾·站位收束】残页夹入厚文件，Víctor常服站书架前。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：20s</x:v>
+      </x:c>
+      <x:c r="G11" s="2" t="str">
+        <x:v>Damián：「Ningún miembro de ninguna familia tocará, investigará ni hará daño a W.」
+Damián：「Quien lo viole… lo demás se quemó.」
+Víctor：「Tu abuelo la protegió hasta el día que murió.」</x:v>
+      </x:c>
+      <x:c r="H11" s="2" t="str">
+        <x:v>第23集
+23-1 家主书房（Estudio, Mansión Vargas） 夜 内
+人物：Víctor、Damián
+△ 镜头特写：一张边缘带有焦痕、质感粗糙的古旧羊皮纸。纸面上排列着整齐的打字机字迹，中间位置有一个醒目的手写大写字母“W”。
+△ 镜头切到 Damián：他低头盯着那张纸，眉头紧锁，神情凝重而迟疑。
+Damián（低声读出纸上的条款）：Ningún miembro de ninguna familia tocará, investigará ni hará daño a W.
+△ 镜头特写：羊皮纸的下半部分缺失，边缘呈现出被火焚烧过后的炭黑色波浪状。
+Damián（抬头看向父亲）：Quien lo viole… lo demás se quemó.
+△ 镜头反打：Víctor 站在书桌对面。他身穿黑金花纹的华丽西装，眼神中透着一股历经沧桑的严厉。他猛地从 Damián 手中夺过那张残破的文件。
+Víctor（语气威严）：Tu abuelo la protegió hasta el día que murió.
+△ 镜头全景：Víctor 转身走到书架旁，将那张残页塞进一叠更厚的文件中。他动作粗鲁，显然情绪并不平静。</x:v>
+      </x:c>
+      <x:c r="I11" s="2" t="str">
+        <x:v>20s</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="200" customHeight="1">
-      <x:c r="A12" s="2"/>
-      <x:c r="B12" s="2"/>
-      <x:c r="C12" s="2"/>
-      <x:c r="D12" s="2"/>
-      <x:c r="E12" s="2"/>
-      <x:c r="F12" s="2"/>
-      <x:c r="G12" s="2"/>
-      <x:c r="H12" s="2"/>
-      <x:c r="I12" s="2"/>
+      <x:c r="A12" s="2" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="B12" s="2" t="str">
+        <x:v>23-1B</x:v>
+      </x:c>
+      <x:c r="C12" s="2" t="str">
+        <x:v>Víctor常服；Damián常服</x:v>
+      </x:c>
+      <x:c r="D12" s="2" t="str">
+        <x:v>家主书房（夜）</x:v>
+      </x:c>
+      <x:c r="E12" s="2" t="str">
+        <x:v>泛黄法律文件；iPhone手机</x:v>
+      </x:c>
+      <x:c r="F12" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+家主书房（夜），9:16竖屏。台灯暖光照纸边；手机仅作暗色玻璃反光，不照亮整张正脸，不出现界面文字。
+[音轨规则]
+远层：书房内安静的室内底噪，门外动静低于台词。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
+0.2s—3.1s，@Víctor常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Tu abuelo también la investigó. Mira.」
+4.1s—6.5s，@Víctor常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Padres biológicos. Apostadores. Endeudados.」
+10.6s—14.7s，@Víctor常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Toda navaja tiene mango. Este es el de ella.」
+[锚定列表]
+场景：@家主书房（夜）
+角色：@Víctor常服；@Damián常服
+道具：@泛黄法律文件；@iPhone手机
+[空间布局总览]
+书桌位于书房北部，Víctor常服在桌北侧主位面向南；Damián常服在桌东端面向西南；客位在桌南侧；门在南墙偏西，书架在西墙，通道沿桌西侧与南侧保留。Víctor常服站西墙书架旁，厚文件在手；Damián常服站桌东，手机放在桌北侧主位附近。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（5个硬切分镜）]
+分镜一：【景别/视角：Víctor常服侧面中近景 | 运镜：沿书架向右短移，落在打开的另一页背面】
+【时长】4.0s
+【构图】Víctor常服翻开调查页，指向面向Damián常服的纸面，示意他看；页面文字背向镜头。
+【音效】纸张轻擦声；台词期间压低动作声。
+【台词】@Víctor常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】厚文件仍在Víctor常服双手之间。
+【镜头结尾·站位收束】厚文件仍在Víctor常服双手之间。
+画面硬切到分镜二。
+分镜二：【景别/视角：Damián常服过肩/前景Víctor常服手与纸边 | 运镜：固定，焦点落在Damián常服脸上】
+【时长】3.5s
+【构图】Víctor常服继续读出调查结论；Damián常服听着，目光从纸边移到父亲，不新增惊呼。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Víctor常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Damián常服站桌东，文件未再交手。
+【镜头结尾·站位收束】Damián常服站桌东，文件未再交手。
+画面硬切到分镜三。
+分镜三：【景别/视角：手部中近景/桌北偏西 | 运镜：向桌面轻摇后固定】
+【时长】3.0s
+【构图】Víctor常服把厚文件放在桌北侧，再以右手拿起iPhone；空出的左手停在桌沿。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】文件已放桌；手机在Víctor常服右手。
+【镜头结尾·站位收束】文件已放桌；手机在Víctor常服右手。
+画面硬切到分镜四。
+分镜四：【景别/视角：Víctor常服侧面近景 | 运镜：从桌西侧缓推，最后落在他向Damián常服抬起的视线】
+【时长】4.0s
+【构图】Víctor常服看一眼背向镜头的手机，抬眼说明如何对付Vera常服；语气压低，句尾收住。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Víctor常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】手机留在右手，左手扶桌，Damián常服仍站桌东。
+【镜头结尾·站位收束】手机留在右手，左手扶桌，Damián常服仍站桌东。
+画面硬切到分镜五。
+分镜五：【景别/视角：Damián常服近景/桌南侧 | 运镜：固定，保持与上一镜同侧视线轴】
+【时长】2.0s
+【构图】Víctor常服的声音延续到完整句尾，Damián常服听完再低眼看桌面文件，身体仍在桌东。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Víctor常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Damián常服站桌东，Víctor常服站桌西侧，手机仍在Víctor常服右手。
+【镜头结尾·站位收束】Damián常服站桌东，Víctor常服站桌西侧，手机仍在Víctor常服右手。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：16.5s</x:v>
+      </x:c>
+      <x:c r="G12" s="2" t="str">
+        <x:v>Víctor：「Tu abuelo también la investigó. Mira.」
+Víctor：「Padres biológicos. Apostadores. Endeudados.」
+Víctor：「Toda navaja tiene mango. Este es el de ella.」</x:v>
+      </x:c>
+      <x:c r="H12" s="2" t="str">
+        <x:v>△ 镜头切到 Víctor 的手部特写：他翻开另一份泛黄的文件，指甲划过纸面，指向一行字迹。
+Víctor：Tu abuelo también la investigó. Mira.
+△ 镜头特写：文件上清晰地写着“Padres biológicos. Apostadores. Endeudados.”
+Víctor：Padres biológicos. Apostadores. Endeudados.
+△ 镜头反打：Damián 站在原地，看着父亲展示的调查结果，眼神中闪过一丝震惊。
+△ 动作特写：Víctor 拿起桌上的 iPhone 手机，屏幕发出的冷光映照在他布满皱纹的脸上。他滑动屏幕，神情冰冷。
+Víctor（语气阴沉）：Toda navaja tiene mango. Este es el de ella.</x:v>
+      </x:c>
+      <x:c r="I12" s="2" t="str">
+        <x:v>16.5s</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="200" customHeight="1">
-      <x:c r="A13" s="2"/>
-      <x:c r="B13" s="2"/>
-      <x:c r="C13" s="2"/>
-      <x:c r="D13" s="2"/>
-      <x:c r="E13" s="2"/>
-      <x:c r="F13" s="2"/>
-      <x:c r="G13" s="2"/>
-      <x:c r="H13" s="2"/>
-      <x:c r="I13" s="2"/>
+      <x:c r="A13" s="2" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="B13" s="2" t="str">
+        <x:v>23-2A</x:v>
+      </x:c>
+      <x:c r="C13" s="2" t="str">
+        <x:v>Vera常服；Renata常服</x:v>
+      </x:c>
+      <x:c r="D13" s="2" t="str">
+        <x:v>高层公寓门口与走廊（文字设定·夜）</x:v>
+      </x:c>
+      <x:c r="E13" s="2" t="str">
+        <x:v>黄色牛皮纸线索信封（文字设定）</x:v>
+      </x:c>
+      <x:c r="F13" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+高层公寓门口与走廊（文字设定·夜），9:16竖屏。走廊顶灯侧照Renata常服，客厅北侧实用灯从门内斜透；门开后形成有来源的明暗交界。
+[音轨规则]
+远层：公寓外远处车流低声，室内维持安静。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段无原定对白或旁白，不新增发声。
+[锚定列表]
+场景：高层公寓门口与走廊（文字设定·夜）
+角色：@Vera常服；@Renata常服
+道具：黄色牛皮纸线索信封（文字设定）
+未带@的本段场景或物件按已授权的文字设计执行，保持下述位置、数量和状态。
+[空间布局总览]
+公寓室内为文字确定的连续空间：入口门在西墙，向室内开启；入口向东进入客厅，茶几在中部、沙发在其北侧；东侧为临街落地窗，东北转角窄玻璃面朝相邻楼；阳台移门在南侧。本文方位为世界参照，不随反打改变。Vera常服从东窗走向西门；Renata常服在门外南侧抱着黄色信封，左脸淤伤和湿发是本场持续状态。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（4个硬切分镜）]
+分镜一：【景别/视角：客厅纵深中景/茶几南侧 | 运镜：随Vera常服由东向西短距离跟随】
+【时长】3.0s
+【构图】Vera常服听见门外动静，从东窗沿茶几南侧通道走向西门，双手空着。
+【音效】门扇与门锁随实际开合发声、脚步随起停出现；台词期间压低动作声。
+【台词】无台词。
+【变化】Vera常服停在门内。
+【镜头结尾·站位收束】Vera常服停在门内。
+画面硬切到分镜二。
+分镜二：【景别/视角：猫眼主观近景 | 运镜：固定在已建立的门内眼位】
+【时长】3.0s
+【构图】Renata常服站门外，湿发贴脸，黄色信封抱在胸前；淤伤在左脸，未换边。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】Renata常服仍在门外，信封未递出。
+【镜头结尾·站位收束】Renata常服仍在门外，信封未递出。
+画面硬切到分镜三。
+分镜三：【景别/视角：门内侧面中景 | 运镜：轻向后让开，完整看见门向室内开启】
+【时长】3.0s
+【构图】Vera常服转动门把，将门向内拉开，身体退到门扇北侧留出入口。
+【音效】门扇与门锁随实际开合发声；台词期间压低动作声。
+【台词】无台词。
+【变化】门打开，Vera常服在门内北侧，Renata常服门外。
+【镜头结尾·站位收束】门打开，Vera常服在门内北侧，Renata常服门外。
+画面硬切到分镜四。
+分镜四：【景别/视角：Renata常服近景/从门内朝外 | 运镜：从门框边短移，露出Renata常服受伤的左脸】
+【时长】3.5s
+【构图】Renata常服看到Vera常服后肩部略松，视线落在她脸上，嘴唇短暂压合；已有泪水沿脸颊自然滑落，不额外抽气尖叫。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】Renata常服抱着信封，仍未跨门槛。
+【镜头结尾·站位收束】Renata常服抱着信封，仍未跨门槛。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：12.5s</x:v>
+      </x:c>
+      <x:c r="G13" s="2" t="str"/>
+      <x:c r="H13" s="2" t="str">
+        <x:v>23-2 高层公寓/走廊 夜 内
+人物：Vera、Renata
+△ 镜头全景：Vera 独自站在落地窗前。窗外是繁华的城市夜景，五彩斑斓的灯光在雨幕中显得有些模糊。
+△ 镜头切到公寓门口：Vera 披着米色风衣，长发盘在脑后。她听到门外的动静，神情警觉地走向房门。
+△ 镜头特写（猫眼视角）：一个浑身湿透的年轻女孩（Renata）站在门外。她穿着米白色的针织毛衣，长发湿漉漉地贴在脸颊上。
+△ 镜头近景：Renata 的左半边脸高高肿起，伴有大片紫红色的淤青，眼眶通红，眼神中充满了极度的惊恐与无助。她怀里死死抱着一个黄色的牛皮纸信封。
+△ 动作特写：Vera 猛地拉开房门。
+△ 镜头切到 Renata：她看到 Vera 后，原本紧绷的肩膀瞬间垮了下来，眼泪夺眶而出，嘴角剧烈颤抖，露出了一个既委屈又带着一丝得救后的惨淡笑容。</x:v>
+      </x:c>
+      <x:c r="I13" s="2" t="str">
+        <x:v>12.5s</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="200" customHeight="1">
-      <x:c r="A14" s="2"/>
-      <x:c r="B14" s="2"/>
-      <x:c r="C14" s="2"/>
-      <x:c r="D14" s="2"/>
-      <x:c r="E14" s="2"/>
-      <x:c r="F14" s="2"/>
-      <x:c r="G14" s="2"/>
-      <x:c r="H14" s="2"/>
-      <x:c r="I14" s="2"/>
+      <x:c r="A14" s="2" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="B14" s="2" t="str">
+        <x:v>23-2B</x:v>
+      </x:c>
+      <x:c r="C14" s="2" t="str">
+        <x:v>Vera常服；Renata常服</x:v>
+      </x:c>
+      <x:c r="D14" s="2" t="str">
+        <x:v>高层公寓门口与客厅（文字设定·夜）</x:v>
+      </x:c>
+      <x:c r="E14" s="2" t="str">
+        <x:v>黄色牛皮纸线索信封（文字设定）</x:v>
+      </x:c>
+      <x:c r="F14" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+高层公寓门口与客厅（文字设定·夜），9:16竖屏。走廊顶灯从Renata常服侧上方照入，室内暖光落在Vera常服肩部，两人面部曝光不随切镜跳变。
+[音轨规则]
+远层：公寓外远处车流低声，室内维持安静。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
+0.2s—4.3s，@Renata常服（对白，声音带疲惫与轻微不稳，词句完整，不加入抽泣语词）：「La casa del lago. La caja fuerte del abuelo.」
+4.5s—9.3s，@Renata常服（对白，声音带疲惫与轻微不稳，词句完整，不加入抽泣语词）：「Lo agarré y corrí. Mi hermano me persiguió. No volteé.」
+[锚定列表]
+场景：高层公寓门口与客厅（文字设定·夜）
+角色：@Vera常服；@Renata常服
+道具：黄色牛皮纸线索信封（文字设定）
+未带@的本段场景或物件按已授权的文字设计执行，保持下述位置、数量和状态。
+[空间布局总览]
+公寓室内为文字确定的连续空间：入口门在西墙，向室内开启；入口向东进入客厅，茶几在中部、沙发在其北侧；东侧为临街落地窗，东北转角窄玻璃面朝相邻楼；阳台移门在南侧。本文方位为世界参照，不随反打改变。门已向室内开启。Vera常服在门内北侧，Renata常服在门外，左脸淤伤，黄色信封起初在Renata常服双手。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（4个硬切分镜）]
+分镜一：【景别/视角：Renata常服中近景/门内向外 | 运镜：固定，信封和受伤左脸同处可读范围】
+【时长】4.0s
+【构图】Renata常服把信封递向Vera常服，声音低且略有停顿；目光仍停在姐姐脸上。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Renata常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】信封两人各持一端，尚未松手。
+【镜头结尾·站位收束】信封两人各持一端，尚未松手。
+画面硬切到分镜二。
+分镜二：【景别/视角：交接近景/门内南侧 | 运镜：轻向右平移，完整保留手指接触】
+【时长】3.0s
+【构图】Vera常服右手托住信封下缘，Renata常服确认她夹稳后松开双手；Renata常服继续叙述逃出的经过。
+【音效】封口与纸张轻擦声；台词期间压低动作声。
+【台词】@Renata常服的对白按本段唯一声音骨架连续发声；@Renata常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】信封归Vera常服右手。
+【镜头结尾·站位收束】信封归Vera常服右手。
+画面硬切到分镜三。
+分镜三：【景别/视角：Vera常服听者近景 | 运镜：从Renata常服肩侧固定观察Vera常服】
+【时长】3.0s
+【构图】Renata常服的声音继续，Vera常服看向她左脸伤处，眉部轻收；右手持信封不再操作。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Renata常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Vera常服左手抬起，停在妹妹左侧脸旁。
+【镜头结尾·站位收束】Vera常服左手抬起，停在妹妹左侧脸旁。
+画面硬切到分镜四。
+分镜四：【景别/视角：双人侧面中景/门内 | 运镜：沿门内通道向东缓退】
+【时长】3.5s
+【构图】Vera常服左指轻触Renata常服伤处后移至其肩背，右手将信封收在身侧，带Renata常服跨门槛进入客厅。
+【音效】门扇与门锁随实际开合发声、封口与纸张轻擦声；台词期间压低动作声。
+【台词】无台词。
+【变化】两人均在室内，Vera常服左手扶Renata常服肩，右手持信封。
+【镜头结尾·站位收束】两人均在室内，Vera常服左手扶Renata常服肩，右手持信封。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：13.5s</x:v>
+      </x:c>
+      <x:c r="G14" s="2" t="str">
+        <x:v>Renata：「La casa del lago. La caja fuerte del abuelo.」
+Renata：「Lo agarré y corrí. Mi hermano me persiguió. No volteé.」</x:v>
+      </x:c>
+      <x:c r="H14" s="2" t="str">
+        <x:v>Renata（抽泣着，将信封递向 Vera）：La casa del lago. La caja fuerte del abuelo.
+△ 镜头切换：Vera 伸出手，动作轻柔地接过信封。
+Renata（语速极快，因恐惧而语无伦次）：Lo agarré y corrí. Mi hermano me persiguió. No volteé.
+△ 镜头近景：Vera 看着 Renata 脸上的伤，眼神瞬间变得冰冷而愤怒。她伸出手，指尖轻触 Renata 脸上的淤青。
+△ 镜头全景：Vera 搂住 Renata 的肩膀，带着她走进房间。</x:v>
+      </x:c>
+      <x:c r="I14" s="2" t="str">
+        <x:v>13.5s</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="200" customHeight="1">
-      <x:c r="A15" s="2"/>
-      <x:c r="B15" s="2"/>
-      <x:c r="C15" s="2"/>
-      <x:c r="D15" s="2"/>
-      <x:c r="E15" s="2"/>
-      <x:c r="F15" s="2"/>
-      <x:c r="G15" s="2"/>
-      <x:c r="H15" s="2"/>
-      <x:c r="I15" s="2"/>
+      <x:c r="A15" s="2" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="B15" s="2" t="str">
+        <x:v>23-3A</x:v>
+      </x:c>
+      <x:c r="C15" s="2" t="str">
+        <x:v>Vera常服；Renata常服；Emiliano常服</x:v>
+      </x:c>
+      <x:c r="D15" s="2" t="str">
+        <x:v>高层公寓客厅（夜）</x:v>
+      </x:c>
+      <x:c r="E15" s="2" t="str">
+        <x:v>黄色牛皮纸线索信封（文字设定）；银色拉杆箱（文字设定）；深绿色薄大衣（文字设定）</x:v>
+      </x:c>
+      <x:c r="F15" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+高层公寓客厅（夜），9:16竖屏。客厅落地灯从沙发北后方侧照，门口走廊散光随开门出现，东窗为冷夜色。
+[音轨规则]
+远层：公寓外远处车流低声，室内维持安静。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
+3.1s—4.2s，@Emiliano常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「¿Es tuya?」
+6.1s—7.2s，@Vera常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Mi hermana.」
+[锚定列表]
+场景：@高层公寓客厅（夜）
+角色：@Vera常服；@Renata常服；@Emiliano常服
+道具：黄色牛皮纸线索信封（文字设定）；银色拉杆箱（文字设定）；深绿色薄大衣（文字设定）
+未带@的本段场景或物件按已授权的文字设计执行，保持下述位置、数量和状态。
+[空间布局总览]
+公寓室内为文字确定的连续空间：入口门在西墙，向室内开启；入口向东进入客厅，茶几在中部、沙发在其北侧；东侧为临街落地窗，东北转角窄玻璃面朝相邻楼；阳台移门在南侧。本文方位为世界参照，不随反打改变。Renata常服坐北侧单人沙发，怀抱靠枕；Vera常服在茶几西侧，信封将放在桌面；Emiliano常服由西门进入，手提银色拉杆箱。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（6个硬切分镜）]
+分镜一：【景别/视角：客厅中全景/南侧 | 运镜：向西短移显出入口与沙发】
+【时长】3.0s
+【构图】Renata常服坐沙发抱着靠枕，Vera常服把信封放在茶几西沿；西门推开，Emiliano常服先入门后把拉杆箱轮落地。
+【音效】门扇与门锁随实际开合发声、封口与纸张轻擦声；台词期间压低动作声。
+【台词】无台词。
+【变化】信封在茶几，Emiliano常服与箱子在入口内。
+【镜头结尾·站位收束】信封在茶几，Emiliano常服与箱子在入口内。
+画面硬切到分镜二。
+分镜二：【景别/视角：Emiliano常服中近景 | 运镜：沿入口至茶几的西侧通道伴随两步】
+【时长】3.0s
+【构图】Emiliano常服看向沙发上的Renata常服，停在Vera常服西侧，用一句短问句确认关系。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Emiliano常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Emiliano常服站茶几西侧偏门口，箱在右手边。
+【镜头结尾·站位收束】Emiliano常服站茶几西侧偏门口，箱在右手边。
+画面硬切到分镜三。
+分镜三：【景别/视角：Vera常服中近景/沙发侧反打 | 运镜：固定，以Renata常服模糊肩线建立关系】
+【时长】3.0s
+【构图】Vera常服看向Emiliano常服，直接回答，未离开妹妹身边。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Vera常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Vera常服站茶几与沙发之间。
+【镜头结尾·站位收束】Vera常服站茶几与沙发之间。
+画面硬切到分镜四。
+分镜四：【景别/视角：拉杆箱及双人中景 | 运镜：轻向后拉，保留箱轮与脚下路径】
+【时长】3.0s
+【构图】Emiliano常服将箱子推到Vera常服身旁的空地，松开拉杆，再向门口退开；箱子不滑进沙发或桌下。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】银箱停在茶几西侧空地，Emiliano常服向西门离开。
+【镜头结尾·站位收束】银箱停在茶几西侧空地，Emiliano常服向西门离开。
+画面硬切到分镜五。
+分镜五：【景别/视角：门口至衣凳侧面中景 | 运镜：镜头留在客厅，随Vera常服向北轻摇】
+【时长】3.0s
+【构图】Emiliano常服退出并带上门；Vera常服到沙发旁衣凳拿起深绿色薄大衣，双手提住肩部。
+【音效】门扇与门锁随实际开合发声；台词期间压低动作声。
+【台词】无台词。
+【变化】西门关闭，薄大衣在Vera常服双手。
+【镜头结尾·站位收束】西门关闭，薄大衣在Vera常服双手。
+画面硬切到分镜六。
+分镜六：【景别/视角：姐妹关系近景/沙发西侧 | 运镜：缓慢靠近，落在披衣后两人的视线高度】
+【时长】3.5s
+【构图】Vera常服把大衣披在Renata常服肩上，手掌离开后衣料自行下垂；她微俯身看妹妹，不堆叠吸气与抿嘴。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】Renata常服仍坐北侧沙发，衣服披在肩，Vera常服站其西侧。
+【镜头结尾·站位收束】Renata常服仍坐北侧沙发，衣服披在肩，Vera常服站其西侧。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：18.5s</x:v>
+      </x:c>
+      <x:c r="G15" s="2" t="str">
+        <x:v>Emiliano：「¿Es tuya?」
+Vera：「Mi hermana.」</x:v>
+      </x:c>
+      <x:c r="H15" s="2" t="str">
+        <x:v>23-3 高层公寓客厅 夜 内
+人物：Vera、Renata、Emiliano
+△ 镜头中景：Renata 坐在单人沙发上，怀里紧紧抱着一个靠枕，身体微微蜷缩，低着头，显得惊魂未定。
+△ 动作特写：Vera 将那个牛皮纸信封放在茶几上，发出一声轻响。
+△ 镜头切换：房门再次被推开。Emiliano 穿着整齐的黑色西装，手里拎着一个银色的拉杆箱走了进来。他神情从容，看向 Vera。
+Emiliano（看向沙发上的 Renata）：¿Es tuya?
+△ 动作特写：Emiliano 将行李箱推向 Vera，金属轮在木地板上发出轻微的摩擦声。
+Vera（语气平静）：Mi hermana.
+△ 镜头切到 Emiliano：他看了一眼受伤的 Renata，微微点头，没有多问，转身退出房间并带上了门。
+△ 镜头全景：Vera 走到一旁的凳子旁，拎起一件深绿色的薄大衣。
+△ 动作特写：Vera 走到沙发旁，将大衣轻轻披在 Renata 的肩膀上。
+△ 镜头切到 Vera 的脸部特写：她微微低头，注视着受惊的妹妹，眼神中原本的冷酷逐渐被一种坚定的守护感所取代。</x:v>
+      </x:c>
+      <x:c r="I15" s="2" t="str">
+        <x:v>18.5s</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="200" customHeight="1">
-      <x:c r="A16" s="2"/>
-      <x:c r="B16" s="2"/>
-      <x:c r="C16" s="2"/>
-      <x:c r="D16" s="2"/>
-      <x:c r="E16" s="2"/>
-      <x:c r="F16" s="2"/>
-      <x:c r="G16" s="2"/>
-      <x:c r="H16" s="2"/>
-      <x:c r="I16" s="2"/>
+      <x:c r="A16" s="2" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="B16" s="2" t="str">
+        <x:v>24-1A</x:v>
+      </x:c>
+      <x:c r="C16" s="2" t="str">
+        <x:v>Vera常服；Renata常服</x:v>
+      </x:c>
+      <x:c r="D16" s="2" t="str">
+        <x:v>高层公寓客厅（夜）</x:v>
+      </x:c>
+      <x:c r="E16" s="2" t="str">
+        <x:v>黄色牛皮纸线索信封（文字设定）；泛黄法律文件；线索信件（文字设定）</x:v>
+      </x:c>
+      <x:c r="F16" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+高层公寓客厅（夜），9:16竖屏。北侧落地灯斜照茶几，东窗城市光形成远层冷色；睡着的Renata常服保持半暗可辨轮廓。
+[音轨规则]
+远层：公寓外远处车流低声，室内维持安静。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段无原定对白或旁白，不新增发声。
+[锚定列表]
+场景：@高层公寓客厅（夜）
+角色：@Vera常服；@Renata常服
+道具：黄色牛皮纸线索信封（文字设定）；@泛黄法律文件；线索信件（文字设定）
+未带@的本段场景或物件按已授权的文字设计执行，保持下述位置、数量和状态。
+[空间布局总览]
+公寓室内为文字确定的连续空间：入口门在西墙，向室内开启；入口向东进入客厅，茶几在中部、沙发在其北侧；东侧为临街落地窗，东北转角窄玻璃面朝相邻楼；阳台移门在南侧。本文方位为世界参照，不随反打改变。Vera常服坐茶几西侧地毯上，Renata常服在北侧沙发睡着，身上盖薄毯；信封在茶几西沿，文件起初在信封内。Vera常服的米色风衣此刻暂搭在沙发旁衣凳上，外套仍属原人物资产，未新增第二件。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（6个硬切分镜）]
+分镜一：【景别/视角：公寓中全景/西南角 | 运镜：沿沙发前空道向东轻移，建立主次层】
+【时长】3.0s
+【构图】前景茶几与Vera常服，中景沙发Renata常服，远景东窗；Vera常服坐稳后将黄色信封拉近。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】Vera常服在地毯，Renata常服睡在沙发，信封到桌西沿。
+【镜头结尾·站位收束】Vera常服在地毯，Renata常服睡在沙发，信封到桌西沿。
+画面硬切到分镜二。
+分镜二：【景别/视角：手部近景/茶几西南角 | 运镜：固定，信封扣线与双手在焦内】
+【时长】3.0s
+【构图】Vera常服解开白色扣线，左手稳袋，右手抽出整叠文件。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】文件已离袋，信封开口朝西。
+【镜头结尾·站位收束】文件已离袋，信封开口朝西。
+画面硬切到分镜三。
+分镜三：【景别/视角：旧文件近景 | 运镜：从纸张背面向焦边轻推，避免拍到字面】
+【时长】3.0s
+【构图】她将烧焦边缘的文件铺在茶几上，指尖停在自己看到的签名位置；镜头只见纸背、焦边与她停住的手。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】旧文件平放，字面不对镜头。
+【镜头结尾·站位收束】旧文件平放，字面不对镜头。
+画面硬切到分镜四。
+分镜四：【景别/视角：Vera常服侧面近景/茶几南侧 | 运镜：固定，视线与纸边同处画面】
+【时长】3.0s
+【构图】Vera常服细看旧文件，眉部向中间轻收，目光在纸面停住。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】她仍坐地毯，未发声。
+【镜头结尾·站位收束】她仍坐地毯，未发声。
+画面硬切到分镜五。
+分镜五：【景别/视角：信件与手部近景 | 运镜：沿桌边向北小幅平移】
+【时长】3.0s
+【构图】Vera常服翻至白色信件，纸面以侧缘朝镜头；阅读由视线和翻页动作表达，画面不出现任何字迹。
+【音效】纸张轻擦声；台词期间压低动作声。
+【台词】无台词。
+【变化】白色信件在旧文件上方，信封留桌西沿。
+【镜头结尾·站位收束】白色信件在旧文件上方，信封留桌西沿。
+画面硬切到分镜六。
+分镜六：【景别/视角：Vera常服与沙发纵深中景 | 运镜：从低位轻抬，落在她望向窗外的侧脸】
+【时长】3.5s
+【构图】Vera常服读完停住，目光转向东窗，唇部轻合后自然放松；Renata常服仍睡在后方。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】Vera常服保持坐姿，所有文件留在茶几。
+【镜头结尾·站位收束】Vera常服保持坐姿，所有文件留在茶几。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：18.5s</x:v>
+      </x:c>
+      <x:c r="G16" s="2" t="str"/>
+      <x:c r="H16" s="2" t="str">
+        <x:v>第24集
+24-1 高层公寓/客厅 夜 内
+人物：Vera、Renata
+△ 画面远景：巨大的落地窗外，改革大道夜景璀璨，蓝色与红色的霓虹灯火交织在雨后的夜幕中。室内灯光柔和，Vera 坐在茶几前的地毯上，正低头处理桌上的物件。Renata 蜷缩在后方的沙发上，似乎已经沉沉睡去，身上盖着一件浅色的薄毯。
+△ 动作特写：Vera 的双手出现在镜头中，她正在拆开那个黄色的牛皮纸信封。信封的封口处有一个白色的圆形扣线锁。
+△ 镜头近景：Vera 熟练地绕开细绳，打开封口。她的动作缓慢而专注，指尖在牛皮纸上轻轻摩擦。
+△ 动作特写：Vera 将手伸进信封内部，从中抽出叠放整齐的文件。最上面的一页泛黄且带有明显的褶皱，边缘有烧焦的痕迹。
+△ 镜头切换：Vera 将文件平铺在深色的木质茶几上。镜头扫过文件内容，上面有旧式官方文头的字样，中间是一个凌厉的手写签名。
+△ 画面特写：镜头聚焦在签名处。那是用钢笔书写的“G. Paredes”，字迹苍劲有力，且带有一丝独特的连笔风格。
+△ 镜头反打：Vera 坐在地毯上，目光紧紧锁住那份文件。她的神情严肃，眉头微微蹙起，似乎在从这些陈旧的字迹中寻找某种关键的线索。
+△ 动作特写：Vera 翻开下一页。这是一张洁白的现代纸张，上面有用钢笔书写的西班牙文手写信，字迹工整且富有美感。
+△ 画面特写：镜头扫过信件正文。
+【字幕：Todo quedó limpio. La niña está a salvo. El seguro está por pagarse.】
+△ 镜头切到 Vera：她读完信件，眼神中闪过一丝复杂的情绪，呼吸变得有些急促。她抬头看向落地窗，玻璃上倒映着她清冷而深沉的面孔。</x:v>
+      </x:c>
+      <x:c r="I16" s="2" t="str">
+        <x:v>18.5s</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="200" customHeight="1">
-      <x:c r="A17" s="2"/>
-      <x:c r="B17" s="2"/>
-      <x:c r="C17" s="2"/>
-      <x:c r="D17" s="2"/>
-      <x:c r="E17" s="2"/>
-      <x:c r="F17" s="2"/>
-      <x:c r="G17" s="2"/>
-      <x:c r="H17" s="2"/>
-      <x:c r="I17" s="2"/>
+      <x:c r="A17" s="2" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="B17" s="2" t="str">
+        <x:v>24-2A</x:v>
+      </x:c>
+      <x:c r="C17" s="2" t="str">
+        <x:v>Vera常服；Renata常服</x:v>
+      </x:c>
+      <x:c r="D17" s="2" t="str">
+        <x:v>高层公寓客厅（夜）</x:v>
+      </x:c>
+      <x:c r="E17" s="2" t="str">
+        <x:v>iPhone手机；米色风衣</x:v>
+      </x:c>
+      <x:c r="F17" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+高层公寓客厅（夜），9:16竖屏。桌边实用灯为侧光，手机屏面偏离镜头，亮度不作为正面美化光。
+[音轨规则]
+远层：公寓外远处车流低声，室内维持安静。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段无原定对白或旁白，不新增发声。
+[锚定列表]
+场景：@高层公寓客厅（夜）
+角色：@Vera常服；@Renata常服
+道具：@iPhone手机；@米色风衣
+[空间布局总览]
+公寓室内为文字确定的连续空间：入口门在西墙，向室内开启；入口向东进入客厅，茶几在中部、沙发在其北侧；东侧为临街落地窗，东北转角窄玻璃面朝相邻楼；阳台移门在南侧。本文方位为世界参照，不随反打改变。Vera常服从茶几西侧地毯起身，Renata常服仍在北侧沙发熟睡。手机在茶几西南角，风衣在衣凳上；南侧移门通阳台。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（4个硬切分镜）]
+分镜一：【景别/视角：桌面手机近景/南侧 | 运镜：固定，屏幕斜背镜头】
+【时长】3.0s
+【构图】iPhone在茶几上振动，光面只露无字反光；Vera常服右手伸向手机。
+【音效】手指与机身接触的低弱摩擦声；台词期间压低动作声。
+【台词】无台词。
+【变化】手机仍在桌上，指尖已到边缘。
+【镜头结尾·站位收束】手机仍在桌上，指尖已到边缘。
+画面硬切到分镜二。
+分镜二：【景别/视角：Vera常服侧面中景 | 运镜：向上摇随她拿起手机，落在看向沙发的视线】
+【时长】3.0s
+【构图】Vera常服拿起手机，先看熟睡的Renata常服，左手撑地准备起身。
+【音效】手指与机身接触的低弱摩擦声；台词期间压低动作声。
+【台词】无台词。
+【变化】手机在右手，左手撑地。
+【镜头结尾·站位收束】手机在右手，左手撑地。
+画面硬切到分镜三。
+分镜三：【景别/视角：客厅至阳台关系中景 | 运镜：沿茶几南侧向南伴随，路径始终在室内】
+【时长】3.5s
+【构图】Vera常服借左手支撑起身，拿起米色风衣披好，走到南侧玻璃移门；手机仍在右手。
+【音效】门扇与门锁随实际开合发声、脚步随起停出现；台词期间压低动作声。
+【台词】无台词。
+【变化】Vera常服在移门内，左手空出。
+【镜头结尾·站位收束】Vera常服在移门内，左手空出。
+画面硬切到分镜四。
+分镜四：【景别/视角：移门侧面全身中景 | 运镜：在门内侧固定，让门扇边界清楚】
+【时长】3.5s
+【构图】她左手滑开玻璃门，跨过门槛，转身用左手合上移门；相机始终停在室内。
+【音效】门扇与门锁随实际开合发声；台词期间压低动作声。
+【台词】无台词。
+【变化】Vera常服已到阳台；移门关上，Renata常服留室内。
+【镜头结尾·站位收束】Vera常服已到阳台；移门关上，Renata常服留室内。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：13s</x:v>
+      </x:c>
+      <x:c r="G17" s="2" t="str"/>
+      <x:c r="H17" s="2" t="str">
+        <x:v>24-2 高层公寓/客厅 夜 内
+人物：Vera、Renata
+△ 镜头近景：放在茶几上的 iPhone 手机突然剧烈震动起来，屏幕亮起，显示来电人。
+【字幕：Veredicto】
+△ 动作特写：手机在光滑的木质桌面上轻微位移。Vera 的手伸向手机。
+△ 镜头切换：Vera 拿起手机，并没有立刻接听，而是看了一眼后方沙发上熟睡的 Renata。Renata 呼吸均匀，双手交叠在胸前，依然沉浸在睡梦中。
+△ 动作特写：Vera 迅速起身，动作轻盈且敏捷，她随手抓起放在一旁的米色风衣，大步走向阳台。
+△ 镜头跟随：Vera 推开通往阳台的玻璃移门，身后的书架排满书籍。她走出去后，反手将门拉上，发出一声轻微的咔哒声。</x:v>
+      </x:c>
+      <x:c r="I17" s="2" t="str">
+        <x:v>13s</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="200" customHeight="1">
-      <x:c r="A18" s="2"/>
-      <x:c r="B18" s="2"/>
-      <x:c r="C18" s="2"/>
-      <x:c r="D18" s="2"/>
-      <x:c r="E18" s="2"/>
-      <x:c r="F18" s="2"/>
-      <x:c r="G18" s="2"/>
-      <x:c r="H18" s="2"/>
-      <x:c r="I18" s="2"/>
+      <x:c r="A18" s="2" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="B18" s="2" t="str">
+        <x:v>24-3A</x:v>
+      </x:c>
+      <x:c r="C18" s="2" t="str">
+        <x:v>Vera常服；Don Ernesto常服</x:v>
+      </x:c>
+      <x:c r="D18" s="2" t="str">
+        <x:v>高层公寓阳台</x:v>
+      </x:c>
+      <x:c r="E18" s="2" t="str">
+        <x:v>iPhone手机</x:v>
+      </x:c>
+      <x:c r="F18" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+高层公寓阳台，9:16竖屏。室内落地灯经玻璃从左后方透出暖光，城市散光形成右侧冷轮廓；不虚构面前灯具。
+[音轨规则]
+远层：公寓外远处车流低声，室内维持安静。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
+3.1s—5.6s，@Don Ernesto常服（VO，电话VO，低沉沙哑，Vera常服只听，不做该句口型）：「Los encontré. A sus «papás».」
+6.6s—12.7s，@Don Ernesto常服（VO，电话VO，低沉沙哑，Vera常服只听，不做该句口型）：「Pareja de apostadores. Hace tres días les cayeron quinientos mil pesos en la cuenta.」
+13.6s—14.7s，@Vera常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「¿De quién?」
+16.6s—20.3s，@Don Ernesto常服（VO，电话VO，低沉沙哑，Vera常服只听，不做该句口型）：「De una empresa fantasma. De la familia Vargas.」
+[锚定列表]
+场景：@高层公寓阳台
+角色：@Vera常服；@Don Ernesto常服
+道具：@iPhone手机
+[空间布局总览]
+公寓室内为文字确定的连续空间：入口门在西墙，向室内开启；入口向东进入客厅，茶几在中部、沙发在其北侧；东侧为临街落地窗，东北转角窄玻璃面朝相邻楼；阳台移门在南侧。本文方位为世界参照，不随反打改变。Vera常服在南侧阳台栏杆内侧，面向城市；Don Ernesto常服只作为电话VO，不入画、不设计其地点。右手持手机，左手可扶栏杆。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（7个硬切分镜）]
+分镜一：【景别/视角：阳台侧后中景 | 运镜：沿阳台门外合法步道短移，停在Vera常服侧后】
+【时长】3.0s
+【构图】Vera常服右拇指接通，再将手机举至右耳；左手落在栏杆内侧。
+【音效】手指与机身接触的低弱摩擦声；台词期间压低动作声。
+【台词】无台词。
+【变化】手机贴右耳，双脚停在栏杆前。
+【镜头结尾·站位收束】手机贴右耳，双脚停在栏杆前。
+画面硬切到分镜二。
+分镜二：【景别/视角：Vera常服侧面近景 | 运镜：固定，视线朝城市而非镜头】
+【时长】3.5s
+【构图】电话中Don Ernesto常服开口，Vera常服没有说话；她的目光由远处落到近处栏杆方向。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Don Ernesto常服的VO按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Vera常服听电话，右手未放下。
+【镜头结尾·站位收束】Vera常服听电话，右手未放下。
+画面硬切到分镜三。
+分镜三：【景别/视角：栏杆与Vera常服中近景 | 运镜：从门侧向外缓推半步后停止】
+【时长】4.0s
+【构图】Don Ernesto常服继续说明转账；Vera常服左手指尖在栏杆上略收，身体仍处安全栏杆内。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Don Ernesto常服的VO按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】左手仍扶栏，右手持手机。
+【镜头结尾·站位收束】左手仍扶栏，右手持手机。
+画面硬切到分镜四。
+分镜四：【景别/视角：Vera常服侧面近景 | 运镜：小幅侧移，保留背景城市视差】
+【时长】3.0s
+【构图】转账信息的声音跨切继续，Vera常服等对方说完，唇部才松开准备提问。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Don Ernesto常服的VO按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】电话信息说完，Vera常服即将接话。
+【镜头结尾·站位收束】电话信息说完，Vera常服即将接话。
+画面硬切到分镜五。
+分镜五：【景别/视角：Vera常服半身近景 | 运镜：固定，给短问句一个清楚停点】
+【时长】3.0s
+【构图】Vera常服不提高音量，直接问来源；右肘自然靠近躯干。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Vera常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】手机仍贴右耳。
+【镜头结尾·站位收束】手机仍贴右耳。
+画面硬切到分镜六。
+分镜六：【景别/视角：背面与城市中景 | 运镜：缓慢后拉显出阳台门和人物距离】
+【时长】4.0s
+【构图】Don Ernesto常服在电话中给出答案，Vera常服目光停住；这次只保留眼睑略收，不叠加颤抖与倒吸气。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Don Ernesto常服的VO按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Vera常服仍在栏杆内侧。
+【镜头结尾·站位收束】Vera常服仍在栏杆内侧。
+画面硬切到分镜七。
+分镜七：【景别/视角：阳台门侧中景 | 运镜：跟随她回转半步，镜头不跨玻璃】
+【时长】3.0s
+【构图】答案结束后Vera常服将手机放低，转身沿原路回阳台门，左手伸向门把。
+【音效】门扇与门锁随实际开合发声、手指与机身接触的低弱摩擦声；台词期间压低动作声。
+【台词】无台词。
+【变化】手机在右手身侧；Vera常服停在门外准备回室内。
+【镜头结尾·站位收束】手机在右手身侧；Vera常服停在门外准备回室内。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：23.5s</x:v>
+      </x:c>
+      <x:c r="G18" s="2" t="str">
+        <x:v>Don Ernesto VO：「Los encontré. A sus «papás».」
+Don Ernesto VO：「Pareja de apostadores. Hace tres días les cayeron quinientos mil pesos en la cuenta.」
+Vera：「¿De quién?」
+Don Ernesto VO：「De una empresa fantasma. De la familia Vargas.」</x:v>
+      </x:c>
+      <x:c r="H18" s="2" t="str">
+        <x:v>24-3 高层公寓阳台 夜 外
+人物：Vera、Don Ernesto VO
+△ 画面全景：Vera 站在阳台上，风衣被高空的冷风吹得猎猎作响。背景是改革大道璀璨的天际线，灯火通明，车流如织，构成了一片迷离的光海。
+△ 动作特写：Vera 划开接听键，将手机贴在耳边。她的眼神变得极其冷冽，直视着远方的灯火。
+Don Ernesto VO（低沉且沙哑的声音）：Los encontré. A sus «papás».
+△ 镜头切到 Vera 的侧脸特写：她微微眯起眼，下颌线紧绷，等待对方的下文。
+Don Ernesto VO：Pareja de apostadores. Hace tres días les cayeron quinientos mil pesos en la cuenta.
+△ 镜头切换：Vera 靠在阳台栏杆上，城市的霓虹灯火在她眼中闪烁，如同跳动的火焰。
+Vera（语气冰冷，开门见山）：¿De quién?
+Don Ernesto VO：De una empresa fantasma. De la familia Vargas.
+△ 镜头近景：Vera 听到“Vargas”时，眼神中闪过一丝预料之中的杀意。她慢慢垂下手，将手机从耳边移开，神情变得阴沉莫测。
+△ 画面特写：Vera 站在阳台上，雨后的城市光影投射在她米色的风衣上。她深吸一口气，整理了一下领口，转身重新走向室内。</x:v>
+      </x:c>
+      <x:c r="I18" s="2" t="str">
+        <x:v>23.5s</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="200" customHeight="1">
-      <x:c r="A19" s="2"/>
-      <x:c r="B19" s="2"/>
-      <x:c r="C19" s="2"/>
-      <x:c r="D19" s="2"/>
-      <x:c r="E19" s="2"/>
-      <x:c r="F19" s="2"/>
-      <x:c r="G19" s="2"/>
-      <x:c r="H19" s="2"/>
-      <x:c r="I19" s="2"/>
+      <x:c r="A19" s="2" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="B19" s="2" t="str">
+        <x:v>24-4A</x:v>
+      </x:c>
+      <x:c r="C19" s="2" t="str">
+        <x:v>Vera常服；Ramón常服；Carmen常服；Escolta A常服</x:v>
+      </x:c>
+      <x:c r="D19" s="2" t="str">
+        <x:v>高层公寓门口与走廊（文字设定·夜）</x:v>
+      </x:c>
+      <x:c r="E19" s="2" t="str"/>
+      <x:c r="F19" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+高层公寓门口与走廊（文字设定·夜），9:16竖屏。走廊顶灯从门外斜上方照入；室内客厅暖光只勾Vera常服侧后轮廓。
+[音轨规则]
+远层：公寓外远处车流低声，室内维持安静。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
+6.1s—9.7s，@Ramón常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Número Siete. Abre. Llegaron papá y mamá.」
+[锚定列表]
+场景：高层公寓门口与走廊（文字设定·夜）
+角色：@Vera常服；@Ramón常服；@Carmen常服；@Escolta A常服
+未带@的本段场景或物件按已授权的文字设计执行，保持下述位置、数量和状态。
+[空间布局总览]
+公寓门在走廊北墙，向公寓内开启；走廊东西向，电梯在东端。Vera常服起初在门内北侧，Ramón常服在门外正前，Carmen常服在其西侧，Escolta A在其东后侧。Vera常服已穿过客厅来到门内；Ramón常服在门外中央、Carmen常服在其西侧、Escolta A在其东后方。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（5个硬切分镜）]
+分镜一：【景别/视角：Vera常服侧后中景/玄关 | 运镜：沿客厅入口向西跟两步，停在门内】
+【时长】3.0s
+【构图】Vera常服走到西门内，先把目光凑近猫眼，右手还未碰门把。
+【音效】门扇与门锁随实际开合发声、脚步随起停出现；台词期间压低动作声。
+【台词】无台词。
+【变化】Vera常服在门内，门关闭。
+【镜头结尾·站位收束】Vera常服在门内，门关闭。
+画面硬切到分镜二。
+分镜二：【景别/视角：猫眼主观中景 | 运镜：固定在Vera常服已建立眼位】
+【时长】3.0s
+【构图】Ramón常服站门外中央，Carmen常服在其西，Escolta A在其东后；三人保持各自距离。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】三人都在走廊，没有进门。
+【镜头结尾·站位收束】三人都在走廊，没有进门。
+画面硬切到分镜三。
+分镜三：【景别/视角：Ramón常服近景/走廊侧 | 运镜：在门外东侧固定，不跨到门内】
+【时长】4.0s
+【构图】Ramón常服抬右手拍门后放下，面对门说话；声线带催逼，不额外加笑声。
+【音效】门扇与门锁随实际开合发声；台词期间压低动作声。
+【台词】@Ramón常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Ramón常服双脚原位，右手已离门板。
+【镜头结尾·站位收束】Ramón常服双脚原位，右手已离门板。
+画面硬切到分镜四。
+分镜四：【景别/视角：门内Vera常服近景 | 运镜：固定，门框与右手同框】
+【时长】3.0s
+【构图】Vera常服听完，目光从猫眼退开，右手握住门把，左手垂在身侧。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】右手转动把手，门仍未大开。
+【镜头结尾·站位收束】右手转动把手，门仍未大开。
+画面硬切到分镜五。
+分镜五：【景别/视角：门缝与人物关系近景 | 运镜：缓向后退，给门扇向内开启留空间】
+【时长】3.0s
+【构图】Vera常服把门向室内拉开一道缝，走廊侧光进入玄关，露出门外Ramón常服的轮廓。
+【音效】门扇与门锁随实际开合发声、脚步随起停出现；台词期间压低动作声。
+【台词】无台词。
+【变化】门向内半开，Vera常服在门内北侧，三人仍门外。
+【镜头结尾·站位收束】门向内半开，Vera常服在门内北侧，三人仍门外。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：16s</x:v>
+      </x:c>
+      <x:c r="G19" s="2" t="str">
+        <x:v>Ramón：「Número Siete. Abre. Llegaron papá y mamá.」</x:v>
+      </x:c>
+      <x:c r="H19" s="2" t="str">
+        <x:v>24-4 高层公寓走廊/门口 夜 内
+人物：Vera、Ramón、Carmen、保镖甲
+△ 镜头全景：Vera 穿过客厅，步伐沉稳地走向公寓大门。她的眼神已经恢复了战斗状态。
+△ 动作特写：Vera 站在门后，并没有直接开门，而是先凑近猫眼观察。
+△ 镜头特写（猫眼视角）：走廊里站着三个人。站在正前方的是穿着棕色夹克、一脸市侩笑容的 Ramón，他身边站着一个同样衣着寒酸、神情萎靡的老妇人 Carmen。两人身后站着一名体型巨大的黑衣保镖，神情肃穆。
+△ 镜头切到 Ramón：他对着猫眼，露出一副夸张且令人作呕的慈祥笑容，眼神中却闪烁着贪婪的光芒。
+Ramón（大声拍门）：Número Siete. Abre. Llegaron papá y mamá.
+△ 镜头反打：Vera 站在门内，面无表情地听着外面的叫喊。她的眼神中没有丝毫见到“父母”的喜悦，只有一种面对猎物的冷酷审视。
+△ 动作特写：Vera 伸出右手，指尖搭在门锁上，缓缓转动把手。
+△ 镜头收尾：门缝开启，走廊的灯光斜射进阴暗的玄关，Vera 的身影被强光勾勒出一个凌厉的轮廓。</x:v>
+      </x:c>
+      <x:c r="I19" s="2" t="str">
+        <x:v>16s</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="200" customHeight="1">
-      <x:c r="A20" s="2"/>
-      <x:c r="B20" s="2"/>
-      <x:c r="C20" s="2"/>
-      <x:c r="D20" s="2"/>
-      <x:c r="E20" s="2"/>
-      <x:c r="F20" s="2"/>
-      <x:c r="G20" s="2"/>
-      <x:c r="H20" s="2"/>
-      <x:c r="I20" s="2"/>
+      <x:c r="A20" s="2" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="B20" s="2" t="str">
+        <x:v>25-1A</x:v>
+      </x:c>
+      <x:c r="C20" s="2" t="str">
+        <x:v>Vera常服；Ramón常服；Carmen常服；Escolta A常服</x:v>
+      </x:c>
+      <x:c r="D20" s="2" t="str">
+        <x:v>高层公寓玄关与走廊（文字设定·夜）</x:v>
+      </x:c>
+      <x:c r="E20" s="2" t="str">
+        <x:v>银色金属球棒</x:v>
+      </x:c>
+      <x:c r="F20" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+高层公寓玄关与走廊（文字设定·夜），9:16竖屏。走廊顶部侧光保留门外人物轮廓，室内落地灯从Vera常服左后方照出侧面。
+[音轨规则]
+远层：公寓外远处车流低声，室内维持安静。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
+3.1s—6.1s，@Carmen常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Quinientos mil pesos nos dieron por ti.」
+6.3s—8.5s，@Carmen常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Todos dijeron que nos estafaron.」
+8.7s—11.6s，@Ramón常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Mírate ahora. Vales un millón, mínimo.」
+11.8s—12.7s，@Vera常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Dinero.」
+13.6s—16.9s，@Ramón常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Un millón de pesos. Llámalo pensión alimenticia.」
+17.1s—18.9s，@Vera常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「¿Y si no pago?」
+[锚定列表]
+场景：高层公寓玄关与走廊（文字设定·夜）
+角色：@Vera常服；@Ramón常服；@Carmen常服；@Escolta A常服
+道具：@银色金属球棒
+未带@的本段场景或物件按已授权的文字设计执行，保持下述位置、数量和状态。
+[空间布局总览]
+公寓门在走廊北墙，向公寓内开启；走廊东西向，电梯在东端。Vera常服起初在门内北侧，Ramón常服在门外正前，Carmen常服在其西侧，Escolta A在其东后侧。门已向室内半开。Vera常服站门内北侧；Escolta A右手持球棒向下，停在Ramón常服东后侧。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（6个硬切分镜）]
+分镜一：【景别/视角：玄关关系中景/门内东侧 | 运镜：向室内退半步，显出门内外距离】
+【时长】3.0s
+【构图】Vera常服把门拉开到可交流宽度，自己留在门内；Ramón常服与Carmen常服没有越门槛，Escolta A持棒在后。
+【音效】门扇与门锁随实际开合发声；台词期间压低动作声。
+【台词】无台词。
+【变化】门开，四人位置清楚。
+【镜头结尾·站位收束】门开，四人位置清楚。
+画面硬切到分镜二。
+分镜二：【景别/视角：Carmen常服近景/门内斜望门外 | 运镜：固定，Ramón常服模糊肩线在前景边缘】
+【时长】4.0s
+【构图】Carmen常服看向Vera常服，说出收到钱的事实，眼神短暂闪避后回到对方；不演额外崩溃。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Carmen常服的对白按本段唯一声音骨架连续发声；@Carmen常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Carmen常服留Ramón常服西侧。
+【镜头结尾·站位收束】Carmen常服留Ramón常服西侧。
+画面硬切到分镜三。
+分镜三：【景别/视角：Ramón常服中近景/走廊东侧 | 运镜：沿门外东侧轻移，不穿过人物】
+【时长】3.5s
+【构图】Ramón常服向门口近半步，视线掠过Vera常服后抬到她脸上，手掌朝上摊开。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Carmen常服的对白按本段唯一声音骨架连续发声；@Ramón常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Ramón常服仍未跨门槛，右手朝上。
+【镜头结尾·站位收束】Ramón常服仍未跨门槛，右手朝上。
+画面硬切到分镜四。
+分镜四：【景别/视角：Vera常服近景/门内西南侧 | 运镜：固定，目光与短回应均清楚】
+【时长】3.0s
+【构图】Vera常服看着Ramón常服，平静说出一个词，双脚没有退让。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Ramón常服的对白按本段唯一声音骨架连续发声；@Vera常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Vera常服门内北侧，右手仍近门把。
+【镜头结尾·站位收束】Vera常服门内北侧，右手仍近门把。
+画面硬切到分镜五。
+分镜五：【景别/视角：Ramón常服侧面近景 | 运镜：短促向前推后落稳】
+【时长】3.5s
+【构图】Ramón常服收起摊开的手掌，给出金额，句尾稍压低；身体仍在门外。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Ramón常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Ramón常服停在门口，Carmen常服在其西侧。
+【镜头结尾·站位收束】Ramón常服停在门口，Carmen常服在其西侧。
+画面硬切到分镜六。
+分镜六：【景别/视角：Vera常服中近景 | 运镜：由门框边短移露出侧脸，随后固定】
+【时长】3.0s
+【构图】Vera常服抬眼看Ramón常服，直接提出条件疑问；音量不变，不机械上扬句尾。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Vera常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Vera常服站位和手部状态未变。
+【镜头结尾·站位收束】Vera常服站位和手部状态未变。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：20s</x:v>
+      </x:c>
+      <x:c r="G20" s="2" t="str">
+        <x:v>Carmen：「Quinientos mil pesos nos dieron por ti.」
+Carmen：「Todos dijeron que nos estafaron.」
+Ramón：「Mírate ahora. Vales un millón, mínimo.」
+Vera：「Dinero.」
+Ramón：「Un millón de pesos. Llámalo pensión alimenticia.」
+Vera：「¿Y si no pago?」</x:v>
+      </x:c>
+      <x:c r="H20" s="2" t="str">
+        <x:v>第25集
+25-1 高层公寓玄关 夜 内
+人物：Vera、Ramón、Carmen、保镖甲
+△ 镜头全景：厚重的木门向内打开。Vera 穿着米色风衣，神情冷峻地站在玄关灯光下，目光如炬，注视着门外的来访者。
+△ 镜头反打：Ramón 站在最前方，身穿深褐色皮夹克和格子衬衫，脸上挂着一抹市侩而虚伪的笑容。他身边站着老妇人 Carmen，她头发灰白凌乱，穿着花色外套，神情委琐，眼神躲闪。一名身材魁梧的黑衣保镖手持金属球棒，如铁塔般矗立在后方。
+△ 镜头特写：Carmen 看着 Vera，眼神中闪过一丝复杂的情绪，随即开口，声音嘶哑而刺耳。
+【字幕：Carmen — Madre biológica de Vera】
+Carmen：Quinientos mil pesos nos dieron por ti.
+△ 镜头近景：Ramón 站在一旁，不断点头附和，神情贪婪。
+Carmen：Todos dijeron que nos estafaron.
+△ 镜头切换：Ramón 走上前半步，上下打量着 Vera 的装束，目光落在她华贵的风衣上，双手不安分地揉搓着。
+【字幕：Ramón — Padre biológico de Vera】
+Ramón：Mírate ahora. Vales un millón, mínimo.
+△ 镜头特写：Vera 的眼神没有任何波动，只是冷冷地吐出一个单词。
+Vera（语气冰冷）：Dinero.
+△ 镜头近景：Ramón 嘿嘿一笑，露出一口残缺不全的牙齿，显得阴险而猥琐。
+Ramón：Un millón de pesos. Llámalo pensión alimenticia.
+△ 镜头切换：Vera 微微扬起下巴，眼神中透出一丝嘲讽。
+Vera：¿Y si no pago?
+△ 镜头特写：Ramón 的笑容逐渐消失，取而代之的是一种扭曲的威胁。他凑近 Vera，压低了声音。</x:v>
+      </x:c>
+      <x:c r="I20" s="2" t="str">
+        <x:v>20s</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="200" customHeight="1">
-      <x:c r="A21" s="2"/>
-      <x:c r="B21" s="2"/>
-      <x:c r="C21" s="2"/>
-      <x:c r="D21" s="2"/>
-      <x:c r="E21" s="2"/>
-      <x:c r="F21" s="2"/>
-      <x:c r="G21" s="2"/>
-      <x:c r="H21" s="2"/>
-      <x:c r="I21" s="2"/>
+      <x:c r="A21" s="2" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="B21" s="2" t="str">
+        <x:v>25-1B</x:v>
+      </x:c>
+      <x:c r="C21" s="2" t="str">
+        <x:v>Vera常服；Ramón常服；Carmen常服；Escolta A常服</x:v>
+      </x:c>
+      <x:c r="D21" s="2" t="str">
+        <x:v>高层公寓玄关与走廊（文字设定·夜）</x:v>
+      </x:c>
+      <x:c r="E21" s="2" t="str">
+        <x:v>银色金属球棒</x:v>
+      </x:c>
+      <x:c r="F21" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+高层公寓玄关与走廊（文字设定·夜），9:16竖屏。门外顶灯冷白与室内侧后暖光保持固定，不随正反打互换。
+[音轨规则]
+远层：公寓外远处车流低声，室内维持安静。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
+0.2s—2.7s，@Ramón常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Entonces… vamos con la prensa.」
+3.1s—8.5s，@Ramón常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「A decirles que a los ocho años le prendiste fuego a nuestra cocina.」
+8.7s—11.3s，@Ramón常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Tu hermanita casi se muere ahí.」
+11.5s—16.5s，@Carmen常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Y ya de paso, igual buscamos al viejo amigo de tu hermana.」
+[锚定列表]
+场景：高层公寓玄关与走廊（文字设定·夜）
+角色：@Vera常服；@Ramón常服；@Carmen常服；@Escolta A常服
+道具：@银色金属球棒
+未带@的本段场景或物件按已授权的文字设计执行，保持下述位置、数量和状态。
+[空间布局总览]
+公寓门在走廊北墙，向公寓内开启；走廊东西向，电梯在东端。Vera常服起初在门内北侧，Ramón常服在门外正前，Carmen常服在其西侧，Escolta A在其东后侧。Ramón常服靠近门外中央，Carmen常服在西侧，Escolta A在东后，右手持棒向下；Vera常服在门内北侧，门向室内开启。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（5个硬切分镜）]
+分镜一：【景别/视角：Ramón常服近景/走廊东侧 | 运镜：固定，视线指向门内Vera常服】
+【时长】3.0s
+【构图】Ramón常服身体略向前，压低声音提到媒体；面部只保留嘴角逐渐收住。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Ramón常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Ramón常服没有进门。
+【镜头结尾·站位收束】Ramón常服没有进门。
+画面硬切到分镜二。
+分镜二：【景别/视角：Vera常服听者近景/门内 | 运镜：向门框内短移，以框架保留她受压的空间】
+【时长】4.0s
+【构图】Ramón常服继续在画外说起火灾；Vera常服目光不离他，右手靠近门把，左手自然垂下。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Ramón常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Vera常服听着，身体不动。
+【镜头结尾·站位收束】Vera常服听着，身体不动。
+画面硬切到分镜三。
+分镜三：【景别/视角：Ramón常服侧面近景 | 运镜：固定，Carmen常服在背景西侧可见】
+【时长】3.0s
+【构图】Ramón常服说到妹妹，目光停在Vera常服脸上；Carmen常服原先低着头，听到这里才抬眼。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Ramón常服的对白按本段唯一声音骨架连续发声；@Ramón常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Ramón常服仍在门外，Carmen常服已抬眼。
+【镜头结尾·站位收束】Ramón常服仍在门外，Carmen常服已抬眼。
+画面硬切到分镜四。
+分镜四：【景别/视角：Carmen常服近景/门外东北侧 | 运镜：缓推至眼神，随后停住】
+【时长】4.0s
+【构图】Carmen常服接过话头，声音偏低沙哑；她看向Vera常服，不安排尖叫或全身发抖。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Ramón常服的对白按本段唯一声音骨架连续发声；@Carmen常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Carmen常服原位，Vera常服在门内听着。
+【镜头结尾·站位收束】Carmen常服原位，Vera常服在门内听着。
+画面硬切到分镜五。
+分镜五：【景别/视角：四人关系中景/门内南侧 | 运镜：缓慢后拉，显出Escolta A持棒与门槛】
+【时长】3.0s
+【构图】Ramón常服回身用左手推一下Escolta A上臂，暗示他上前；球棒仍在Escolta A右手。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Carmen常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Escolta A重心前移，尚未越过门槛。
+【镜头结尾·站位收束】Escolta A重心前移，尚未越过门槛。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：17s</x:v>
+      </x:c>
+      <x:c r="G21" s="2" t="str">
+        <x:v>Ramón：「Entonces… vamos con la prensa.」
+Ramón：「A decirles que a los ocho años le prendiste fuego a nuestra cocina.」
+Ramón：「Tu hermanita casi se muere ahí.」
+Carmen：「Y ya de paso, igual buscamos al viejo amigo de tu hermana.」</x:v>
+      </x:c>
+      <x:c r="H21" s="2" t="str">
+        <x:v>Ramón：Entonces… vamos con la prensa.
+△ 镜头反打：Vera 依旧纹丝不动，冷冷地看着他表演。
+Ramón：A decirles que a los ocho años le prendiste fuego a nuestra cocina.
+△ 镜头特写：Carmen 在一旁低下头，似乎陷入了某种痛苦的回忆。
+Ramón：Tu hermanita casi se muere ahí.
+△ 镜头近景：Carmen 突然抬起头，眼神中带着一种病态的报复感。
+Carmen：Y ya de paso, igual buscamos al viejo amigo de tu hermana.
+△ 动作特写：Ramón 见 Vera 沉默，显得有些不耐烦，他用力推了一下身后的保镖甲。</x:v>
+      </x:c>
+      <x:c r="I21" s="2" t="str">
+        <x:v>17s</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="200" customHeight="1">
-      <x:c r="A22" s="2"/>
-      <x:c r="B22" s="2"/>
-      <x:c r="C22" s="2"/>
-      <x:c r="D22" s="2"/>
-      <x:c r="E22" s="2"/>
-      <x:c r="F22" s="2"/>
-      <x:c r="G22" s="2"/>
-      <x:c r="H22" s="2"/>
-      <x:c r="I22" s="2"/>
+      <x:c r="A22" s="2" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="B22" s="2" t="str">
+        <x:v>25-1C</x:v>
+      </x:c>
+      <x:c r="C22" s="2" t="str">
+        <x:v>Vera常服；Ramón常服；Carmen常服；Escolta A常服</x:v>
+      </x:c>
+      <x:c r="D22" s="2" t="str">
+        <x:v>高层公寓玄关与走廊（文字设定·夜）</x:v>
+      </x:c>
+      <x:c r="E22" s="2" t="str">
+        <x:v>银色金属球棒</x:v>
+      </x:c>
+      <x:c r="F22" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+高层公寓玄关与走廊（文字设定·夜），9:16竖屏。沿用走廊冷白侧光与玄关暖侧逆光，脸部不新增正面光。
+[音轨规则]
+远层：公寓外远处车流低声，室内维持安静。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
+0.2s—2.8s，@Vera常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Ustedes saben dónde está mi hermana.」
+3.6s—5.3s，@Ramón常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「¿Quieres saber? Paga.」
+[锚定列表]
+场景：高层公寓玄关与走廊（文字设定·夜）
+角色：@Vera常服；@Ramón常服；@Carmen常服；@Escolta A常服
+道具：@银色金属球棒
+未带@的本段场景或物件按已授权的文字设计执行，保持下述位置、数量和状态。
+[空间布局总览]
+公寓门在走廊北墙，向公寓内开启；走廊东西向，电梯在东端。Vera常服起初在门内北侧，Ramón常服在门外正前，Carmen常服在其西侧，Escolta A在其东后侧。Vera常服在门内，Ramón常服在门外，Carmen常服西侧，Escolta A东后方准备上前，右手持棒。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（3个硬切分镜）]
+分镜一：【景别/视角：Vera常服近景/门内西南侧 | 运镜：缓慢前推，落在她压住的唇部与视线】
+【时长】3.5s
+【构图】Vera常服目光收紧，先看Ramón常服再停住，问出妹妹的下落；发声低沉，不加咆哮。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Vera常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Vera常服右手仍靠近门把。
+【镜头结尾·站位收束】Vera常服右手仍靠近门把。
+画面硬切到分镜二。
+分镜二：【景别/视角：Ramón常服中近景/门外东侧 | 运镜：固定，保留朝门内伸出的手】
+【时长】3.0s
+【构图】Ramón常服伸出右手，先反问再索价；动作不触到Vera常服身体。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Ramón常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】右手停在胸前，仍在走廊。
+【镜头结尾·站位收束】右手停在胸前，仍在走廊。
+画面硬切到分镜三。
+分镜三：【景别/视角：Escolta A低位中景 | 运镜：沿走廊东侧短移，落在跨步前的脚与持棒手】
+【时长】3.0s
+【构图】Escolta A从Ramón常服东后侧向门口迈半步，右手抬起球棒；Ramón常服让出门口东侧的窄道。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】球棒接近门洞，Vera常服在门内准备关门。
+【镜头结尾·站位收束】球棒接近门洞，Vera常服在门内准备关门。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：9.5s</x:v>
+      </x:c>
+      <x:c r="G22" s="2" t="str">
+        <x:v>Vera：「Ustedes saben dónde está mi hermana.」
+Ramón：「¿Quieres saber? Paga.」</x:v>
+      </x:c>
+      <x:c r="H22" s="2" t="str">
+        <x:v>△ 镜头切到 Vera：她的瞳孔微缩，声音变得低沉而危险。
+Vera：Ustedes saben dónde está mi hermana.
+△ 镜头特写：Ramón 再次露出那副令人作呕的笑容，伸出一只手做讨要状。
+Ramón：¿Quieres saber? Paga.</x:v>
+      </x:c>
+      <x:c r="I22" s="2" t="str">
+        <x:v>9.5s</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="200" customHeight="1">
-      <x:c r="A23" s="2"/>
-      <x:c r="B23" s="2"/>
-      <x:c r="C23" s="2"/>
-      <x:c r="D23" s="2"/>
-      <x:c r="E23" s="2"/>
-      <x:c r="F23" s="2"/>
-      <x:c r="G23" s="2"/>
-      <x:c r="H23" s="2"/>
-      <x:c r="I23" s="2"/>
+      <x:c r="A23" s="2" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="B23" s="2" t="str">
+        <x:v>25-2A</x:v>
+      </x:c>
+      <x:c r="C23" s="2" t="str">
+        <x:v>Vera常服；Ramón常服；Carmen常服；Escolta A常服</x:v>
+      </x:c>
+      <x:c r="D23" s="2" t="str">
+        <x:v>高层公寓玄关与电梯厅（文字设定·夜）</x:v>
+      </x:c>
+      <x:c r="E23" s="2" t="str">
+        <x:v>银色金属球棒</x:v>
+      </x:c>
+      <x:c r="F23" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+高层公寓玄关与电梯厅（文字设定·夜），9:16竖屏。走廊顶灯照清门缝与球棒接触，室内侧光只补轮廓，动作不藏在暗处。
+[音轨规则]
+远层：公寓外远处车流低声，室内维持安静。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
+6.1s—12.9s，@Vera常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「No te voltees. Si te volteas, vas a ver esta cara en cada pesadilla que tengas.」
+[锚定列表]
+场景：高层公寓玄关与电梯厅（文字设定·夜）
+角色：@Vera常服；@Ramón常服；@Carmen常服；@Escolta A常服
+道具：@银色金属球棒
+未带@的本段场景或物件按已授权的文字设计执行，保持下述位置、数量和状态。
+[空间布局总览]
+公寓门在走廊北墙，向公寓内开启；走廊东西向，电梯在东端。Vera常服起初在门内北侧，Ramón常服在门外正前，Carmen常服在其西侧，Escolta A在其东后侧。门扇向室内开。Escolta A从门外东侧伸棒逼近；Ramón常服、Carmen常服退到走廊西侧；Vera常服在门内右手握门把。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（6个硬切分镜）]
+分镜一：【景别/视角：门槛侧面中景/走廊东侧 | 运镜：固定，门扇运动与棒身完整入画】
+【时长】3.0s
+【构图】Escolta A右手将球棒探入门洞，Vera常服右手把门向外侧门框方向推合；棒身卡在门缝，门保留一条窄缝而未完全关闭。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】球棒卡住，Escolta A在门外拉住棒柄，Vera常服在门内。
+【镜头结尾·站位收束】球棒卡住，Escolta A在门外拉住棒柄，Vera常服在门内。
+画面硬切到分镜二。
+分镜二：【景别/视角：门内斜侧中景 | 运镜：向室内退半步，让出真实通道】
+【时长】3.0s
+【构图】Vera常服左手稳住门边、右手将门重新向室内拉开，球棒解卡；她从门外西侧空隙侧身跨到走廊，绕至Escolta A西后侧。
+【音效】门扇与门锁随实际开合发声、脚步随起停出现；台词期间压低动作声。
+【台词】无台词。
+【变化】门向内重新打开；Vera常服已在走廊，Escolta A仍面向门洞。
+【镜头结尾·站位收束】门向内重新打开；Vera常服已在走廊，Escolta A仍面向门洞。
+画面硬切到分镜三。
+分镜三：【景别/视角：Vera常服侧面近景/走廊西侧 | 运镜：伴随她停在Escolta A侧后方后固定】
+【时长】4.0s
+【构图】Vera常服靠近对方耳侧低声警告，双脚一前一后支撑，双手尚未夺棒；Escolta A握棒停住。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Vera常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Vera常服在其西后侧，Escolta A右手仍持棒。
+【镜头结尾·站位收束】Vera常服在其西后侧，Escolta A右手仍持棒。
+画面硬切到分镜四。
+分镜四：【景别/视角：Escolta A侧面中景 | 运镜：沿走廊北侧短移，保留Vera常服与对方的距离】
+【时长】4.0s
+【构图】警告声音跨切继续；Escolta A头部想转又停，右手对棒柄的握力略松，身体没有提前逃走。
+【音效】脚步随起停出现；台词期间压低动作声。
+【台词】@Vera常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】警告说完，Vera常服已站稳支撑脚。
+【镜头结尾·站位收束】警告说完，Vera常服已站稳支撑脚。
+画面硬切到分镜五。
+分镜五：【景别/视角：双人全身中景/走廊南侧 | 运镜：固定，脚部发力、接触与持棒手都在画内】
+【时长】3.5s
+【构图】Vera常服左手扣住Escolta A右腕，右脚支撑、左脚踹向其腰侧，接触后他向东踉跄；Vera常服右手抓棒身，左手压低对方手腕，对方松手后球棒转归她右手。
+【音效】鞋底接触地面声、棒身与接触物的短促撞击声；台词期间压低动作声。
+【台词】无台词。
+【变化】Escolta A向东失衡，Vera常服右手持棒、左手已放开其腕。
+【镜头结尾·站位收束】Escolta A向东失衡，Vera常服右手持棒、左手已放开其腕。
+画面硬切到分镜六。
+分镜六：【景别/视角：走廊纵深中景/西端望东 | 运镜：随Escolta A向东轻摇，保持Vera常服留在近景一侧】
+【时长】3.0s
+【构图】Escolta A站稳一脚后向东逃离，退出电梯厅画外；Vera常服停在门外，不追赶。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】Escolta A已离开；Vera常服右手持球棒，Ramón常服与Carmen常服仍在西侧。
+【镜头结尾·站位收束】Escolta A已离开；Vera常服右手持球棒，Ramón常服与Carmen常服仍在西侧。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：20.5s</x:v>
+      </x:c>
+      <x:c r="G23" s="2" t="str">
+        <x:v>Vera：「No te voltees. Si te volteas, vas a ver esta cara en cada pesadilla que tengas.」</x:v>
+      </x:c>
+      <x:c r="H23" s="2" t="str">
+        <x:v>25-2 高层公寓/电梯厅 夜 内
+人物：Vera、Ramón、Carmen、保镖甲
+△ 画面全景：保镖甲猛地跨步上前，手中的金属球棒在灯光下闪着寒光。他神情凶恶，意图闯入房间。
+△ 动作特写：Vera 的反应极快。她猛地发力，右手用力一甩，沉重的实木房门“砰”的一声合上。
+△ 镜头反打：保镖甲反应不及，金属球棒直接卡在了门缝中，发出一声刺耳的撞击声。
+△ 动作特写：Vera 并没有停止。她隔着门再次发力狠推，同时侧身闪出房门，借着冲劲直接冲向电梯厅的众人。
+△ 镜头切换：Vera 一个闪身绕到保镖甲的侧后方，动作如行云流水。
+△ 镜头特写：Vera 眼神凌厉，贴近保镖甲的耳边，声音如冰刃般刺骨。
+Vera（低声警告）：No te voltees. Si te volteas, vas a ver esta cara en cada pesadilla que tengas.
+△ 动作特写：保镖甲被这股强大的气场所震慑，竟僵在原地不敢动弹。他握着球棒的手微微颤抖。
+△ 镜头全景：Vera 猛地一脚踹在保镖甲的腰部，同时顺势夺下球棒。
+△ 镜头切换：保镖甲狼狈地踉跄了几步，惊恐地看了一眼 Vera，随即转头拔腿就跑，丢下了 Ramón 和 Carmen。</x:v>
+      </x:c>
+      <x:c r="I23" s="2" t="str">
+        <x:v>20.5s</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="200" customHeight="1">
-      <x:c r="A24" s="2"/>
-      <x:c r="B24" s="2"/>
-      <x:c r="C24" s="2"/>
-      <x:c r="D24" s="2"/>
-      <x:c r="E24" s="2"/>
-      <x:c r="F24" s="2"/>
-      <x:c r="G24" s="2"/>
-      <x:c r="H24" s="2"/>
-      <x:c r="I24" s="2"/>
+      <x:c r="A24" s="2" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="B24" s="2" t="str">
+        <x:v>25-2B</x:v>
+      </x:c>
+      <x:c r="C24" s="2" t="str">
+        <x:v>Vera常服；Ramón常服；Carmen常服</x:v>
+      </x:c>
+      <x:c r="D24" s="2" t="str">
+        <x:v>高层公寓玄关与电梯厅（文字设定·夜）</x:v>
+      </x:c>
+      <x:c r="E24" s="2" t="str">
+        <x:v>银色金属球棒</x:v>
+      </x:c>
+      <x:c r="F24" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+高层公寓玄关与电梯厅（文字设定·夜），9:16竖屏。走廊顶灯从上侧照清腕部接触，侧后壁灯勾出人物轮廓；动作关键区保持可读。
+[音轨规则]
+远层：公寓外远处车流低声，室内维持安静。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
+3.1s—4.4s，@Ramón常服（对白，疼痛下的急促声演，原定呼喊词照原文发出，不再叠加额外叫声）：「¡Ahhh! ¡Alto!」
+6.1s—7.2s，@Vera常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「¿Dónde está?」
+9.1s—12.9s，@Ramón常服（对白，疼痛下的急促声演，原定呼喊词照原文发出，不再叠加额外叫声）：「Si me la rompes, nunca la vas a encontrar.」
+13.1s—20.5s，@Ramón常服（对白，疼痛下的急促声演，原定呼喊词照原文发出，不再叠加额外叫声）：「¡Al sur! ¡La vendimos al sur! A un hombre… ¡con tatuajes rojos en todo el cuello!」
+[锚定列表]
+场景：高层公寓玄关与电梯厅（文字设定·夜）
+角色：@Vera常服；@Ramón常服；@Carmen常服
+道具：@银色金属球棒
+未带@的本段场景或物件按已授权的文字设计执行，保持下述位置、数量和状态。
+[空间布局总览]
+公寓门在走廊北墙，向公寓内开启；走廊东西向，电梯在东端。Vera常服起初在门内北侧，Ramón常服在门外正前，Carmen常服在其西侧，Escolta A在其东后侧。Escolta A已向东逃走。Vera常服在门外中央，右手持棒；Ramón常服在她西前方，Carmen常服在Ramón常服西侧；东端电梯门关闭。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（7个硬切分镜）]
+分镜一：【景别/视角：双人腰部中近景/走廊南侧 | 运镜：向西短移，落在Vera常服左手与Ramón常服右腕】
+【时长】3.0s
+【构图】Ramón常服后退，Vera常服先以左手扣住他的右腕，将右手球棒放低倚在门外北墙，确认棒底落地后右手离开球棒。
+【音效】门扇与门锁随实际开合发声、棒身与接触物的短促撞击声；台词期间压低动作声。
+【台词】无台词。
+【变化】球棒在门边地面；Vera常服左手控Ramón常服右腕，右手已空出。
+【镜头结尾·站位收束】球棒在门边地面；Vera常服左手控Ramón常服右腕，右手已空出。
+画面硬切到分镜二。
+分镜二：【景别/视角：手臂接触与全身中景 | 运镜：固定，让手腕、肘与跪地过程都可见】
+【时长】3.0s
+【构图】Vera常服右手接住Ramón常服前臂，双手形成反关节控制，向下带动其重心；Ramón常服屈膝跪下，先接触地面再发出疼痛声。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Ramón常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Ramón常服跪地，右腕仍受控，Carmen常服在西侧站着。
+【镜头结尾·站位收束】Ramón常服跪地，右腕仍受控，Carmen常服在西侧站着。
+画面硬切到分镜三。
+分镜三：【景别/视角：Vera常服侧面近景 | 运镜：沿走廊西侧轻推，落在她问话的脸】
+【时长】3.0s
+【构图】Vera常服略俯身看Ramón常服，左手保持腕部控制，右手稳住其前臂，不反复重新扭动。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Vera常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】她等回答，力道暂时保持。
+【镜头结尾·站位收束】她等回答，力道暂时保持。
+画面硬切到分镜四。
+分镜四：【景别/视角：Ramón常服侧面近景 | 运镜：固定，左手撑地维持身体支撑】
+【时长】4.0s
+【构图】Ramón常服跪在地上，左手撑地，说出威胁；声线不稳但原文清楚，呼吸不盖住词语。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Ramón常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Ramón常服仍跪地，Vera常服尚未松手。
+【镜头结尾·站位收束】Ramón常服仍跪地，Vera常服尚未松手。
+画面硬切到分镜五。
+分镜五：【景别/视角：双人中景/走廊南侧 | 运镜：微向后拉，保留受控手臂与两张脸】
+【时长】4.0s
+【构图】Vera常服手腕再下压一个小幅度，Ramón常服身体随之低下；一次低弱关节声后，他立即说出方向与纹身线索。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Ramón常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Vera常服听着，双手仍固定在原有接触点。
+【镜头结尾·站位收束】Vera常服听着，双手仍固定在原有接触点。
+画面硬切到分镜六。
+分镜六：【景别/视角：Carmen常服肩侧望向Vera常服与Ramón常服 | 运镜：固定，关键发声继续跨切，镜头不逼拍创伤】
+【时长】4.0s
+【构图】Ramón常服的整句供述继续到完整结尾；Vera常服目光停在他脸上，不新增情绪性吸气，Carmen常服保持站立。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Ramón常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】供述说完，Vera常服准备松开。
+【镜头结尾·站位收束】供述说完，Vera常服准备松开。
+画面硬切到分镜七。
+分镜七：【景别/视角：电梯厅纵深全景 | 运镜：镜头向东轻摇，落在电梯门前】
+【时长】3.5s
+【构图】Vera常服先松开腕部再松开前臂，Ramón常服捧住受伤右腕，Carmen常服从西侧上前搀扶其左臂，两人沿走廊东行进入已开启的电梯，门合上。
+【音效】门扇与门锁随实际开合发声、脚步随起停出现；台词期间压低动作声。
+【台词】无台词。
+【变化】两人已入电梯，Vera常服留门口，球棒仍靠门边北墙。
+【镜头结尾·站位收束】两人已入电梯，Vera常服留门口，球棒仍靠门边北墙。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：24.5s</x:v>
+      </x:c>
+      <x:c r="G24" s="2" t="str">
+        <x:v>Ramón：「¡Ahhh! ¡Alto!」
+Vera：「¿Dónde está?」
+Ramón：「Si me la rompes, nunca la vas a encontrar.」
+Ramón：「¡Al sur! ¡La vendimos al sur! A un hombre… ¡con tatuajes rojos en todo el cuello!」</x:v>
+      </x:c>
+      <x:c r="H24" s="2" t="str">
+        <x:v>△ 镜头特写：Ramón 见势不妙，原本嚣张的气焰瞬间熄灭。他惊慌失措地想要后退，却被 Vera 一个箭步冲上，精准地扣住了他的右手腕。
+△ 动作特写：Vera 猛地向下发力，反关节拧动。
+△ 镜头切换：Ramón 的身体随着 Vera 的动作颓然跪地，发出一声杀猪般的惨叫。
+Ramón（痛苦哀嚎）：¡Ahhh! ¡Alto!
+△ 镜头近景：Carmen 站在一旁，惊恐地捂住嘴，浑身发抖，却不敢上前帮忙。
+△ 镜头特写：Vera 俯下身，脸部贴近跪在地上不断喘息的 Ramón。她的眼神中充满了压迫感。
+Vera（语气森寒）：¿Dónde está?
+△ 镜头切到 Ramón：他由于剧痛而满头大汗，眼神中充满了恐惧，但仍试图顽抗。
+Ramón（颤抖着）：Si me la rompes, nunca la vas a encontrar.
+△ 动作特写：Vera 眼神一冷，手上的力道再次加重。骨骼错位的“咔吧”声在走廊里清晰可闻。
+Ramón（声嘶力竭）：¡Al sur! ¡La vendimos al sur! A un hombre… ¡con tatuajes rojos en todo el cuello!
+△ 镜头特写：Vera 听到“tatuajes rojos”这个细节，眼神瞬间变得极其复杂。她缓缓松开了手。
+△ 镜头全景：Ramón 捧着折断的手腕，在 Carmen 的搀扶下，连滚带爬地逃进电梯。电梯门缓缓合上。</x:v>
+      </x:c>
+      <x:c r="I24" s="2" t="str">
+        <x:v>24.5s</x:v>
+      </x:c>
     </x:row>
     <x:row r="25" ht="200" customHeight="1">
-      <x:c r="A25" s="2"/>
-      <x:c r="B25" s="2"/>
-      <x:c r="C25" s="2"/>
-      <x:c r="D25" s="2"/>
-      <x:c r="E25" s="2"/>
-      <x:c r="F25" s="2"/>
-      <x:c r="G25" s="2"/>
-      <x:c r="H25" s="2"/>
-      <x:c r="I25" s="2"/>
+      <x:c r="A25" s="2" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="B25" s="2" t="str">
+        <x:v>25-2C</x:v>
+      </x:c>
+      <x:c r="C25" s="2" t="str">
+        <x:v>Vera常服</x:v>
+      </x:c>
+      <x:c r="D25" s="2" t="str">
+        <x:v>高层公寓玄关（文字设定·夜）</x:v>
+      </x:c>
+      <x:c r="E25" s="2" t="str">
+        <x:v>银色金属球棒</x:v>
+      </x:c>
+      <x:c r="F25" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+高层公寓玄关（文字设定·夜），9:16竖屏。走廊顶灯冷光照门口，室内暖侧光照到地毯边缘；暗部仍能读出肢体支撑。
+[音轨规则]
+远层：公寓外远处车流低声，室内维持安静。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段无原定对白或旁白，不新增发声。
+[锚定列表]
+场景：高层公寓玄关（文字设定·夜）
+角色：@Vera常服
+道具：@银色金属球棒
+未带@的本段场景或物件按已授权的文字设计执行，保持下述位置、数量和状态。
+[空间布局总览]
+公寓门在走廊北墙，向公寓内开启；走廊东西向，电梯在东端。Vera常服起初在门内北侧，Ramón常服在门外正前，Carmen常服在其西侧，Escolta A在其东后侧。电梯已关闭，Escolta A已逃离。Vera常服站公寓门外，门仍向内打开，球棒倚门外北墙。室内客厅通道在她身后。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（4个硬切分镜）]
+分镜一：【景别/视角：走廊关系全景 | 运镜：由东端电梯方向缓拉向门口】
+【时长】3.0s
+【构图】电梯门已经合拢，Vera常服独站门口；右手捡起靠墙球棒，转身退入玄关。
+【音效】门扇与门锁随实际开合发声、棒身与接触物的短促撞击声；台词期间压低动作声。
+【台词】无台词。
+【变化】Vera常服进入门内，右手持棒。
+【镜头结尾·站位收束】Vera常服进入门内，右手持棒。
+画面硬切到分镜二。
+分镜二：【景别/视角：玄关侧面中景 | 运镜：相机在门内固定，让身体下降过程完整可见】
+【时长】3.0s
+【构图】Vera常服将球棒平放在门内地面，右手离开；背靠门板慢慢屈膝坐下，左手扶地支撑。
+【音效】门扇与门锁随实际开合发声、棒身与接触物的短促撞击声；台词期间压低动作声。
+【台词】无台词。
+【变化】球棒横放门内地面；Vera常服坐在门内，门未凭空改变开向。
+【镜头结尾·站位收束】球棒横放门内地面；Vera常服坐在门内，门未凭空改变开向。
+画面硬切到分镜三。
+分镜三：【景别/视角：Vera常服近景/玄关侧面 | 运镜：缓慢靠近，落在她低垂的眼睑】
+【时长】3.5s
+【构图】Vera常服短暂低头，呼吸由偏快逐渐变匀；已有紧张留在下颌，肩部只略松。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】Vera常服仍坐地，没有新增哭喊。
+【镜头结尾·站位收束】Vera常服仍坐地，没有新增哭喊。
+画面硬切到分镜四。
+分镜四：【景别/视角：低位全身中景 | 运镜：随她起身平缓上抬，保持脚与手的支撑关系】
+【时长】3.5s
+【构图】Vera常服左掌撑地，右手扶门框，先收脚再起身；站定后视线回到室内，球棒留在地面。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】Vera常服在玄关站稳，双手离开支撑点，球棒仍在门内地面。
+【镜头结尾·站位收束】Vera常服在玄关站稳，双手离开支撑点，球棒仍在门内地面。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：13s</x:v>
+      </x:c>
+      <x:c r="G25" s="2" t="str"/>
+      <x:c r="H25" s="2" t="str">
+        <x:v>△ 镜头切换：走廊重新恢复了寂静。Vera 独自站在灯光下，背影显得孤傲而萧索。
+△ 动作特写：Vera 缓缓退回房间，身体靠在门框上，似乎所有的力气都在这一瞬间被抽走。
+△ 镜头近景：Vera 顺着门板滑落在地，坐在地板上。她低着头，呼吸急促，眼中闪过一丝从未流露过的脆弱。
+△ 镜头俯拍：空荡荡的玄关，落在地板上的金属球棒，以及蜷缩在阴影中的 Vera。
+△ 镜头收尾：Vera 抬起头，眼神重新变得坚定，她单手撑地，摇摇晃晃地站了起来。</x:v>
+      </x:c>
+      <x:c r="I25" s="2" t="str">
+        <x:v>13s</x:v>
+      </x:c>
     </x:row>
     <x:row r="26" ht="200" customHeight="1">
       <x:c r="A26" s="2"/>

</xml_diff>

<commit_message>
Re-audit source scene definitions and correct existing corridor bindings
</commit_message>
<xml_diff>
--- a/archive/projects/la-reina-del-bajo-mundo/deliverables/前夫黑道酵母_分镜_21-33.xlsx
+++ b/archive/projects/la-reina-del-bajo-mundo/deliverables/前夫黑道酵母_分镜_21-33.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分镜脚本" sheetId="1" r:id="R3937f7487433491c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分镜脚本" sheetId="1" r:id="Rc08d745346ed4f45"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -807,19 +807,19 @@
         <x:v>Vera常服</x:v>
       </x:c>
       <x:c r="D5" s="2" t="str">
-        <x:v>高层公寓窗边与入口（文字设定·夜）</x:v>
+        <x:v>高层公寓客厅（夜）；公寓入口（文字设定·夜）</x:v>
       </x:c>
       <x:c r="E5" s="2" t="str"/>
       <x:c r="F5" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
-高层公寓窗边与入口（文字设定·夜），9:16竖屏。城市夜光从窗外勾勒肩部；楼下门灯只照入口与两位保镖。
+高层公寓客厅（夜）；公寓入口（文字设定·夜），9:16竖屏。城市夜光从窗外勾勒肩部；楼下门灯只照入口与两位保镖。
 [音轨规则]
 远层：公寓外远处车流低声，室内维持安静。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
 本段无原定对白或旁白，不新增发声。
 [锚定列表]
-场景：高层公寓窗边与入口（文字设定·夜）
+场景：@高层公寓客厅（夜）；公寓入口（文字设定·夜）
 角色：@Vera常服
 未带@的本段场景或物件按已授权的文字设计执行，保持下述位置、数量和状态。
 [空间布局总览]
@@ -1584,7 +1584,7 @@
         <x:v>Vera常服；Renata常服</x:v>
       </x:c>
       <x:c r="D13" s="2" t="str">
-        <x:v>高层公寓门口与走廊（文字设定·夜）</x:v>
+        <x:v>高层公寓客厅（夜）；公寓大楼走廊</x:v>
       </x:c>
       <x:c r="E13" s="2" t="str">
         <x:v>黄色牛皮纸线索信封（文字设定）</x:v>
@@ -1593,12 +1593,12 @@
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
-高层公寓门口与走廊（文字设定·夜），9:16竖屏。走廊顶灯侧照Renata常服，客厅北侧实用灯从门内斜透；门开后形成有来源的明暗交界。
+高层公寓客厅（夜）；公寓大楼走廊，9:16竖屏。走廊顶灯侧照Renata常服，客厅北侧实用灯从门内斜透；门开后形成有来源的明暗交界。
 [音轨规则]
 远层：公寓外远处车流低声，室内维持安静。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
 本段无原定对白或旁白，不新增发声。
 [锚定列表]
-场景：高层公寓门口与走廊（文字设定·夜）
+场景：@高层公寓客厅（夜）；@公寓大楼走廊
 角色：@Vera常服；@Renata常服
 道具：黄色牛皮纸线索信封（文字设定）
 未带@的本段场景或物件按已授权的文字设计执行，保持下述位置、数量和状态。
@@ -1671,7 +1671,7 @@
         <x:v>Vera常服；Renata常服</x:v>
       </x:c>
       <x:c r="D14" s="2" t="str">
-        <x:v>高层公寓门口与客厅（文字设定·夜）</x:v>
+        <x:v>高层公寓客厅（夜）；公寓大楼走廊</x:v>
       </x:c>
       <x:c r="E14" s="2" t="str">
         <x:v>黄色牛皮纸线索信封（文字设定）</x:v>
@@ -1680,14 +1680,14 @@
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
-高层公寓门口与客厅（文字设定·夜），9:16竖屏。走廊顶灯从Renata常服侧上方照入，室内暖光落在Vera常服肩部，两人面部曝光不随切镜跳变。
+高层公寓客厅（夜）；公寓大楼走廊，9:16竖屏。走廊顶灯从Renata常服侧上方照入，室内暖光落在Vera常服肩部，两人面部曝光不随切镜跳变。
 [音轨规则]
 远层：公寓外远处车流低声，室内维持安静。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
 本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
 0.2s—4.3s，@Renata常服（对白，声音带疲惫与轻微不稳，词句完整，不加入抽泣语词）：「La casa del lago. La caja fuerte del abuelo.」
 4.5s—9.3s，@Renata常服（对白，声音带疲惫与轻微不稳，词句完整，不加入抽泣语词）：「Lo agarré y corrí. Mi hermano me persiguió. No volteé.」
 [锚定列表]
-场景：高层公寓门口与客厅（文字设定·夜）
+场景：@高层公寓客厅（夜）；@公寓大楼走廊
 角色：@Vera常服；@Renata常服
 道具：黄色牛皮纸线索信封（文字设定）
 未带@的本段场景或物件按已授权的文字设计执行，保持下述位置、数量和状态。
@@ -2190,22 +2190,21 @@
         <x:v>Vera常服；Ramón常服；Carmen常服；Escolta A常服</x:v>
       </x:c>
       <x:c r="D19" s="2" t="str">
-        <x:v>高层公寓门口与走廊（文字设定·夜）</x:v>
+        <x:v>高层公寓客厅（夜）；公寓大楼走廊</x:v>
       </x:c>
       <x:c r="E19" s="2" t="str"/>
       <x:c r="F19" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
-高层公寓门口与走廊（文字设定·夜），9:16竖屏。走廊顶灯从门外斜上方照入；室内客厅暖光只勾Vera常服侧后轮廓。
+高层公寓客厅（夜）；公寓大楼走廊，9:16竖屏。走廊顶灯从门外斜上方照入；室内客厅暖光只勾Vera常服侧后轮廓。
 [音轨规则]
 远层：公寓外远处车流低声，室内维持安静。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
 本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
 6.1s—9.7s，@Ramón常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Número Siete. Abre. Llegaron papá y mamá.」
 [锚定列表]
-场景：高层公寓门口与走廊（文字设定·夜）
+场景：@高层公寓客厅（夜）；@公寓大楼走廊
 角色：@Vera常服；@Ramón常服；@Carmen常服；@Escolta A常服
-未带@的本段场景或物件按已授权的文字设计执行，保持下述位置、数量和状态。
 [空间布局总览]
 公寓门在走廊北墙，向公寓内开启；走廊东西向，电梯在东端。Vera常服起初在门内北侧，Ramón常服在门外正前，Carmen常服在其西侧，Escolta A在其东后侧。Vera常服已穿过客厅来到门内；Ramón常服在门外中央、Carmen常服在其西侧、Escolta A在其东后方。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
 [运镜时间线（5个硬切分镜）]
@@ -2287,7 +2286,7 @@
         <x:v>Vera常服；Ramón常服；Carmen常服；Escolta A常服</x:v>
       </x:c>
       <x:c r="D20" s="2" t="str">
-        <x:v>高层公寓玄关与走廊（文字设定·夜）</x:v>
+        <x:v>高层公寓客厅（夜）；公寓大楼走廊</x:v>
       </x:c>
       <x:c r="E20" s="2" t="str">
         <x:v>银色金属球棒</x:v>
@@ -2296,7 +2295,7 @@
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
-高层公寓玄关与走廊（文字设定·夜），9:16竖屏。走廊顶部侧光保留门外人物轮廓，室内落地灯从Vera常服左后方照出侧面。
+高层公寓客厅（夜）；公寓大楼走廊，9:16竖屏。走廊顶部侧光保留门外人物轮廓，室内落地灯从Vera常服左后方照出侧面。
 [音轨规则]
 远层：公寓外远处车流低声，室内维持安静。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
 本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
@@ -2307,10 +2306,9 @@
 13.6s—16.9s，@Ramón常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Un millón de pesos. Llámalo pensión alimenticia.」
 17.1s—18.9s，@Vera常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「¿Y si no pago?」
 [锚定列表]
-场景：高层公寓玄关与走廊（文字设定·夜）
+场景：@高层公寓客厅（夜）；@公寓大楼走廊
 角色：@Vera常服；@Ramón常服；@Carmen常服；@Escolta A常服
 道具：@银色金属球棒
-未带@的本段场景或物件按已授权的文字设计执行，保持下述位置、数量和状态。
 [空间布局总览]
 公寓门在走廊北墙，向公寓内开启；走廊东西向，电梯在东端。Vera常服起初在门内北侧，Ramón常服在门外正前，Carmen常服在其西侧，Escolta A在其东后侧。门已向室内半开。Vera常服站门内北侧；Escolta A右手持球棒向下，停在Ramón常服东后侧。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
 [运镜时间线（6个硬切分镜）]
@@ -2415,7 +2413,7 @@
         <x:v>Vera常服；Ramón常服；Carmen常服；Escolta A常服</x:v>
       </x:c>
       <x:c r="D21" s="2" t="str">
-        <x:v>高层公寓玄关与走廊（文字设定·夜）</x:v>
+        <x:v>高层公寓客厅（夜）；公寓大楼走廊</x:v>
       </x:c>
       <x:c r="E21" s="2" t="str">
         <x:v>银色金属球棒</x:v>
@@ -2424,7 +2422,7 @@
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
-高层公寓玄关与走廊（文字设定·夜），9:16竖屏。门外顶灯冷白与室内侧后暖光保持固定，不随正反打互换。
+高层公寓客厅（夜）；公寓大楼走廊，9:16竖屏。门外顶灯冷白与室内侧后暖光保持固定，不随正反打互换。
 [音轨规则]
 远层：公寓外远处车流低声，室内维持安静。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
 本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
@@ -2433,10 +2431,9 @@
 8.7s—11.3s，@Ramón常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Tu hermanita casi se muere ahí.」
 11.5s—16.5s，@Carmen常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Y ya de paso, igual buscamos al viejo amigo de tu hermana.」
 [锚定列表]
-场景：高层公寓玄关与走廊（文字设定·夜）
+场景：@高层公寓客厅（夜）；@公寓大楼走廊
 角色：@Vera常服；@Ramón常服；@Carmen常服；@Escolta A常服
 道具：@银色金属球棒
-未带@的本段场景或物件按已授权的文字设计执行，保持下述位置、数量和状态。
 [空间布局总览]
 公寓门在走廊北墙，向公寓内开启；走廊东西向，电梯在东端。Vera常服起初在门内北侧，Ramón常服在门外正前，Carmen常服在其西侧，Escolta A在其东后侧。Ramón常服靠近门外中央，Carmen常服在西侧，Escolta A在东后，右手持棒向下；Vera常服在门内北侧，门向室内开启。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
 [运镜时间线（5个硬切分镜）]
@@ -2519,7 +2516,7 @@
         <x:v>Vera常服；Ramón常服；Carmen常服；Escolta A常服</x:v>
       </x:c>
       <x:c r="D22" s="2" t="str">
-        <x:v>高层公寓玄关与走廊（文字设定·夜）</x:v>
+        <x:v>高层公寓客厅（夜）；公寓大楼走廊</x:v>
       </x:c>
       <x:c r="E22" s="2" t="str">
         <x:v>银色金属球棒</x:v>
@@ -2528,17 +2525,16 @@
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
-高层公寓玄关与走廊（文字设定·夜），9:16竖屏。沿用走廊冷白侧光与玄关暖侧逆光，脸部不新增正面光。
+高层公寓客厅（夜）；公寓大楼走廊，9:16竖屏。沿用走廊冷白侧光与玄关暖侧逆光，脸部不新增正面光。
 [音轨规则]
 远层：公寓外远处车流低声，室内维持安静。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
 本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
 0.2s—2.8s，@Vera常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Ustedes saben dónde está mi hermana.」
 3.6s—5.3s，@Ramón常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「¿Quieres saber? Paga.」
 [锚定列表]
-场景：高层公寓玄关与走廊（文字设定·夜）
+场景：@高层公寓客厅（夜）；@公寓大楼走廊
 角色：@Vera常服；@Ramón常服；@Carmen常服；@Escolta A常服
 道具：@银色金属球棒
-未带@的本段场景或物件按已授权的文字设计执行，保持下述位置、数量和状态。
 [空间布局总览]
 公寓门在走廊北墙，向公寓内开启；走廊东西向，电梯在东端。Vera常服起初在门内北侧，Ramón常服在门外正前，Carmen常服在其西侧，Escolta A在其东后侧。Vera常服在门内，Ramón常服在门外，Carmen常服西侧，Escolta A东后方准备上前，右手持棒。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
 [运镜时间线（3个硬切分镜）]
@@ -2599,7 +2595,7 @@
         <x:v>Vera常服；Ramón常服；Carmen常服；Escolta A常服</x:v>
       </x:c>
       <x:c r="D23" s="2" t="str">
-        <x:v>高层公寓玄关与电梯厅（文字设定·夜）</x:v>
+        <x:v>高层公寓客厅（夜）；公寓大楼走廊</x:v>
       </x:c>
       <x:c r="E23" s="2" t="str">
         <x:v>银色金属球棒</x:v>
@@ -2608,16 +2604,15 @@
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
-高层公寓玄关与电梯厅（文字设定·夜），9:16竖屏。走廊顶灯照清门缝与球棒接触，室内侧光只补轮廓，动作不藏在暗处。
+高层公寓客厅（夜）；公寓大楼走廊，9:16竖屏。走廊顶灯照清门缝与球棒接触，室内侧光只补轮廓，动作不藏在暗处。
 [音轨规则]
 远层：公寓外远处车流低声，室内维持安静。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
 本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
 6.1s—12.9s，@Vera常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「No te voltees. Si te volteas, vas a ver esta cara en cada pesadilla que tengas.」
 [锚定列表]
-场景：高层公寓玄关与电梯厅（文字设定·夜）
+场景：@高层公寓客厅（夜）；@公寓大楼走廊
 角色：@Vera常服；@Ramón常服；@Carmen常服；@Escolta A常服
 道具：@银色金属球棒
-未带@的本段场景或物件按已授权的文字设计执行，保持下述位置、数量和状态。
 [空间布局总览]
 公寓门在走廊北墙，向公寓内开启；走廊东西向，电梯在东端。Vera常服起初在门内北侧，Ramón常服在门外正前，Carmen常服在其西侧，Escolta A在其东后侧。门扇向室内开。Escolta A从门外东侧伸棒逼近；Ramón常服、Carmen常服退到走廊西侧；Vera常服在门内右手握门把。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
 [运镜时间线（6个硬切分镜）]
@@ -2709,7 +2704,7 @@
         <x:v>Vera常服；Ramón常服；Carmen常服</x:v>
       </x:c>
       <x:c r="D24" s="2" t="str">
-        <x:v>高层公寓玄关与电梯厅（文字设定·夜）</x:v>
+        <x:v>高层公寓客厅（夜）；公寓大楼走廊</x:v>
       </x:c>
       <x:c r="E24" s="2" t="str">
         <x:v>银色金属球棒</x:v>
@@ -2718,7 +2713,7 @@
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
-高层公寓玄关与电梯厅（文字设定·夜），9:16竖屏。走廊顶灯从上侧照清腕部接触，侧后壁灯勾出人物轮廓；动作关键区保持可读。
+高层公寓客厅（夜）；公寓大楼走廊，9:16竖屏。走廊顶灯从上侧照清腕部接触，侧后壁灯勾出人物轮廓；动作关键区保持可读。
 [音轨规则]
 远层：公寓外远处车流低声，室内维持安静。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
 本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
@@ -2727,10 +2722,9 @@
 9.1s—12.9s，@Ramón常服（对白，疼痛下的急促声演，原定呼喊词照原文发出，不再叠加额外叫声）：「Si me la rompes, nunca la vas a encontrar.」
 13.1s—20.5s，@Ramón常服（对白，疼痛下的急促声演，原定呼喊词照原文发出，不再叠加额外叫声）：「¡Al sur! ¡La vendimos al sur! A un hombre… ¡con tatuajes rojos en todo el cuello!」
 [锚定列表]
-场景：高层公寓玄关与电梯厅（文字设定·夜）
+场景：@高层公寓客厅（夜）；@公寓大楼走廊
 角色：@Vera常服；@Ramón常服；@Carmen常服
 道具：@银色金属球棒
-未带@的本段场景或物件按已授权的文字设计执行，保持下述位置、数量和状态。
 [空间布局总览]
 公寓门在走廊北墙，向公寓内开启；走廊东西向，电梯在东端。Vera常服起初在门内北侧，Ramón常服在门外正前，Carmen常服在其西侧，Escolta A在其东后侧。Escolta A已向东逃走。Vera常服在门外中央，右手持棒；Ramón常服在她西前方，Carmen常服在Ramón常服西侧；东端电梯门关闭。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
 [运镜时间线（7个硬切分镜）]
@@ -2834,7 +2828,7 @@
         <x:v>Vera常服</x:v>
       </x:c>
       <x:c r="D25" s="2" t="str">
-        <x:v>高层公寓玄关（文字设定·夜）</x:v>
+        <x:v>高层公寓客厅（夜）；公寓大楼走廊</x:v>
       </x:c>
       <x:c r="E25" s="2" t="str">
         <x:v>银色金属球棒</x:v>
@@ -2843,15 +2837,14 @@
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
-高层公寓玄关（文字设定·夜），9:16竖屏。走廊顶灯冷光照门口，室内暖侧光照到地毯边缘；暗部仍能读出肢体支撑。
+高层公寓客厅（夜）；公寓大楼走廊，9:16竖屏。走廊顶灯冷光照门口，室内暖侧光照到地毯边缘；暗部仍能读出肢体支撑。
 [音轨规则]
 远层：公寓外远处车流低声，室内维持安静。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
 本段无原定对白或旁白，不新增发声。
 [锚定列表]
-场景：高层公寓玄关（文字设定·夜）
+场景：@高层公寓客厅（夜）；@公寓大楼走廊
 角色：@Vera常服
 道具：@银色金属球棒
-未带@的本段场景或物件按已授权的文字设计执行，保持下述位置、数量和状态。
 [空间布局总览]
 公寓门在走廊北墙，向公寓内开启；走廊东西向，电梯在东端。Vera常服起初在门内北侧，Ramón常服在门外正前，Carmen常服在其西侧，Escolta A在其东后侧。电梯已关闭，Escolta A已逃离。Vera常服站公寓门外，门仍向内打开，球棒倚门外北墙。室内客厅通道在她身后。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
 [运镜时间线（4个硬切分镜）]

</xml_diff>

<commit_message>
Reconcile all 56 completed screenshot scene assets and bind existing car interior
</commit_message>
<xml_diff>
--- a/archive/projects/la-reina-del-bajo-mundo/deliverables/前夫黑道酵母_分镜_21-33.xlsx
+++ b/archive/projects/la-reina-del-bajo-mundo/deliverables/前夫黑道酵母_分镜_21-33.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分镜脚本" sheetId="1" r:id="Rc08d745346ed4f45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分镜脚本" sheetId="1" r:id="R3955e759d2fb4282"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -490,7 +490,7 @@
         <x:v>Vera常服；Emiliano常服</x:v>
       </x:c>
       <x:c r="D2" s="2" t="str">
-        <x:v>轿车内（文字设定·夜）</x:v>
+        <x:v>轿车内</x:v>
       </x:c>
       <x:c r="E2" s="2" t="str">
         <x:v>白色卡片（文字设定）</x:v>
@@ -499,7 +499,7 @@
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
-轿车内（文字设定·夜），9:16竖屏。车外旅馆霓虹在侧窗形成冷蓝边光，道路灯经前挡风玻璃斜侧透入；面部保留暗部。
+轿车内，9:16竖屏。车外旅馆霓虹在侧窗形成冷蓝边光，道路灯经前挡风玻璃斜侧透入；面部保留暗部。
 [音轨规则]
 远层：旅馆入口外的雨后道路车流与夜间底噪。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
 本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
@@ -508,7 +508,7 @@
 9.6s—11.1s，@Emiliano常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Entonces llámalo inversión.」
 11.3s—13.5s，@Emiliano常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Si pierdes, pierdo mi dinero.」
 [锚定列表]
-场景：轿车内（文字设定·夜）
+场景：@轿车内
 角色：@Vera常服；@Emiliano常服
 道具：白色卡片（文字设定）
 未带@的本段场景或物件按已授权的文字设计执行，保持下述位置、数量和状态。
@@ -600,7 +600,7 @@
         <x:v>Vera常服；Emiliano常服</x:v>
       </x:c>
       <x:c r="D3" s="2" t="str">
-        <x:v>汽车旅馆103房（外·夜）</x:v>
+        <x:v>汽车旅馆103房（外·夜）；轿车内</x:v>
       </x:c>
       <x:c r="E3" s="2" t="str">
         <x:v>白色卡片（文字设定）；轿车（文字设定）</x:v>
@@ -609,13 +609,13 @@
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
-汽车旅馆103房（外·夜），9:16竖屏。旅馆蓝色灯光形成侧逆光，门边实用灯照亮人行道；招牌光面不含字样。
+汽车旅馆103房（外·夜）；轿车内，9:16竖屏。旅馆蓝色灯光形成侧逆光，门边实用灯照亮人行道；招牌光面不含字样。
 [音轨规则]
 远层：旅馆入口外的雨后道路车流与夜间底噪。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
 本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
 6.6s—8.4s，@Vera常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Bonitos zapatos, por cierto.」
 [锚定列表]
-场景：@汽车旅馆103房（外·夜）
+场景：@汽车旅馆103房（外·夜）；@轿车内
 角色：@Vera常服；@Emiliano常服
 道具：白色卡片（文字设定）；轿车（文字设定）
 未带@的本段场景或物件按已授权的文字设计执行，保持下述位置、数量和状态。

</xml_diff>

<commit_message>
Complete episodes 26–30 storyboards with textual blocking and Loop checks
</commit_message>
<xml_diff>
--- a/archive/projects/la-reina-del-bajo-mundo/deliverables/前夫黑道酵母_分镜_21-33.xlsx
+++ b/archive/projects/la-reina-del-bajo-mundo/deliverables/前夫黑道酵母_分镜_21-33.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分镜脚本" sheetId="1" r:id="R3955e759d2fb4282"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分镜脚本" sheetId="1" r:id="R662051841b0a4ddf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2901,235 +2901,2195 @@
       </x:c>
     </x:row>
     <x:row r="26" ht="200" customHeight="1">
-      <x:c r="A26" s="2"/>
-      <x:c r="B26" s="2"/>
-      <x:c r="C26" s="2"/>
-      <x:c r="D26" s="2"/>
-      <x:c r="E26" s="2"/>
-      <x:c r="F26" s="2"/>
-      <x:c r="G26" s="2"/>
-      <x:c r="H26" s="2"/>
-      <x:c r="I26" s="2"/>
+      <x:c r="A26" s="2" t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B26" s="2" t="str">
+        <x:v>26-1A</x:v>
+      </x:c>
+      <x:c r="C26" s="2" t="str">
+        <x:v>Vera常服；Emiliano常服</x:v>
+      </x:c>
+      <x:c r="D26" s="2" t="str">
+        <x:v>高层公寓客厅（夜）</x:v>
+      </x:c>
+      <x:c r="E26" s="2" t="str">
+        <x:v>医用纱布；牛皮纸线索信封</x:v>
+      </x:c>
+      <x:c r="F26" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+高层公寓客厅（夜），9:16竖屏。客厅落地灯从北侧斜照手腕，东窗冷色夜光勾人物轮廓，纱布层次和指尖接触可读。
+[音轨规则]
+远层：公寓外远处车流低声，室内维持安静。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
+0.2s—1.3s，@Emiliano常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Última vuelta.」
+3.1s—4.6s，@Vera常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Está ganando tiempo.」
+[锚定列表]
+场景：@高层公寓客厅（夜）
+角色：@Vera常服；@Emiliano常服
+道具：医用纱布；牛皮纸线索信封
+未带@的物件仅作剧本所需普通文字描述，不冒充已完成资产或新增绑定。
+[空间布局总览]
+公寓入口在西墙，茶几位于客厅中部、沙发在北侧，东墙落地窗可见城市，书桌工作区位于窗侧；南侧移门通阳台，桌椅之间保留南侧通道。世界方位不随反打改变。Vera常服坐茶几东侧，Emiliano常服坐茶几西侧，两人面对面。Vera常服左前臂横放茶几；纱布已绕过腕部，卷筒在Emiliano常服右手，左手托其腕。信封在Vera常服右手边。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（5个硬切分镜）]
+分镜一：【景别/视角：双手近景/茶几南侧 | 运镜：沿桌沿缓移，落在最后一圈纱布】
+【时长】3.0s
+【构图】Emiliano常服左手托住Vera常服左腕，右手将最后一圈纱布沿既有方向绕好；卷筒不穿过手臂。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Emiliano常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】最后一圈已绕到腕背，Vera常服左手掌保持放松。
+【镜头结尾·站位收束】最后一圈已绕到腕背，Vera常服左手掌保持放松。
+画面硬切到分镜二。
+分镜二：【景别/视角：Vera常服侧面近景/茶几北侧 | 运镜：固定，Emiliano常服虚化肩线留在画边】
+【时长】3.0s
+【构图】Vera常服看着对方，眼睑稍收，直接指出他在拖延；左腕留在桌面，不抽手打断包扎。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Vera常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Vera常服仍坐桌东，左腕由Emiliano常服托着。
+【镜头结尾·站位收束】Vera常服仍坐桌东，左腕由Emiliano常服托着。
+画面硬切到分镜三。
+分镜三：【景别/视角：手腕与Emiliano常服中近景 | 运镜：从桌南侧轻推，保持结头和指尖可见】
+【时长】3.5s
+【构图】Emiliano常服放下纱布卷，将末端塞入已绕好的层间，再打平整小结，确认后双手离开。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】包扎完成，纱布卷留在桌西沿，Vera常服左腕自由。
+【镜头结尾·站位收束】包扎完成，纱布卷留在桌西沿，Vera常服左腕自由。
+画面硬切到分镜四。
+分镜四：【景别/视角：Emiliano常服近景/桌东南侧 | 运镜：固定，焦点从手腕回到脸部】
+【时长】3.0s
+【构图】Emiliano常服抬眼看Vera常服，再低眼看自己腕表；只保留一次短停顿，不补写对白。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】Emiliano常服仍坐桌西，目光回到信封。
+【镜头结尾·站位收束】Emiliano常服仍坐桌西，目光回到信封。
+画面硬切到分镜五。
+分镜五：【景别/视角：双人侧面中景 | 运镜：沿桌南侧短移，显示推送与接取】
+【时长】3.5s
+【构图】Vera常服左指轻触信封，改以右手把信封平推过茶几；Emiliano常服右手按住后取到自己面前。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】信封归Emiliano常服；他右手取出其中文件低头看纸背，Vera常服左腕纱布保持同一方向。
+【镜头结尾·站位收束】信封归Emiliano常服；他右手取出其中文件低头看纸背，Vera常服左腕纱布保持同一方向。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：16s</x:v>
+      </x:c>
+      <x:c r="G26" s="2" t="str">
+        <x:v>Emiliano：「Última vuelta.」
+Vera：「Está ganando tiempo.」</x:v>
+      </x:c>
+      <x:c r="H26" s="2" t="str">
+        <x:v>第26集
+26-1 高层公寓/客厅（Departamento ejecutivo, Piso 21, Reforma） 夜 内
+人物：Vera、Emiliano
+△ 镜头特写：Emiliano修长且指骨分明的手正在忙碌。他拿着一卷白色的医用纱布，一圈又一圈地缠绕在 Vera 的手腕上。
+Emiliano（低头专注，语气温和）：Última vuelta.
+△ 镜头近景：Vera 穿着米色风衣坐在对面，她的长发微乱，发丝垂在脸颊边。她静静地看着 Emiliano的动作，眼神中带着审视。
+Vera（语气冷淡，直接拆穿）：Está ganando tiempo.
+△ 动作特写：Emiliano将纱布的末端熟练地塞进缠绕好的缝隙中，并细心地打了一个平整的结。
+△ 镜头近景：Emiliano抬起头，他穿着笔挺的黑色三件套西装，神情深沉且难以捉摸。他并没有反驳，而是看了一眼手腕上的腕表。
+△ 镜头反打：Vera 抬起缠着白色纱布的左手，指尖轻触那个棕色的牛皮纸信封。她的指甲上还有些许干涸的血迹。
+△ 动作特写：Vera 伸出手，将信封推向Emiliano 的方向。
+△ 镜头切换：Emiliano 伸手接过信封，眼神在 Vera 脸上停留了片刻，随后低头看向信封内的文件。</x:v>
+      </x:c>
+      <x:c r="I26" s="2" t="str">
+        <x:v>16s</x:v>
+      </x:c>
     </x:row>
     <x:row r="27" ht="200" customHeight="1">
-      <x:c r="A27" s="2"/>
-      <x:c r="B27" s="2"/>
-      <x:c r="C27" s="2"/>
-      <x:c r="D27" s="2"/>
-      <x:c r="E27" s="2"/>
-      <x:c r="F27" s="2"/>
-      <x:c r="G27" s="2"/>
-      <x:c r="H27" s="2"/>
-      <x:c r="I27" s="2"/>
+      <x:c r="A27" s="2" t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B27" s="2" t="str">
+        <x:v>26-2A</x:v>
+      </x:c>
+      <x:c r="C27" s="2" t="str">
+        <x:v>Vera常服；Ramón常服；Carmen常服</x:v>
+      </x:c>
+      <x:c r="D27" s="2" t="str">
+        <x:v>汽车旅馆103房（内·夜）</x:v>
+      </x:c>
+      <x:c r="E27" s="2" t="str">
+        <x:v>纸质证据；房屋照片</x:v>
+      </x:c>
+      <x:c r="F27" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+汽车旅馆103房（内·夜），9:16竖屏。床头暖灯与书桌屏幕侧后冷光分区；屏幕背向摄影机，光面无文字，脸部曝光不随切镜改变。
+[音轨规则]
+远层：夜间空间的低弱环境底噪。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
+6.1s—9.6s，@Ramón常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Tú... tú no puedes probar nada.」
+9.8s—16.5s，@Vera常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Incendio por el seguro. Quinientos mil pesos por una niña. Ese caso nunca se cerró.」
+[锚定列表]
+场景：@汽车旅馆103房（内·夜）
+角色：@Vera常服；@Ramón常服；@Carmen常服
+道具：纸质证据；房屋照片
+未带@的物件仅作剧本所需普通文字描述，不冒充已完成资产或新增绑定。
+[空间布局总览]
+103房门位于西墙并向室内开启，床在北侧，书桌在东墙窗边，门旁柜在西南角。Vera常服在书桌西侧，Ramón常服与Carmen常服由西门入内后留在南侧床尾空道。门已打开，Vera常服左腕纱布仍在，笔记本在书桌东侧、纸质证据在桌面中央。照片起初压在纸叠下。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（6个硬切分镜）]
+分镜一：【景别/视角：房间全景/门内南侧 | 运镜：由门边向东短移，展示床尾通道】
+【时长】3.0s
+【构图】Ramón常服与Carmen常服跨门槛进来后停在床尾，Vera常服在书桌西侧面对他们；入口仍在两人身后。
+【音效】门扇与门锁随实际开合发声；台词期间压低动作声。
+【台词】无台词。
+【变化】三人分处门侧与桌侧，笔记本朝Vera常服。
+【镜头结尾·站位收束】三人分处门侧与桌侧，笔记本朝Vera常服。
+画面硬切到分镜二。
+分镜二：【景别/视角：纸张与Vera常服中近景 | 运镜：固定，纸叠与两位来客同框】
+【时长】3.0s
+【构图】Vera常服右手抓起桌上纸叠，向两人面前低位甩出；纸页散开后落在床尾空道，不遮住人物整个身体。
+【音效】纸张轻擦声；台词期间压低动作声。
+【台词】无台词。
+【变化】右手已放开纸叠，部分纸页落地。
+【镜头结尾·站位收束】右手已放开纸叠，部分纸页落地。
+画面硬切到分镜三。
+分镜三：【景别/视角：Ramón常服近景/桌侧反打 | 运镜：缓推至他停住的视线】
+【时长】3.5s
+【构图】Ramón常服盯着落地纸张，再抬眼看Vera常服，说话先迟疑后试图否认；Carmen常服在他旁边。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Ramón常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Ramón常服双脚仍在床尾，未跨到书桌。
+【镜头结尾·站位收束】Ramón常服双脚仍在床尾，未跨到书桌。
+画面硬切到分镜四。
+分镜四：【景别/视角：Vera常服中近景/床尾向东 | 运镜：固定，手指与纸背在画面下部】
+【时长】4.0s
+【构图】Vera常服左手指向桌上发黄单据的边缘，字面朝自己；她平稳说出金额与纵火案事实，右手撑桌。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Ramón常服的对白按本段唯一声音骨架连续发声；@Vera常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】左腕纱布不变，单据在桌面。
+【镜头结尾·站位收束】左腕纱布不变，单据在桌面。
+画面硬切到分镜五。
+分镜五：【景别/视角：Ramón常服与桌沿关系中景 | 运镜：向南侧短移形成照片与听者的纵深】
+【时长】3.0s
+【构图】Vera常服的原声继续，右手将房屋照片从纸叠下滑出，转向两位来客；照片仅呈建筑影像。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Vera常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】照片平放桌西沿，字面不入画，Ramón常服看向它。
+【镜头结尾·站位收束】照片平放桌西沿，字面不入画，Ramón常服看向它。
+画面硬切到分镜六。
+分镜六：【景别/视角：Carmen常服侧面近景 | 运镜：固定，Ramón常服肩部为前景】
+【时长】3.0s
+【构图】Carmen常服左手攥住自己衣袖，Ramón常服下颌停住，二人不再对视；不新增同步颤抖与抽气。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】两人留床尾，Vera常服在书桌边。
+【镜头结尾·站位收束】两人留床尾，Vera常服在书桌边。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：19.5s</x:v>
+      </x:c>
+      <x:c r="G27" s="2" t="str">
+        <x:v>Ramón：「Tú... tú no puedes probar nada.」
+Vera：「Incendio por el seguro. Quinientos mil pesos por una niña. Ese caso nunca se cerró.」</x:v>
+      </x:c>
+      <x:c r="H27" s="2" t="str">
+        <x:v>26-2 汽车旅馆103房（Motel Vista Pacífico, 103） 夜 内
+人物：Vera、Ramón、Carmen
+△ 镜头特写：一扇墨绿色的木门被推开。
+△ 镜头近景：Ramón 和 Carmen 局促地站在门口，两人的衣服都显得有些破旧。Ramón 依然是一脸市侩的苦相，而 Carmen 眼神躲闪，显得非常不安。
+△ 镜头全景：这是一间昏暗且简陋的汽车旅馆房间。Vera 穿着米色风衣站在桌边，桌上放着一台运行中的笔记本电脑，屏幕上显示着复杂的建筑结构图和账目。
+△ 动作特写：Vera 冷漠地抓起桌上的一叠文件，用力一挥。
+△ 镜头切换：白色纸张如雪片般撒向对面的两人，在空中凌乱飞舞。
+Ramón（神情紧绷，试图狡辩）：Tú... tú no puedes probar nada.
+△ 动作特写：Vera 伸出缠着纱布的手指，重重地按在桌上的一张发黄的单据上。
+△ 镜头特写：单据的抬头印着"COMERCIALIZADORA DEL GOLFO Y CIA."，底部金额显示为"$500,000.00"。
+Vera（语气冰冷）：Incendio por el seguro. Quinientos mil pesos por una niña. Ese caso nunca se cerró.
+△ 动作特写：Vera 挪动手拍在另一张彩色照片上。照片里是一栋城郊的老式独栋住宅。
+△ 镜头近景：Ramón 盯着照片，喉结上下滚动，额头渗出冷汗。</x:v>
+      </x:c>
+      <x:c r="I27" s="2" t="str">
+        <x:v>19.5s</x:v>
+      </x:c>
     </x:row>
     <x:row r="28" ht="200" customHeight="1">
-      <x:c r="A28" s="2"/>
-      <x:c r="B28" s="2"/>
-      <x:c r="C28" s="2"/>
-      <x:c r="D28" s="2"/>
-      <x:c r="E28" s="2"/>
-      <x:c r="F28" s="2"/>
-      <x:c r="G28" s="2"/>
-      <x:c r="H28" s="2"/>
-      <x:c r="I28" s="2"/>
+      <x:c r="A28" s="2" t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B28" s="2" t="str">
+        <x:v>26-2B</x:v>
+      </x:c>
+      <x:c r="C28" s="2" t="str">
+        <x:v>Vera常服；Ramón常服；Carmen常服</x:v>
+      </x:c>
+      <x:c r="D28" s="2" t="str">
+        <x:v>汽车旅馆103房（内·夜）</x:v>
+      </x:c>
+      <x:c r="E28" s="2" t="str">
+        <x:v>纸质证据；房屋照片</x:v>
+      </x:c>
+      <x:c r="F28" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+汽车旅馆103房（内·夜），9:16竖屏。暖床头灯切出两名来客的侧脸，屏幕冷光仅在桌边和Vera常服侧面提供低弱反射。
+[音轨规则]
+远层：夜间空间的低弱环境底噪。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
+0.2s—7.8s，@Vera常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「¿Y la casa donde se esconden? Es de un prestamista que ni los Vargas se atreven a cruzar.」
+8.1s—12.3s，@Vera常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Dos opciones. La cárcel... o leen mi guion.」
+12.5s—14.7s，@Carmen常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「¡De cualquier modo estamos muertos!」
+[锚定列表]
+场景：@汽车旅馆103房（内·夜）
+角色：@Vera常服；@Ramón常服；@Carmen常服
+道具：纸质证据；房屋照片
+未带@的物件仅作剧本所需普通文字描述，不冒充已完成资产或新增绑定。
+[空间布局总览]
+103房门位于西墙并向室内开启，床在北侧，书桌在东墙窗边，门旁柜在西南角。Vera常服在书桌西侧，Ramón常服与Carmen常服由西门入内后留在南侧床尾空道。Vera常服站书桌西侧，Ramón常服与Carmen常服在南侧床尾。房屋照片在桌西沿，笔记本朝Vera常服，装订文件压在桌北侧。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（5个硬切分镜）]
+分镜一：【景别/视角：Vera常服侧面中近景 | 运镜：沿桌南侧轻推，落在她指向照片的右手】
+【时长】4.0s
+【构图】Vera常服点一下房屋照片后抬眼看Ramón常服，明确说出房屋背后的威胁；右手离开照片后停在桌沿。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Vera常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】照片未换位置，两人仍在床尾。
+【镜头结尾·站位收束】照片未换位置，两人仍在床尾。
+画面硬切到分镜二。
+分镜二：【景别/视角：Ramón常服听者近景 | 运镜：从Vera常服肩后固定观察，不反复重启反应】
+【时长】4.0s
+【构图】Vera常服的声音跨切继续；Ramón常服目光从照片移开，唇部短暂压紧；Carmen常服不抢话。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Vera常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】上句完整结束，Ramón常服还没有回应。
+【镜头结尾·站位收束】上句完整结束，Ramón常服还没有回应。
+画面硬切到分镜三。
+分镜三：【景别/视角：文件与双人中景 | 运镜：向桌西侧轻移，保留推送路径】
+【时长】4.0s
+【构图】Vera常服从桌北拿起装订文件，平推到床尾方向的桌沿，给出两种选择；纸面侧背镜头。
+【音效】纸张轻擦声；台词期间压低动作声。
+【台词】@Vera常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】装订文件在桌西沿，Vera常服双手已离文件。
+【镜头结尾·站位收束】装订文件在桌西沿，Vera常服双手已离文件。
+画面硬切到分镜四。
+分镜四：【景别/视角：Carmen常服近景 | 运镜：固定，手部抓住Ramón常服袖口的动作在画内】
+【时长】3.0s
+【构图】Carmen常服抓住Ramón常服左袖，开口说出原定感叹句；声音沙哑急促，词语清楚，不另添尖叫。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Vera常服的对白按本段唯一声音骨架连续发声；@Carmen常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Carmen常服仍抓左袖，Ramón常服保持站立。
+【镜头结尾·站位收束】Carmen常服仍抓左袖，Ramón常服保持站立。
+画面硬切到分镜五。
+分镜五：【景别/视角：Vera常服与门口纵深中景 | 运镜：轻向后拉，留出西侧出口方向】
+【时长】3.0s
+【构图】Vera常服听完后收回放在桌沿的手，身体转向西门；两位来客仍在原位置。
+【音效】门扇与门锁随实际开合发声；台词期间压低动作声。
+【台词】无台词。
+【变化】Vera常服面向出口，文件与照片留在桌上。
+【镜头结尾·站位收束】Vera常服面向出口，文件与照片留在桌上。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：18s</x:v>
+      </x:c>
+      <x:c r="G28" s="2" t="str">
+        <x:v>Vera：「¿Y la casa donde se esconden? Es de un prestamista que ni los Vargas se atreven a cruzar.」
+Vera：「Dos opciones. La cárcel... o leen mi guion.」
+Carmen：「¡De cualquier modo estamos muertos!」</x:v>
+      </x:c>
+      <x:c r="H28" s="2" t="str">
+        <x:v>Vera：¿Y la casa donde se esconden? Es de un prestamista que ni los Vargas se atreven a cruzar.
+△ 镜头反打：Vera 盯着两人，眼神犀利如刃，她从桌上推过去一份装订好的纸质文件。
+Vera（给出最后通牒）：Dos opciones. La cárcel... o leen mi guion.
+△ 镜头切到 Carmen：她由于极度的恐惧，苍老的双手剧烈颤抖，紧紧抓着 Ramón 的衣袖，近乎崩溃地哭喊出来。
+Carmen（声音嘶哑）：¡De cualquier modo estamos muertos!</x:v>
+      </x:c>
+      <x:c r="I28" s="2" t="str">
+        <x:v>18s</x:v>
+      </x:c>
     </x:row>
     <x:row r="29" ht="200" customHeight="1">
-      <x:c r="A29" s="2"/>
-      <x:c r="B29" s="2"/>
-      <x:c r="C29" s="2"/>
-      <x:c r="D29" s="2"/>
-      <x:c r="E29" s="2"/>
-      <x:c r="F29" s="2"/>
-      <x:c r="G29" s="2"/>
-      <x:c r="H29" s="2"/>
-      <x:c r="I29" s="2"/>
+      <x:c r="A29" s="2" t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B29" s="2" t="str">
+        <x:v>26-3A</x:v>
+      </x:c>
+      <x:c r="C29" s="2" t="str">
+        <x:v>Vera常服；Ramón常服；Carmen常服</x:v>
+      </x:c>
+      <x:c r="D29" s="2" t="str">
+        <x:v>汽车旅馆103房（内·夜）</x:v>
+      </x:c>
+      <x:c r="E29" s="2" t="str">
+        <x:v>现金；纸质证据</x:v>
+      </x:c>
+      <x:c r="F29" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+汽车旅馆103房（内·夜），9:16竖屏。床头暖灯从侧后照人物，门口落暗但门把与柜台接触区可读。
+[音轨规则]
+远层：夜间空间的低弱环境底噪。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
+3.1s—7.7s，@Vera常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Los Vargas les pagaron quinientos mil por leer el de ellos.」
+10.1s—15.1s，@Vera常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Pregúntense... después de la conferencia, ¿los van a dejar gastarlo?」
+[锚定列表]
+场景：@汽车旅馆103房（内·夜）
+角色：@Vera常服；@Ramón常服；@Carmen常服
+道具：现金；纸质证据
+未带@的物件仅作剧本所需普通文字描述，不冒充已完成资产或新增绑定。
+[空间布局总览]
+103房门位于西墙并向室内开启，床在北侧，书桌在东墙窗边，门旁柜在西南角。Vera常服在书桌西侧，Ramón常服与Carmen常服由西门入内后留在南侧床尾空道。Vera常服由书桌西侧沿床尾北边的空道走向西门，左腕有纱布；Ramón常服与Carmen常服在床尾南侧，不堵门。现金在Vera常服右侧外套口袋内，门边柜台空着。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（6个硬切分镜）]
+分镜一：【景别/视角：侧后中景/书桌至门口 | 运镜：向西跟随Vera常服，速度随她停步减缓】
+【时长】3.0s
+【构图】Vera常服离开书桌走到门口，左手搭门把，右手仍垂在外套口袋旁；两位来客留在后方。
+【音效】门扇与门锁随实际开合发声、脚步随起停出现；台词期间压低动作声。
+【台词】无台词。
+【变化】Vera常服站门内，门还未推开。
+【镜头结尾·站位收束】Vera常服站门内，门还未推开。
+画面硬切到分镜二。
+分镜二：【景别/视角：Vera常服侧面近景/门旁柜侧 | 运镜：固定，视线回到两位来客】
+【时长】4.0s
+【构图】Vera常服稍回头看向Ramón常服与Carmen常服，提醒他们已收过Vargas的钱，语气平而冷。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Vera常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】左手仍搭门把，右手尚未取现金。
+【镜头结尾·站位收束】左手仍搭门把，右手尚未取现金。
+画面硬切到分镜三。
+分镜三：【景别/视角：现金与柜台近景 | 运镜：沿门边柜面短移后停住】
+【时长】3.0s
+【构图】Vera常服右手从口袋取出整叠现金，低位放到门边柜台，指尖离开后纸钞落稳；现金正面不呈现字样。
+【音效】门扇与门锁随实际开合发声、纸张轻擦声；台词期间压低动作声。
+【台词】@Vera常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】现金留柜台，Vera常服右手空出。
+【镜头结尾·站位收束】现金留柜台，Vera常服右手空出。
+画面硬切到分镜四。
+分镜四：【景别/视角：Ramón常服听者近景/床尾 | 运镜：固定，以门边现金作模糊前景】
+【时长】4.0s
+【构图】Ramón常服看向现金后抬眼，Vera常服在画外发出第二句警告；Carmen常服目光也落到柜边。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Vera常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】两人仍未上前取钱。
+【镜头结尾·站位收束】两人仍未上前取钱。
+画面硬切到分镜五。
+分镜五：【景别/视角：双人中景/床尾南侧 | 运镜：缓慢后拉，让出口与两人保持同框】
+【时长】3.0s
+【构图】Vera常服的声音完整结束，两位来客短暂交换目光；Carmen常服手指放开袖口，不新增倒吸气。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Vera常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Ramón常服与Carmen常服都留在床尾，现金留柜台。
+【镜头结尾·站位收束】Ramón常服与Carmen常服都留在床尾，现金留柜台。
+画面硬切到分镜六。
+分镜六：【景别/视角：门侧全身中景 | 运镜：固定，完整保留门扇与门槛】
+【时长】3.0s
+【构图】Vera常服左手推开门，侧身跨出门槛后带上门；相机留在房内，不穿过门板。
+【音效】门扇与门锁随实际开合发声；台词期间压低动作声。
+【台词】无台词。
+【变化】Vera常服已离场，门关上，现金与两人留室内。
+【镜头结尾·站位收束】Vera常服已离场，门关上，现金与两人留室内。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：20s</x:v>
+      </x:c>
+      <x:c r="G29" s="2" t="str">
+        <x:v>Vera：「Los Vargas les pagaron quinientos mil por leer el de ellos.」
+Vera：「Pregúntense... después de la conferencia, ¿los van a dejar gastarlo?」</x:v>
+      </x:c>
+      <x:c r="H29" s="2" t="str">
+        <x:v>26-3 汽车旅馆103房/门口（Motel Vista Pacífico, 103） 夜 内
+人物：Vera、Ramón、Carmen
+△ 动作特写：Vera 并没有理会老妇人的哀求，她转过身，米色风衣的衣摆在空中划过一个冷硬的弧度，径直向门口走去。
+△ 镜头跟随：Vera 走到门口，手搭在门把手上，身姿笔挺而孤傲。
+△ 镜头切到 Vera 的侧脸特写：她停下脚步，微微侧过头，眼角的余光扫过身后颓然的两人。
+Vera（声音不带一丝温度）：Los Vargas les pagaron quinientos mil por leer el de ellos.
+△ 动作特写：Vera 反手将厚厚的一叠现金摔在门边的柜子上。钞票发出沉闷的撞击声。
+△ 镜头近景：Ramón 的目光瞬间被那叠现金锁死，原本绝望的眼神中透出一丝疯狂的贪婪。
+Vera：Pregúntense... después de la conferencia, ¿los van a dejar gastarlo?
+△ 镜头切到 Ramón 和 Carmen：两人面面相觑，Ramón 的眼中充满了极度的动摇，而 Carmen 惊恐地瞪大了双眼，倒吸一口冷气。
+△ 画面收尾：Vera 果断推门而出，将两人留在了充满死亡气息的沉默中。</x:v>
+      </x:c>
+      <x:c r="I29" s="2" t="str">
+        <x:v>20s</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="200" customHeight="1">
-      <x:c r="A30" s="2"/>
-      <x:c r="B30" s="2"/>
-      <x:c r="C30" s="2"/>
-      <x:c r="D30" s="2"/>
-      <x:c r="E30" s="2"/>
-      <x:c r="F30" s="2"/>
-      <x:c r="G30" s="2"/>
-      <x:c r="H30" s="2"/>
-      <x:c r="I30" s="2"/>
+      <x:c r="A30" s="2" t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="B30" s="2" t="str">
+        <x:v>27-1A</x:v>
+      </x:c>
+      <x:c r="C30" s="2" t="str">
+        <x:v>Ramón常服；Vera常服；Emiliano常服；Damián常服；Bárbara常服；Carmen常服；Escolta A常服</x:v>
+      </x:c>
+      <x:c r="D30" s="2" t="str">
+        <x:v>发布会现场</x:v>
+      </x:c>
+      <x:c r="E30" s="2" t="str">
+        <x:v>白色发言稿；麦克风</x:v>
+      </x:c>
+      <x:c r="F30" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+发布会现场，9:16竖屏。会场顶灯均匀照亮座席，讲台侧方已有摄影灯给人物侧光；背景板保留色块，不出现文字或标志字形。
+[音轨规则]
+远层：日间会场低弱人群底噪，快门声低于原台词。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
+3.1s—5.5s，@Ramón常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Mi hija Vera Saldaña...」
+6.1s—8.8s，@Ramón常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「...es una buena chica.」
+9.1s—14.1s，@Ramón常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Los Vargas vinieron a vernos... nos dieron quinientos mil pesos.」
+15.1s—20.8s，@Ramón常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Nos dijeron que la llamáramos loca. Que dijéramos que ella prendió el fuego.」
+[锚定列表]
+场景：@发布会现场
+角色：@Ramón常服；@Vera常服；@Emiliano常服；@Damián常服；@Bárbara常服；@Carmen常服；@Escolta A常服
+道具：白色发言稿；麦克风
+未带@的物件仅作剧本所需普通文字描述，不冒充已完成资产或新增绑定。
+[空间布局总览]
+发布会讲台在北侧矮台上，座席面向北；中央通道南北向，两侧各有通行边道，出入口在南墙。Ramón常服在讲台后，Vera常服坐前排西侧，Emiliano常服在其西侧，Damián常服与Bárbara常服坐后排东侧相邻座位。Carmen常服起初在讲台东侧台下，Escolta A在东边道。三名背景员工在后排西侧，仅作观众。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（7个硬切分镜）]
+分镜一：【景别/视角：会场关系全景/南端中央通道 | 运镜：沿中轴向北短推，落在讲台与前排关系】
+【时长】3.0s
+【构图】Ramón常服站讲台后，Vera常服与Emiliano常服在前排西侧，Damián常服与Bárbara常服在后排东侧；Carmen常服在舞台东端台下。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】所有人物的楼层与座席关系成立。
+【镜头结尾·站位收束】所有人物的楼层与座席关系成立。
+画面硬切到分镜二。
+分镜二：【景别/视角：Ramón常服正面偏侧近景 | 运镜：从讲台西侧固定，麦克风仍固定于讲台支架、在嘴前下方】
+【时长】3.0s
+【构图】Ramón常服面对记者开口，声音略沙哑；说到女儿名字后稍停，右手落在稿纸边。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Ramón常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Ramón常服停顿，未离开讲台。
+【镜头结尾·站位收束】Ramón常服停顿，未离开讲台。
+画面硬切到分镜三。
+分镜三：【景别/视角：Vera常服近景/前排东南侧 | 运镜：轻向左平移，露出她与舞台的视线线索】
+【时长】3.0s
+【构图】Vera常服看向讲台，唇角略松但不夸张笑；Ramón常服声音从北侧画外补完句子。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Ramón常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Vera常服仍坐前排，Emiliano常服在她西侧。
+【镜头结尾·站位收束】Vera常服仍坐前排，Emiliano常服在她西侧。
+画面硬切到分镜四。
+分镜四：【景别/视角：讲台稿纸手部近景 | 运镜：由讲台西侧向纸背轻推】
+【时长】3.0s
+【构图】Ramón常服右手从台下取出白色发言稿，左手扶稿，纸面朝自己；抬头继续读。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Ramón常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】稿纸在Ramón常服双手，画面不呈现字迹。
+【镜头结尾·站位收束】稿纸在Ramón常服双手，画面不呈现字迹。
+画面硬切到分镜五。
+分镜五：【景别/视角：Ramón常服侧面中近景 | 运镜：固定，台下听众虚化在背景】
+【时长】3.0s
+【构图】Ramón常服的原声继续到完整金额，手指只在纸边轻擦一次。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Ramón常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】第一项指控完整结束，纸张仍在双手。
+【镜头结尾·站位收束】第一项指控完整结束，纸张仍在双手。
+画面硬切到分镜六。
+分镜六：【景别/视角：Vera常服过肩望Ramón常服中景 | 运镜：在前排西侧向北轻推，保持舞台距离】
+【时长】4.0s
+【构图】Ramón常服继续说出被要求造谣的内容，Vera常服背影留在近处；听众视线逐渐集中于讲台。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Ramón常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Ramón常服站位未变，稿纸仍在讲台上方。
+【镜头结尾·站位收束】Ramón常服站位未变，稿纸仍在讲台上方。
+画面硬切到分镜七。
+分镜七：【景别/视角：后排关系中景/东边道 | 运镜：横移显出Damián常服与Bárbara常服相邻座位】
+【时长】3.0s
+【构图】Ramón常服声音结束，Damián常服手掌在膝上收紧；Bárbara常服看向讲台，嘴唇稍分开后收住。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Ramón常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】两人仍坐在后排，Escolta A在东边道。
+【镜头结尾·站位收束】两人仍坐在后排，Escolta A在东边道。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：22s</x:v>
+      </x:c>
+      <x:c r="G30" s="2" t="str">
+        <x:v>Ramón：「Mi hija Vera Saldaña...」
+Ramón：「...es una buena chica.」
+Ramón：「Los Vargas vinieron a vernos... nos dieron quinientos mil pesos.」
+Ramón：「Nos dijeron que la llamáramos loca. Que dijéramos que ella prendió el fuego.」</x:v>
+      </x:c>
+      <x:c r="H30" s="2" t="str">
+        <x:v>第27集
+27-1 发布会现场（Sala de prensa） 日 内
+人物：Ramón、Vera、Bárbara、Damián、Emiliano、Carmen、Escolta A、Empleado A、Empleado B、Empleado C
+△ 画面特写：Ramón 站在讲台后，微微低头靠近麦克风，眼神深沉。他由于情绪激动，呼吸显得有些沉重。
+Ramón（声音沙哑，带着一丝决绝）：Mi hija Vera Saldaña...
+△ 镜头反打：Vera 坐在台下，神情恬淡。她微微侧头，嘴角挂着一抹若有若无的笑意，眼神中透着一种掌控全局的自信。
+Ramón：...es una buena chica.
+△ 镜头特写：Vera 轻轻眨动眼睫，眼神明亮。
+△ 镜头切到 Ramón：他从讲台下拿出一份白色的文件，手指在纸张边缘摩擦。
+Ramón（低头读稿，声音略微颤抖）：Los Vargas vinieron a vernos... nos dieron quinientos mil pesos.
+△ 镜头全景：发布会大厅内灯光亮堂。Ramón 站在台上，背后是印有蓝色圆形标志的背景板。
+Ramón：Nos dijeron que la llamáramos loca. Que dijéramos que ella prendió el fuego.</x:v>
+      </x:c>
+      <x:c r="I30" s="2" t="str">
+        <x:v>22s</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="200" customHeight="1">
-      <x:c r="A31" s="2"/>
-      <x:c r="B31" s="2"/>
-      <x:c r="C31" s="2"/>
-      <x:c r="D31" s="2"/>
-      <x:c r="E31" s="2"/>
-      <x:c r="F31" s="2"/>
-      <x:c r="G31" s="2"/>
-      <x:c r="H31" s="2"/>
-      <x:c r="I31" s="2"/>
+      <x:c r="A31" s="2" t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="B31" s="2" t="str">
+        <x:v>27-1B</x:v>
+      </x:c>
+      <x:c r="C31" s="2" t="str">
+        <x:v>Ramón常服；Carmen常服；Bárbara常服；Escolta A常服；Vera常服；Emiliano常服；Damián常服</x:v>
+      </x:c>
+      <x:c r="D31" s="2" t="str">
+        <x:v>发布会现场</x:v>
+      </x:c>
+      <x:c r="E31" s="2" t="str">
+        <x:v>麦克风；白色发言稿</x:v>
+      </x:c>
+      <x:c r="F31" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+发布会现场，9:16竖屏。沿用会场顶灯与讲台侧光，快门闪光仅短促出现，不持续洗白脸部。
+[音轨规则]
+远层：日间会场低弱人群底噪，快门声低于原台词。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
+3.1s—5.6s，@Carmen常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「¡No teníamos nada! ¡Nos usaron!」
+6.6s—9.7s，@Carmen常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「¡Nos vamos a retractar! Ellos...」
+12.6s—13.5s，@Bárbara常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「¡Esperen!」
+[锚定列表]
+场景：@发布会现场
+角色：@Ramón常服；@Carmen常服；@Bárbara常服；@Escolta A常服；@Vera常服；@Emiliano常服；@Damián常服
+道具：麦克风；白色发言稿
+未带@的物件仅作剧本所需普通文字描述，不冒充已完成资产或新增绑定。
+[空间布局总览]
+发布会讲台在北侧矮台上，座席面向北；中央通道南北向，两侧各有通行边道，出入口在南墙。Ramón常服在讲台后，Vera常服坐前排西侧，Emiliano常服在其西侧，Damián常服与Bárbara常服坐后排东侧相邻座位。Carmen常服起初在讲台东侧台下，Escolta A在东边道。三名背景员工在后排西侧，仅作观众。Ramón常服站讲台后，麦克风固定于讲台支架，稿纸压在讲台。Carmen常服将从东侧台阶上台；Bárbara常服仍坐后排东侧。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（6个硬切分镜）]
+分镜一：【景别/视角：讲台侧面中景/东侧台阶 | 运镜：沿东边道向北轻摇，完整跟到台阶顶】
+【时长】3.0s
+【构图】Carmen常服沿台阶上台，走到Ramón常服右侧；右手握住麦克风下部，从支架抽起后举到嘴前，Ramón常服不再靠近支架。
+【音效】脚步随起停出现；台词期间压低动作声。
+【台词】无台词。
+【变化】Carmen常服站台上，麦克风在右手，Ramón常服退开半步。
+【镜头结尾·站位收束】Carmen常服站台上，麦克风在右手，Ramón常服退开半步。
+画面硬切到分镜二。
+分镜二：【景别/视角：Carmen常服近景 | 运镜：固定在讲台西侧，保护发声口型】
+【时长】3.5s
+【构图】Carmen常服举麦克风说出原句，声音激动但不把全部词都喊破；左手按讲台边。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Carmen常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Carmen常服在台上站稳，麦克风未换手。
+【镜头结尾·站位收束】Carmen常服在台上站稳，麦克风未换手。
+画面硬切到分镜三。
+分镜三：【景别/视角：听众中景/西边道 | 运镜：由前排向后短移，显示不同人物反应】
+【时长】3.0s
+【构图】Carmen常服继续发声，观众转头交换目光；三名背景员工留后排西侧，Damián常服和Bárbara常服仍在东侧。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Carmen常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】听众未涌向舞台。
+【镜头结尾·站位收束】听众未涌向舞台。
+画面硬切到分镜四。
+分镜四：【景别/视角：东边道全景 | 运镜：由台阶向南摇摄，落在Bárbara常服座位区】
+【时长】3.0s
+【构图】一名普通安保到台阶边维持秩序，Escolta A沿东边道走到后排Bárbara常服座侧；不从舞台直接跳到座席。
+【音效】脚步随起停出现；台词期间压低动作声。
+【台词】@Carmen常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Escolta A在Bárbara常服右侧，另一安保在台阶边。
+【镜头结尾·站位收束】Escolta A在Bárbara常服右侧，另一安保在台阶边。
+画面硬切到分镜五。
+分镜五：【景别/视角：Bárbara常服与Escolta A双人中近景 | 运镜：在座位前侧固定，手臂接触清楚】
+【时长】3.0s
+【构图】Escolta A握住Bárbara常服两上臂，Bárbara常服先把双脚收至座椅下方，借力起身并说出原定阻止词。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Bárbara常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Bárbara常服已离座，Escolta A仍控制其上臂。
+【镜头结尾·站位收束】Bárbara常服已离座，Escolta A仍控制其上臂。
+画面硬切到分镜六。
+分镜六：【景别/视角：后排座位与边道中景 | 运镜：向后拉出离开座席的空道】
+【时长】3.0s
+【构图】Bárbara常服踉跄一步后稳住脚，Escolta A将她带到东边道；Damián常服留在座位旁，Vera常服仍在前排。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】Bárbara常服进入东边道，舞台两人仍在台上。
+【镜头结尾·站位收束】Bárbara常服进入东边道，舞台两人仍在台上。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：18.5s</x:v>
+      </x:c>
+      <x:c r="G31" s="2" t="str">
+        <x:v>Carmen：「¡No teníamos nada! ¡Nos usaron!」
+Carmen：「¡Nos vamos a retractar! Ellos...」
+Bárbara：「¡Esperen!」</x:v>
+      </x:c>
+      <x:c r="H31" s="2" t="str">
+        <x:v>△ 动作特写：老妇人 Carmen 突然冲上台，她头发凌乱，神情惊恐且扭曲，猛地夺过 Ramón 手中的麦克风。
+Carmen（声嘶力竭地尖叫）：¡No teníamos nada! ¡Nos usaron!
+△ 镜头全景：台下乱成一团。原本整齐坐着的宾客和员工们纷纷侧头，露出震惊和不可思议的表情。
+Carmen：¡Nos vamos a retractar! Ellos...
+△ 镜头近景：后排的员工们（Empleado A、Empleado B、Empleado C）面露惊惧。Damián 穿着棕灰色西装站在人群中，眉头紧锁，脸色极其难看。他身边的 Bárbara 穿着粉色丝绸礼服，张大嘴巴，眼神中充满了难以置信。
+△ 动作特写：两名安保人员冲上台。Escolta A 粗鲁地抓住 Bárbara 的双臂，试图将她从座位上带走。
+Bárbara（惊恐地挣扎）：¡Esperen!
+△ 镜头切到 Bárbara：她被 Escolta A 强行拉起，身体失衡，在混乱中显得狼狈不堪。</x:v>
+      </x:c>
+      <x:c r="I31" s="2" t="str">
+        <x:v>18.5s</x:v>
+      </x:c>
     </x:row>
     <x:row r="32" ht="200" customHeight="1">
-      <x:c r="A32" s="2"/>
-      <x:c r="B32" s="2"/>
-      <x:c r="C32" s="2"/>
-      <x:c r="D32" s="2"/>
-      <x:c r="E32" s="2"/>
-      <x:c r="F32" s="2"/>
-      <x:c r="G32" s="2"/>
-      <x:c r="H32" s="2"/>
-      <x:c r="I32" s="2"/>
+      <x:c r="A32" s="2" t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="B32" s="2" t="str">
+        <x:v>27-2A</x:v>
+      </x:c>
+      <x:c r="C32" s="2" t="str">
+        <x:v>Damián常服；Víctor常服</x:v>
+      </x:c>
+      <x:c r="D32" s="2" t="str">
+        <x:v>庄园大厅</x:v>
+      </x:c>
+      <x:c r="E32" s="2" t="str">
+        <x:v>白色方巾；老式电话机</x:v>
+      </x:c>
+      <x:c r="F32" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+庄园大厅，9:16竖屏。壁炉暖火为近处侧光，窗帘缝隙透日间冷白环境光，镜框与裂纹有真实反射；不照出虚构人影。
+[音轨规则]
+远层：夜间空间的低弱环境底噪。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
+6.1s—7.6s，@Víctor常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「No es suerte.」
+9.1s—12.4s，@Víctor常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Nos lleva tres pasos de ventaja. Siempre.」
+15.6s—17.4s，@Víctor常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Consígueme a Ernesto Miranda.」
+18.6s—22.4s，@Víctor常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Dile... que tenemos un problema en común.」
+[锚定列表]
+场景：@庄园大厅
+角色：@Damián常服；@Víctor常服
+道具：白色方巾；老式电话机
+未带@的物件仅作剧本所需普通文字描述，不冒充已完成资产或新增绑定。
+[空间布局总览]
+庄园大厅北墙为壁炉及裂镜，沙发在中部偏西，电话几在东墙，南门通前庭，桌椅之间保留南北通道。Damián常服在大厅中部，Víctor常服站北侧壁炉旁，裂镜与碎片在壁炉下方。沿原资产结构，仅按原剧本时段改变窗外为日光。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（7个硬切分镜）]
+分镜一：【景别/视角：裂镜近景/壁炉侧 | 运镜：固定，镜面与落地碎片同框】
+【时长】3.0s
+【构图】开场承接重物撞击后的裂纹扩散，少量玻璃碎片落到壁炉前；不虚构是谁扔的重物。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】镜面已裂，碎片留北墙下。
+【镜头结尾·站位收束】镜面已裂，碎片留北墙下。
+画面硬切到分镜二。
+分镜二：【景别/视角：大厅关系全景/南门内侧 | 运镜：向北轻推，建立两人及电话几的位置】
+【时长】3.0s
+【构图】Damián常服在中部来回两步后停住，Víctor常服在壁炉侧，东墙电话几清楚可见。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】两人未踩进碎玻璃区域。
+【镜头结尾·站位收束】两人未踩进碎玻璃区域。
+画面硬切到分镜三。
+分镜三：【景别/视角：Víctor常服手部与侧脸近景 | 运镜：由方巾轻摇到他的眼神】
+【时长】3.0s
+【构图】Víctor常服取出白色方巾，擦一下右手掌再折回左手，平稳说出判断。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Víctor常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】方巾在Víctor常服左手，Damián常服留中部。
+【镜头结尾·站位收束】方巾在Víctor常服左手，Damián常服留中部。
+画面硬切到分镜四。
+分镜四：【景别/视角：Damián常服听者近景 | 运镜：从壁炉南侧固定，裂镜退至画外】
+【时长】3.5s
+【构图】Víctor常服的原声继续，Damián常服下颌绷紧后不再踱步，看向父亲。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Víctor常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Damián常服站定，听完句尾。
+【镜头结尾·站位收束】Damián常服站定，听完句尾。
+画面硬切到分镜五。
+分镜五：【景别/视角：Víctor常服侧后中景 | 运镜：沿家具间通道向东跟随】
+【时长】3.0s
+【构图】Víctor常服把方巾收回口袋，走到东墙电话几，右手提起话筒，左手拨号码；相机不绕进墙面。
+【音效】脚步随起停出现；台词期间压低动作声。
+【台词】无台词。
+【变化】话筒在右耳，左手离开拨盘。
+【镜头结尾·站位收束】话筒在右耳，左手离开拨盘。
+画面硬切到分镜六。
+分镜六：【景别/视角：Víctor常服侧面近景 | 运镜：固定，电话几与手部仍留画面下缘】
+【时长】3.0s
+【构图】Víctor常服向电话中的功能性受话者发出指令，身体留在电话几旁。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Víctor常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】电话还未挂断，右手仍持话筒。
+【镜头结尾·站位收束】电话还未挂断，右手仍持话筒。
+画面硬切到分镜七。
+分镜七：【景别/视角：大厅纵深中景 | 运镜：缓慢向后拉，显出中部的Damián常服】
+【时长】4.0s
+【构图】Víctor常服补充共同难题，Damián常服在中部听着；话筒不换手，不新增对方回答。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Víctor常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Víctor常服在东墙电话几，Damián常服站大厅中部。
+【镜头结尾·站位收束】Víctor常服在东墙电话几，Damián常服站大厅中部。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：22.5s</x:v>
+      </x:c>
+      <x:c r="G32" s="2" t="str">
+        <x:v>Víctor：「No es suerte.」
+Víctor：「Nos lleva tres pasos de ventaja. Siempre.」
+Víctor：「Consígueme a Ernesto Miranda.」
+Víctor：「Dile... que tenemos un problema en común.」</x:v>
+      </x:c>
+      <x:c r="H32" s="2" t="str">
+        <x:v>27-2 庄园大厅（Mansión Vargas, salón principal） 日 内
+人物：Damián、Víctor
+△ 画面特写：伴随着一声清脆的玻璃破碎声，大厅内的一面巨大装饰镜被重物击穿，裂纹如蛛网般迅速蔓延。
+△ 镜头全景：Damián 穿着红棕色西装，领带松散，他愤怒地在大厅中央踱步，拳头紧握。背景的壁炉内火焰熊熊燃烧。
+△ 动作特写：Víctor穿着黑金花纹西装，神情冷峻地站在破碎的镜子前。他从胸前口袋掏出一块整齐叠放的白色方巾。
+△ 镜头近景：Víctor 慢条斯理地用方巾擦拭自己的双手，指间闪烁着一枚厚重的金戒指。他的眼神深邃而阴狠，完全没有了刚才在台上的颓势。
+Víctor：No es suerte.
+△ 镜头切换：镜子破碎的特写。玻璃碴散落在地，映照着跳动的火光。
+Víctor：Nos lleva tres pasos de ventaja. Siempre.
+△ 动作特写：Víctor走到电话几旁，那上面放着一台黑色的老式拨盘电话机。
+△ 镜头近景：Víctor伸手抓住话筒，熟练地拨动号码。
+Víctor（对着话筒，语气冰冷且果断）：Consígueme a Ernesto Miranda.
+△ 镜头特写：Víctor 侧脸，眼神锁向远方，下颌线绷得极紧。
+Víctor：Dile... que tenemos un problema en común.</x:v>
+      </x:c>
+      <x:c r="I32" s="2" t="str">
+        <x:v>22.5s</x:v>
+      </x:c>
     </x:row>
     <x:row r="33" ht="200" customHeight="1">
-      <x:c r="A33" s="2"/>
-      <x:c r="B33" s="2"/>
-      <x:c r="C33" s="2"/>
-      <x:c r="D33" s="2"/>
-      <x:c r="E33" s="2"/>
-      <x:c r="F33" s="2"/>
-      <x:c r="G33" s="2"/>
-      <x:c r="H33" s="2"/>
-      <x:c r="I33" s="2"/>
+      <x:c r="A33" s="2" t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="B33" s="2" t="str">
+        <x:v>27-3A</x:v>
+      </x:c>
+      <x:c r="C33" s="2" t="str">
+        <x:v>Damián常服；Escorpión常服；Vera常服</x:v>
+      </x:c>
+      <x:c r="D33" s="2" t="str">
+        <x:v>巴尔加斯庄园主卧（夜）；家主书房（夜）</x:v>
+      </x:c>
+      <x:c r="E33" s="2" t="str">
+        <x:v>iPhone手机；电视画面</x:v>
+      </x:c>
+      <x:c r="F33" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+巴尔加斯庄园主卧（夜）；家主书房（夜），9:16竖屏。主卧床头灯从侧后照Damián常服，电视为低弱冷反射；书房暖台灯只切出Escorpión常服侧面，两处曝光分别连续。
+[音轨规则]
+远层：书房内安静的室内底噪，门外动静低于台词。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
+3.1s—4.2s，@Escorpión常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Una pregunta.」
+6.1s—7.9s，@Escorpión常服（VO，Escorpión常服电话VO，略窄频，Damián常服只听，不做该句口型）：「¿Ella es la Viuda?」
+9.1s—10.9s，@Damián常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Me casé con ella.」
+12.1s—14.3s，@Damián常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Me casé con la Viuda.」
+[锚定列表]
+场景：@巴尔加斯庄园主卧（夜）；@家主书房（夜）
+角色：@Damián常服；@Escorpión常服；@Vera常服
+道具：@iPhone手机；电视画面
+未带@的物件仅作剧本所需普通文字描述，不冒充已完成资产或新增绑定。
+[空间布局总览]
+主卧北侧是床与床头灯、电视在南侧墙；书房桌在北侧、客椅在桌南、书架在西墙。通话交叉剪辑明确分两地：Damián常服坐主卧床沿，电视在床前；Escorpión常服独坐书房南侧客椅，手机贴右耳。Vera常服只出现在电视回放的发布会影像中，不进入主卧或书房。人物造型全部使用已有常服。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（6个硬切分镜）]
+分镜一：【景别/视角：主卧中景/床侧 | 运镜：从床前斜侧轻推，电视边缘留前景】
+【时长】3.0s
+【构图】Damián常服坐床沿看电视回放，右手手机已贴耳；电视只呈先前发布会人物影像，不出现文字。
+【音效】手指与机身接触的低弱摩擦声；台词期间压低动作声。
+【台词】无台词。
+【变化】Damián常服仍在主卧，电视回放不是同场真人。
+【镜头结尾·站位收束】Damián常服仍在主卧，电视回放不是同场真人。
+画面硬切到分镜二。
+分镜二：【景别/视角：书房Escorpión常服侧面近景 | 运镜：硬切到书房固定机位，后方书架建立不同地点】
+【时长】3.0s
+【构图】Escorpión常服坐客椅，右手持手机，面向空桌发问，目光不看Damián常服所在方向。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Escorpión常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Escorpión常服留在书房，右手未换位。
+【镜头结尾·站位收束】Escorpión常服留在书房，右手未换位。
+画面硬切到分镜三。
+分镜三：【景别/视角：主卧Damián常服近景 | 运镜：固定，电视边光只在面部一侧】
+【时长】3.0s
+【构图】Escorpión常服后半问句以电话VO进入主卧，Damián常服听着，嘴部不代说。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Escorpión常服的VO按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Damián常服目光从电视降到床前。
+【镜头结尾·站位收束】Damián常服目光从电视降到床前。
+画面硬切到分镜四。
+分镜四：【景别/视角：Damián常服侧面近景 | 运镜：微向前推后停住】
+【时长】3.0s
+【构图】Damián常服听完，嘴角稍松，用压低的声音回答；身体没有站起。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Damián常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】手机仍在右耳，另一手撑床沿。
+【镜头结尾·站位收束】手机仍在右耳，另一手撑床沿。
+画面硬切到分镜五。
+分镜五：【景别/视角：书房Escorpión常服近景 | 运镜：固定，焦点停在静止的唇部和眼神】
+【时长】3.0s
+【构图】Damián常服的第二句通过电话传来，Escorpión常服不说话，仅目光停住，避免把画外词配到其口型。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Damián常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Escorpión常服仍坐客椅。
+【镜头结尾·站位收束】Escorpión常服仍坐客椅。
+画面硬切到分镜六。
+分镜六：【景别/视角：主卧Damián常服中近景 | 运镜：向侧方小幅移，露出电视与床沿距离】
+【时长】3.0s
+【构图】Damián常服说完后抬头，短促地笑出原定非语言声一次，幅度收小；不新增词语。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】Damián常服仍坐床沿，通话状态持续。
+【镜头结尾·站位收束】Damián常服仍坐床沿，通话状态持续。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：18s</x:v>
+      </x:c>
+      <x:c r="G33" s="2" t="str">
+        <x:v>Escorpión：「Una pregunta.」
+Escorpión VO：「¿Ella es la Viuda?」
+Damián：「Me casé con ella.」
+Damián：「Me casé con la Viuda.」</x:v>
+      </x:c>
+      <x:c r="H33" s="2" t="str">
+        <x:v>27-3 豪宅/发布会后台/卧室（Mansión Vargas） 夜 内
+人物：Damián、Escorpión、Vera
+△ 画面全景：电视屏幕上正重播着发布会的混乱画面。Damián 穿着棕色夹克，坐在电视机前，低着头，神情阴沉到了极点。
+△ 镜头特写：Damián 的侧脸。他微微抬起眼皮，瞳孔中映着电视屏幕的冷光。
+△ 镜头切换：Escorpión 坐在书房的阴影中。他手里拿着手机贴在耳边，面部轮廓在微弱的灯光下显得冷峻而立体。
+Escorpión：Una pregunta.
+△ 镜头反打：Damián 坐在床沿，手中同样拿着手机，眼神中透着一股复杂的情绪。
+Escorpión VO：¿Ella es la Viuda?
+△ 镜头特写：Damián 沉默了片刻，嘴角竟微微上扬，露出一抹极具侵略性的笑容。
+Damián（低声，语气中带着一丝病态的自豪）：Me casé con ella.
+△ 镜头切换：Escorpión 的嘴唇特写。他听着电话那头的回答，没有说话。
+Damián：Me casé con la Viuda.
+△ 镜头特写：Damián 坐在床边，他抬起头，眼神中闪烁着疯狂而兴奋的光芒。他突然笑出了声，笑声在空荡的房间里显得格外刺耳。</x:v>
+      </x:c>
+      <x:c r="I33" s="2" t="str">
+        <x:v>18s</x:v>
+      </x:c>
     </x:row>
     <x:row r="34" ht="200" customHeight="1">
-      <x:c r="A34" s="2"/>
-      <x:c r="B34" s="2"/>
-      <x:c r="C34" s="2"/>
-      <x:c r="D34" s="2"/>
-      <x:c r="E34" s="2"/>
-      <x:c r="F34" s="2"/>
-      <x:c r="G34" s="2"/>
-      <x:c r="H34" s="2"/>
-      <x:c r="I34" s="2"/>
+      <x:c r="A34" s="2" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B34" s="2" t="str">
+        <x:v>28-1A</x:v>
+      </x:c>
+      <x:c r="C34" s="2" t="str">
+        <x:v>Víctor常服；Don Ernesto常服；Escolta A常服</x:v>
+      </x:c>
+      <x:c r="D34" s="2" t="str">
+        <x:v>游艇甲板</x:v>
+      </x:c>
+      <x:c r="E34" s="2" t="str">
+        <x:v>香槟杯</x:v>
+      </x:c>
+      <x:c r="F34" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+游艇甲板，9:16竖屏。桌上烛光从两人侧下方照出局部反射，甲板边灯勾轮廓，湖岸灯火在栏杆外；人物不过度均匀补亮。
+[音轨规则]
+远层：湖面低弱水声、游艇轻微船体底噪。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
+3.1s—6.5s，@Víctor常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Su hijo no pudo guardársela en los pantalones.」
+7.1s—8.6s，@Víctor常服（VO，现场画外原声，保持原说话人声线，画面内听者不代说）：「Ahí empezó todo.」
+10.1s—15.1s，@Don Ernesto常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Y tú criaste un perro por veinte años que al final mordió.」
+[锚定列表]
+场景：@游艇甲板
+角色：@Víctor常服；@Don Ernesto常服；@Escolta A常服
+道具：香槟杯
+未带@的物件仅作剧本所需普通文字描述，不冒充已完成资产或新增绑定。
+[空间布局总览]
+游艇艉部甲板中央是双人餐桌，Víctor常服坐桌西侧朝东，Don Ernesto常服坐桌东侧朝西；Escolta A在北侧通往船舱的入口旁站岗。南侧栏杆外为湖面，餐桌南侧留相机通道。两人的右手酒杯放在各自靠身前桌沿，文件起初收在Don Ernesto常服衣内。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（6个硬切分镜）]
+分镜一：【景别/视角：甲板关系全景/南侧栏杆内 | 运镜：沿桌南侧短移，展示两人相对位置与船舱入口】
+【时长】3.0s
+【构图】Víctor常服坐西侧，Don Ernesto常服坐东侧；Escolta A在北侧船舱口，香槟杯在各自手边。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】餐桌与人物位置已建立，栏杆始终在南侧。
+【镜头结尾·站位收束】餐桌与人物位置已建立，栏杆始终在南侧。
+画面硬切到分镜二。
+分镜二：【景别/视角：Víctor常服侧面近景/桌南偏东 | 运镜：缓推至他前倾后的眼神】
+【时长】4.0s
+【构图】Víctor常服双前臂仍靠自己一侧桌沿，上身略前倾，低声说出挑衅；酒杯未举起。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Víctor常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Víctor常服仍坐西侧，视线锁住对方。
+【镜头结尾·站位收束】Víctor常服仍坐西侧，视线锁住对方。
+画面硬切到分镜三。
+分镜三：【景别/视角：Don Ernesto常服听者近景 | 运镜：在桌南偏西固定，远岸灯点位于身后】
+【时长】3.0s
+【构图】Víctor常服追加一句以现场画外VO承接，Don Ernesto常服嘴角收住，左手停在桌沿；不做别人台词的口型。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Víctor常服的VO按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Don Ernesto常服坐东侧，未突然站起。
+【镜头结尾·站位收束】Don Ernesto常服坐东侧，未突然站起。
+画面硬切到分镜四。
+分镜四：【景别/视角：Don Ernesto常服侧面近景 | 运镜：沿桌南侧轻移，落在其迎视Víctor常服的目光】
+【时长】4.0s
+【构图】Don Ernesto常服抬眼直接回应，声音压低；手指不敲杯，不用伤疤抽动代替表演。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Don Ernesto常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】两人仍相对而坐。
+【镜头结尾·站位收束】两人仍相对而坐。
+画面硬切到分镜五。
+分镜五：【景别/视角：Víctor常服听者中近景 | 运镜：固定，Don Ernesto常服杯沿在前景边缘】
+【时长】3.0s
+【构图】Don Ernesto常服的原声跨切到句尾，Víctor常服下颌略收，右手开始靠近酒杯杯梗。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Don Ernesto常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】回应说完，双方右手各近自己的杯。
+【镜头结尾·站位收束】回应说完，双方右手各近自己的杯。
+画面硬切到分镜六。
+分镜六：【景别/视角：双手与杯口近景 | 运镜：固定，手、杯、桌面都在清楚焦平面】
+【时长】3.0s
+【构图】两人以右手各举一杯，沿桌面上方靠近，杯口轻碰一次再分开；酒液只随真实惯性微晃。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】两只杯分开，仍由各自右手持住。
+【镜头结尾·站位收束】两只杯分开，仍由各自右手持住。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：20s</x:v>
+      </x:c>
+      <x:c r="G34" s="2" t="str">
+        <x:v>Víctor：「Su hijo no pudo guardársela en los pantalones.」
+Víctor VO：「Ahí empezó todo.」
+Don Ernesto：「Y tú criaste un perro por veinte años que al final mordió.」</x:v>
+      </x:c>
+      <x:c r="H34" s="2" t="str">
+        <x:v>第28集
+28-1 游艇甲板（Yate "El Patrón", lago de Valle de Bravo） 夜 外
+人物：Víctor、Don Ernesto、Escolta A
+△ 镜头全景：夜晚的湖面上，一艘豪华游艇灯火通明。甲板上摆放着精致的餐桌，桌上点缀着蜡烛，香槟桶里冰镇着酒。背景是远处湖岸模糊的灯火。
+△ 镜头近景：Víctor 坐在餐桌一侧，他穿着剪裁得体、带有金色暗纹的黑色西装，银发梳理得一丝不苟。他神情从容，嘴角带着一抹似笑非笑的弧度。
+△ 镜头反打：Don Ernesto 坐在对面，他穿着黑色西装内搭黑衬衫，银色的短发下，左眼角有一道醒目的交叉状伤疤，眼神凌厉如鹰。
+Víctor（身体微微前倾，语气带着嘲讽）：Su hijo no pudo guardársela en los pantalones.
+△ 镜头特写：Don Ernesto 的面部特写。听到这句话，他的眼神瞬间变得阴沉，眼角伤疤微微抽动，充满了压抑的怒火。
+Víctor VO：Ahí empezó todo.
+△ 镜头切到 Don Ernesto：他深吸一口气，直视着 Víctor，声音低沉且沙哑。
+Don Ernesto（语气冰冷且危险）：Y tú criaste un perro por veinte años que al final mordió.
+△ 动作特写：两只手分别举起盛满香槟的高脚杯，在空中轻轻碰撞，发出清脆的叮当声。杯中细密的泡沫不断上升。</x:v>
+      </x:c>
+      <x:c r="I34" s="2" t="str">
+        <x:v>20s</x:v>
+      </x:c>
     </x:row>
     <x:row r="35" ht="200" customHeight="1">
-      <x:c r="A35" s="2"/>
-      <x:c r="B35" s="2"/>
-      <x:c r="C35" s="2"/>
-      <x:c r="D35" s="2"/>
-      <x:c r="E35" s="2"/>
-      <x:c r="F35" s="2"/>
-      <x:c r="G35" s="2"/>
-      <x:c r="H35" s="2"/>
-      <x:c r="I35" s="2"/>
+      <x:c r="A35" s="2" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B35" s="2" t="str">
+        <x:v>28-1B</x:v>
+      </x:c>
+      <x:c r="C35" s="2" t="str">
+        <x:v>Víctor常服；Don Ernesto常服；Escolta A常服</x:v>
+      </x:c>
+      <x:c r="D35" s="2" t="str">
+        <x:v>游艇甲板</x:v>
+      </x:c>
+      <x:c r="E35" s="2" t="str">
+        <x:v>联合声明文件；香槟杯</x:v>
+      </x:c>
+      <x:c r="F35" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+游艇甲板，9:16竖屏。烛光保持同一方向，纸张只显边缘与背面，金属栏杆反射随机位短移改变。
+[音轨规则]
+远层：湖面低弱水声、游艇轻微船体底噪。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
+0.2s—1.7s，@Don Ernesto常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Una declaración conjunta.」
+3.1s—7.7s，@Don Ernesto常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Matrimonio fraudulento. Extorsión. Inestabilidad mental. Vínculos con el crimen.」
+10.1s—13.4s，@Don Ernesto常服（VO，现场画外原声，保持原说话人声线，画面内听者不代说）：「Y mi parte. El terreno sobre Reforma.」
+14.1s—16.8s，@Don Ernesto常服（VO，现场画外原声，保持原说话人声线，画面内听者不代说）：「Tuyo... por una firma.」
+[锚定列表]
+场景：@游艇甲板
+角色：@Víctor常服；@Don Ernesto常服；@Escolta A常服
+道具：联合声明文件；香槟杯
+未带@的物件仅作剧本所需普通文字描述，不冒充已完成资产或新增绑定。
+[空间布局总览]
+游艇艉部甲板中央是双人餐桌，Víctor常服坐桌西侧朝东，Don Ernesto常服坐桌东侧朝西；Escolta A在北侧通往船舱的入口旁站岗。南侧栏杆外为湖面，餐桌南侧留相机通道。两人的右手酒杯放在各自靠身前桌沿，文件起初收在Don Ernesto常服衣内。上段举杯后，两人先将杯底落回各自身前杯垫；右手松开后再取文件。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（6个硬切分镜）]
+分镜一：【景别/视角：酒杯与Don Ernesto常服中景 | 运镜：从杯底轻抬到衣内取物的手】
+【时长】3.0s
+【构图】两只酒杯已各自放回；Don Ernesto常服右手松杯后，从衣内取出折叠声明，左手扶住纸边展开。
+【音效】纸张轻擦声；台词期间压低动作声。
+【台词】@Don Ernesto常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】纸张在Don Ernesto常服双手，杯子留在桌面。
+【镜头结尾·站位收束】纸张在Don Ernesto常服双手，杯子留在桌面。
+画面硬切到分镜二。
+分镜二：【景别/视角：文件交接中近景/餐桌南侧 | 运镜：短距离向西平移，保留文件路径】
+【时长】4.0s
+【构图】Don Ernesto常服把文件平放并向西推到桌中，右指依次点出条款；纸面朝向Víctor常服，镜头只见侧边。
+【音效】纸张轻擦声；台词期间压低动作声。
+【台词】@Don Ernesto常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】文件到桌中偏西，双方手未相叠。
+【镜头结尾·站位收束】文件到桌中偏西，双方手未相叠。
+画面硬切到分镜三。
+分镜三：【景别/视角：Víctor常服过肩望文件中景 | 运镜：固定，Don Ernesto常服置于画外侧】
+【时长】3.0s
+【构图】Don Ernesto常服的条款原声继续，Víctor常服用右手食中二指压住纸边，将文件拉到自己一侧。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Don Ernesto常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】文件停在Víctor常服身前，纸张无跳位。
+【镜头结尾·站位收束】文件停在Víctor常服身前，纸张无跳位。
+画面硬切到分镜四。
+分镜四：【景别/视角：Víctor常服近景/餐桌南偏东 | 运镜：缓推至其低头阅读后抬眼】
+【时长】4.0s
+【构图】Don Ernesto常服以现场画外VO补充土地交易，Víctor常服看向文件，再抬眼；字面不入画。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Don Ernesto常服的VO按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Víctor常服右手仍按纸边。
+【镜头结尾·站位收束】Víctor常服右手仍按纸边。
+画面硬切到分镜五。
+分镜五：【景别/视角：Don Ernesto常服手部近景 | 运镜：固定在桌南侧，仅呈手部与文件边沿】
+【时长】3.0s
+【构图】Don Ernesto常服保持坐姿，以原现场画外声说出签名条件；镜头不呈其嘴部，左手掌朝上停在自己一侧桌面，未提前握手。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Don Ernesto常服的VO按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】条件说完，Don Ernesto常服才伸出右手。
+【镜头结尾·站位收束】条件说完，Don Ernesto常服才伸出右手。
+画面硬切到分镜六。
+分镜六：【景别/视角：双人中景/甲板南侧 | 运镜：缓慢后拉显出桌沿和双方前臂】
+【时长】3.0s
+【构图】Víctor常服把文件放平并松指，伸出右手与Don Ernesto常服右手相握；双方左手留桌侧，杯子未再拿起。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】两人右手握在桌上方，文件与酒杯各在原位置。
+【镜头结尾·站位收束】两人右手握在桌上方，文件与酒杯各在原位置。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：20s</x:v>
+      </x:c>
+      <x:c r="G35" s="2" t="str">
+        <x:v>Don Ernesto：「Una declaración conjunta.」
+Don Ernesto：「Matrimonio fraudulento. Extorsión. Inestabilidad mental. Vínculos con el crimen.」
+Don Ernesto VO：「Y mi parte. El terreno sobre Reforma.」
+Don Ernesto VO：「Tuyo... por una firma.」</x:v>
+      </x:c>
+      <x:c r="H35" s="2" t="str">
+        <x:v>△ 镜头全景：Don Ernesto 靠在椅背上，从怀中掏出一份折叠的文件，动作沉稳而有力。
+Don Ernesto：Una declaración conjunta.
+△ 动作特写：Don Ernesto 将文件在桌面上推向 Víctor。
+Don Ernesto（依次指点文件内容）：Matrimonio fraudulento. Extorsión. Inestabilidad mental. Vínculos con el crimen.
+△ 镜头切换：Víctor 的双手出现在画面中，他伸出食指和中指，压在文件的边缘，缓缓将其拉向自己。
+△ 镜头特写：文件正文内容。上面用花体字印着法律条款，包含"padres biológicos"等字样。
+Don Ernesto VO：Y mi parte. El terreno sobre Reforma.
+△ 镜头切到 Víctor：他低头看着文件，手指在纸面上有节奏地轻点，眼神中闪烁着精明的算计。
+Don Ernesto VO：Tuyo... por una firma.
+△ 动作特写：两人的手在茶几上方紧紧握在一起。Víctor 的右手戴着一块醒目的金色劳力士腕表。
+△ 镜头虚化：画面在有力的握手中迅速变焦并淡出。</x:v>
+      </x:c>
+      <x:c r="I35" s="2" t="str">
+        <x:v>20s</x:v>
+      </x:c>
     </x:row>
     <x:row r="36" ht="200" customHeight="1">
-      <x:c r="A36" s="2"/>
-      <x:c r="B36" s="2"/>
-      <x:c r="C36" s="2"/>
-      <x:c r="D36" s="2"/>
-      <x:c r="E36" s="2"/>
-      <x:c r="F36" s="2"/>
-      <x:c r="G36" s="2"/>
-      <x:c r="H36" s="2"/>
-      <x:c r="I36" s="2"/>
+      <x:c r="A36" s="2" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B36" s="2" t="str">
+        <x:v>28-2A</x:v>
+      </x:c>
+      <x:c r="C36" s="2" t="str">
+        <x:v>Vera常服</x:v>
+      </x:c>
+      <x:c r="D36" s="2" t="str">
+        <x:v>高层公寓客厅（夜）</x:v>
+      </x:c>
+      <x:c r="E36" s="2" t="str">
+        <x:v>黑色信封</x:v>
+      </x:c>
+      <x:c r="F36" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+高层公寓客厅（夜），9:16竖屏。北侧落地灯斜照入口地面，东窗夜光勾人物侧脸；卡片表面保持空白，无可读字形。
+[音轨规则]
+远层：公寓外远处车流低声，室内维持安静。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段无原定对白或旁白，不新增发声。
+[锚定列表]
+场景：@高层公寓客厅（夜）
+角色：@Vera常服
+道具：@黑色信封
+[空间布局总览]
+公寓入口在西墙，茶几位于客厅中部、沙发在北侧，东墙落地窗可见城市，书桌工作区位于窗侧；南侧移门通阳台，桌椅之间保留南侧通道。世界方位不随反打改变。黑色信封在西侧入口内地面；Vera常服从客厅南侧通道经过，右手起初空着。她全程使用Vera常服，沿用现有服装与鞋履，不派生赤脚新造型。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（5个硬切分镜）]
+分镜一：【景别/视角：脚步与信封低位近景 | 运镜：沿入口地面向东短移，落在停步位置】
+【时长】3.0s
+【构图】Vera常服走近黑色信封，先停稳双脚；镜头用原有鞋履承接，不另设计赤脚身份版本。
+【音效】鞋底接触地面声、脚步随起停出现；台词期间压低动作声。
+【台词】无台词。
+【变化】信封仍在地面，Vera常服在它东侧。
+【镜头结尾·站位收束】信封仍在地面，Vera常服在它东侧。
+画面硬切到分镜二。
+分镜二：【景别/视角：Vera常服侧面中景 | 运镜：固定，保留弯腰、拾取、直身过程】
+【时长】3.0s
+【构图】Vera常服屈膝俯身，右手捡起黑色信封，左手扶膝支撑，直身后左手接住信封下缘。
+【音效】封口与纸张轻擦声；台词期间压低动作声。
+【台词】无台词。
+【变化】信封在双手，已离地。
+【镜头结尾·站位收束】信封在双手，已离地。
+画面硬切到分镜三。
+分镜三：【景别/视角：窗侧中景 | 运镜：与Vera常服向东同行两步，最后停在她侧面】
+【时长】3.0s
+【构图】Vera常服沿客厅南侧通道走到东窗内侧，避开茶几；信封保持在胸前。
+【音效】脚步随起停出现、封口与纸张轻擦声；台词期间压低动作声。
+【台词】无台词。
+【变化】Vera常服在东窗内侧，未穿过玻璃。
+【镜头结尾·站位收束】Vera常服在东窗内侧，未穿过玻璃。
+画面硬切到分镜四。
+分镜四：【景别/视角：信封与手部近景 | 运镜：固定，封口及卡片接触可读】
+【时长】3.5s
+【构图】Vera常服左手稳住黑信封，右手撕开封口，抽出乳白卡片；卡片朝自己，镜头只见空白背面。
+【音效】封口与纸张轻擦声；台词期间压低动作声。
+【台词】无台词。
+【变化】卡片在右手，黑信封在左手。
+【镜头结尾·站位收束】卡片在右手，黑信封在左手。
+画面硬切到分镜五。
+分镜五：【景别/视角：Vera常服侧面近景 | 运镜：轻向侧方移，框入窗框和她停住的视线】
+【时长】3.5s
+【构图】Vera常服看完后目光停住，唇缝短暂压合；右手握卡边略紧，不新增瞪眼、退步或抽气。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】她留窗边，卡片与信封分在左右手。
+【镜头结尾·站位收束】她留窗边，卡片与信封分在左右手。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：16s</x:v>
+      </x:c>
+      <x:c r="G36" s="2" t="str"/>
+      <x:c r="H36" s="2" t="str">
+        <x:v>28-2 高层公寓/走廊（Departamento ejecutivo, Piso 21, Reforma） 夜 内
+人物：Vera
+△ 镜头俯拍特写：Vera 赤着脚走在深色的木质地板上，步履轻盈。地板上静静地躺着一个黑色的信封，封口没有任何标志。
+△ 动作特写：Vera 弯腰捡起信封。信封质感高级，呈现磨砂质感。
+△ 镜头近景：Vera 走到窗边，侧脸被微弱的月光勾勒。她用修长的手指熟练地撕开封口，从里面抽出一张质地坚硬的乳白色卡片。
+△ 画面特写：卡片上只有三个巨大的黑色手写字母。
+【字幕：CORRE】
+△ 镜头切到 Vera：她紧紧盯着手中的卡片，瞳孔微微收缩。她的头发有些湿润地贴在颈部，眼神中闪过一丝极度的震惊与不安，呼吸明显变得急促。</x:v>
+      </x:c>
+      <x:c r="I36" s="2" t="str">
+        <x:v>16s</x:v>
+      </x:c>
     </x:row>
     <x:row r="37" ht="200" customHeight="1">
-      <x:c r="A37" s="2"/>
-      <x:c r="B37" s="2"/>
-      <x:c r="C37" s="2"/>
-      <x:c r="D37" s="2"/>
-      <x:c r="E37" s="2"/>
-      <x:c r="F37" s="2"/>
-      <x:c r="G37" s="2"/>
-      <x:c r="H37" s="2"/>
-      <x:c r="I37" s="2"/>
+      <x:c r="A37" s="2" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B37" s="2" t="str">
+        <x:v>29-1A</x:v>
+      </x:c>
+      <x:c r="C37" s="2" t="str">
+        <x:v>Vera常服；Damián常服</x:v>
+      </x:c>
+      <x:c r="D37" s="2" t="str">
+        <x:v>高层公寓入口处（外·日）</x:v>
+      </x:c>
+      <x:c r="E37" s="2" t="str">
+        <x:v>红玫瑰花束</x:v>
+      </x:c>
+      <x:c r="F37" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+高层公寓入口处（外·日），9:16竖屏。日光从广场西侧斜照，建筑檐口给门内Vera常服提供软阴影，玻璃只反射真实广场方向。
+[音轨规则]
+远层：日间入口广场远处车流，人物附近保持清楚。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
+3.1s—4.9s，@Damián常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Vera, empecemos de nuevo.」
+6.1s—12.5s，@Damián常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Tú eres la Viuda, yo soy un Vargas. Juntos podríamos ser dueños de esta ciudad.」
+13.1s—15.3s，@Vera常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「¿Y su compromiso con Bárbara?」
+16.1s—19.4s，@Damián常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Eso no fue nada. Puedo acabarlo hoy.」
+[锚定列表]
+场景：@高层公寓入口处（外·日）
+角色：@Vera常服；@Damián常服
+道具：@红玫瑰花束
+[空间布局总览]
+高层公寓入口玻璃门位于大楼北侧立面、向大厅内开启；大楼室内在南，室外广场向北展开。Vera常服在半开门内南侧，Damián常服在门外北侧，面向Vera常服，双手托着红玫瑰束；门外东侧空地可供一步接近。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（6个硬切分镜）]
+分镜一：【景别/视角：入口关系全景/门外东侧 | 运镜：从广场向半开门短推，保留玻璃门边界】
+【时长】3.0s
+【构图】Vera常服在门内南侧，Damián常服在门外北侧，两人相距约两步；玫瑰束由Damián常服双手托在胸腹前。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】双方位置与门的开启方向清楚。
+【镜头结尾·站位收束】双方位置与门的开启方向清楚。
+画面硬切到分镜二。
+分镜二：【景别/视角：Damián常服近景/门侧反打 | 运镜：固定，花束上缘留前景】
+【时长】3.0s
+【构图】Damián常服看着Vera常服，先提出重新开始，语气试探而急切；双手保持托花。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Damián常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Damián常服未向前迈步。
+【镜头结尾·站位收束】Damián常服未向前迈步。
+画面硬切到分镜三。
+分镜三：【景别/视角：双人侧面中景/广场东侧 | 运镜：沿门前向南小幅侧移，形成门框与人物层次】
+【时长】4.0s
+【构图】Damián常服继续说出权力设想；Vera常服留在门内，右手在身侧慢慢握紧，不握住不存在物件。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Damián常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Damián常服仍在原位，Vera常服右手已收紧。
+【镜头结尾·站位收束】Damián常服仍在原位，Vera常服右手已收紧。
+画面硬切到分镜四。
+分镜四：【景别/视角：Vera常服近景/门内偏东 | 运镜：固定，焦点留眼神与唇部】
+【时长】3.0s
+【构图】Damián常服的声音继续到完整句尾，Vera常服等他说完才准备回应，不提前做说话口型。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Damián常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Vera常服仍在门内。
+【镜头结尾·站位收束】Vera常服仍在门内。
+画面硬切到分镜五。
+分镜五：【景别/视角：Vera常服侧面近景 | 运镜：轻向前推后落稳】
+【时长】3.0s
+【构图】Vera常服抬眼提到Bárbara常服，音量平稳，疑问按语义收尾，不机械上扬。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Vera常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Vera常服右手慢慢松开，身体未前移。
+【镜头结尾·站位收束】Vera常服右手慢慢松开，身体未前移。
+画面硬切到分镜六。
+分镜六：【景别/视角：Damián常服近景 | 运镜：固定，保持花束和双手可见】
+【时长】4.0s
+【构图】Damián常服先低眼看一眼花，再看向Vera常服，立即回答；双手一直托着花束。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Damián常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】回答结束，两人距离仍约两步。
+【镜头结尾·站位收束】回答结束，两人距离仍约两步。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：20s</x:v>
+      </x:c>
+      <x:c r="G37" s="2" t="str">
+        <x:v>Damián：「Vera, empecemos de nuevo.」
+Damián：「Tú eres la Viuda, yo soy un Vargas. Juntos podríamos ser dueños de esta ciudad.」
+Vera：「¿Y su compromiso con Bárbara?」
+Damián：「Eso no fue nada. Puedo acabarlo hoy.」</x:v>
+      </x:c>
+      <x:c r="H37" s="2" t="str">
+        <x:v>第29集
+29-1 高层公寓/入口处（Departamento ejecutivo, Piso 21, Reforma） 日 外
+人物：Vera、Damián
+△ 画面特写：Vera 侧身站在半开的厚重玻璃门后。她穿着米色风衣，长发随意披散，神情冷静且透着一种疏离感。
+△ 镜头切换：Damián 站在阳光下的广场上。他穿着一套深红棕色的西装，内搭白色衬衫，领带略显凌乱。他双手捧着一大束鲜艳的红玫瑰，金色的腕表在阳光下闪闪发光。
+△ 镜头近景：Damián 眼神中充满了急切与渴望，他紧紧盯着 Vera，呼吸有些急促。
+Damián：Vera, empecemos de nuevo.
+△ 镜头特写：Vera 的面部特写。她的绿眼睛平静地注视着 Damián，没有任何波动。
+Damián：Tú eres la Viuda, yo soy un Vargas. Juntos podríamos ser dueños de esta ciudad.
+△ 动作特写：镜头移向 Vera 的手部。她原本自然垂在风衣口袋旁的手慢慢收紧，指尖陷入掌心，随后在大腿外侧紧紧攥成了拳头。
+△ 镜头切到 Vera：她微微抬起下巴，眼神中闪过一丝嘲讽。
+Vera：¿Y su compromiso con Bárbara?
+△ 动作特写：Damián 听到这个名字，神情微微一滞。他迅速低头看了一眼手中的玫瑰，又立刻抬头，眼神变得坚定而狠厉。
+Damián：Eso no fue nada. Puedo acabarlo hoy.</x:v>
+      </x:c>
+      <x:c r="I37" s="2" t="str">
+        <x:v>20s</x:v>
+      </x:c>
     </x:row>
     <x:row r="38" ht="200" customHeight="1">
-      <x:c r="A38" s="2"/>
-      <x:c r="B38" s="2"/>
-      <x:c r="C38" s="2"/>
-      <x:c r="D38" s="2"/>
-      <x:c r="E38" s="2"/>
-      <x:c r="F38" s="2"/>
-      <x:c r="G38" s="2"/>
-      <x:c r="H38" s="2"/>
-      <x:c r="I38" s="2"/>
+      <x:c r="A38" s="2" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B38" s="2" t="str">
+        <x:v>29-1B</x:v>
+      </x:c>
+      <x:c r="C38" s="2" t="str">
+        <x:v>Vera常服；Damián常服</x:v>
+      </x:c>
+      <x:c r="D38" s="2" t="str">
+        <x:v>高层公寓入口处（外·日）</x:v>
+      </x:c>
+      <x:c r="E38" s="2" t="str">
+        <x:v>红玫瑰花束</x:v>
+      </x:c>
+      <x:c r="F38" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+高层公寓入口处（外·日），9:16竖屏。沿用西侧日光与建筑阴影，脸部受光随跨门槛自然变化，不临时新增正面灯。
+[音轨规则]
+远层：日间入口广场远处车流，人物附近保持清楚。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
+0.2s—5.0s，@Damián常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Te perdono. Las mentiras, la trampa, todo. No me importa.」
+5.2s—7.0s，@Vera常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「¿Me perdona a MÍ?」
+10.1s—14.6s，@Vera常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「No se enamoró de mí. Se enamoró de sentirse vivo.」
+14.8s—20.1s，@Vera常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「No está aquí porque me quiera. Está aquí porque le aterra morir.」
+[锚定列表]
+场景：@高层公寓入口处（外·日）
+角色：@Vera常服；@Damián常服
+道具：@红玫瑰花束
+[空间布局总览]
+高层公寓入口玻璃门位于大楼北侧立面、向大厅内开启；大楼室内在南，室外广场向北展开。Vera常服在半开门内南侧，Damián常服在门外北侧，面向Vera常服，双手托着红玫瑰束；门外东侧空地可供一步接近。两人仍隔两步，Vera常服在门内，Damián常服手持花束在广场。Damián常服本段只前进一步，Vera常服随后跨出门槛半步。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（6个硬切分镜）]
+分镜一：【景别/视角：双人侧面中景 | 运镜：从门外东侧短距离伴随Damián常服前移后停住】
+【时长】4.0s
+【构图】Damián常服向门口走一步，停在门外近处，压低声音说原话；花束仍在双手，不借花遮住双方嘴部。
+【音效】门扇与门锁随实际开合发声、脚步随起停出现；台词期间压低动作声。
+【台词】@Damián常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】距离缩为一步，Vera常服仍在门内。
+【镜头结尾·站位收束】距离缩为一步，Vera常服仍在门内。
+画面硬切到分镜二。
+分镜二：【景别/视角：Vera常服近景/门框内侧 | 运镜：固定，保护她从停顿到开口的变化】
+【时长】3.0s
+【构图】Damián常服声音结束后Vera常服眉部略收，平静反问；重音落在原文强调词，身体不突然后仰。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Damián常服的对白按本段唯一声音骨架连续发声；@Vera常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Vera常服直视对方，右手已松开。
+【镜头结尾·站位收束】Vera常服直视对方，右手已松开。
+画面硬切到分镜三。
+分镜三：【景别/视角：Damián常服听者近景 | 运镜：轻向侧移，门框在背景保持同一方向】
+【时长】3.0s
+【构图】Damián常服嘴唇动一下后停住，没有新增台词；花束仍在胸腹前。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】Damián常服停在门外一步内。
+【镜头结尾·站位收束】Damián常服停在门外一步内。
+画面硬切到分镜四。
+分镜四：【景别/视角：Vera常服侧面中近景 | 运镜：从门外东南侧向北短移，落在她的目光】
+【时长】4.0s
+【构图】Vera常服拆穿他的动机，声音清楚偏低；她说话时自然开合嘴唇，不同时要求紧闭唇缝。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Vera常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Vera常服仍站门槛南侧。
+【镜头结尾·站位收束】Vera常服仍站门槛南侧。
+画面硬切到分镜五。
+分镜五：【景别/视角：双人关系中近景 | 运镜：向广场东侧退半步，为Vera常服过门槛留空间】
+【时长】4.0s
+【构图】Vera常服跨出门槛半步，站到门外正对Damián常服的位置，继续说出死亡恐惧的判断；脚步发生一次。
+【音效】门扇与门锁随实际开合发声、鞋底接触地面声；台词期间压低动作声。
+【台词】@Vera常服的对白按本段唯一声音骨架连续发声；@Vera常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Vera常服已在门外近处，Damián常服仍双手持花。
+【镜头结尾·站位收束】Vera常服已在门外近处，Damián常服仍双手持花。
+画面硬切到分镜六。
+分镜六：【景别/视角：Damián常服近景/门外西侧 | 运镜：固定，镜头停在听者残留状态】
+【时长】3.0s
+【构图】Vera常服原声完整结束，Damián常服下颌逐渐绷住，目光没有离开她；不新增瞳孔剧变。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Vera常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】双方在门外近距站定，花束仍在两人之间。
+【镜头结尾·站位收束】双方在门外近距站定，花束仍在两人之间。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：21s</x:v>
+      </x:c>
+      <x:c r="G38" s="2" t="str">
+        <x:v>Damián：「Te perdono. Las mentiras, la trampa, todo. No me importa.」
+Vera：「¿Me perdona a MÍ?」
+Vera：「No se enamoró de mí. Se enamoró de sentirse vivo.」
+Vera：「No está aquí porque me quiera. Está aquí porque le aterra morir.」</x:v>
+      </x:c>
+      <x:c r="H38" s="2" t="str">
+        <x:v>△ 镜头近景：Damián 走近了一步，两人的距离缩短。他压低声音，语气中带着一种近乎偏执的真诚。
+Damián：Te perdono. Las mentiras, la trampa, todo. No me importa.
+△ 镜头特写：Vera 的眼神中突然燃起一丝怒火，她直视着 Damián 的眼睛，声音低沉但字字铿锵。
+Vera：¿Me perdona a MÍ?
+△ 镜头特写：Damián 的眼部特写。他的瞳孔中倒映着 Vera 的身影，眼神显得有些迷乱。
+△ 动作特写：Damián 的嘴唇微微动了一下，欲言又止。
+△ 镜头切到 Vera 的侧脸：阳光洒在她的侧颜上，她的眼神中透着一种看穿一切的冷漠。
+Vera：No se enamoró de mí. Se enamoró de sentirse vivo.
+△ 镜头近景：Vera 逼近 Damián，声音在他耳边响起。
+Vera：No está aquí porque me quiera. Está aquí porque le aterra morir.
+△ 镜头特写：Damián 的表情瞬间凝固，瞳孔由于极度的震惊和被拆穿的愤怒而放大。</x:v>
+      </x:c>
+      <x:c r="I38" s="2" t="str">
+        <x:v>21s</x:v>
+      </x:c>
     </x:row>
     <x:row r="39" ht="200" customHeight="1">
-      <x:c r="A39" s="2"/>
-      <x:c r="B39" s="2"/>
-      <x:c r="C39" s="2"/>
-      <x:c r="D39" s="2"/>
-      <x:c r="E39" s="2"/>
-      <x:c r="F39" s="2"/>
-      <x:c r="G39" s="2"/>
-      <x:c r="H39" s="2"/>
-      <x:c r="I39" s="2"/>
+      <x:c r="A39" s="2" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B39" s="2" t="str">
+        <x:v>29-2A</x:v>
+      </x:c>
+      <x:c r="C39" s="2" t="str">
+        <x:v>Vera常服；Damián常服</x:v>
+      </x:c>
+      <x:c r="D39" s="2" t="str">
+        <x:v>高层公寓入口处（外·日）</x:v>
+      </x:c>
+      <x:c r="E39" s="2" t="str">
+        <x:v>红玫瑰花束</x:v>
+      </x:c>
+      <x:c r="F39" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+高层公寓入口处（外·日），9:16竖屏。沿用西侧日光，门内为自然檐影，花瓣只在真实接触后散落。
+[音轨规则]
+远层：日间入口广场远处车流，人物附近保持清楚。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
+9.1s—11.7s，@Damián常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「¡Vas a desear no haberlo hecho!」
+[锚定列表]
+场景：@高层公寓入口处（外·日）
+角色：@Vera常服；@Damián常服
+道具：@红玫瑰花束
+[空间布局总览]
+高层公寓入口玻璃门位于大楼北侧立面、向大厅内开启；大楼室内在南，室外广场向北展开。Vera常服在半开门内南侧，Damián常服在门外北侧，面向Vera常服，双手托着红玫瑰束；门外东侧空地可供一步接近。Vera常服刚跨到门外半步，Damián常服站门外面对她，双手持花。门向大厅内半开，Vera常服可沿原路回去。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（5个硬切分镜）]
+分镜一：【景别/视角：花束与双人中景 | 运镜：固定，Vera常服手掌、花束、Damián常服持握点均清楚】
+【时长】3.0s
+【构图】Vera常服右手从身侧抬起，推开玫瑰束上部，Damián常服仍握束柄，几片花瓣接触后落地。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】花束偏向Damián常服胸前，未转交Vera常服。
+【镜头结尾·站位收束】花束偏向Damián常服胸前，未转交Vera常服。
+画面硬切到分镜二。
+分镜二：【景别/视角：侧后全身中景 | 运镜：伴随Vera常服回身走向门内，机位留广场】
+【时长】3.0s
+【构图】Vera常服收回右手，转身跨回门槛进入大厅；Damián常服不跟进，花束还在其双手。
+【音效】门扇与门锁随实际开合发声；台词期间压低动作声。
+【台词】无台词。
+【变化】Vera常服到门内，Damián常服留门外。
+【镜头结尾·站位收束】Vera常服到门内，Damián常服留门外。
+画面硬切到分镜三。
+分镜三：【景别/视角：Damián常服手部与肩部近景 | 运镜：缓推至握住花束的指节】
+【时长】3.0s
+【构图】Damián常服把散乱花束收近，握力加重，肩部略起后稳住；不连续全身颤抖。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】花束在胸前，双脚仍在原地。
+【镜头结尾·站位收束】花束在胸前，双脚仍在原地。
+画面硬切到分镜四。
+分镜四：【景别/视角：Damián常服近景/门外东侧 | 运镜：固定，前景门框保留离场方向】
+【时长】4.0s
+【构图】Damián常服朝Vera常服背影发出原定威胁，重音清楚，不新增咆哮语词。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Damián常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】台词结束，Vera常服已在大厅远处。
+【镜头结尾·站位收束】台词结束，Vera常服已在大厅远处。
+画面硬切到分镜五。
+分镜五：【景别/视角：入口关系远中景 | 运镜：缓慢后拉，拉开门内外距离】
+【时长】2.5s
+【构图】Vera常服沿大厅通道继续走远，Damián常服独留广场，脚边是落下的花瓣。
+【音效】鞋底接触地面声、脚步随起停出现；台词期间压低动作声。
+【台词】无台词。
+【变化】门内外人物不再形成近距对话。
+【镜头结尾·站位收束】门内外人物不再形成近距对话。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：15.5s</x:v>
+      </x:c>
+      <x:c r="G39" s="2" t="str">
+        <x:v>Damián：「¡Vas a desear no haberlo hecho!」</x:v>
+      </x:c>
+      <x:c r="H39" s="2" t="str">
+        <x:v>29-2 高层公寓/入口处（Departamento ejecutivo, Piso 21, Reforma） 日 外
+人物：Vera、Damián
+△ 动作特写：Vera 伸手猛地推开面前的红玫瑰束。红色的花瓣在推搡中散落。
+△ 镜头全景：Vera 决绝地转身走向公寓内部，风衣的下摆划出一个冷冽的弧度。Damián 捧着被推乱的花束站在原地，背影显得僵硬且愤怒。
+△ 动作特写：Damián 紧紧抓着花束的手在剧烈颤抖，手背上青筋暴起。
+△ 镜头切到 Damián 的正面特写：他五官扭曲，发疯似地对着 Vera 的背影咆哮，声音中充满了威胁。
+Damián（愤怒嘶吼）：¡Vas a desear no haberlo hecho!</x:v>
+      </x:c>
+      <x:c r="I39" s="2" t="str">
+        <x:v>15.5s</x:v>
+      </x:c>
     </x:row>
     <x:row r="40" ht="200" customHeight="1">
-      <x:c r="A40" s="2"/>
-      <x:c r="B40" s="2"/>
-      <x:c r="C40" s="2"/>
-      <x:c r="D40" s="2"/>
-      <x:c r="E40" s="2"/>
-      <x:c r="F40" s="2"/>
-      <x:c r="G40" s="2"/>
-      <x:c r="H40" s="2"/>
-      <x:c r="I40" s="2"/>
+      <x:c r="A40" s="2" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B40" s="2" t="str">
+        <x:v>29-3A</x:v>
+      </x:c>
+      <x:c r="C40" s="2" t="str">
+        <x:v>Guardia常服</x:v>
+      </x:c>
+      <x:c r="D40" s="2" t="str">
+        <x:v>庄园铁门与前庭（夜）</x:v>
+      </x:c>
+      <x:c r="E40" s="2" t="str">
+        <x:v>金色蝴蝶结礼盒；手电筒</x:v>
+      </x:c>
+      <x:c r="F40" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+庄园铁门与前庭（夜），9:16竖屏。庄园门灯作侧上方实用光，货车大灯朝街道，不直射Guardia常服正脸；手电只照车斗和吊坠。
+[音轨规则]
+远层：夜间空间的低弱环境底噪。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段无原定对白或旁白，不新增发声。
+[锚定列表]
+场景：@庄园铁门与前庭（夜）
+角色：@Guardia常服
+道具：@金色蝴蝶结礼盒；手电筒
+未带@的物件仅作剧本所需普通文字描述，不冒充已完成资产或新增绑定。
+[空间布局总览]
+庄园铁门沿东西向，庄园内部在北，街道在南，货车停在门外南侧，后车斗朝门口；Guardia常服在门内东侧岗亭，手电在右手。银色礼盒固定在后车斗中央，金色缎带与吊坠保持为同一套配件。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（5个硬切分镜）]
+分镜一：【景别/视角：铁门关系全景/门内东北侧 | 运镜：沿门内车道向南短推，停在铁门一侧】
+【时长】3.0s
+【构图】黑货车停门外，车斗中央为银色礼盒；Guardia常服从门内东侧岗亭走到门边，右手持手电。
+【音效】门扇与门锁随实际开合发声、脚步随起停出现；台词期间压低动作声。
+【台词】无台词。
+【变化】Guardia常服仍在门内，货车未开进庄园。
+【镜头结尾·站位收束】Guardia常服仍在门内，货车未开进庄园。
+画面硬切到分镜二。
+分镜二：【景别/视角：Guardia常服侧面中景 | 运镜：沿门内向西短移，保持铁门为前景】
+【时长】3.0s
+【构图】Guardia常服把手电从车轮上方移到后车斗，左手扶门栏，视线跟随光束。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】光束落到礼盒，右手未换持。
+【镜头结尾·站位收束】光束落到礼盒，右手未换持。
+画面硬切到分镜三。
+分镜三：【景别/视角：礼盒近景/铁门空隙取景 | 运镜：固定，金缎带与银色箱面产生不同反射】
+【时长】3.0s
+【构图】光束扫过金色蝴蝶结，再落到礼盒前左角吊坠；吊坠转动只随细链自然摆动。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】吊坠进入亮区，箱体保持固定。
+【镜头结尾·站位收束】吊坠进入亮区，箱体保持固定。
+画面硬切到分镜四。
+分镜四：【景别/视角：吊坠手电光特写 | 运镜：缓推至轮廓后停住，刻字面背向镜头】
+【时长】3.0s
+【构图】银吊坠以形状、链条与金缎带关系建立辨认，按全片政策不呈现其字母刻痕。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】吊坠仍挂在箱角，没有被拿走。
+【镜头结尾·站位收束】吊坠仍挂在箱角，没有被拿走。
+画面硬切到分镜五。
+分镜五：【景别/视角：Guardia常服近景 | 运镜：固定，手电留在下缘，视线有明确目标】
+【时长】3.0s
+【构图】Guardia常服看清后呼吸短停，手电光束轻偏后稳住；不新增脸色突变与夸张瞪眼。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】Guardia常服停在门内，目光留在礼盒上。
+【镜头结尾·站位收束】Guardia常服停在门内，目光留在礼盒上。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：15s</x:v>
+      </x:c>
+      <x:c r="G40" s="2" t="str"/>
+      <x:c r="H40" s="2" t="str">
+        <x:v>29-3 庄园铁门与前庭（Portón y explanada, Mansión Vargas） 夜 外
+人物：Guardia
+△ 画面全景：深夜，一辆黑色的厢式货车亮着刺眼的大灯，停在一座宏伟的庄园铁门前。庄园内主楼灯火通明，气氛森严。
+△ 动作特写：Guardia 穿着灰色的保安大衣，头戴大檐帽。他神情紧张，手里拿着一支手电筒，在大雨后的寒风中匆匆跑向铁门。
+△ 镜头切换：Guardia 跑到门边，将手电光照向货车的后车斗。
+△ 镜头特写：货车车斗上放着一个巨大的银色金属立方体礼盒。礼盒上缠绕着金色的缎带，顶端打着一个巨大的金色蝴蝶结。
+△ 镜头近景：Guardia 疑惑地皱起眉，将光束移向礼盒的侧面。
+△ 镜头特写：在礼盒的一角，挂着一个圆形的银色吊坠。吊坠中央刻着一个独特的字母"V"，在手电光下折射出冰冷的银光。
+△ 镜头切到 Guardia：他看清吊坠的瞬间，瞳孔骤然收缩，脸色变得惨白，整个人如同被定住了一般，眼神中充满了极度的惊恐。</x:v>
+      </x:c>
+      <x:c r="I40" s="2" t="str">
+        <x:v>15s</x:v>
+      </x:c>
     </x:row>
     <x:row r="41" ht="200" customHeight="1">
-      <x:c r="A41" s="2"/>
-      <x:c r="B41" s="2"/>
-      <x:c r="C41" s="2"/>
-      <x:c r="D41" s="2"/>
-      <x:c r="E41" s="2"/>
-      <x:c r="F41" s="2"/>
-      <x:c r="G41" s="2"/>
-      <x:c r="H41" s="2"/>
-      <x:c r="I41" s="2"/>
+      <x:c r="A41" s="2" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="B41" s="2" t="str">
+        <x:v>30-1A</x:v>
+      </x:c>
+      <x:c r="C41" s="2" t="str">
+        <x:v>Damián常服；Guardia常服</x:v>
+      </x:c>
+      <x:c r="D41" s="2" t="str">
+        <x:v>庄园铁门与前庭（夜）</x:v>
+      </x:c>
+      <x:c r="E41" s="2" t="str">
+        <x:v>金色蝴蝶结礼盒；手电筒</x:v>
+      </x:c>
+      <x:c r="F41" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+庄园铁门与前庭（夜），9:16竖屏。门灯与货车灯方向保持29-3一致，金缎带只反射真实光源。
+[音轨规则]
+远层：夜间空间的低弱环境底噪。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段无原定对白或旁白，不新增发声。
+[锚定列表]
+场景：@庄园铁门与前庭（夜）
+角色：@Damián常服；@Guardia常服
+道具：@金色蝴蝶结礼盒；手电筒
+未带@的物件仅作剧本所需普通文字描述，不冒充已完成资产或新增绑定。
+[空间布局总览]
+庄园铁门沿东西向，庄园内部在北，街道在南，货车停在门外南侧，后车斗朝门口；Guardia常服在门内东侧岗亭，手电在右手。银色礼盒固定在后车斗中央，金色缎带与吊坠保持为同一套配件。Guardia常服已在门内，礼盒仍在车斗。Damián常服从北侧主楼方向走向铁门，两名普通背景保镖随在其后，不复制Escolta A身份。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（4个硬切分镜）]
+分镜一：【景别/视角：车斗与Guardia常服中景 | 运镜：在门内东侧固定，保持前后位置一致】
+【时长】3.0s
+【构图】Guardia常服手电仍照礼盒前左角；黑色车身和湿地反射留在后景，箱体没有自行进门。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】Guardia常服在门边，礼盒仍在货车。
+【镜头结尾·站位收束】Guardia常服在门边，礼盒仍在货车。
+画面硬切到分镜二。
+分镜二：【景别/视角：Damián常服侧后全身中景 | 运镜：沿门内车道向南跟随，随他停步减速】
+【时长】3.0s
+【构图】Damián常服从主楼走到铁门内侧停下，两名背景保镖在其后一步收住。
+【音效】门扇与门锁随实际开合发声、脚步随起停出现；台词期间压低动作声。
+【台词】无台词。
+【变化】Damián常服到门内中央，Guardia常服在其东侧。
+【镜头结尾·站位收束】Damián常服到门内中央，Guardia常服在其东侧。
+画面硬切到分镜三。
+分镜三：【景别/视角：Damián常服近景/铁门东北侧 | 运镜：固定，视线越过门栏落在箱体】
+【时长】3.0s
+【构图】Damián常服先看蝴蝶结再看吊坠，眼睑略收；原造型保持Damián常服。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】Damián常服还未触碰礼盒。
+【镜头结尾·站位收束】Damián常服还未触碰礼盒。
+画面硬切到分镜四。
+分镜四：【景别/视角：缎带与吊坠近景 | 运镜：向箱角轻推后停住】
+【时长】3.0s
+【构图】金色缎带在夜风中略动，吊坠仍背向镜头，形状与银箱唤起回忆。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】以缎带的形状切入下一段闪回。
+【镜头结尾·站位收束】以缎带的形状切入下一段闪回。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：12s</x:v>
+      </x:c>
+      <x:c r="G41" s="2" t="str"/>
+      <x:c r="H41" s="2" t="str">
+        <x:v>第30集
+30-1 庄园铁门与前庭（Portón y explanada, Mansión Vargas） 夜 外
+人物：Damián、Guardia、Vera (Flashback)
+△ 镜头全景：夜晚的暴雨初歇，宏伟的庄园铁门在灯光下泛着冷冽的金属光泽。一辆黑色的厢式货车停在门外，大灯刺眼。
+△ 镜头特写：Guardia 穿着灰色保安制服，神情紧绷，手中颤抖的手电筒光束打在货车后座那个巨大的银色礼盒上。
+△ 镜头近景：Guardia 的视线死死盯着礼盒边缘挂着的银色"V"字吊坠。他的脸色由红转白，额头渗出细密的汗珠。
+△ 镜头切换：Damián 穿着深红棕色西装，神情冷峻地从庄园内走来，身后跟着两名保镖。他的脚步在大门口戛然而止，目光锁定了那个巨大的礼盒。
+△ 镜头特写：巨大的金色蝴蝶结在晚风中微微颤动。Damián 眯起双眼，眼神中透出一丝危险的怀疑。</x:v>
+      </x:c>
+      <x:c r="I41" s="2" t="str">
+        <x:v>12s</x:v>
+      </x:c>
     </x:row>
     <x:row r="42" ht="200" customHeight="1">
-      <x:c r="A42" s="2"/>
-      <x:c r="B42" s="2"/>
-      <x:c r="C42" s="2"/>
-      <x:c r="D42" s="2"/>
-      <x:c r="E42" s="2"/>
-      <x:c r="F42" s="2"/>
-      <x:c r="G42" s="2"/>
-      <x:c r="H42" s="2"/>
-      <x:c r="I42" s="2"/>
+      <x:c r="A42" s="2" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="B42" s="2" t="str">
+        <x:v>30-1B</x:v>
+      </x:c>
+      <x:c r="C42" s="2" t="str">
+        <x:v>Vera常服</x:v>
+      </x:c>
+      <x:c r="D42" s="2" t="str">
+        <x:v>庄园铁门与前庭</x:v>
+      </x:c>
+      <x:c r="E42" s="2" t="str">
+        <x:v>金色蝴蝶结礼盒</x:v>
+      </x:c>
+      <x:c r="F42" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+庄园铁门与前庭，9:16竖屏。前庭已有灯具在薄雾中形成柔和侧逆光，以空间与速度变化区分闪回，不叠加字幕或年代字样。
+[音轨规则]
+远层：夜间空间的低弱环境底噪。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段无原定对白或旁白，不新增发声。
+[锚定列表]
+场景：@庄园铁门与前庭
+角色：@Vera常服
+道具：@金色蝴蝶结礼盒
+[空间布局总览]
+本段为明确闪回：沿用已有庄园前庭空间，Vera常服使用已确认Vera常服，不派生白衬衫红领带新造型。入口在南，雾中主楼在北，礼盒位于前庭通道旁；相机不把闪回人物置入当前门口人群。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（2个硬切分镜）]
+分镜一：【景别/视角：Vera常服侧后全身中景 | 运镜：沿前庭通道向北伴随，避免冲入人物路线】
+【时长】3.0s
+【构图】Vera常服沿前庭空道向主楼跑过，衣摆随真实步速摆动；侧后机位保留同一身份与已有造型。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】Vera常服向北离开近景，未与当前时空人物同框。
+【镜头结尾·站位收束】Vera常服向北离开近景，未与当前时空人物同框。
+画面硬切到分镜二。
+分镜二：【景别/视角：礼盒与缎带近景 | 运镜：横向短移，落在金色缎带形状】
+【时长】3.0s
+【构图】银色箱体与金色蝴蝶结占据画面，光线与薄雾沿已有来源成立；镜头在形状落稳后切回现在。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】闪回结束于礼盒形状，未改变当前礼盒归属。
+【镜头结尾·站位收束】闪回结束于礼盒形状，未改变当前礼盒归属。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：6s</x:v>
+      </x:c>
+      <x:c r="G42" s="2" t="str"/>
+      <x:c r="H42" s="2" t="str">
+        <x:v>△ 镜头反打（闪回）：Vera 穿着白色衬衫，系着深红色领带，在豪宅前奔跑。背景是层叠的枯树和雾气中的大宅。
+△ 镜头特写（闪回）：一个巨大的银色保险箱状礼盒，上面系着金色的鳞片状缎带。</x:v>
+      </x:c>
+      <x:c r="I42" s="2" t="str">
+        <x:v>6s</x:v>
+      </x:c>
     </x:row>
     <x:row r="43" ht="200" customHeight="1">
-      <x:c r="A43" s="2"/>
-      <x:c r="B43" s="2"/>
-      <x:c r="C43" s="2"/>
-      <x:c r="D43" s="2"/>
-      <x:c r="E43" s="2"/>
-      <x:c r="F43" s="2"/>
-      <x:c r="G43" s="2"/>
-      <x:c r="H43" s="2"/>
-      <x:c r="I43" s="2"/>
+      <x:c r="A43" s="2" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="B43" s="2" t="str">
+        <x:v>30-2A</x:v>
+      </x:c>
+      <x:c r="C43" s="2" t="str">
+        <x:v>Damián常服；Don Ernesto常服；Víctor常服；Guardia常服；Reportera D VO</x:v>
+      </x:c>
+      <x:c r="D43" s="2" t="str">
+        <x:v>庄园大厅</x:v>
+      </x:c>
+      <x:c r="E43" s="2" t="str">
+        <x:v>金色蝴蝶结礼盒；礼盒内车辆徽章与便签；电视画面</x:v>
+      </x:c>
+      <x:c r="F43" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+庄园大厅，9:16竖屏。壁炉暖光从北侧形成轮廓，低亮吊灯照清箱盖接触区；电视冷光只作局部反射，无标题条或可读文字。
+[音轨规则]
+远层：夜间空间的低弱环境底噪。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
+6.1s—12.7s，Reportera D VO（VO，电视新闻VO，清晰平稳，不绑定未提供的音频）：「En cuarenta y ocho horas, las familias Vargas y Miranda ofrecerán una conferencia de prensa conjunta.」
+[锚定列表]
+场景：@庄园大厅
+角色：@Damián常服；@Don Ernesto常服；@Víctor常服；@Guardia常服；Reportera D VO
+道具：@金色蝴蝶结礼盒；礼盒内车辆徽章与便签；电视画面
+未带@的物件仅作剧本所需普通文字描述，不冒充已完成资产或新增绑定。
+[空间布局总览]
+庄园大厅北墙为壁炉及裂镜，沙发在中部偏西，电话几在东墙，南门通前庭，桌椅之间保留南北通道。本场与门外之间明确省略搬运过程：礼盒已被移到大厅中部稳固矮台上，Guardia常服在南门内，Damián常服站箱南侧，Víctor常服在其东后，Don Ernesto常服坐西侧沙发。箱盖起初仍闭合，电视在东侧墙面。Reportera D仅电视声源，按已授权作文字设定。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（7个硬切分镜）]
+分镜一：【景别/视角：大厅关系全景/南门内 | 运镜：向北短推，明确礼盒已在室内及各人位置】
+【时长】3.0s
+【构图】Damián常服站礼盒南侧，双手扶住箱盖边缘；Víctor常服在东后，Don Ernesto常服坐西侧沙发，Guardia常服守南门。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】箱体在矮台上固定，双手准备开盖。
+【镜头结尾·站位收束】箱体在矮台上固定，双手准备开盖。
+画面硬切到分镜二。
+分镜二：【景别/视角：箱盖与双手近景 | 运镜：固定在箱侧，留出盖子开启弧线】
+【时长】3.0s
+【构图】Damián常服先松开已解好的缎带，将盖子沿铰接方向掀起，双手避开夹缝；缎带留箱侧。
+【音效】箱体或扣锁的实际接触声；台词期间压低动作声。
+【台词】无台词。
+【变化】箱盖开启，箱体未移动。
+【镜头结尾·站位收束】箱盖开启，箱体未移动。
+画面硬切到分镜三。
+分镜三：【景别/视角：Don Ernesto常服侧面近景 | 运镜：从箱西南角轻摇到沙发】
+【时长】3.0s
+【构图】Don Ernesto常服听到开盖声抬眼，把原握酒杯放回沙发旁小几；电视新闻声从东墙开始。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】Reportera D VO的VO按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Don Ernesto常服空出右手，仍坐沙发。
+【镜头结尾·站位收束】Don Ernesto常服空出右手，仍坐沙发。
+画面硬切到分镜四。
+分镜四：【景别/视角：电视中景/大厅西侧 | 运镜：固定，避免镜头冲进屏幕】
+【时长】3.0s
+【构图】屏幕只呈金发女主持人的新闻影像和色块，不显示任何字形；Reportera D原VO持续，画面中人物口型属于电视节目。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】Reportera D VO的VO按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】新闻持续，大厅人物不代说。
+【镜头结尾·站位收束】新闻持续，大厅人物不代说。
+画面硬切到分镜五。
+分镜五：【景别/视角：Damián常服听者近景 | 运镜：回到箱南侧固定，保持同一手部状态】
+【时长】3.0s
+【构图】新闻VO跨切继续到完整句尾；Damián常服向箱内看，嘴唇轻合，双手已经离开开合边。
+【音效】箱体或扣锁的实际接触声；台词期间压低动作声。
+【台词】Reportera D VO的VO按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】新闻播报结束，Damián常服目光落向箱内。
+【镜头结尾·站位收束】新闻播报结束，Damián常服目光落向箱内。
+画面硬切到分镜六。
+分镜六：【景别/视角：箱内物件近景 | 运镜：由箱南侧轻俯，聚焦边沿而不探入液面】
+【时长】3.0s
+【构图】箱内金色流动表面反射暖光；徽章和便签放在高于液面的箱内边沿托片上，车辆剪影可见，便签字面不出现。
+【音效】箱体或扣锁的实际接触声；台词期间压低动作声。
+【台词】无台词。
+【变化】徽章与便签在干燥托片上，未滑入液体。
+【镜头结尾·站位收束】徽章与便签在干燥托片上，未滑入液体。
+画面硬切到分镜七。
+分镜七：【景别/视角：手指与徽章特写 | 运镜：固定，指尖接触点清楚可见】
+【时长】3.0s
+【构图】Damián常服右指只触干燥托片上的车辆徽章边缘，不把手伸入金色液面；随后松指，视线转到旁边便签。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】徽章留托片，右手准备取便签。
+【镜头结尾·站位收束】徽章留托片，右手准备取便签。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：21s</x:v>
+      </x:c>
+      <x:c r="G43" s="2" t="str">
+        <x:v>Reportera D VO：「En cuarenta y ocho horas, las familias Vargas y Miranda ofrecerán una conferencia de prensa conjunta.」</x:v>
+      </x:c>
+      <x:c r="H43" s="2" t="str">
+        <x:v>30-2 庄园大厅（Mansión Vargas, salón principal） 夜 内
+人物：Damián、Don Ernesto、Víctor、Guardia、Reportera D
+△ 动作特写：随着沉重的金属摩擦声，银色礼盒的盖子被 Damián 亲手缓缓推开。
+△ 镜头近景：Damián 的面部特写。他的瞳孔骤然放大，原本冷峻的神情被一种难以言喻的惊愕所取代。
+△ 镜头切换：Don Ernesto 坐在沙发上，原本正在端详手中的酒杯。他感觉到气氛不对，猛地抬起头，眼神中透出极度的警觉。
+△ 镜头全景：大厅内的电视屏幕亮起，正播报着突发新闻。画面中是那个熟悉的金发女主持人。
+【字幕：NOTICIAS DE ÚLTIMA HORA】
+Reportera D VO：En cuarenta y ocho horas, las familias Vargas y Miranda ofrecerán una conferencia de prensa conjunta.
+△ 镜头切换：Damián 站在礼盒前，他的视线缓缓下移。礼盒内部并不是什么恐怖的威胁，而是盛满了如液体般流动的熔融金水，正在灯光下泛着诡异的波光。
+△ 动作特写：Damián 伸出手指，触碰礼盒边缘的一枚徽章。徽章上刻着一辆复古小轿车的剪影。
+△ 镜头特写：徽章旁放着一张白色的便签纸。
+【字幕：Por el incendio Vargas. Sospechoso principal.】</x:v>
+      </x:c>
+      <x:c r="I43" s="2" t="str">
+        <x:v>21s</x:v>
+      </x:c>
     </x:row>
     <x:row r="44" ht="200" customHeight="1">
-      <x:c r="A44" s="2"/>
-      <x:c r="B44" s="2"/>
-      <x:c r="C44" s="2"/>
-      <x:c r="D44" s="2"/>
-      <x:c r="E44" s="2"/>
-      <x:c r="F44" s="2"/>
-      <x:c r="G44" s="2"/>
-      <x:c r="H44" s="2"/>
-      <x:c r="I44" s="2"/>
+      <x:c r="A44" s="2" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="B44" s="2" t="str">
+        <x:v>30-2B</x:v>
+      </x:c>
+      <x:c r="C44" s="2" t="str">
+        <x:v>Damián常服；Víctor常服；Don Ernesto常服；Guardia常服</x:v>
+      </x:c>
+      <x:c r="D44" s="2" t="str">
+        <x:v>庄园大厅</x:v>
+      </x:c>
+      <x:c r="E44" s="2" t="str">
+        <x:v>金色蝴蝶结礼盒；礼盒内便签</x:v>
+      </x:c>
+      <x:c r="F44" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+庄园大厅，9:16竖屏。沿用暖壁炉与低亮吊灯，纸面不呈现字形，人物转头后受光自然改变。
+[音轨规则]
+远层：夜间空间的低弱环境底噪。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
+3.1s—6.8s，@Damián常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「El rastro del Tejedor. Lleva diez años invisible.」
+[锚定列表]
+场景：@庄园大厅
+角色：@Damián常服；@Víctor常服；@Don Ernesto常服；@Guardia常服
+道具：@金色蝴蝶结礼盒；礼盒内便签
+未带@的物件仅作剧本所需普通文字描述，不冒充已完成资产或新增绑定。
+[空间布局总览]
+庄园大厅北墙为壁炉及裂镜，沙发在中部偏西，电话几在东墙，南门通前庭，桌椅之间保留南北通道。箱盖已开，箱内便签在干燥边沿托片。Damián常服在箱南侧，Víctor常服在东后，Don Ernesto常服仍坐西侧沙发，Guardia常服在南门。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（3个硬切分镜）]
+分镜一：【景别/视角：便签与Damián常服近景 | 运镜：由手部轻抬至脸，保持纸背朝镜头】
+【时长】3.0s
+【构图】Damián常服右手夹起便签，看完后转上身朝东后的Víctor常服；双脚留在箱南侧，不碰到液面。
+【音效】鞋底接触地面声、箱体或扣锁的实际接触声；台词期间压低动作声。
+【台词】无台词。
+【变化】便签在右手，Víctor常服处于他的视线方向。
+【镜头结尾·站位收束】便签在右手，Víctor常服处于他的视线方向。
+画面硬切到分镜二。
+分镜二：【景别/视角：Damián常服侧面中近景 | 运镜：固定，Víctor常服肩侧留作前景】
+【时长】4.0s
+【构图】Damián常服用低哑声线说出原句，重音在追踪的时间跨度，未新增任何解释。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Damián常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Damián常服右手持便签，箱盖仍开着。
+【镜头结尾·站位收束】Damián常服右手持便签，箱盖仍开着。
+画面硬切到分镜三。
+分镜三：【景别/视角：三人关系中景 | 运镜：缓慢后拉，露出西侧沙发上的Don Ernesto常服】
+【时长】3.0s
+【构图】Damián常服的声音延续至完整句尾，Víctor常服和Don Ernesto常服各看向他；物件和人员没有交换位置。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】句尾落在三人的沉默关系中，Guardia常服仍在门侧。
+【镜头结尾·站位收束】句尾落在三人的沉默关系中，Guardia常服仍在门侧。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：10s</x:v>
+      </x:c>
+      <x:c r="G44" s="2" t="str">
+        <x:v>Damián：「El rastro del Tejedor. Lleva diez años invisible.」</x:v>
+      </x:c>
+      <x:c r="H44" s="2" t="str">
+        <x:v>△ 镜头近景：Damián 拿起那张便签，手在微微颤抖。他猛地转过身，看向身后的 Víctor 和 Don Ernesto。
+Damián（声音嘶哑，带着压抑的愤怒）：El rastro del Tejedor. Lleva diez años invisible.</x:v>
+      </x:c>
+      <x:c r="I44" s="2" t="str">
+        <x:v>10s</x:v>
+      </x:c>
     </x:row>
     <x:row r="45" ht="200" customHeight="1">
-      <x:c r="A45" s="2"/>
-      <x:c r="B45" s="2"/>
-      <x:c r="C45" s="2"/>
-      <x:c r="D45" s="2"/>
-      <x:c r="E45" s="2"/>
-      <x:c r="F45" s="2"/>
-      <x:c r="G45" s="2"/>
-      <x:c r="H45" s="2"/>
-      <x:c r="I45" s="2"/>
+      <x:c r="A45" s="2" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="B45" s="2" t="str">
+        <x:v>30-3A</x:v>
+      </x:c>
+      <x:c r="C45" s="2" t="str">
+        <x:v>Vera常服；El Zorro Blanco VO</x:v>
+      </x:c>
+      <x:c r="D45" s="2" t="str">
+        <x:v>高层公寓客厅（夜）</x:v>
+      </x:c>
+      <x:c r="E45" s="2" t="str">
+        <x:v>iPhone手机；黑色皮手套；旧发票</x:v>
+      </x:c>
+      <x:c r="F45" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+高层公寓客厅（夜），9:16竖屏。窗外城市冷色与书桌边已有暖灯形成侧光，桌面文字背向镜头，手机无界面字形。
+[音轨规则]
+远层：公寓外远处车流低声，室内维持安静。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
+7.1s—13.9s，El Zorro Blanco VO（VO，电话VO，略窄频，仅文字设定声源，不绑定未提供的音频）：「El rastro del Tejedor. Lleva diez años invisible, pero el mes pasado salió a la superficie.」
+15.1s—16.0s，@Vera常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「¿Dónde?」
+18.1s—19.6s，El Zorro Blanco VO（VO，电话VO，略窄频，仅文字设定声源，不绑定未提供的音频）：「Valle de Bravo.」
+[锚定列表]
+场景：@高层公寓客厅（夜）
+角色：@Vera常服；El Zorro Blanco VO
+道具：@iPhone手机；@黑色皮手套；旧发票
+未带@的物件仅作剧本所需普通文字描述，不冒充已完成资产或新增绑定。
+[空间布局总览]
+公寓入口在西墙，茶几位于客厅中部、沙发在北侧，东墙落地窗可见城市，书桌工作区位于窗侧；南侧移门通阳台，桌椅之间保留南侧通道。世界方位不随反打改变。按本场实际动作与落地窗描述取既有公寓的窗侧书桌工作区，不新增独立密室结构。Vera常服坐书桌西侧面向东窗，已有米色风衣暂搭在南侧衣凳，旧发票和黑色皮手套平放桌上，手机在其右手边。El Zorro Blanco只作为电话VO，不入画。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（6个硬切分镜）]
+分镜一：【景别/视角：桌面与右手近景 | 运镜：沿桌沿向东短移，落在手套与发票边缘】
+【时长】3.0s
+【构图】Vera常服右指从旧发票边缘移到黑色皮手套，左手留在桌沿；发票纸面朝自己，镜头只见背面和旧纸纹理。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】发票与手套仍在桌面，右手准备拿手机。
+【镜头结尾·站位收束】发票与手套仍在桌面，右手准备拿手机。
+画面硬切到分镜二。
+分镜二：【景别/视角：Vera常服侧面近景 | 运镜：固定，手机背面与她的反应同时可读】
+【时长】4.0s
+【构图】Vera常服拿起手机，右指触屏发起第一次拨号；听到未接通的简短提示后停一下，再发起第二次通话；不显示号码或联系人文字。
+【音效】手指与机身接触的低弱摩擦声；台词期间压低动作声。
+【台词】无台词。
+【变化】第二次电话接通，Vera常服把手机贴右耳。
+【镜头结尾·站位收束】第二次电话接通，Vera常服把手机贴右耳。
+画面硬切到分镜三。
+分镜三：【景别/视角：Vera常服中近景/书桌南侧 | 运镜：缓推后停在她聆听的眼神】
+【时长】4.0s
+【构图】El Zorro Blanco以电话VO给出追踪消息，声音经电话略窄但词语清楚；Vera常服不做该句口型。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】El Zorro Blanco VO的VO按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Vera常服仍坐书桌前，右手持手机。
+【镜头结尾·站位收束】Vera常服仍坐书桌前，右手持手机。
+画面硬切到分镜四。
+分镜四：【景别/视角：手套与Vera常服侧后中景 | 运镜：沿书桌南侧短移，保留东窗与人物关系】
+【时长】4.0s
+【构图】电话原声跨切持续；Vera常服左手在桌沿停住，没有新增抓挠、颤抖或吸气。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】El Zorro Blanco VO的VO按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】来电者消息完整说完，Vera常服准备追问。
+【镜头结尾·站位收束】来电者消息完整说完，Vera常服准备追问。
+画面硬切到分镜五。
+分镜五：【景别/视角：Vera常服侧面近景 | 运镜：固定，给短问句一个清晰停点】
+【时长】3.0s
+【构图】Vera常服抬眼看向窗外，用一个短问句追问地点；右肘自然贴近身体。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Vera常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】手机还在右耳。
+【镜头结尾·站位收束】手机还在右耳。
+画面硬切到分镜六。
+分镜六：【景别/视角：Vera常服听者近景 | 运镜：轻向后拉，留出桌面与手部】
+【时长】3.0s
+【构图】El Zorro Blanco回答地名，Vera常服听完后目光停住，左手掌落在桌沿准备起身。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】El Zorro Blanco VO的VO按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】第二句VO结束，Vera常服仍坐稳。
+【镜头结尾·站位收束】第二句VO结束，Vera常服仍坐稳。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：21s</x:v>
+      </x:c>
+      <x:c r="G45" s="2" t="str">
+        <x:v>El Zorro Blanco VO：「El rastro del Tejedor. Lleva diez años invisible, pero el mes pasado salió a la superficie.」
+Vera：「¿Dónde?」
+El Zorro Blanco VO：「Valle de Bravo.」</x:v>
+      </x:c>
+      <x:c r="H45" s="2" t="str">
+        <x:v>30-3 高层公寓/密室（Departamento ejecutivo, Piso 21, Reforma） 夜 内
+人物：Vera、El Zorro Blanco (VO)
+△ 镜头近景：一张精致的木质桌面上，放着一张发黄的旧发票，抬头是"COMERCIALIZADORA DEL GOLFO Y CIA."，金额显示为"$500,000.00"。
+△ 动作特写：一只涂着深咖啡色指甲油的纤细右手伸入镜头，缓缓抚过桌上的一只黑色皮质手套。
+△ 镜头特写：手机屏幕亮起。手指在拨号盘上快速按下了"9"字键。
+△ 镜头反打：屏幕显示"LLAMADA FALLIDA"。Vera 眼神冷冽，没有丝毫犹豫，迅速按下了另一个快捷键。
+△ 镜头特写：屏幕上跳出联系人姓名——"El Zorro Blanco"。
+△ 镜头近景：Vera 坐在黑暗中，将手机贴在耳边。月光从窗外洒入，勾勒出她优越的轮廓。她的眼神深邃得如同深不见底的海潭。
+El Zorro Blanco VO：El rastro del Tejedor. Lleva diez años invisible, pero el mes pasado salió a la superficie.
+Vera（语气冷淡，带着一丝志在必得）：¿Dónde?
+El Zorro Blanco VO：Valle de Bravo.</x:v>
+      </x:c>
+      <x:c r="I45" s="2" t="str">
+        <x:v>21s</x:v>
+      </x:c>
     </x:row>
     <x:row r="46" ht="200" customHeight="1">
-      <x:c r="A46" s="2"/>
-      <x:c r="B46" s="2"/>
-      <x:c r="C46" s="2"/>
-      <x:c r="D46" s="2"/>
-      <x:c r="E46" s="2"/>
-      <x:c r="F46" s="2"/>
-      <x:c r="G46" s="2"/>
-      <x:c r="H46" s="2"/>
-      <x:c r="I46" s="2"/>
+      <x:c r="A46" s="2" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="B46" s="2" t="str">
+        <x:v>30-3B</x:v>
+      </x:c>
+      <x:c r="C46" s="2" t="str">
+        <x:v>Vera常服</x:v>
+      </x:c>
+      <x:c r="D46" s="2" t="str">
+        <x:v>高层公寓客厅（夜）</x:v>
+      </x:c>
+      <x:c r="E46" s="2" t="str">
+        <x:v>iPhone手机；米色风衣；黑色皮手套</x:v>
+      </x:c>
+      <x:c r="F46" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+高层公寓客厅（夜），9:16竖屏。落地窗外城市楼体只保留无字的红色光面，不显示时间或倒计时；室内暖灯继续形成侧逆光。
+[音轨规则]
+远层：公寓外远处车流低声，室内维持安静。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段无原定对白或旁白，不新增发声。
+[锚定列表]
+场景：@高层公寓客厅（夜）
+角色：@Vera常服
+道具：@iPhone手机；@米色风衣；@黑色皮手套
+[空间布局总览]
+公寓入口在西墙，茶几位于客厅中部、沙发在北侧，东墙落地窗可见城市，书桌工作区位于窗侧；南侧移门通阳台，桌椅之间保留南侧通道。世界方位不随反打改变。Vera常服在窗侧书桌西侧，手机在右手，手套和旧发票留桌面；外套为Vera常服已有米色风衣，不派生黑风衣。衣凳在她南侧，客厅向西通入口。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（4个硬切分镜）]
+分镜一：【景别/视角：Vera常服全身中景/书桌南侧 | 运镜：顺她起身轻抬，保留支撑手与双脚】
+【时长】3.0s
+【构图】Vera常服左手撑桌起身，右手把手机从耳边放低；双脚收稳后身体站直，不用镜头切换代替起身。
+【音效】鞋底接触地面声、手指与机身接触的低弱摩擦声；台词期间压低动作声。
+【台词】无台词。
+【变化】Vera常服站在书桌西侧，右手持手机。
+【镜头结尾·站位收束】Vera常服站在书桌西侧，右手持手机。
+画面硬切到分镜二。
+分镜二：【景别/视角：衣凳与人物中景 | 运镜：沿南侧通道短移，留出披衣动作空间】
+【时长】3.0s
+【构图】Vera常服把手机暂放桌沿，双手取起已有米色风衣披好，沿用原资产型制；不改变人物造型。
+【音效】手指与机身接触的低弱摩擦声；台词期间压低动作声。
+【台词】无台词。
+【变化】风衣已披好，手机在桌沿。
+【镜头结尾·站位收束】风衣已披好，手机在桌沿。
+画面硬切到分镜三。
+分镜三：【景别/视角：手部与口袋近景 | 运镜：固定，衣袋口与手机移动路径清楚】
+【时长】3.0s
+【构图】Vera常服右手从桌沿拿回手机，将机身收入右侧口袋，手指离开袋口；画面不出现屏幕内容。
+【音效】手指与机身接触的低弱摩擦声；台词期间压低动作声。
+【台词】无台词。
+【变化】手机在口袋，双手空出。
+【镜头结尾·站位收束】手机在口袋，双手空出。
+画面硬切到分镜四。
+分镜四：【景别/视角：客厅纵深中景/东窗朝西 | 运镜：在书桌侧固定，缓慢摇摄跟随人物离开工作区】
+【时长】3.5s
+【构图】Vera常服从书桌西侧沿客厅南侧通道走入较暗处；远处楼体红色光面只提供无字反射，手套留桌上。
+【音效】脚步随起停出现；台词期间压低动作声。
+【台词】无台词。
+【变化】Vera常服走向西侧入口方向，桌面手套与发票未随她移动。
+【镜头结尾·站位收束】Vera常服走向西侧入口方向，桌面手套与发票未随她移动。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：12.5s</x:v>
+      </x:c>
+      <x:c r="G46" s="2" t="str"/>
+      <x:c r="H46" s="2" t="str">
+        <x:v>△ 动作特写：Vera 猛地站起身，反手抓起桌上的黑色风衣，动作利落而充满力量感。
+△ 镜头切换：Vera 将手机塞入风衣内侧口袋。手机屏幕上赫然显示着当前时间：5:48 de la mañana。
+△ 镜头全景：落地窗外，改革大道夜景斑斓。远处最高建筑的顶端，巨大的红色 LED 倒计时显示屏正在跳动。
+【字幕：48:06:09】
+△ 镜头收尾：倒计时的红光映在 Vera 冰冷的双眸中，她转身步入阴影。</x:v>
+      </x:c>
+      <x:c r="I46" s="2" t="str">
+        <x:v>12.5s</x:v>
+      </x:c>
     </x:row>
     <x:row r="47" ht="200" customHeight="1">
       <x:c r="A47" s="2"/>

</xml_diff>

<commit_message>
Complete episodes 31–33 and verify the full 21–33 storyboard workbook
</commit_message>
<xml_diff>
--- a/archive/projects/la-reina-del-bajo-mundo/deliverables/前夫黑道酵母_分镜_21-33.xlsx
+++ b/archive/projects/la-reina-del-bajo-mundo/deliverables/前夫黑道酵母_分镜_21-33.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分镜脚本" sheetId="1" r:id="R662051841b0a4ddf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分镜脚本" sheetId="1" r:id="Rcda49bf7d9264f2f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5092,139 +5092,1523 @@
       </x:c>
     </x:row>
     <x:row r="47" ht="200" customHeight="1">
-      <x:c r="A47" s="2"/>
-      <x:c r="B47" s="2"/>
-      <x:c r="C47" s="2"/>
-      <x:c r="D47" s="2"/>
-      <x:c r="E47" s="2"/>
-      <x:c r="F47" s="2"/>
-      <x:c r="G47" s="2"/>
-      <x:c r="H47" s="2"/>
-      <x:c r="I47" s="2"/>
+      <x:c r="A47" s="2" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="B47" s="2" t="str">
+        <x:v>31-1A</x:v>
+      </x:c>
+      <x:c r="C47" s="2" t="str">
+        <x:v>Vera黑色晚宴装</x:v>
+      </x:c>
+      <x:c r="D47" s="2" t="str">
+        <x:v>高层公寓阳台</x:v>
+      </x:c>
+      <x:c r="E47" s="2" t="str">
+        <x:v>红色马克笔；白色法律文件</x:v>
+      </x:c>
+      <x:c r="F47" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+高层公寓阳台，9:16竖屏。暮色由城市方向映入，红色光面只形成无字的建筑反射；桌面受门内既有灯的间接侧光，文件不出现任何字形。
+[音轨规则]
+远层：公寓外远处车流低声，室内维持安静。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段无原定对白或旁白，不新增发声。
+[锚定列表]
+场景：@高层公寓阳台
+角色：@Vera黑色晚宴装
+道具：红色马克笔；白色法律文件
+普通物件及用户另行确认的文字设计项不带@，不冒充已完成资产或新增绑定。
+[空间布局总览]
+阳台北侧为通向公寓的推拉门，南侧栏杆外是城市天际线；Vera黑色晚宴装站阳台北侧小桌前，左手压文件，右手持红色马克笔。开场只从既有阳台向外取城市楼体局部，手部插镜仍在同一阳台，不把她放到楼外高空。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（4个硬切分镜）]
+分镜一：【景别/视角：城市楼体局部/阳台外望 | 运镜：在栏杆内固定，轻向上摇到楼体红色光面】
+【时长】3.0s
+【构图】开场越过栏杆观察改革大道楼体，红色光面由常亮变为一次短闪，再稳定；只呈无字色块。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】城市暮色仍在南侧，未显示数字或标题。
+【镜头结尾·站位收束】城市暮色仍在南侧，未显示数字或标题。
+画面硬切到分镜二。
+分镜二：【景别/视角：文件与双手俯拍近景 | 运镜：从阳台桌上方垂直观察，沿纸边短移】
+【时长】3.0s
+【构图】Vera黑色晚宴装左手压住白色文件一角，右手将马克笔笔尖落在纸面，沿横向画第一道红线；纸面不显示原印刷文字。
+【音效】马克笔尖擦过纸面的低弱声；台词期间压低动作声。
+【台词】无台词。
+【变化】第一道线完成，笔尖离纸，文件未移动。
+【镜头结尾·站位收束】第一道线完成，笔尖离纸，文件未移动。
+画面硬切到分镜三。
+分镜三：【景别/视角：右手侧面特写 | 运镜：固定在桌东侧，保留指尖和纸面接触】
+【时长】3.0s
+【构图】右手落笔画第二道红线，笔尖在第三处留白上方停住；不凭空出现字母或再次重画第一道。
+【音效】马克笔尖擦过纸面的低弱声；台词期间压低动作声。
+【台词】无台词。
+【变化】两道红线留纸面，右手停笔。
+【镜头结尾·站位收束】两道红线留纸面，右手停笔。
+画面硬切到分镜四。
+分镜四：【景别/视角：Vera黑色晚宴装侧后中景/阳台东侧 | 运镜：沿空置门前通道后拉，显出栏杆与桌的关系】
+【时长】3.0s
+【构图】Vera黑色晚宴装看着文件，肩背保持直立，手指将笔握稳；红色楼体反光只留在远处，不投出文字。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】Vera黑色晚宴装留桌前，文件与笔仍由左右手分别控制。
+【镜头结尾·站位收束】Vera黑色晚宴装留桌前，文件与笔仍由左右手分别控制。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：12s</x:v>
+      </x:c>
+      <x:c r="G47" s="2" t="str"/>
+      <x:c r="H47" s="2" t="str">
+        <x:v>第31集
+31-1 豪华大楼/外 暮 外
+人物：Vera
+△ 镜头俯拍特写：摩天大楼的玻璃幕墙上，一个巨大的红色数字显示屏正散发着刺眼的红光。显示屏上的数字固定在“00:00:00”。
+△ 镜头切换：画面闪烁，红色显示屏上的文字发生改变，背景是暗蓝色的改革大道天际线。
+【字幕：CONFERENCIA DE PRENSA: EN VIVO EN 24 HORAS】
+△ 镜头特写：Vera 戴着黑色皮质长手套的右手出现在镜头中。她正拿着一支鲜红色的马克笔，在一份白色的法律文件上用力划线。
+△ 动作特写：笔尖在“MATRIMONIO”和“EXTORSIÓN”这两个词上留下了粗重的红杠，最后停在了“ENFERMEDAD MENTAL”这一项上。</x:v>
+      </x:c>
+      <x:c r="I47" s="2" t="str">
+        <x:v>12s</x:v>
+      </x:c>
     </x:row>
     <x:row r="48" ht="200" customHeight="1">
-      <x:c r="A48" s="2"/>
-      <x:c r="B48" s="2"/>
-      <x:c r="C48" s="2"/>
-      <x:c r="D48" s="2"/>
-      <x:c r="E48" s="2"/>
-      <x:c r="F48" s="2"/>
-      <x:c r="G48" s="2"/>
-      <x:c r="H48" s="2"/>
-      <x:c r="I48" s="2"/>
+      <x:c r="A48" s="2" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="B48" s="2" t="str">
+        <x:v>31-2A</x:v>
+      </x:c>
+      <x:c r="C48" s="2" t="str">
+        <x:v>Vera黑色晚宴装；Emiliano常服</x:v>
+      </x:c>
+      <x:c r="D48" s="2" t="str">
+        <x:v>高层公寓客厅（日）</x:v>
+      </x:c>
+      <x:c r="E48" s="2" t="str">
+        <x:v>白色法律文件；红色马克笔</x:v>
+      </x:c>
+      <x:c r="F48" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+高层公寓客厅（日），9:16竖屏。沿用日景公寓结构，将东窗光写为临近日落的弱侧光，已有落地灯提供暖侧逆光；不把暮色改成正午。
+[音轨规则]
+远层：公寓外远处车流低声，室内维持安静。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
+0.2s—2.4s，@Emiliano常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Valle de Bravo puede esperar.」
+6.1s—9.5s，@Vera黑色晚宴装（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Cuarenta y ocho horas me bastan para callarlos.」
+[锚定列表]
+场景：@高层公寓客厅（日）
+角色：@Vera黑色晚宴装；@Emiliano常服
+道具：白色法律文件；红色马克笔
+普通物件及用户另行确认的文字设计项不带@，不冒充已完成资产或新增绑定。
+[空间布局总览]
+客厅东侧为落地窗，北侧是沙发，餐桌在西侧，阳台在南；Vera黑色晚宴装已由阳台进屋坐北侧沙发，马克笔与文件放茶几。Emiliano常服站餐桌东侧，手上没有文件；两人隔茶几与空道交流。沿用已有对应造型，不新增黑皮风衣版本。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（5个硬切分镜）]
+分镜一：【景别/视角：客厅关系中全景/南侧通道 | 运镜：由阳台门内侧向北短移，落在餐桌与沙发关系】
+【时长】3.0s
+【构图】Emiliano常服站西侧餐桌边，Vera黑色晚宴装坐北侧沙发；他理平已有西装袖口，向她开口。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Emiliano常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】两人不因反打换座或换造型。
+【镜头结尾·站位收束】两人不因反打换座或换造型。
+画面硬切到分镜二。
+分镜二：【景别/视角：Vera黑色晚宴装侧面中近景 | 运镜：从茶几东侧固定，沙发扶手构成边界】
+【时长】3.0s
+【构图】Emiliano常服句尾跨切传来，Vera黑色晚宴装看向他，右手整理既有晚宴装肩侧布料后落回扶手；不另披未确认黑风衣。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】Vera黑色晚宴装仍坐沙发，手已放稳。
+【镜头结尾·站位收束】Vera黑色晚宴装仍坐沙发，手已放稳。
+画面硬切到分镜三。
+分镜三：【景别/视角：Vera黑色晚宴装近景/茶几南侧 | 运镜：从沙发对角缓推至目光落点】
+【时长】4.0s
+【构图】Vera黑色晚宴装说出原句，声音偏低但清楚，重音落在时间与行动意图；不额外发笑。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Vera黑色晚宴装的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Vera黑色晚宴装说话时自然开合嘴唇。
+【镜头结尾·站位收束】Vera黑色晚宴装说话时自然开合嘴唇。
+画面硬切到分镜四。
+分镜四：【景别/视角：Emiliano常服听者中近景 | 运镜：在餐桌南侧固定，以沙发边缘作远景】
+【时长】3.0s
+【构图】Vera黑色晚宴装原声到完整句尾，Emiliano常服目光留在她脸上，手指松开袖口。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】Emiliano常服留餐桌旁，无新增回答。
+【镜头结尾·站位收束】Emiliano常服留餐桌旁，无新增回答。
+画面硬切到分镜五。
+分镜五：【景别/视角：双人关系中景 | 运镜：沿南侧通道向西后拉，显出两人之间的空道】
+【时长】3.0s
+【构图】Vera黑色晚宴装下颌稍抬后停住，Emiliano常服保持站姿；纸笔留茶几，为出发前的决定留短停顿。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】人物与桌面物件均在原位。
+【镜头结尾·站位收束】人物与桌面物件均在原位。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：16s</x:v>
+      </x:c>
+      <x:c r="G48" s="2" t="str">
+        <x:v>Emiliano：「Valle de Bravo puede esperar.」
+Vera：「Cuarenta y ocho horas me bastan para callarlos.」</x:v>
+      </x:c>
+      <x:c r="H48" s="2" t="str">
+        <x:v>31-2 高层公寓/客厅 暮 内
+人物：Emiliano、Vera
+△ 镜头中景：Emiliano 穿着一套修身的黑色三件套西装，白色衬衫领口微微敞开。他站在餐桌旁，双手整理着脱下的黑色大衣，神情冷峻而忧郁。
+Emiliano（低声，语气果断）：Valle de Bravo puede esperar.
+△ 镜头反打：Vera 坐在沙发上，她穿着一件抹胸式的黑色修身长裙，长发如海藻般披散在肩头。她微微侧身，将黑色皮质长风衣披在身上，动作优雅且充满攻击性。
+△ 镜头特写：Vera 的面部特写。她画着深邃的烟熏妆，眼神犀利如刀，嘴角勾起一抹冷酷的弧度。
+Vera（语气冰冷且自信）：Cuarenta y ocho horas me bastan para callarlos.</x:v>
+      </x:c>
+      <x:c r="I48" s="2" t="str">
+        <x:v>16s</x:v>
+      </x:c>
     </x:row>
     <x:row r="49" ht="200" customHeight="1">
-      <x:c r="A49" s="2"/>
-      <x:c r="B49" s="2"/>
-      <x:c r="C49" s="2"/>
-      <x:c r="D49" s="2"/>
-      <x:c r="E49" s="2"/>
-      <x:c r="F49" s="2"/>
-      <x:c r="G49" s="2"/>
-      <x:c r="H49" s="2"/>
-      <x:c r="I49" s="2"/>
+      <x:c r="A49" s="2" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="B49" s="2" t="str">
+        <x:v>31-3A</x:v>
+      </x:c>
+      <x:c r="C49" s="2" t="str">
+        <x:v>Oficial A常服</x:v>
+      </x:c>
+      <x:c r="D49" s="2" t="str">
+        <x:v>酒店正门（外·日）</x:v>
+      </x:c>
+      <x:c r="E49" s="2" t="str">
+        <x:v>两辆警车；黑色轿车</x:v>
+      </x:c>
+      <x:c r="F49" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+酒店正门（外·日），9:16竖屏。午后日光从西南侧斜照立面，入口檐口提供自然阴影；警灯只在车身和地面形成短促红蓝反射，招牌无字。
+[音轨规则]
+远层：门外实际车流底噪，车辆停稳后发动机声降低，人物附近安静。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段无原定对白或旁白，不新增发声。
+[锚定列表]
+场景：酒店正门（外·日）
+角色：@Oficial A常服
+道具：两辆警车；黑色轿车
+普通物件及用户另行确认的文字设计项不带@，不冒充已完成资产或新增绑定。
+[空间布局总览]
+酒店正门沿东西向立面，门内大厅在北、门外车道在南；门前有三层宽台阶，东侧留缓坡。黑色轿车沿东西向停在台阶南侧，右后车门朝北面向台阶；门外西侧留相机通道。外景按已获授权的文字设计，保持日夜为同一建筑，不冒用其他场景标签。Oficial A站门口东侧，另一名普通警员站西侧，功能性警员不另绑定人物身份。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（3个硬切分镜）]
+分镜一：【景别/视角：酒店外景全景/车道西侧 | 运镜：沿人行空道向东平移，落在正门与两辆警车关系】
+【时长】3.0s
+【构图】黑色豪车停在门前车道，两辆警车分停入口东西两侧；门口警员在台阶两端维持通道，车辆不封住台阶。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】酒店入口与通行路线清楚，车门均关闭。
+【镜头结尾·站位收束】酒店入口与通行路线清楚，车门均关闭。
+画面硬切到分镜二。
+分镜二：【景别/视角：警员与入口中景/台阶西南侧 | 运镜：从车身前景向北短移，显出门前的警员】
+【时长】3.0s
+【构图】Oficial A留东侧，普通警员在西侧抬手示意来客沿中央入口通行；只作无词手势，不新增口令。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】中央入口保持畅通，警员没有离岗。
+【镜头结尾·站位收束】中央入口保持畅通，警员没有离岗。
+画面硬切到分镜三。
+分镜三：【景别/视角：酒店门面中全景 | 运镜：从台阶下方轻向上摇到入口檐口后停住】
+【时长】3.0s
+【构图】入口玻璃反射车道与日光，原招牌位置仅留建筑色面；原稿酒店名和会务标题不显示。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】以门框结构切入同一酒店大厅。
+【镜头结尾·站位收束】以门框结构切入同一酒店大厅。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：9s</x:v>
+      </x:c>
+      <x:c r="G49" s="2" t="str"/>
+      <x:c r="H49" s="2" t="str">
+        <x:v>31-3 晚宴酒店/大厅 日 外/内
+人物：Víctor、Don Ernesto、Vera、Empleado A、Empleado B、Empleado C、Reportero C、Oficial A、Oficial B
+△ 镜头全景：阳光明媚。圣安琪尔大酒店的正门口停满了黑色豪车。两辆警车闪烁着红蓝警灯停在入口处，多名警察正在维持秩序。
+【字幕：HOTEL SAN ÁNGEL IMPERIAL】
+【字幕：CUMBRE FUTURO GLOBAL 2025 - CONFERENCIA DE PRENSA -】</x:v>
+      </x:c>
+      <x:c r="I49" s="2" t="str">
+        <x:v>9s</x:v>
+      </x:c>
     </x:row>
     <x:row r="50" ht="200" customHeight="1">
-      <x:c r="A50" s="2"/>
-      <x:c r="B50" s="2"/>
-      <x:c r="C50" s="2"/>
-      <x:c r="D50" s="2"/>
-      <x:c r="E50" s="2"/>
-      <x:c r="F50" s="2"/>
-      <x:c r="G50" s="2"/>
-      <x:c r="H50" s="2"/>
-      <x:c r="I50" s="2"/>
+      <x:c r="A50" s="2" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="B50" s="2" t="str">
+        <x:v>31-3B</x:v>
+      </x:c>
+      <x:c r="C50" s="2" t="str">
+        <x:v>Víctor常服；Don Ernesto常服；Reportero C常服；Mujer OS</x:v>
+      </x:c>
+      <x:c r="D50" s="2" t="str">
+        <x:v>晚宴酒店大厅</x:v>
+      </x:c>
+      <x:c r="E50" s="2" t="str">
+        <x:v>单反相机；麦克风</x:v>
+      </x:c>
+      <x:c r="F50" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+晚宴酒店大厅，9:16竖屏。沿用大厅吊灯与侧窗日光：窗光由西侧斜照，吊灯提供低弱环境亮度；背景板为无字色块，快门闪光短促，不把全场反复洗白。
+[音轨规则]
+远层：日间发布会低弱人群底噪，快门与无词议论声低于台词。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
+3.1s—7.3s，Mujer OS（OS，台下未具名年轻女子的现场OS，嘴部不入画，声音从座位方向传来，不改为旁白）：「Cada noche sueño que está parada junto a mi cama.」
+15.6s—18.2s，@Víctor常服（对白，发布会现场发声，重音与音量随语义提高，字词不破音，不新增吼叫词）：「Hoy vamos a desenmascarar un fraude.」
+[锚定列表]
+场景：@晚宴酒店大厅
+角色：@Víctor常服；@Don Ernesto常服；@Reportero C常服；Mujer OS
+道具：单反相机；麦克风
+普通物件及用户另行确认的文字设计项不带@，不冒充已完成资产或新增绑定。
+[空间布局总览]
+会场设于既有晚宴酒店大厅：讲台在北侧矮台，座席面向北；中央通道南北向，主入口在南墙向厅内开，东侧有台阶通矮台。Vera黑色晚宴装在前排西侧靠中央通道座位，Damián常服在前排东侧；Reportero C常服在西侧边道拍摄。Víctor常服在讲台后，Don Ernesto常服站台上东侧，Carmen常服站台上西侧。三名功能性员工在后排西侧，其中一名负责传递文件，不冒充人物表Empleada A。讲台只有一支无线手持麦克风，起初固定于支架；谁拿到它谁发声扩声，其他现场对白保持真实空间声源，不复制麦克风。此时Vera黑色晚宴装尚未进场；Mujer为台下未具名年轻女子的现场OS，只作普通群众和声源描述，不新增身份资产。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（7个硬切分镜）]
+分镜一：【景别/视角：会场全景/南端中央通道 | 运镜：从入口向北短推，前排座位框出舞台】
+【时长】3.0s
+【构图】Reportero C常服在西侧边道举相机，记者与宾客已经入座；Vera黑色晚宴装前排西侧位置暂空。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】记者留各自座席或边道，中央通道畅通。
+【镜头结尾·站位收束】记者留各自座席或边道，中央通道畅通。
+画面硬切到分镜二。
+分镜二：【景别/视角：年轻女子眼部与手部近景 | 运镜：固定在座位斜前方，嘴部留画外】
+【时长】3.0s
+【构图】未具名年轻女子坐台下，指尖压住膝上衣料，眼角已有泪痕；其原定OS从同一座位方向传来，嘴部始终不入画。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】Mujer OS的OS按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】女子仍坐着，声源没有改为旁白。
+【镜头结尾·站位收束】女子仍坐着，声源没有改为旁白。
+画面硬切到分镜三。
+分镜三：【景别/视角：前排听众侧后中景 | 运镜：沿西侧边道短移，露出相机与听众的不同深度】
+【时长】3.5s
+【构图】女子OS连续说完，附近记者举起手机和相机；画面只见机身背面，不出现文字界面。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】Mujer OS的OS按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】所有设备留各自拍摄者手中。
+【镜头结尾·站位收束】所有设备留各自拍摄者手中。
+画面硬切到分镜四。
+分镜四：【景别/视角：舞台侧面中全景/东侧台阶 | 运镜：从台阶南端向北伴随，落在台阶上段】
+【时长】3.0s
+【构图】Víctor常服踏上东侧台阶，Don Ernesto常服随后登阶，二人顺序不变；沿用各自已有造型。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】Víctor常服已上台，Don Ernesto常服到台阶上段。
+【镜头结尾·站位收束】Víctor常服已上台，Don Ernesto常服到台阶上段。
+画面硬切到分镜五。
+分镜五：【景别/视角：讲台关系中景/台前东南侧 | 运镜：从台阶向西短摇，跟到两人各自停步】
+【时长】3.0s
+【构图】Víctor常服沿台前走到讲台后，Don Ernesto常服上完台阶停在台上东侧，右手理平原有领口；按已有造型不新增眼镜。
+【音效】脚步随起停出现；台词期间压低动作声。
+【台词】无台词。
+【变化】Víctor常服到讲台，Don Ernesto常服留台上东侧。
+【镜头结尾·站位收束】Víctor常服到讲台，Don Ernesto常服留台上东侧。
+画面硬切到分镜六。
+分镜六：【景别/视角：Víctor常服侧面近景 | 运镜：在讲台西南侧轻推，保护嘴部和麦克风距离】
+【时长】3.0s
+【构图】Víctor常服双手搭讲台边，靠近支架麦克风，发出原定开场句。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Víctor常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Víctor常服站位不变，麦克风仍在支架。
+【镜头结尾·站位收束】Víctor常服站位不变，麦克风仍在支架。
+画面硬切到分镜七。
+分镜七：【景别/视角：记者与台上关系中景 | 运镜：从西边道向南短拉，以相机形成前景】
+【时长】3.0s
+【构图】Víctor常服原声结束，Reportero C常服继续对准讲台，听众目光集中；不新增欢呼或音乐。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】会场秩序仍完整，入口保持空置。
+【镜头结尾·站位收束】会场秩序仍完整，入口保持空置。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：21.5s</x:v>
+      </x:c>
+      <x:c r="G50" s="2" t="str">
+        <x:v>Mujer OS：「Cada noche sueño que está parada junto a mi cama.」
+Víctor：「Hoy vamos a desenmascarar un fraude.」</x:v>
+      </x:c>
+      <x:c r="H50" s="2" t="str">
+        <x:v>△ 镜头切换：发布会大厅内。几十名穿着正装的记者和宾客已经入座。Reportero C 拿着单反相机正对准讲台，快门声此起彼伏，闪光灯不断闪烁。
+△ 镜头特写：一名年轻女子坐在台下，眼眶湿润，一颗硕大的泪珠顺着脸颊滑落。她神情哀戚，嘴唇微微颤抖。
+Mujer OS：Cada noche sueño que está parada junto a mi cama.
+△ 镜头全景：台下的记者们神情严肃，纷纷举起手机或相机进行拍摄。
+△ 动作特写：背景板上印着“CUMBRE FUTURO GLOBAL 2025 - CONFERENCIA DE PRENSA -”。Víctor 迈着稳健的步伐走上讲台，他穿着一套黑金花纹的华丽西装，神情倨傲。Don Ernesto 穿着灰色西装紧随其后。
+△ 镜头近景：Don Ernesto 走到发言席，他伸手推了推架在鼻梁上的无框眼镜，眼神中透着一种老辣的精明。
+△ 镜头切到 Víctor：他站在麦克风前，双手撑在讲台上，目光扫视全场，声音低沉洪亮。
+Víctor：Hoy vamos a desenmascarar un fraude.</x:v>
+      </x:c>
+      <x:c r="I50" s="2" t="str">
+        <x:v>21.5s</x:v>
+      </x:c>
     </x:row>
     <x:row r="51" ht="200" customHeight="1">
-      <x:c r="A51" s="2"/>
-      <x:c r="B51" s="2"/>
-      <x:c r="C51" s="2"/>
-      <x:c r="D51" s="2"/>
-      <x:c r="E51" s="2"/>
-      <x:c r="F51" s="2"/>
-      <x:c r="G51" s="2"/>
-      <x:c r="H51" s="2"/>
-      <x:c r="I51" s="2"/>
+      <x:c r="A51" s="2" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="B51" s="2" t="str">
+        <x:v>31-3C</x:v>
+      </x:c>
+      <x:c r="C51" s="2" t="str">
+        <x:v>Vera黑色晚宴装；Víctor常服；Don Ernesto常服；Reportero C常服</x:v>
+      </x:c>
+      <x:c r="D51" s="2" t="str">
+        <x:v>晚宴酒店大厅</x:v>
+      </x:c>
+      <x:c r="E51" s="2" t="str">
+        <x:v>单反相机；麦克风</x:v>
+      </x:c>
+      <x:c r="F51" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+晚宴酒店大厅，9:16竖屏。沿用大厅吊灯与侧窗日光：窗光由西侧斜照，吊灯提供低弱环境亮度；背景板为无字色块，快门闪光短促，不把全场反复洗白。
+[音轨规则]
+远层：日间发布会低弱人群底噪，快门与无词议论声低于台词。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段无原定对白或旁白，不新增发声。
+[锚定列表]
+场景：@晚宴酒店大厅
+角色：@Vera黑色晚宴装；@Víctor常服；@Don Ernesto常服；@Reportero C常服
+道具：单反相机；麦克风
+普通物件及用户另行确认的文字设计项不带@，不冒充已完成资产或新增绑定。
+[空间布局总览]
+会场设于既有晚宴酒店大厅：讲台在北侧矮台，座席面向北；中央通道南北向，主入口在南墙向厅内开，东侧有台阶通矮台。Vera黑色晚宴装在前排西侧靠中央通道座位，Damián常服在前排东侧；Reportero C常服在西侧边道拍摄。Víctor常服在讲台后，Don Ernesto常服站台上东侧，Carmen常服站台上西侧。三名功能性员工在后排西侧，其中一名负责传递文件，不冒充人物表Empleada A。讲台只有一支无线手持麦克风，起初固定于支架；谁拿到它谁发声扩声，其他现场对白保持真实空间声源，不复制麦克风。Vera黑色晚宴装从南门进入，前排西侧靠中央通道的座位空着。Emiliano常服尚未走入本段镜头。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（5个硬切分镜）]
+分镜一：【景别/视角：鞋与门槛低位近景 | 运镜：从门内西侧侧向伴随，落在完整跨门后的支撑脚】
+【时长】3.0s
+【构图】Vera黑色晚宴装穿已有晚宴装与原鞋履跨过南门槛，裙摆随步伐摆动，门扇已开，不穿过玻璃。
+【音效】门扇与门锁随实际开合发声；台词期间压低动作声。
+【台词】无台词。
+【变化】Vera黑色晚宴装双脚已到厅内。
+【镜头结尾·站位收束】Vera黑色晚宴装双脚已到厅内。
+画面硬切到分镜二。
+分镜二：【景别/视角：Vera黑色晚宴装侧后全身中景 | 运镜：沿中央通道同向跟随，保持前排目标可见】
+【时长】4.0s
+【构图】Vera黑色晚宴装沿中央通道向北走，记者转头看她；相机在其侧后，未同时要求看到正面细微表情。
+【音效】脚步随起停出现；台词期间压低动作声。
+【台词】无台词。
+【变化】她到前排西侧座位旁。
+【镜头结尾·站位收束】她到前排西侧座位旁。
+画面硬切到分镜三。
+分镜三：【景别/视角：Vera黑色晚宴装与空座侧面中景 | 运镜：沿座排前侧空道短弧移动，落在入座动作】
+【时长】3.0s
+【构图】Vera黑色晚宴装由通道移到空椅前，背朝椅背、面向北侧讲台，手扶椅侧，屈膝坐下；裙摆落稳后才交叠双腿。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】Vera黑色晚宴装坐前排西侧，双脚与裙摆位置稳定。
+【镜头结尾·站位收束】Vera黑色晚宴装坐前排西侧，双脚与裙摆位置稳定。
+画面硬切到分镜四。
+分镜四：【景别/视角：Vera黑色晚宴装近景/讲台侧向南 | 运镜：固定，以座椅靠背呈框架】
+【时长】3.0s
+【构图】她把双手放到膝上，看向北侧讲台的Víctor常服；相机位于该视线旁侧，不要求直视镜头。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】双手留膝上，目光落在讲台。
+【镜头结尾·站位收束】双手留膝上，目光落在讲台。
+画面硬切到分镜五。
+分镜五：【景别/视角：前排至舞台关系高角度中全景 | 运镜：由西侧边道较高处轻向东摇，显出台下与台上距离】
+【时长】2.5s
+【构图】Vera黑色晚宴装在前排坐定，Víctor常服在讲台后；Don Ernesto常服在台上东侧，中央通道未被占满。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】发布会双方位置成立，进入下一集对峙。
+【镜头结尾·站位收束】发布会双方位置成立，进入下一集对峙。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：15.5s</x:v>
+      </x:c>
+      <x:c r="G51" s="2" t="str"/>
+      <x:c r="H51" s="2" t="str">
+        <x:v>△ 镜头特写：Vera 踩着细高跟鞋步入会场。她穿着黑色抹胸裙，黑色皮质长手套拉至肘部，眼神冷漠而高傲。
+△ 动作特写：Vera 在众人的注视下，从容地走到前排空位坐下。她优雅地叠起双腿，双手交叠放在膝盖上，直视着台上的 Víctor。
+△ 镜头定格：Vera 的正面近景。她面无表情地看着镜头，眼神中充满了挑衅与不屑，仿佛在等待一场好戏开幕。</x:v>
+      </x:c>
+      <x:c r="I51" s="2" t="str">
+        <x:v>15.5s</x:v>
+      </x:c>
     </x:row>
     <x:row r="52" ht="200" customHeight="1">
-      <x:c r="A52" s="2"/>
-      <x:c r="B52" s="2"/>
-      <x:c r="C52" s="2"/>
-      <x:c r="D52" s="2"/>
-      <x:c r="E52" s="2"/>
-      <x:c r="F52" s="2"/>
-      <x:c r="G52" s="2"/>
-      <x:c r="H52" s="2"/>
-      <x:c r="I52" s="2"/>
+      <x:c r="A52" s="2" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B52" s="2" t="str">
+        <x:v>32-1A</x:v>
+      </x:c>
+      <x:c r="C52" s="2" t="str">
+        <x:v>Vera黑色晚宴装；Víctor常服；Don Ernesto常服；Damián常服；Carmen常服；Reportero C常服；Escolta A常服</x:v>
+      </x:c>
+      <x:c r="D52" s="2" t="str">
+        <x:v>晚宴酒店大厅</x:v>
+      </x:c>
+      <x:c r="E52" s="2" t="str">
+        <x:v>麦克风；单反相机</x:v>
+      </x:c>
+      <x:c r="F52" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+晚宴酒店大厅，9:16竖屏。沿用大厅吊灯与侧窗日光：窗光由西侧斜照，吊灯提供低弱环境亮度；背景板为无字色块，快门闪光短促，不把全场反复洗白。
+[音轨规则]
+远层：日间发布会低弱人群底噪，快门与无词议论声低于台词。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
+3.1s—4.2s，@Víctor常服（对白，发布会现场发声，重音与音量随语义提高，字词不破音，不新增吼叫词）：「Vera Saldaña.」
+6.1s—8.6s，@Víctor常服（对白，发布会现场发声，重音与音量随语义提高，字词不破音，不新增吼叫词）：「Mentalmente inestable. Con tendencias violentas.」
+9.6s—11.8s，@Carmen常服（对白，现场发声带轻微不稳，句子完整，不加入哭声语词）：「Mi hija nunca fue normal.」
+12.6s—16.3s，@Carmen常服（对白，现场发声带轻微不稳，句子完整，不加入哭声语词）：「Mentía, robaba, golpeaba gente. La aguantamos veinte años.」
+[锚定列表]
+场景：@晚宴酒店大厅
+角色：@Vera黑色晚宴装；@Víctor常服；@Don Ernesto常服；@Damián常服；@Carmen常服；@Reportero C常服；@Escolta A常服
+道具：麦克风；单反相机
+普通物件及用户另行确认的文字设计项不带@，不冒充已完成资产或新增绑定。
+[空间布局总览]
+会场设于既有晚宴酒店大厅：讲台在北侧矮台，座席面向北；中央通道南北向，主入口在南墙向厅内开，东侧有台阶通矮台。Vera黑色晚宴装在前排西侧靠中央通道座位，Damián常服在前排东侧；Reportero C常服在西侧边道拍摄。Víctor常服在讲台后，Don Ernesto常服站台上东侧，Carmen常服站台上西侧。三名功能性员工在后排西侧，其中一名负责传递文件，不冒充人物表Empleada A。讲台只有一支无线手持麦克风，起初固定于支架；谁拿到它谁发声扩声，其他现场对白保持真实空间声源，不复制麦克风。Escolta A常服在南门东侧边道，Carmen常服在上一场间隔已到台上西侧；Emiliano常服在南端中央通道外，尚未到前排。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（7个硬切分镜）]
+分镜一：【景别/视角：Vera黑色晚宴装侧面近景/前排东南侧 | 运镜：缓推，北侧讲台留画外视线目标】
+【时长】3.0s
+【构图】Vera黑色晚宴装坐前排西侧，目光向北，头部仅稍抬；双手仍在膝上，不重做入座。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】Vera黑色晚宴装在原座位。
+【镜头结尾·站位收束】Vera黑色晚宴装在原座位。
+画面硬切到分镜二。
+分镜二：【景别/视角：Víctor常服近景/讲台西南侧 | 运镜：固定，支架麦克风与嘴部同框】
+【时长】3.0s
+【构图】Víctor常服点出Vera黑色晚宴装全名，稍停后眼睑收窄；原资产伤疤保持，不重设计标记。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Víctor常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Víctor常服仍在讲台后。
+【镜头结尾·站位收束】Víctor常服仍在讲台后。
+画面硬切到分镜三。
+分镜三：【景别/视角：Vera黑色晚宴装过肩望台上中景 | 运镜：在前排西侧固定，Vera黑色晚宴装肩背为近景、Víctor常服为中景】
+【时长】3.5s
+【构图】Víctor常服继续抛出指控，Vera黑色晚宴装肩背不动；背景板不出现文字。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Víctor常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】指控句尾完整落下。
+【镜头结尾·站位收束】指控句尾完整落下。
+画面硬切到分镜四。
+分镜四：【景别/视角：Carmen常服近景/讲台东南侧 | 运镜：从Víctor常服侧面短摇到Carmen常服，落稳后保护口型】
+【时长】3.0s
+【构图】Carmen常服靠近讲台西侧的同一麦克风说话范围，Víctor常服向东让半步；她看向记者开口，声音不稳但词句完整。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Carmen常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Carmen常服站台上西侧，麦克风未离支架。
+【镜头结尾·站位收束】Carmen常服站台上西侧，麦克风未离支架。
+画面硬切到分镜五。
+分镜五：【景别/视角：Carmen常服侧面近景 | 运镜：沿台前空道向西短移，背景听众形成纵深】
+【时长】4.0s
+【构图】Carmen常服继续控诉，手掌压在讲台侧沿；已有泪痕不再叠加抽泣声或面部扭曲。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Carmen常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Carmen常服手留台侧，句尾完整。
+【镜头结尾·站位收束】Carmen常服手留台侧，句尾完整。
+画面硬切到分镜六。
+分镜六：【景别/视角：Damián常服手臂与上身中景 | 运镜：固定在前排东侧边道，保留他与座位关系】
+【时长】3.0s
+【构图】Damián常服站到座椅旁，左手把右袖往上推到前臂，右脚向中央通道挪半步后停住；沿用现有常服。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】Damián常服在座侧站定，未冲上舞台。
+【镜头结尾·站位收束】Damián常服在座侧站定，未冲上舞台。
+画面硬切到分镜七。
+分镜七：【景别/视角：记者前景与人群中景 | 运镜：沿西边道向南侧移，显出相机和听众转头】
+【时长】3.0s
+【构图】Reportero C常服按快门，背景三名员工与宾客交换目光；议论保持无词低声，不新增可辨台词。
+【音效】实际快门声，次数随画内按键出现；台词期间压低动作声。
+【台词】无台词。
+【变化】中央通道仍可通行，Damián常服留座侧。
+【镜头结尾·站位收束】中央通道仍可通行，Damián常服留座侧。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：22.5s</x:v>
+      </x:c>
+      <x:c r="G52" s="2" t="str">
+        <x:v>Víctor：「Vera Saldaña.」
+Víctor：「Mentalmente inestable. Con tendencias violentas.」
+Carmen：「Mi hija nunca fue normal.」
+Carmen：「Mentía, robaba, golpeaba gente. La aguantamos veinte años.」</x:v>
+      </x:c>
+      <x:c r="H52" s="2" t="str">
+        <x:v>第32集
+32-1 发布会大厅 日 内
+人物：Vera、Víctor、Don Ernesto、Damián、Emiliano、Carmen、EscoltaA、Empleado A、Empleado B、Empleado C、Reportero C
+△ 画面特写：Vera 的侧脸。她微微抬起下巴，神情冷峻而从容。她的睫毛纤长，眼神中透着一种洞察一切的锐利。
+△ 镜头切换：Víctor 站在讲台后，身着黑金花纹西装。他身体微微前倾，靠近麦克风，眼神阴鸷。
+Víctor：Vera Saldaña.
+△ 画面特写：Víctor 脸部近景。他额角的伤疤在灯光下清晰可见，咬牙切齿地吐出后续的词句。
+Víctor：Mentalmente inestable. Con tendencias violentas.
+△ 镜头反打：Carmen 站在 Víctor 身边，她面容憔悴，眼眶通红，泪水顺着布满皱纹的脸颊滑落。她神情激动地对着镜头控诉。
+Carmen（声音颤抖，带着哭腔）：Mi hija nunca fue normal.
+△ 画面特写：Carmen 的侧脸。她因为极度的表演性情绪而面部扭曲，眼神中透着一种疯狂的虚假。
+Carmen：Mentía, robaba, golpeaba gente. La aguantamos veinte años.
+△ 动作特写：台下，Damián 穿着棕色麂皮夹克，正愤怒地伸手撸起右手的衣袖，露出结实的小臂，作势要冲上台。
+△ 镜头快速切换：多名记者按下快门，镁光灯如雨点般密集闪烁。Reportero C 举着相机，神情紧绷。
+△ 镜头切到台下宾客：人们交头接耳，露出震惊和鄙夷的神色。</x:v>
+      </x:c>
+      <x:c r="I52" s="2" t="str">
+        <x:v>22.5s</x:v>
+      </x:c>
     </x:row>
     <x:row r="53" ht="200" customHeight="1">
-      <x:c r="A53" s="2"/>
-      <x:c r="B53" s="2"/>
-      <x:c r="C53" s="2"/>
-      <x:c r="D53" s="2"/>
-      <x:c r="E53" s="2"/>
-      <x:c r="F53" s="2"/>
-      <x:c r="G53" s="2"/>
-      <x:c r="H53" s="2"/>
-      <x:c r="I53" s="2"/>
+      <x:c r="A53" s="2" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B53" s="2" t="str">
+        <x:v>32-1B</x:v>
+      </x:c>
+      <x:c r="C53" s="2" t="str">
+        <x:v>Vera黑色晚宴装；Emiliano常服；Víctor常服；Carmen常服；Don Ernesto常服；Damián常服</x:v>
+      </x:c>
+      <x:c r="D53" s="2" t="str">
+        <x:v>晚宴酒店大厅</x:v>
+      </x:c>
+      <x:c r="E53" s="2" t="str">
+        <x:v>麦克风；公证文件</x:v>
+      </x:c>
+      <x:c r="F53" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+晚宴酒店大厅，9:16竖屏。沿用大厅吊灯与侧窗日光：窗光由西侧斜照，吊灯提供低弱环境亮度；背景板为无字色块，快门闪光短促，不把全场反复洗白。
+[音轨规则]
+远层：日间发布会低弱人群底噪，快门与无词议论声低于台词。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
+0.2s—1.7s，@Emiliano常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Soy su abogado.」
+3.6s—5.4s，@Emiliano常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Tiene derecho a réplica.」
+16.6s—20.3s，@Vera黑色晚宴装（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Hace dos semanas… ¿qué fue lo que firmaste?」
+[锚定列表]
+场景：@晚宴酒店大厅
+角色：@Vera黑色晚宴装；@Emiliano常服；@Víctor常服；@Carmen常服；@Don Ernesto常服；@Damián常服
+道具：麦克风；公证文件
+普通物件及用户另行确认的文字设计项不带@，不冒充已完成资产或新增绑定。
+[空间布局总览]
+会场设于既有晚宴酒店大厅：讲台在北侧矮台，座席面向北；中央通道南北向，主入口在南墙向厅内开，东侧有台阶通矮台。Vera黑色晚宴装在前排西侧靠中央通道座位，Damián常服在前排东侧；Reportero C常服在西侧边道拍摄。Víctor常服在讲台后，Don Ernesto常服站台上东侧，Carmen常服站台上西侧。三名功能性员工在后排西侧，其中一名负责传递文件，不冒充人物表Empleada A。讲台只有一支无线手持麦克风，起初固定于支架；谁拿到它谁发声扩声，其他现场对白保持真实空间声源，不复制麦克风。Emiliano常服从中央通道南端向前排走，左手持厚文件靠身侧；Vera黑色晚宴装仍坐前排西侧。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（7个硬切分镜）]
+分镜一：【景别/视角：Emiliano常服侧后中景/中央通道 | 运镜：沿通道向北跟随，保持空位和讲台可见】
+【时长】3.5s
+【构图】Emiliano常服走向前排，在Vera黑色晚宴装座后放慢脚步，抬眼朝讲台发声；左手文件不换手。
+【音效】鞋底接触地面声、脚步随起停出现；台词期间压低动作声。
+【台词】@Emiliano常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】他到Vera黑色晚宴装身后约半步。
+【镜头结尾·站位收束】他到Vera黑色晚宴装身后约半步。
+画面硬切到分镜二。
+分镜二：【景别/视角：Emiliano常服与Vera黑色晚宴装双人侧面中景 | 运镜：从西侧座排前方向东短弧，落在站者与坐者关系】
+【时长】3.0s
+【构图】Emiliano常服站定，低眼看向Vera黑色晚宴装后向台上补充回应；Vera黑色晚宴装仍坐着听完。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Emiliano常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Emiliano常服站座后，Vera黑色晚宴装准备起身。
+【镜头结尾·站位收束】Emiliano常服站座后，Vera黑色晚宴装准备起身。
+画面硬切到分镜三。
+分镜三：【景别/视角：Vera黑色晚宴装起身全身中景 | 运镜：从座椅侧面固定，完整呈现支撑与站起】
+【时长】3.0s
+【构图】Vera黑色晚宴装双手从膝上移到椅侧，双脚收稳后起身；Emiliano常服后退半步给她让出通道。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】Vera黑色晚宴装站在前排中央通道边。
+【镜头结尾·站位收束】Vera黑色晚宴装站在前排中央通道边。
+画面硬切到分镜四。
+分镜四：【景别/视角：Vera黑色晚宴装侧后全身中景 | 运镜：沿台前空道向东跟随，东侧台阶保持在画面前方】
+【时长】4.0s
+【构图】Vera黑色晚宴装从前排沿台前空道走到东侧台阶，手扶栏边，踏上前两级；步速正常。
+【音效】脚步随起停出现；台词期间压低动作声。
+【台词】无台词。
+【变化】Vera黑色晚宴装到台阶上段，未瞬移到讲台。
+【镜头结尾·站位收束】Vera黑色晚宴装到台阶上段，未瞬移到讲台。
+画面硬切到分镜五。
+分镜五：【景别/视角：讲台关系中景/台阶西南侧 | 运镜：轻向北摇，跟到她在讲台南侧站稳】
+【时长】3.0s
+【构图】Vera黑色晚宴装上完台阶，沿台上前沿走到讲台南侧；Víctor常服与Carmen常服退到讲台后东、西两侧，Don Ernesto常服仍在更东侧。
+【音效】脚步随起停出现；台词期间压低动作声。
+【台词】无台词。
+【变化】Vera黑色晚宴装在麦克风南侧可及处，未改变其他人方位。
+【镜头结尾·站位收束】Vera黑色晚宴装在麦克风南侧可及处，未改变其他人方位。
+画面硬切到分镜六。
+分镜六：【景别/视角：Vera黑色晚宴装近景/台前东南侧 | 运镜：轻推到她与Carmen常服对视的落点】
+【时长】4.0s
+【构图】Vera黑色晚宴装抬眼看Carmen常服，发出原问句；麦克风仍在支架，她没有抢夺它。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Vera黑色晚宴装的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Vera黑色晚宴装说完，目光留Carmen常服。
+【镜头结尾·站位收束】Vera黑色晚宴装说完，目光留Carmen常服。
+画面硬切到分镜七。
+分镜七：【景别/视角：Carmen常服听者近景 | 运镜：固定，讲台边线形成斜线】
+【时长】2.5s
+【构图】Carmen常服唇部短暂张开又收住，没有回答；Víctor常服肩侧留背景，未新增可辨低语。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】Carmen常服停在讲台后西侧。
+【镜头结尾·站位收束】Carmen常服停在讲台后西侧。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：23s</x:v>
+      </x:c>
+      <x:c r="G53" s="2" t="str">
+        <x:v>Emiliano：「Soy su abogado.」
+Emiliano：「Tiene derecho a réplica.」
+Vera：「Hace dos semanas… ¿qué fue lo que firmaste?」</x:v>
+      </x:c>
+      <x:c r="H53" s="2" t="str">
+        <x:v>△ 镜头全景：大厅中央的过道上。Emiliano 穿着一身笔挺的黑色三件套西装，金发梳理得整齐划一，正大步走向台前。
+Emiliano（语气平稳但充满威慑力）：Soy su abogado.
+△ 镜头特写：Emiliano 走到 Vera 身后站定，低头看向正坐着的 Vera。Vera 依旧保持着优雅的坐姿，面无表情。
+Emiliano：Tiene derecho a réplica.
+△ 动作特写：Vera 站起身，黑色抹胸长裙勾勒出她曼妙而冷硬的线条。她踩着细高跟鞋，从容地走上讲台，站在了 Víctor 和 Carmen 面前。
+△ 镜头近景：Vera 直视着 Carmen，眼神冰冷如铁。Carmen 眼神闪躲，不敢与她对视。
+Vera：Hace dos semanas… ¿qué fue lo que firmaste?
+△ 镜头切换：Carmen 愣在原地，嘴唇微微颤动，却发不出声音。Víctor 在一旁脸色铁青。</x:v>
+      </x:c>
+      <x:c r="I53" s="2" t="str">
+        <x:v>23s</x:v>
+      </x:c>
     </x:row>
     <x:row r="54" ht="200" customHeight="1">
-      <x:c r="A54" s="2"/>
-      <x:c r="B54" s="2"/>
-      <x:c r="C54" s="2"/>
-      <x:c r="D54" s="2"/>
-      <x:c r="E54" s="2"/>
-      <x:c r="F54" s="2"/>
-      <x:c r="G54" s="2"/>
-      <x:c r="H54" s="2"/>
-      <x:c r="I54" s="2"/>
+      <x:c r="A54" s="2" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B54" s="2" t="str">
+        <x:v>32-1C</x:v>
+      </x:c>
+      <x:c r="C54" s="2" t="str">
+        <x:v>Vera黑色晚宴装；Emiliano常服；Víctor常服；Carmen常服；Don Ernesto常服；Reportero C常服</x:v>
+      </x:c>
+      <x:c r="D54" s="2" t="str">
+        <x:v>晚宴酒店大厅</x:v>
+      </x:c>
+      <x:c r="E54" s="2" t="str">
+        <x:v>公证文件；麦克风；单反相机</x:v>
+      </x:c>
+      <x:c r="F54" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+晚宴酒店大厅，9:16竖屏。沿用大厅吊灯与侧窗日光：窗光由西侧斜照，吊灯提供低弱环境亮度；背景板为无字色块，快门闪光短促，不把全场反复洗白。
+[音轨规则]
+远层：日间发布会低弱人群底噪，快门与无词议论声低于台词。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
+0.2s—3.5s，@Emiliano常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Notariada. Firmada por toda la familia Saldaña.」
+6.1s—10.7s，@Emiliano常服（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Declarando a la señorita Saldaña «en pleno uso de sus facultades».」
+10.9s—16.3s，@Vera黑色晚宴装（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「El día que se llevaron mis doscientos mil pesos, ahí sí estaba cuerda.」
+17.1s—21.2s，@Vera黑色晚宴装（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「Se acabó el dinero… y de pronto estoy loca.」
+[锚定列表]
+场景：@晚宴酒店大厅
+角色：@Vera黑色晚宴装；@Emiliano常服；@Víctor常服；@Carmen常服；@Don Ernesto常服；@Reportero C常服
+道具：公证文件；麦克风；单反相机
+普通物件及用户另行确认的文字设计项不带@，不冒充已完成资产或新增绑定。
+[空间布局总览]
+会场设于既有晚宴酒店大厅：讲台在北侧矮台，座席面向北；中央通道南北向，主入口在南墙向厅内开，东侧有台阶通矮台。Vera黑色晚宴装在前排西侧靠中央通道座位，Damián常服在前排东侧；Reportero C常服在西侧边道拍摄。Víctor常服在讲台后，Don Ernesto常服站台上东侧，Carmen常服站台上西侧。三名功能性员工在后排西侧，其中一名负责传递文件，不冒充人物表Empleada A。讲台只有一支无线手持麦克风，起初固定于支架；谁拿到它谁发声扩声，其他现场对白保持真实空间声源，不复制麦克风。Vera黑色晚宴装站讲台南侧，Víctor常服在讲台后东侧，Carmen常服在后西侧。Emiliano常服已由座后走到台前西侧，左手持成套文件副本；一名功能性员工在其西侧准备接件。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（7个硬切分镜）]
+分镜一：【景别/视角：文件交接侧面近景/台前西侧 | 运镜：固定，双方接触和松手都在画内】
+【时长】3.0s
+【构图】Emiliano常服左手把成套公证文件递向员工，员工双手接住底边并夹稳，Emiliano常服才松手；他同时说明文件性质。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Emiliano常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】副本归员工，Emiliano常服左手空出。
+【镜头结尾·站位收束】副本归员工，Emiliano常服左手空出。
+画面硬切到分镜二。
+分镜二：【景别/视角：员工与前排中景 | 运镜：沿前排通行空道向北短移，落在分发过程】
+【时长】3.0s
+【构图】员工把文件分成已装订的副本，递给两位前排记者；每次记者握稳后员工才松手。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Emiliano常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】两份副本分别在两名记者手中，其余留员工。
+【镜头结尾·站位收束】两份副本分别在两名记者手中，其余留员工。
+画面硬切到分镜三。
+分镜三：【景别/视角：记者翻阅手部俯视近景 | 运镜：由西侧边道较高机位向下观察，保留纸背与订口】
+【时长】4.0s
+【构图】Emiliano常服在台前现场继续说明公证内容，声音自然转画外；记者只翻一次页，纸面不出现字迹。
+【音效】纸张轻擦声；台词期间压低动作声。
+【台词】@Emiliano常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】副本保持各自归属，Emiliano常服仍在台前西侧。
+【镜头结尾·站位收束】副本保持各自归属，Emiliano常服仍在台前西侧。
+画面硬切到分镜四。
+分镜四：【景别/视角：Vera黑色晚宴装侧面近景/台前东南侧 | 运镜：从文件方向轻摇回Vera黑色晚宴装，落稳在开口】
+【时长】3.5s
+【构图】Emiliano常服说完后Vera黑色晚宴装接话，略侧头看文件方向，再把目光转回Carmen常服；语气清楚，嘴角只轻收。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Emiliano常服的对白按本段唯一声音骨架连续发声；@Vera黑色晚宴装的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Vera黑色晚宴装留讲台南侧，话筒仍在支架。
+【镜头结尾·站位收束】Vera黑色晚宴装留讲台南侧，话筒仍在支架。
+画面硬切到分镜五。
+分镜五：【景别/视角：Carmen常服与Víctor常服听者中景 | 运镜：固定在讲台南方，保留两人实际间距】
+【时长】3.5s
+【构图】Vera黑色晚宴装上句连续跨切到句尾，Carmen常服视线移向纸背，Víctor常服下颌绷紧；二人不做她的口型。
+【音效】纸张轻擦声；台词期间压低动作声。
+【台词】@Vera黑色晚宴装的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】两名听者仍在台后原位。
+【镜头结尾·站位收束】两名听者仍在台后原位。
+画面硬切到分镜六。
+分镜六：【景别/视角：Vera黑色晚宴装正侧近景 | 运镜：沿台前向东短弧，落在她看向听众的眼神】
+【时长】4.0s
+【构图】Vera黑色晚宴装继续补完第二句判断，按省略号自然停顿；不把一句拆成两次重新起音。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Vera黑色晚宴装的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Vera黑色晚宴装说完，右手仍空着。
+【镜头结尾·站位收束】Vera黑色晚宴装说完，右手仍空着。
+画面硬切到分镜七。
+分镜七：【景别/视角：讲台与台前关系中景 | 运镜：短拉显示Víctor常服与麦克风之间的半步距离】
+【时长】2.0s
+【构图】Vera黑色晚宴装看向台下，Víctor常服从东后方准备上前，Carmen常服让开侧边；文件仍在记者和员工手中。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Vera黑色晚宴装的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Víctor常服尚未取走话筒，下一动作有明确起点。
+【镜头结尾·站位收束】Víctor常服尚未取走话筒，下一动作有明确起点。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：23s</x:v>
+      </x:c>
+      <x:c r="G54" s="2" t="str">
+        <x:v>Emiliano：「Notariada. Firmada por toda la familia Saldaña.」
+Emiliano：「Declarando a la señorita Saldaña «en pleno uso de sus facultades».」
+Vera：「El día que se llevaron mis doscientos mil pesos, ahí sí estaba cuerda.」
+Vera：「Se acabó el dinero… y de pronto estoy loca.」</x:v>
+      </x:c>
+      <x:c r="H54" s="2" t="str">
+        <x:v>△ 镜头切到 Emiliano：他将一份厚厚的文件递给台下的工作人员，动作利落。
+Emiliano：Notariada. Firmada por toda la familia Saldaña.
+△ 动作特写：工作人员接过文件，分发给前排的记者。记者们纷纷低头翻阅。
+Emiliano：Declarando a la señorita Saldaña «en pleno uso de sus facultades».
+△ 镜头近景：Vera 站在麦克风前，微微侧头看向那份文件，嘴角勾起一抹讥讽的笑意。
+Vera：El día que se llevaron mis doscientos mil pesos, ahí sí estaba cuerda.
+△ 镜头特写：Vera 眼神如炬，逼视着台下的众人，声音清冷而有力。
+Vera：Se acabó el dinero… y de pronto estoy loca.</x:v>
+      </x:c>
+      <x:c r="I54" s="2" t="str">
+        <x:v>23s</x:v>
+      </x:c>
     </x:row>
     <x:row r="55" ht="200" customHeight="1">
-      <x:c r="A55" s="2"/>
-      <x:c r="B55" s="2"/>
-      <x:c r="C55" s="2"/>
-      <x:c r="D55" s="2"/>
-      <x:c r="E55" s="2"/>
-      <x:c r="F55" s="2"/>
-      <x:c r="G55" s="2"/>
-      <x:c r="H55" s="2"/>
-      <x:c r="I55" s="2"/>
+      <x:c r="A55" s="2" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B55" s="2" t="str">
+        <x:v>32-1D</x:v>
+      </x:c>
+      <x:c r="C55" s="2" t="str">
+        <x:v>Vera黑色晚宴装；Víctor常服；Don Ernesto常服；Carmen常服；Emiliano常服；Escolta A常服；Tiburcio常服；Reportero C常服</x:v>
+      </x:c>
+      <x:c r="D55" s="2" t="str">
+        <x:v>晚宴酒店大厅</x:v>
+      </x:c>
+      <x:c r="E55" s="2" t="str">
+        <x:v>麦克风；单反相机</x:v>
+      </x:c>
+      <x:c r="F55" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+晚宴酒店大厅，9:16竖屏。沿用大厅吊灯与侧窗日光：窗光由西侧斜照，吊灯提供低弱环境亮度；背景板为无字色块，快门闪光短促，不把全场反复洗白。
+[音轨规则]
+远层：日间发布会低弱人群底噪，快门与无词议论声低于台词。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
+3.1s—5.2s，@Víctor常服（对白，发布会现场发声，重音与音量随语义提高，字词不破音，不新增吼叫词）：「¿Cuerda? ¡Entonces explique ESTO!」
+6.1s—9.1s，@Víctor常服（对白，发布会现场发声，重音与音量随语义提高，字词不破音，不新增吼叫词）：「¡Hace diez años esta mujer no EXISTÍA!」
+10.1s—11.6s，@Víctor常服（对白，发布会现场发声，重音与音量随语义提高，字词不破音，不新增吼叫词）：「¡Traigan al testigo!」
+[锚定列表]
+场景：@晚宴酒店大厅
+角色：@Vera黑色晚宴装；@Víctor常服；@Don Ernesto常服；@Carmen常服；@Emiliano常服；@Escolta A常服；@Tiburcio常服；@Reportero C常服
+道具：麦克风；单反相机
+普通物件及用户另行确认的文字设计项不带@，不冒充已完成资产或新增绑定。
+[空间布局总览]
+会场设于既有晚宴酒店大厅：讲台在北侧矮台，座席面向北；中央通道南北向，主入口在南墙向厅内开，东侧有台阶通矮台。Vera黑色晚宴装在前排西侧靠中央通道座位，Damián常服在前排东侧；Reportero C常服在西侧边道拍摄。Víctor常服在讲台后，Don Ernesto常服站台上东侧，Carmen常服站台上西侧。三名功能性员工在后排西侧，其中一名负责传递文件，不冒充人物表Empleada A。讲台只有一支无线手持麦克风，起初固定于支架；谁拿到它谁发声扩声，其他现场对白保持真实空间声源，不复制麦克风。Vera黑色晚宴装在讲台南侧，Víctor常服在东后半步，Carmen常服在后西侧。Tiburcio常服在南门外，Escolta A常服与一名普通安保各扶其一侧上臂；不复制Escolta A常服身份。Emiliano常服在台前西侧。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（8个硬切分镜）]
+分镜一：【景别/视角：麦克风与两人中近景/台前东南侧 | 运镜：固定，手掌与支架接触清楚】
+【时长】3.0s
+【构图】Víctor常服跨前半步，右手从支架抽走麦克风；Vera黑色晚宴装把右侧肩线向西让出，手不与他争夺。
+【音效】手与话筒支架实际接触的轻响；台词期间压低动作声。
+【台词】无台词。
+【变化】话筒在Víctor常服右手，支架留空。
+【镜头结尾·站位收束】话筒在Víctor常服右手，支架留空。
+画面硬切到分镜二。
+分镜二：【景别/视角：Víctor常服近景 | 运镜：缓推至其开口，话筒不遮嘴】
+【时长】3.0s
+【构图】Víctor常服靠近右手话筒，发出质问，音量提高但字词不破音；Vera黑色晚宴装在他西侧半步。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Víctor常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Víctor常服右手未换位。
+【镜头结尾·站位收束】Víctor常服右手未换位。
+画面硬切到分镜三。
+分镜三：【景别/视角：Víctor常服侧面中景 | 运镜：由讲台西南侧向南摇少许，保留指向入口的左手】
+【时长】4.0s
+【构图】Víctor常服左手指向南门，给出关于十年前的指控；右手始终持话筒。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Víctor常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】左手指向入口，右手话筒在嘴前。
+【镜头结尾·站位收束】左手指向入口，右手话筒在嘴前。
+画面硬切到分镜四。
+分镜四：【景别/视角：Vera黑色晚宴装听者近景/台前东侧 | 运镜：固定，入口留在她视线转向的画外方向】
+【时长】2.5s
+【构图】Víctor常服下令带证人，Vera黑色晚宴装只把视线转向南门；下令词保留同一现场声源。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Víctor常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Vera黑色晚宴装看向南门，未离开舞台。
+【镜头结尾·站位收束】Vera黑色晚宴装看向南门，未离开舞台。
+画面硬切到分镜五。
+分镜五：【景别/视角：南门至通道中全景/西边道 | 运镜：先对南门固定，开门后沿通道同向短移】
+【时长】4.0s
+【构图】普通安保先用空出的外侧手推门，再重新扶住Tiburcio常服上臂；Escolta A常服扶另一侧，两人带他跨门槛进入中央通道。
+【音效】门扇与门锁随实际开合发声；台词期间压低动作声。
+【台词】无台词。
+【变化】三人都已在厅内，门扇不穿过身体。
+【镜头结尾·站位收束】三人都已在厅内，门扇不穿过身体。
+画面硬切到分镜六。
+分镜六：【景别/视角：证人侧后全身中景 | 运镜：沿中央通道向北跟随，舞台保持前方目标】
+【时长】4.0s
+【构图】Tiburcio常服被带到台前中央，双脚仍自行落地；两名看管者在其两侧随行，帽檐遮住上半脸。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】三人到台前中央停下，Escolta A常服在证人东侧。
+【镜头结尾·站位收束】三人到台前中央停下，Escolta A常服在证人东侧。
+画面硬切到分镜七。
+分镜七：【景别/视角：Tiburcio常服近景/台前西侧 | 运镜：从手臂接触轻摇至帽檐下的眼神】
+【时长】3.0s
+【构图】Tiburcio常服抬头少许，嘴唇压合，目光不与Vera黑色晚宴装对上；不新加吞咽声。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】他站台下中央，两臂仍被扶住。
+【镜头结尾·站位收束】他站台下中央，两臂仍被扶住。
+画面硬切到分镜八。
+分镜八：【景别/视角：会场关系高角度中全景 | 运镜：从西边道较高位置向东短摇，显出舞台与证人】
+【时长】2.5s
+【构图】记者同时举机，短促快门与闪光集中到证人；背景板仍无可读文字。
+【音效】实际快门声，次数随画内按键出现；台词期间压低动作声。
+【台词】无台词。
+【变化】台上台下位置成立，证人未上台。
+【镜头结尾·站位收束】台上台下位置成立，证人未上台。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：26s</x:v>
+      </x:c>
+      <x:c r="G55" s="2" t="str">
+        <x:v>Víctor：「¿Cuerda? ¡Entonces explique ESTO!」
+Víctor：「¡Hace diez años esta mujer no EXISTÍA!」
+Víctor：「¡Traigan al testigo!」</x:v>
+      </x:c>
+      <x:c r="H55" s="2" t="str">
+        <x:v>△ 镜头切换：Víctor 猛地跨前一步，一把夺过麦克风，对着 Vera 怒吼，五官因愤怒而显得狰狞。
+Víctor：¿Cuerda? ¡Entonces explique ESTO!
+△ 镜头特写：Víctor 伸手一指大厅入口处，眼神中充满了报复的快感。
+Víctor：¡Hace diez años esta mujer no EXISTÍA!
+△ 镜头切到 Víctor：他对着台下大声下令，气势汹汹。
+Víctor：¡Traigan al testigo!
+△ 动作特写：大厅后方的大门被推开。两名保镖架着一个身材瘦削、神情颓废的男人走了进来。男人戴着一顶破旧的棕色棒球帽，低着头，看不清面容。
+△ 镜头近景：那个戴帽子的男人被带到台前。他穿着一件脏旧的军绿色夹克，整个人显得畏畏缩缩。
+△ 镜头特写：男人微微抬起头，帽子下的双眼透着一种复杂的恐惧。他的胡渣凌乱，嘴唇紧闭。
+△ 镜头全景：全场一片死寂，随后爆发出的快门声掩盖了一切。几十部手机同时举起，闪光灯疯狂跳动，对准了台上的所有人。
+【字幕：CUMBRE FUTURO GLOBAL 2025 - CONFERENCIA DE PRENSA -】</x:v>
+      </x:c>
+      <x:c r="I55" s="2" t="str">
+        <x:v>26s</x:v>
+      </x:c>
     </x:row>
     <x:row r="56" ht="200" customHeight="1">
-      <x:c r="A56" s="2"/>
-      <x:c r="B56" s="2"/>
-      <x:c r="C56" s="2"/>
-      <x:c r="D56" s="2"/>
-      <x:c r="E56" s="2"/>
-      <x:c r="F56" s="2"/>
-      <x:c r="G56" s="2"/>
-      <x:c r="H56" s="2"/>
-      <x:c r="I56" s="2"/>
+      <x:c r="A56" s="2" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="B56" s="2" t="str">
+        <x:v>33-1A</x:v>
+      </x:c>
+      <x:c r="C56" s="2" t="str">
+        <x:v>Tiburcio常服；Escolta A常服；Vera黑色晚宴装；Víctor常服；Don Ernesto常服；Damián常服；Carmen常服；Emiliano常服；Reportero C常服</x:v>
+      </x:c>
+      <x:c r="D56" s="2" t="str">
+        <x:v>晚宴酒店大厅</x:v>
+      </x:c>
+      <x:c r="E56" s="2" t="str">
+        <x:v>麦克风；单反相机</x:v>
+      </x:c>
+      <x:c r="F56" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+晚宴酒店大厅，9:16竖屏。沿用大厅吊灯与侧窗日光：窗光由西侧斜照，吊灯提供低弱环境亮度；背景板为无字色块，快门闪光短促，不把全场反复洗白。
+[音轨规则]
+远层：日间发布会低弱人群底噪，快门与无词议论声低于台词。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
+3.1s—10.6s，@Tiburcio常服（对白，低而沙哑，迟疑服从原句标点，不新增喘词）：「Hace tres años… el incendio del muelle. Yo vi con mis propios ojos cómo ella lo prendió.」
+[锚定列表]
+场景：@晚宴酒店大厅
+角色：@Tiburcio常服；@Escolta A常服；@Vera黑色晚宴装；@Víctor常服；@Don Ernesto常服；@Damián常服；@Carmen常服；@Emiliano常服；@Reportero C常服
+道具：麦克风；单反相机
+普通物件及用户另行确认的文字设计项不带@，不冒充已完成资产或新增绑定。
+[空间布局总览]
+会场设于既有晚宴酒店大厅：讲台在北侧矮台，座席面向北；中央通道南北向，主入口在南墙向厅内开，东侧有台阶通矮台。Vera黑色晚宴装在前排西侧靠中央通道座位，Damián常服在前排东侧；Reportero C常服在西侧边道拍摄。Víctor常服在讲台后，Don Ernesto常服站台上东侧，Carmen常服站台上西侧。三名功能性员工在后排西侧，其中一名负责传递文件，不冒充人物表Empleada A。讲台只有一支无线手持麦克风，起初固定于支架；谁拿到它谁发声扩声，其他现场对白保持真实空间声源，不复制麦克风。Tiburcio常服站台下中央，两名看管者在两侧，Escolta A常服在东侧。Víctor常服站讲台后东侧，右手持话筒；Vera黑色晚宴装站讲台南侧偏西，Carmen常服在后西侧；Damián常服在前排东侧座旁。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（5个硬切分镜）]
+分镜一：【景别/视角：证人与舞台关系中全景/西边道 | 运镜：侧移绕过已存在的相机前景，落在证人被看管的关系】
+【时长】3.0s
+【构图】Tiburcio常服帽檐低垂，两名看管者仍扶上臂；舞台人物看向他，记者留通道两侧。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】证人仍在台下中央，不站到讲台后。
+【镜头结尾·站位收束】证人仍在台下中央，不站到讲台后。
+画面硬切到分镜二。
+分镜二：【景别/视角：Tiburcio常服侧面近景 | 运镜：从台前西侧轻推，落在他抬头后的嘴部】
+【时长】4.0s
+【构图】Tiburcio常服抬头发出原定证词，声音低而沙哑；眼神短暂看向Vera黑色晚宴装后移开。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Tiburcio常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】证词尚在连续发声，两名看管者未松手。
+【镜头结尾·站位收束】证词尚在连续发声，两名看管者未松手。
+画面硬切到分镜三。
+分镜三：【景别/视角：Damián常服听者中近景/前排东侧 | 运镜：固定，以证人肩部作远处关系参照】
+【时长】4.0s
+【构图】证词跨切持续，Damián常服把双手插进西装裤袋，目光转向台上的Víctor常服，头部随后跟上。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Tiburcio常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Damián常服留座旁，没有走向证人。
+【镜头结尾·站位收束】Damián常服留座旁，没有走向证人。
+画面硬切到分镜四。
+分镜四：【景别/视角：Víctor常服侧面近景 | 运镜：从台前西南侧固定，话筒在他右手下方】
+【时长】3.0s
+【构图】证词完整结束，Víctor常服看向Damián常服，单侧嘴角轻抬后停住；不新增笑声。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】话筒仍在Víctor常服右手。
+【镜头结尾·站位收束】话筒仍在Víctor常服右手。
+画面硬切到分镜五。
+分镜五：【景别/视角：舞台三人关系中景 | 运镜：沿台前向东短移，显出空支架与Vera黑色晚宴装的可及距离】
+【时长】3.0s
+【构图】Víctor常服把话筒放回讲台支架并松手，Vera黑色晚宴装向讲台靠半步；Carmen常服留后西侧，Don Ernesto常服留东侧。
+【音效】手与话筒支架实际接触的轻响；台词期间压低动作声。
+【台词】无台词。
+【变化】麦克风回到支架，Vera黑色晚宴装有明确可发声位置。
+【镜头结尾·站位收束】麦克风回到支架，Vera黑色晚宴装有明确可发声位置。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：17s</x:v>
+      </x:c>
+      <x:c r="G56" s="2" t="str">
+        <x:v>Tiburcio：「Hace tres años… el incendio del muelle. Yo vi con mis propios ojos cómo ella lo prendió.」</x:v>
+      </x:c>
+      <x:c r="H56" s="2" t="str">
+        <x:v>第33集
+33-1 发布会大厅 日 内
+人物：Vera、Víctor、Don Ernesto、Emiliano、Renata、Damián、Carmen、Tiburcio、Reportero C、Empleado A、EscoltaA
+△ 镜头全景：发布会现场气氛凝重。巨大的背景板上印着“CUMBRE FUTURO GLOBAL 2025 CONFERENCIA DE PRENSA”。一名戴着棕色棒球帽、身穿破旧军绿色夹克的消瘦男人（Tiburcio）在两名保镖的看管下站在台前。
+△ 镜头特写：Tiburcio 微微抬起头，帽檐阴影遮住了上半张脸，露出凌乱的胡渣和紧闭的嘴唇，神情显得局促而畏缩。
+Tiburcio（声音低沉嘶哑）：Hace tres años… el incendio del muelle. Yo vi con mis propios ojos cómo ella lo prendió.
+△ 镜头反打：Damián 站在台下，双手插在西装裤口袋里，眼神中透着一股狠戾。他转过头，目光如利刃般射向站在台上的 Víctor。
+△ 镜头特写：Víctor 嘴角勾起一抹胜券在握的冷笑，他挑衅地对着 Damián 挑了挑眉，眼神中充满了报复的快感。</x:v>
+      </x:c>
+      <x:c r="I56" s="2" t="str">
+        <x:v>17s</x:v>
+      </x:c>
     </x:row>
     <x:row r="57" ht="200" customHeight="1">
-      <x:c r="A57" s="2"/>
-      <x:c r="B57" s="2"/>
-      <x:c r="C57" s="2"/>
-      <x:c r="D57" s="2"/>
-      <x:c r="E57" s="2"/>
-      <x:c r="F57" s="2"/>
-      <x:c r="G57" s="2"/>
-      <x:c r="H57" s="2"/>
-      <x:c r="I57" s="2"/>
+      <x:c r="A57" s="2" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="B57" s="2" t="str">
+        <x:v>33-1B</x:v>
+      </x:c>
+      <x:c r="C57" s="2" t="str">
+        <x:v>Vera黑色晚宴装；Tiburcio常服；Víctor常服；Escolta A常服；Carmen常服；Don Ernesto常服；Emiliano常服</x:v>
+      </x:c>
+      <x:c r="D57" s="2" t="str">
+        <x:v>晚宴酒店大厅</x:v>
+      </x:c>
+      <x:c r="E57" s="2" t="str">
+        <x:v>麦克风</x:v>
+      </x:c>
+      <x:c r="F57" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+晚宴酒店大厅，9:16竖屏。沿用大厅吊灯与侧窗日光：窗光由西侧斜照，吊灯提供低弱环境亮度；背景板为无字色块，快门闪光短促，不把全场反复洗白。
+[音轨规则]
+远层：日间发布会低弱人群底噪，快门与无词议论声低于台词。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
+0.2s—1.7s，@Vera黑色晚宴装（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「¿Usted estuvo ahí?」
+3.1s—4.0s，@Tiburcio常服（对白，低而沙哑，迟疑服从原句标点，不新增喘词）：「Sí.」
+5.1s—8.1s，@Vera黑色晚宴装（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「¿Hacia dónde soplaba el viento esa noche?」
+9.1s—10.6s，@Tiburcio常服（对白，低而沙哑，迟疑服从原句标点，不新增喘词）：「Hacia el norte.」
+12.1s—17.0s，@Vera黑色晚宴装（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「El reporte de rescate es público. El viento soplaba del SUR.」
+[锚定列表]
+场景：@晚宴酒店大厅
+角色：@Vera黑色晚宴装；@Tiburcio常服；@Víctor常服；@Escolta A常服；@Carmen常服；@Don Ernesto常服；@Emiliano常服
+道具：麦克风
+普通物件及用户另行确认的文字设计项不带@，不冒充已完成资产或新增绑定。
+[空间布局总览]
+会场设于既有晚宴酒店大厅：讲台在北侧矮台，座席面向北；中央通道南北向，主入口在南墙向厅内开，东侧有台阶通矮台。Vera黑色晚宴装在前排西侧靠中央通道座位，Damián常服在前排东侧；Reportero C常服在西侧边道拍摄。Víctor常服在讲台后，Don Ernesto常服站台上东侧，Carmen常服站台上西侧。三名功能性员工在后排西侧，其中一名负责传递文件，不冒充人物表Empleada A。讲台只有一支无线手持麦克风，起初固定于支架；谁拿到它谁发声扩声，其他现场对白保持真实空间声源，不复制麦克风。话筒已回讲台支架，Vera黑色晚宴装在南侧偏西，Víctor常服在讲台后东侧；Tiburcio常服站台下中央，Escolta A常服与普通安保各扶一侧上臂。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（6个硬切分镜）]
+分镜一：【景别/视角：Vera黑色晚宴装近景/台前东南侧 | 运镜：轻推，停在她与台下证人的视线关系】
+【时长】3.0s
+【构图】Vera黑色晚宴装靠近支架麦克风，直接问证人是否在场；下颌放松，问句清楚短促。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Vera黑色晚宴装的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Vera黑色晚宴装未触碰话筒。
+【镜头结尾·站位收束】Vera黑色晚宴装未触碰话筒。
+画面硬切到分镜二。
+分镜二：【景别/视角：Tiburcio常服近景/台前西侧 | 运镜：固定，Vera黑色晚宴装在画外较高视线方向】
+【时长】2.0s
+【构图】Tiburcio常服避开Vera黑色晚宴装视线，低头快速肯定；声源在台下，声音不从舞台话筒发出。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Tiburcio常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Tiburcio常服仍被两侧看管。
+【镜头结尾·站位收束】Tiburcio常服仍被两侧看管。
+画面硬切到分镜三。
+分镜三：【景别/视角：Vera黑色晚宴装俯视证人过肩中景 | 运镜：从Vera黑色晚宴装西后肩旁向南下方观察，帽檐和看管者构成中景】
+【时长】4.0s
+【构图】Vera黑色晚宴装问风向，身体留在台上；证人抬眼试图判断她的意思。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Vera黑色晚宴装的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】问题完整结束，双方距离未改变。
+【镜头结尾·站位收束】问题完整结束，双方距离未改变。
+画面硬切到分镜四。
+分镜四：【景别/视角：Tiburcio常服侧面近景 | 运镜：固定，帽檐阴影有可读眼神】
+【时长】3.0s
+【构图】Tiburcio常服稍停才答，目光飘向台上的Víctor常服；只保留一次短促迟疑，不加吞咽音。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Tiburcio常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】回答完整，Tiburcio常服未挪脚。
+【镜头结尾·站位收束】回答完整，Tiburcio常服未挪脚。
+画面硬切到分镜五。
+分镜五：【景别/视角：Vera黑色晚宴装侧面中近景 | 运镜：从台前西南侧向东短弧，落在她转向记者的姿态】
+【时长】4.0s
+【构图】Vera黑色晚宴装直起身体，指出救援报告与原定风向词；表情以唇角轻收表达，不新增解释性台词。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Vera黑色晚宴装的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Vera黑色晚宴装仍在讲台南侧，右手空着。
+【镜头结尾·站位收束】Vera黑色晚宴装仍在讲台南侧，右手空着。
+画面硬切到分镜六。
+分镜六：【景别/视角：Tiburcio常服与Víctor常服纵深中景 | 运镜：由证人西侧轻向后拉，揭出他目光的台上落点】
+【时长】3.0s
+【构图】Vera黑色晚宴装句尾跨切说完，Tiburcio常服看向Víctor常服，嘴唇不再抿紧；Víctor常服留在台后东侧。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Vera黑色晚宴装的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】台下求助目光与台上接收方明确。
+【镜头结尾·站位收束】台下求助目光与台上接收方明确。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：19s</x:v>
+      </x:c>
+      <x:c r="G57" s="2" t="str">
+        <x:v>Vera：「¿Usted estuvo ahí?」
+Tiburcio：「Sí.」
+Vera：「¿Hacia dónde soplaba el viento esa noche?」
+Tiburcio：「Hacia el norte.」
+Vera：「El reporte de rescate es público. El viento soplaba del SUR.」</x:v>
+      </x:c>
+      <x:c r="H57" s="2" t="str">
+        <x:v>△ 镜头近景：Vera 站在讲台一侧，身体微微前倾，靠近麦克风。她眼神犀利，直视着 Tiburcio，语气冷静且充满压迫感。
+Vera：¿Usted estuvo ahí?
+△ 镜头特写：Tiburcio 避开 Vera 的视线，有些不安地低下头，语速飞快。
+Tiburcio：Sí.
+Vera：¿Hacia dónde soplaba el viento esa noche?
+△ 镜头特写：Tiburcio 吞咽了一下，喉结上下滚动。他由于紧张，嘴角微微抽动。
+Tiburcio（迟疑了一下）：Hacia el norte.
+△ 镜头近景：Vera 露出一丝嘲讽的笑意，她直起身体，扫视全场记者，声音清冷。
+Vera：El reporte de rescate es público. El viento soplaba del SUR.
+△ 镜头特写：Tiburcio 的瞳孔由于谎言被戳穿而剧烈震动，他眼神慌乱地看向侧方的 Víctor。</x:v>
+      </x:c>
+      <x:c r="I57" s="2" t="str">
+        <x:v>19s</x:v>
+      </x:c>
     </x:row>
     <x:row r="58" ht="200" customHeight="1">
-      <x:c r="A58" s="2"/>
-      <x:c r="B58" s="2"/>
-      <x:c r="C58" s="2"/>
-      <x:c r="D58" s="2"/>
-      <x:c r="E58" s="2"/>
-      <x:c r="F58" s="2"/>
-      <x:c r="G58" s="2"/>
-      <x:c r="H58" s="2"/>
-      <x:c r="I58" s="2"/>
+      <x:c r="A58" s="2" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="B58" s="2" t="str">
+        <x:v>33-1C</x:v>
+      </x:c>
+      <x:c r="C58" s="2" t="str">
+        <x:v>Vera黑色晚宴装；Tiburcio常服；Víctor常服；Escolta A常服；Reportero C常服；Carmen常服；Don Ernesto常服</x:v>
+      </x:c>
+      <x:c r="D58" s="2" t="str">
+        <x:v>晚宴酒店大厅</x:v>
+      </x:c>
+      <x:c r="E58" s="2" t="str">
+        <x:v>麦克风；单反相机</x:v>
+      </x:c>
+      <x:c r="F58" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+晚宴酒店大厅，9:16竖屏。沿用大厅吊灯与侧窗日光：窗光由西侧斜照，吊灯提供低弱环境亮度；背景板为无字色块，快门闪光短促，不把全场反复洗白。
+[音轨规则]
+远层：日间发布会低弱人群底噪，快门与无词议论声低于台词。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
+0.2s—2.8s，@Vera黑色晚宴装（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「¿De qué color era el fuego?」
+3.6s—4.5s，@Tiburcio常服（对白，低而沙哑，迟疑服从原句标点，不新增喘词）：「Rojo.」
+5.6s—12.0s，@Vera黑色晚宴装（对白，语气低而清楚，按语义停顿，感叹号不自动变为尖叫）：「El fuego de una bodega de químicos arde AZUL. Cualquiera que estuvo ahí lo sabe.」
+[锚定列表]
+场景：@晚宴酒店大厅
+角色：@Vera黑色晚宴装；@Tiburcio常服；@Víctor常服；@Escolta A常服；@Reportero C常服；@Carmen常服；@Don Ernesto常服
+道具：麦克风；单反相机
+普通物件及用户另行确认的文字设计项不带@，不冒充已完成资产或新增绑定。
+[空间布局总览]
+会场设于既有晚宴酒店大厅：讲台在北侧矮台，座席面向北；中央通道南北向，主入口在南墙向厅内开，东侧有台阶通矮台。Vera黑色晚宴装在前排西侧靠中央通道座位，Damián常服在前排东侧；Reportero C常服在西侧边道拍摄。Víctor常服在讲台后，Don Ernesto常服站台上东侧，Carmen常服站台上西侧。三名功能性员工在后排西侧，其中一名负责传递文件，不冒充人物表Empleada A。讲台只有一支无线手持麦克风，起初固定于支架；谁拿到它谁发声扩声，其他现场对白保持真实空间声源，不复制麦克风。Vera黑色晚宴装在台上讲台南侧，Tiburcio常服在台下中央，两名看管者仍在其两侧；Víctor常服在讲台后东侧，麦克风固定支架。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（5个硬切分镜）]
+分镜一：【景别/视角：Vera黑色晚宴装近景/台前东南侧 | 运镜：短推后稳住，留出她问完后的停顿】
+【时长】3.5s
+【构图】Vera黑色晚宴装把目光重新落到Tiburcio常服，问火焰颜色；不额外前冲缩短台阶距离。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Vera黑色晚宴装的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Vera黑色晚宴装站位不变。
+【镜头结尾·站位收束】Vera黑色晚宴装站位不变。
+画面硬切到分镜二。
+分镜二：【景别/视角：Tiburcio常服近景 | 运镜：固定，在他开口时保护嘴部可读】
+【时长】2.0s
+【构图】Tiburcio常服立即答出原色词，句尾落下后目光停住，不新增第二个词。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Tiburcio常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】证人仍在台下中央。
+【镜头结尾·站位收束】证人仍在台下中央。
+画面硬切到分镜三。
+分镜三：【景别/视角：Vera黑色晚宴装侧面中近景 | 运镜：沿台前从西向东短移，停在她朝记者说话的位置】
+【时长】4.0s
+【构图】Vera黑色晚宴装指出化学品仓库火焰特征，原文大写只作自然语义重音，未安排尖叫。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Vera黑色晚宴装的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】她的原声保持连续，讲台支架不移动。
+【镜头结尾·站位收束】她的原声保持连续，讲台支架不移动。
+画面硬切到分镜四。
+分镜四：【景别/视角：Reportero C常服与证人关系中景 | 运镜：从西边道向北侧移，以镜头机身产生前景视差】
+【时长】4.0s
+【构图】Vera黑色晚宴装原声跨切说完整句，Reportero C常服举相机对准Tiburcio常服；背景记者随后举机，听众低声议论无可辨新词。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Vera黑色晚宴装的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】拍摄目标转为证人，通道仍不被围堵。
+【镜头结尾·站位收束】拍摄目标转为证人，通道仍不被围堵。
+画面硬切到分镜五。
+分镜五：【景别/视角：Víctor常服听者近景 | 运镜：从台前西南侧固定，Vera黑色晚宴装虚化侧影在画边】
+【时长】3.0s
+【构图】Víctor常服听完后鼻翼略张又收住，下颌紧张保留；没有剧烈喘气、变色或新增咒骂。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】Víctor常服还在讲台后东侧，准备转向后排声源。
+【镜头结尾·站位收束】Víctor常服还在讲台后东侧，准备转向后排声源。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：16.5s</x:v>
+      </x:c>
+      <x:c r="G58" s="2" t="str">
+        <x:v>Vera：「¿De qué color era el fuego?」
+Tiburcio：「Rojo.」
+Vera：「El fuego de una bodega de químicos arde AZUL. Cualquiera que estuvo ahí lo sabe.」</x:v>
+      </x:c>
+      <x:c r="H58" s="2" t="str">
+        <x:v>△ 镜头切换：Vera 步步紧逼，声音更冷了几分。
+Vera：¿De qué color era el fuego?
+Tiburcio（脱口而出）：Rojo.
+△ 镜头特写：Vera 的唇角上扬，露出了一个充满杀气的冷笑，眼神如看死人一般。
+Vera：El fuego de una bodega de químicos arde AZUL. Cualquiera que estuvo ahí lo sabe.
+△ 镜头全景：台下爆发出一阵嘈杂的议论声，记者们纷纷举起相机对着 Tiburcio 疯狂拍照。Víctor 脸色铁青，呼吸变得急促。</x:v>
+      </x:c>
+      <x:c r="I58" s="2" t="str">
+        <x:v>16.5s</x:v>
+      </x:c>
     </x:row>
-    <x:row r="59" ht="200" customHeight="1"/>
-    <x:row r="60" ht="200" customHeight="1"/>
+    <x:row r="59" ht="200" customHeight="1">
+      <x:c r="A59" s="2" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="B59" s="2" t="str">
+        <x:v>33-1D</x:v>
+      </x:c>
+      <x:c r="C59" s="2" t="str">
+        <x:v>Renata常服；Vera黑色晚宴装；Víctor常服；Damián常服；Carmen常服；Don Ernesto常服；Emiliano常服；Tiburcio常服；Escolta A常服；Reportero C常服</x:v>
+      </x:c>
+      <x:c r="D59" s="2" t="str">
+        <x:v>晚宴酒店大厅</x:v>
+      </x:c>
+      <x:c r="E59" s="2" t="str">
+        <x:v>麦克风；单反相机</x:v>
+      </x:c>
+      <x:c r="F59" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+晚宴酒店大厅，9:16竖屏。沿用大厅吊灯与侧窗日光：窗光由西侧斜照，吊灯提供低弱环境亮度；背景板为无字色块，快门闪光短促，不把全场反复洗白。
+[音轨规则]
+远层：日间发布会低弱人群底噪，快门与无词议论声低于台词。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段采用唯一声音骨架，镜头切换时持续发声，不在镜头栏重念；各区间为自然西语声演预算：
+3.1s—8.8s，@Renata常服（对白，向舞台发声，清楚坚决，受刺激处有轻微声线不稳，句子完整，不加入抽泣语词）：「¡Los moretones de mi hermana… el taco de billar estaba en SU mano!」
+10.1s—15.4s，@Renata常服（对白，向舞台发声，清楚坚决，受刺激处有轻微声线不稳，句子完整，不加入抽泣语词）：「¡Él la atacó a ELLA! ¡Yo lo vi con mis propios ojos!」
+15.6s—16.9s，@Víctor常服（对白，发布会现场发声，重音与音量随语义提高，字词不破音，不新增吼叫词）：「¡Renata! ¡SIÉNTATE!」
+17.1s—24.3s，@Renata常服（对白，向舞台发声，清楚坚决，受刺激处有轻微声线不稳，句子完整，不加入抽泣语词）：「¡La tuvieron encerrada en el ático tres años! ¿Quién de ustedes puede decir que no lo sabía?」
+[锚定列表]
+场景：@晚宴酒店大厅
+角色：@Renata常服；@Vera黑色晚宴装；@Víctor常服；@Damián常服；@Carmen常服；@Don Ernesto常服；@Emiliano常服；@Tiburcio常服；@Escolta A常服；@Reportero C常服
+道具：麦克风；单反相机
+普通物件及用户另行确认的文字设计项不带@，不冒充已完成资产或新增绑定。
+[空间布局总览]
+会场设于既有晚宴酒店大厅：讲台在北侧矮台，座席面向北；中央通道南北向，主入口在南墙向厅内开，东侧有台阶通矮台。Vera黑色晚宴装在前排西侧靠中央通道座位，Damián常服在前排东侧；Reportero C常服在西侧边道拍摄。Víctor常服在讲台后，Don Ernesto常服站台上东侧，Carmen常服站台上西侧。三名功能性员工在后排西侧，其中一名负责传递文件，不冒充人物表Empleada A。讲台只有一支无线手持麦克风，起初固定于支架；谁拿到它谁发声扩声，其他现场对白保持真实空间声源，不复制麦克风。Renata常服一直坐后排东侧靠边道位置，本段起身发声；Vera黑色晚宴装在台上讲台南侧，Víctor常服在后东侧，话筒固定支架。Tiburcio常服在台下中央，Escolta A常服与普通安保仍在两侧，Damián常服在前排东侧座旁。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（8个硬切分镜）]
+分镜一：【景别/视角：Renata常服侧后全身中景/东边道 | 运镜：由后排空座间向上轻抬，跟到她站稳】
+【时长】3.0s
+【构图】Renata常服双脚收稳后从后排起身，手掌离开椅背，面向北侧舞台；脸上已有伤痕沿用先前状态，不新增伤口。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】Renata常服站后排座侧，不走入中央通道。
+【镜头结尾·站位收束】Renata常服站后排座侧，不走入中央通道。
+画面硬切到分镜二。
+分镜二：【景别/视角：Renata常服近景/后排西南侧 | 运镜：缓推后稳住，让面部与指向有清楚边界】
+【时长】4.0s
+【构图】Renata常服说出第一句控诉，声音带不稳但词语完整；右手由身侧抬起指向舞台，幅度不盖住脸。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Renata常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】右手指向北侧，Renata常服仍站座旁。
+【镜头结尾·站位收束】右手指向北侧，Renata常服仍站座旁。
+画面硬切到分镜三。
+分镜三：【景别/视角：Vera黑色晚宴装听者近景/台前东南侧 | 运镜：先随她视线向南转，再在侧面落稳】
+【时长】3.0s
+【构图】Renata常服原声跨切说完，Vera黑色晚宴装视线先转向后排，头部跟随；她不代说后排台词。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Renata常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】Vera黑色晚宴装留舞台，目光到后排东侧。
+【镜头结尾·站位收束】Vera黑色晚宴装留舞台，目光到后排东侧。
+画面硬切到分镜四。
+分镜四：【景别/视角：Renata常服侧面中近景 | 运镜：从东边道固定，后排座椅形成纵深】
+【时长】4.0s
+【构图】Renata常服继续作证，句中的代词重音按原文保留；右手保持指向后放低，不反复挥动。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Renata常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】第二句控诉连续发声，双脚不移。
+【镜头结尾·站位收束】第二句控诉连续发声，双脚不移。
+画面硬切到分镜五。
+分镜五：【景别/视角：Víctor常服与麦克风中近景 | 运镜：从台前西侧短移，跟到他靠近话筒】
+【时长】3.0s
+【构图】Renata常服说完后Víctor常服从讲台后东侧跨近半步，右掌拍讲台一次，对麦克风发出原定制止词；不取下话筒。
+【音效】右掌与讲台一次短促接触声；台词期间压低动作声。
+【台词】@Renata常服的对白按本段唯一声音骨架连续发声；@Víctor常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】右掌落在台面，话筒仍在支架。
+【镜头结尾·站位收束】右掌落在台面，话筒仍在支架。
+画面硬切到分镜六。
+分镜六：【景别/视角：Renata常服近景/后排西南侧 | 运镜：固定，给她回击的声音完整起点】
+【时长】4.0s
+【构图】Renata常服迎视台上，追问被关阁楼的事实；声音清楚坚决，只在句中自然换气，不叠加尖叫。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Renata常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】她仍站后排，原声跨切继续。
+【镜头结尾·站位收束】她仍站后排，原声跨切继续。
+画面硬切到分镜七。
+分镜七：【景别/视角：台上台下关系高角度中全景 | 运镜：由西侧边道较高处向北慢摇，以后排Renata常服至台上Víctor常服为对角线】
+【时长】4.0s
+【构图】Renata常服整句连续说完，宾客视线在后排与台上之间转移；Vera黑色晚宴装仍在讲台南侧，证人与看管者留台前。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】@Renata常服的对白按本段唯一声音骨架连续发声；切到听者或手部时原声转画外，听者不代说。
+【变化】声源与所有人位置保持，不新增可辨人群台词。
+【镜头结尾·站位收束】声源与所有人位置保持，不新增可辨人群台词。
+画面硬切到分镜八。
+分镜八：【景别/视角：Víctor常服近景/台前西南侧 | 运镜：固定，停在他未能接话的状态】
+【时长】3.0s
+【构图】Víctor常服看向后排，原来准备张口的唇缝合住，右掌仍压在讲台；不重复拍台或再喊一次。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】Víctor常服留讲台后，Renata常服站后排，冲突落在沉默。
+【镜头结尾·站位收束】Víctor常服留讲台后，Renata常服站后排，冲突落在沉默。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：28s</x:v>
+      </x:c>
+      <x:c r="G59" s="2" t="str">
+        <x:v>Renata：「¡Los moretones de mi hermana… el taco de billar estaba en SU mano!」
+Renata：「¡Él la atacó a ELLA! ¡Yo lo vi con mis propios ojos!」
+Víctor：「¡Renata! ¡SIÉNTATE!」
+Renata：「¡La tuvieron encerrada en el ático tres años! ¿Quién de ustedes puede decir que no lo sabía?」</x:v>
+      </x:c>
+      <x:c r="H59" s="2" t="str">
+        <x:v>△ 镜头特写：会场后方，一名面部带伤、眼眶红肿的年轻女子（Renata）猛地站起身，她神情激愤，泪水盈满眼眶。
+        Renata（尖声控诉，声音颤抖）：¡Los moretones de mi hermana… el taco de billar estaba en SU mano!
+△ 镜头反打：Vera 站在台上，面无表情地看着 Renata。
+Renata（嘶吼着）：¡Él la atacó a ELLA! ¡Yo lo vi con mis propios ojos!
+△ 镜头切换：Víctor 猛地冲向麦克风，对着 Renata 疯狂咆哮，右手重重地拍击在讲台上。
+Víctor（怒吼）：¡Renata! ¡SIÉNTATE!
+△ 镜头近景：Renata 丝毫不退缩，她指着 Víctor 和台上的众人，泪流满面，声音因极度的悲愤而破碎。
+Renata：¡La tuvieron encerrada en el ático tres años! ¿Quién de ustedes puede decir que no lo sabía?
+△ 镜头特写：Víctor 僵在原地，眼神中闪过一丝惊恐和被揭穿的恼羞成怒。</x:v>
+      </x:c>
+      <x:c r="I59" s="2" t="str">
+        <x:v>28s</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="200" customHeight="1">
+      <x:c r="A60" s="2" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="B60" s="2" t="str">
+        <x:v>33-2A</x:v>
+      </x:c>
+      <x:c r="C60" s="2" t="str">
+        <x:v>Vera黑色晚宴装；Escolta A常服</x:v>
+      </x:c>
+      <x:c r="D60" s="2" t="str">
+        <x:v>酒店正门（外·夜）；轿车内</x:v>
+      </x:c>
+      <x:c r="E60" s="2" t="str">
+        <x:v>金色衔尾蛇纹章黑色文件夹</x:v>
+      </x:c>
+      <x:c r="F60" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+酒店正门（外·夜）；轿车内，9:16竖屏。酒店檐口既有暖灯从侧上方照台阶，车内顶灯只在车门开启后亮起；玻璃幕墙反射真实车道灯，不显示招牌文字。
+[音轨规则]
+远层：门外实际车流底噪，车辆停稳后发动机声降低，人物附近安静。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段无原定对白或旁白，不新增发声。
+[锚定列表]
+场景：酒店正门（外·夜）；@轿车内
+角色：@Vera黑色晚宴装；@Escolta A常服
+道具：金色衔尾蛇纹章黑色文件夹
+普通物件及用户另行确认的文字设计项不带@，不冒充已完成资产或新增绑定。
+[空间布局总览]
+酒店正门沿东西向立面，门内大厅在北、门外车道在南；门前有三层宽台阶，东侧留缓坡。黑色轿车沿东西向停在台阶南侧，右后车门朝北面向台阶；门外西侧留相机通道。外景按已获授权的文字设计，保持日夜为同一建筑，不冒用其他场景标签。从日间会场到夜间门外明确省略离场过程。Vera黑色晚宴装站台阶上第二层、面向南侧车道，双臂起初交叠；Escolta A常服坐轿车右后座，文件夹平放在其左侧空座，封面金色蛇咬尾图形朝上，不含可读字形。人物沿用已有造型，不另创黑风衣或全黑西装版本。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（7个硬切分镜）]
+分镜一：【景别/视角：酒店与车辆关系全景/车道西侧 | 运镜：沿人行空道向东短移，随轿车停稳后落稳】
+【时长】3.0s
+【构图】黑色轿车缓慢驶到台阶南侧停住，Vera黑色晚宴装在第二层台阶双臂交叠，面向车；她不同时出现在车内。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】轿车停稳，右后门仍关闭。
+【镜头结尾·站位收束】轿车停稳，右后门仍关闭。
+画面硬切到分镜二。
+分镜二：【景别/视角：右后车门侧面中景/车道东北侧 | 运镜：固定，完整呈现开门与落脚】
+【时长】4.0s
+【构图】Escolta A常服从车内推开右后门，先落右脚再转身站到车门外；空出的门扇停在开启位置，车内文件夹还在左侧空座。
+【音效】门扇与门锁随实际开合发声、鞋底接触地面声；台词期间压低动作声。
+【台词】无台词。
+【变化】Escolta A常服站车外，门已开，文件夹未移动。
+【镜头结尾·站位收束】Escolta A常服站车外，门已开，文件夹未移动。
+画面硬切到分镜三。
+分镜三：【景别/视角：车内文件夹与手部近景/开启车门外 | 运镜：在门外俯视后座，轻推到两手接触点】
+【时长】3.0s
+【构图】Escolta A常服俯身从开启门口伸入双手，分别托文件夹两侧下缘，抬离座垫并收回身前；相机不穿过车壳。
+【音效】门扇与门锁随实际开合发声；台词期间压低动作声。
+【台词】无台词。
+【变化】文件夹由双手托住，封面朝上，车门仍开启。
+【镜头结尾·站位收束】文件夹由双手托住，封面朝上，车门仍开启。
+画面硬切到分镜四。
+分镜四：【景别/视角：台阶侧面双人中景 | 运镜：沿台阶西侧空道侧向伴随，停在交接距离】
+【时长】3.0s
+【构图】Escolta A常服持文件夹走到第一层台阶，Vera黑色晚宴装在第二层放开交叠双臂，双手伸向文件夹两侧；两人相距一臂。
+【音效】脚步随起停出现；台词期间压低动作声。
+【台词】无台词。
+【变化】双方手指均已接触文件夹，Escolta A常服仍托底。
+【镜头结尾·站位收束】双方手指均已接触文件夹，Escolta A常服仍托底。
+画面硬切到分镜五。
+分镜五：【景别/视角：文件夹交接手部近景 | 运镜：固定，两侧手指与托底手掌在同一焦平面】
+【时长】3.0s
+【构图】Vera黑色晚宴装双手夹稳文件夹两侧并托住下缘后，Escolta A常服才松手退回半步；不在切镜时转移归属。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】文件夹归Vera黑色晚宴装，Escolta A常服双手空出。
+【镜头结尾·站位收束】文件夹归Vera黑色晚宴装，Escolta A常服双手空出。
+画面硬切到分镜六。
+分镜六：【景别/视角：文件夹封面特写 | 运镜：沿封面边缘短移，落在金色圆环蛇纹章】
+【时长】3.0s
+【构图】Vera黑色晚宴装左手托底、右手扶侧边，将封面略向自己倾斜；金色蛇咬尾图形随灯光改变反射，小字区域为无字黑面。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】纹章为图形，无任何可读字母，文件夹仍在双手。
+【镜头结尾·站位收束】纹章为图形，无任何可读字母，文件夹仍在双手。
+画面硬切到分镜七。
+分镜七：【景别/视角：双人关系中景/台阶西侧 | 运镜：由文件夹轻向上摇至Vera黑色晚宴装与Escolta A常服的目光关系】
+【时长】3.0s
+【构图】Vera黑色晚宴装抬眼看Escolta A常服一瞬，再把文件夹靠近身前；Escolta A常服留下一层台阶，车门仍开，两人都不发声。
+【音效】门扇与门锁随实际开合发声；台词期间压低动作声。
+【台词】无台词。
+【变化】Vera黑色晚宴装持文件夹站第二层台阶，Escolta A常服站第一层，结尾归属与位置明确。
+【镜头结尾·站位收束】Vera黑色晚宴装持文件夹站第二层台阶，Escolta A常服站第一层，结尾归属与位置明确。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：22s</x:v>
+      </x:c>
+      <x:c r="G60" s="2" t="str"/>
+      <x:c r="H60" s="2" t="str">
+        <x:v>33-2 豪华酒店/正门 夜 外
+人物：Vera、EscoltaA
+△ 镜头全景：夜幕降临，一辆黑色的豪华轿车稳稳地停在酒店门前。大楼的玻璃幕墙在灯光下闪烁着冰冷的光泽。
+△ 镜头近景：Vera 穿着黑色抹胸长裙，披着黑色长风衣，戴着黑色皮质长手套。她双手抱胸站在台阶上，神情孤傲而冷漠。
+△ 镜头特写：一名穿着全黑西装、戴着黑色手套的男保镖（EscoltaA）从车内走出，动作利落而恭敬。
+△ 动作特写：EscoltaA 弯腰捡起车座上的一个黑色硬质文件夹，随后双手递到 Vera 面前，微微低头。
+△ 镜头近景：Vera 伸出戴着手套的手接管文件夹。她眼神深邃地看了一眼 EscoltaA，没有言语。
+△ 镜头特写：文件夹的封面上，印着一个金色的“衔尾蛇”纹章——一条蛇正咬着自己的尾巴形成一个圆环。
+△ 镜头推近特写：纹章下方印着一行金色的小字。
+【字幕：DE ORO Y MERCURIO】</x:v>
+      </x:c>
+      <x:c r="I60" s="2" t="str">
+        <x:v>22s</x:v>
+      </x:c>
+    </x:row>
     <x:row r="61" ht="200" customHeight="1"/>
     <x:row r="62" ht="200" customHeight="1"/>
     <x:row r="63" ht="200" customHeight="1"/>

</xml_diff>

<commit_message>
Recheck storyboards and fix staging resets, occupied hands, and exit timing
</commit_message>
<xml_diff>
--- a/archive/projects/la-reina-del-bajo-mundo/deliverables/前夫黑道酵母_分镜_21-33.xlsx
+++ b/archive/projects/la-reina-del-bajo-mundo/deliverables/前夫黑道酵母_分镜_21-33.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分镜脚本" sheetId="1" r:id="Rcda49bf7d9264f2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分镜脚本" sheetId="1" r:id="R6f0b4baad72e4605"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -716,11 +716,11 @@
 道具：牛皮纸档案袋（文字设定）；两张便利贴（文字设定）；黑色胶卷转盘（文字设定）
 未带@的本段场景或物件按已授权的文字设计执行，保持下述位置、数量和状态。
 [空间布局总览]
-公寓室内为文字确定的连续空间：入口门在西墙，向室内开启；入口向东进入客厅，茶几在中部、沙发在其北侧；东侧为临街落地窗，东北转角窄玻璃面朝相邻楼；阳台移门在南侧。本文方位为世界参照，不随反打改变。Vera常服从西侧入口进入，档案袋和两层便利贴在茶几中央；胶卷转盘起初在袋内。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+公寓室内为文字确定的连续空间：入口门在南墙西端，向室内开启；入口向东进入客厅，茶几在中部、沙发在其北侧；东侧为临街落地窗，东北转角窄玻璃面朝相邻楼；阳台移门在南墙东端。本文方位为世界参照，不随反打改变。Vera常服从南墙西端入口进入，档案袋和两层便利贴在茶几中央；胶卷转盘起初在袋内。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
 [运镜时间线（6个硬切分镜）]
 分镜一：【景别/视角：客厅远景/入口内侧 | 运镜：沿入口向东短移，展示门、茶几与落地窗的关系】
 【时长】3.0s
-【构图】Vera常服从西门走进室内，先停在茶几西侧观察房间。
+【构图】Vera常服从入口门走进室内，先停在茶几西侧观察房间。
 【音效】门扇与门锁随实际开合发声、脚步随起停出现；台词期间压低动作声。
 【台词】无台词。
 【变化】Vera常服在茶几西侧，档案袋在桌中央。
@@ -823,7 +823,7 @@
 角色：@Vera常服
 未带@的本段场景或物件按已授权的文字设计执行，保持下述位置、数量和状态。
 [空间布局总览]
-公寓室内为文字确定的连续空间：入口门在西墙，向室内开启；入口向东进入客厅，茶几在中部、沙发在其北侧；东侧为临街落地窗，东北转角窄玻璃面朝相邻楼；阳台移门在南侧。本文方位为世界参照，不随反打改变。Vera常服在东窗内侧。楼下门卫两人为普通背景保镖，各守入口两侧，身份不与Escolta A合并。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+公寓室内为文字确定的连续空间：入口门在南墙西端，向室内开启；入口向东进入客厅，茶几在中部、沙发在其北侧；东侧为临街落地窗，东北转角窄玻璃面朝相邻楼；阳台移门在南墙东端。本文方位为世界参照，不随反打改变。Vera常服在东窗内侧。楼下门卫两人为普通背景保镖，各守入口两侧，身份不与Escolta A合并。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
 [运镜时间线（4个硬切分镜）]
 分镜一：【景别/视角：背面中景/客厅西侧望东 | 运镜：缓慢向东推进，落在Vera常服与窗框构成的关系画面】
 【时长】3.0s
@@ -908,7 +908,7 @@
 道具：狙击镜观察画面（文字设定）
 未带@的本段场景或物件按已授权的文字设计执行，保持下述位置、数量和状态。
 [空间布局总览]
-公寓室内为文字确定的连续空间：入口门在西墙，向室内开启；入口向东进入客厅，茶几在中部、沙发在其北侧；东侧为临街落地窗，东北转角窄玻璃面朝相邻楼；阳台移门在南侧。本文方位为世界参照，不随反打改变。Vera常服位于东窗偏北，身体朝东南看夜景；东北转角玻璃使相邻楼斜后方视线能看到她肩背。观察者始终在对楼，镜头不穿玻璃。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+公寓室内为文字确定的连续空间：入口门在南墙西端，向室内开启；入口向东进入客厅，茶几在中部、沙发在其北侧；东侧为临街落地窗，东北转角窄玻璃面朝相邻楼；阳台移门在南墙东端。本文方位为世界参照，不随反打改变。Vera常服位于东窗偏北，身体朝东南看夜景；东北转角玻璃使相邻楼斜后方视线能看到她肩背。观察者始终在对楼，镜头不穿玻璃。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
 [运镜时间线（3个硬切分镜）]
 分镜一：【景别/视角：远距主观特写/狙击镜视角 | 运镜：微幅调整朝向，保持远距机位不平移】
 【时长】3.0s
@@ -985,7 +985,7 @@
 道具：狙击镜观察画面（文字设定）
 未带@的本段场景或物件按已授权的文字设计执行，保持下述位置、数量和状态。
 [空间布局总览]
-公寓室内为文字确定的连续空间：入口门在西墙，向室内开启；入口向东进入客厅，茶几在中部、沙发在其北侧；东侧为临街落地窗，东北转角窄玻璃面朝相邻楼；阳台移门在南侧。本文方位为世界参照，不随反打改变。沿用Vera常服在东窗偏北面向东南的站位；东北侧窄窗允许对楼观察其肩背。红光先在后心附近，随她侧头调整到头后侧。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+公寓室内为文字确定的连续空间：入口门在南墙西端，向室内开启；入口向东进入客厅，茶几在中部、沙发在其北侧；东侧为临街落地窗，东北转角窄玻璃面朝相邻楼；阳台移门在南墙东端。本文方位为世界参照，不随反打改变。沿用Vera常服在东窗偏北面向东南的站位；东北侧窄窗允许对楼观察其肩背。红光先在后心附近，随她侧头调整到头后侧。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
 [运镜时间线（4个硬切分镜）]
 分镜一：【景别/视角：肩背近景/东北侧斜望 | 运镜：固定，避免让玻璃同时映出不可能的完整背面】
 【时长】3.0s
@@ -1603,11 +1603,11 @@
 道具：黄色牛皮纸线索信封（文字设定）
 未带@的本段场景或物件按已授权的文字设计执行，保持下述位置、数量和状态。
 [空间布局总览]
-公寓室内为文字确定的连续空间：入口门在西墙，向室内开启；入口向东进入客厅，茶几在中部、沙发在其北侧；东侧为临街落地窗，东北转角窄玻璃面朝相邻楼；阳台移门在南侧。本文方位为世界参照，不随反打改变。Vera常服从东窗走向西门；Renata常服在门外南侧抱着黄色信封，左脸淤伤和湿发是本场持续状态。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+公寓室内为文字确定的连续空间：入口门在南墙西端，向室内开启；入口向东进入客厅，茶几在中部、沙发在其北侧；东侧为临街落地窗，东北转角窄玻璃面朝相邻楼；阳台移门在南墙东端。本文方位为世界参照，不随反打改变。Vera常服从东窗走向入口门；Renata常服在门外南侧抱着黄色信封，左脸淤伤和湿发是本场持续状态。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
 [运镜时间线（4个硬切分镜）]
 分镜一：【景别/视角：客厅纵深中景/茶几南侧 | 运镜：随Vera常服由东向西短距离跟随】
 【时长】3.0s
-【构图】Vera常服听见门外动静，从东窗沿茶几南侧通道走向西门，双手空着。
+【构图】Vera常服听见门外动静，从东窗沿茶几南侧通道走向入口门，双手空着。
 【音效】门扇与门锁随实际开合发声、脚步随起停出现；台词期间压低动作声。
 【台词】无台词。
 【变化】Vera常服停在门内。
@@ -1692,7 +1692,7 @@
 道具：黄色牛皮纸线索信封（文字设定）
 未带@的本段场景或物件按已授权的文字设计执行，保持下述位置、数量和状态。
 [空间布局总览]
-公寓室内为文字确定的连续空间：入口门在西墙，向室内开启；入口向东进入客厅，茶几在中部、沙发在其北侧；东侧为临街落地窗，东北转角窄玻璃面朝相邻楼；阳台移门在南侧。本文方位为世界参照，不随反打改变。门已向室内开启。Vera常服在门内北侧，Renata常服在门外，左脸淤伤，黄色信封起初在Renata常服双手。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+公寓室内为文字确定的连续空间：入口门在南墙西端，向室内开启；入口向东进入客厅，茶几在中部、沙发在其北侧；东侧为临街落地窗，东北转角窄玻璃面朝相邻楼；阳台移门在南墙东端。本文方位为世界参照，不随反打改变。门已向室内开启。Vera常服在门内北侧，Renata常服在门外，左脸淤伤，黄色信封起初在Renata常服双手。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
 [运镜时间线（4个硬切分镜）]
 分镜一：【景别/视角：Renata常服中近景/门内向外 | 运镜：固定，信封和受伤左脸同处可读范围】
 【时长】4.0s
@@ -1781,11 +1781,11 @@
 道具：黄色牛皮纸线索信封（文字设定）；银色拉杆箱（文字设定）；深绿色薄大衣（文字设定）
 未带@的本段场景或物件按已授权的文字设计执行，保持下述位置、数量和状态。
 [空间布局总览]
-公寓室内为文字确定的连续空间：入口门在西墙，向室内开启；入口向东进入客厅，茶几在中部、沙发在其北侧；东侧为临街落地窗，东北转角窄玻璃面朝相邻楼；阳台移门在南侧。本文方位为世界参照，不随反打改变。Renata常服坐北侧单人沙发，怀抱靠枕；Vera常服在茶几西侧，信封将放在桌面；Emiliano常服由西门进入，手提银色拉杆箱。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+公寓室内为文字确定的连续空间：入口门在南墙西端，向室内开启；入口向东进入客厅，茶几在中部、沙发在其北侧；东侧为临街落地窗，东北转角窄玻璃面朝相邻楼；阳台移门在南墙东端。本文方位为世界参照，不随反打改变。Renata常服坐北侧单人沙发，怀抱靠枕；Vera常服在茶几西侧，信封将放在桌面；Emiliano常服由入口门进入，手提银色拉杆箱。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
 [运镜时间线（6个硬切分镜）]
 分镜一：【景别/视角：客厅中全景/南侧 | 运镜：向西短移显出入口与沙发】
 【时长】3.0s
-【构图】Renata常服坐沙发抱着靠枕，Vera常服把信封放在茶几西沿；西门推开，Emiliano常服先入门后把拉杆箱轮落地。
+【构图】Renata常服坐沙发抱着靠枕，Vera常服把信封放在茶几西沿；入口门推开，Emiliano常服先入门后把拉杆箱轮落地。
 【音效】门扇与门锁随实际开合发声、封口与纸张轻擦声；台词期间压低动作声。
 【台词】无台词。
 【变化】信封在茶几，Emiliano常服与箱子在入口内。
@@ -1812,16 +1812,16 @@
 【构图】Emiliano常服将箱子推到Vera常服身旁的空地，松开拉杆，再向门口退开；箱子不滑进沙发或桌下。
 【音效】保留本场环境底噪与自然呼吸，不添加强调音。
 【台词】无台词。
-【变化】银箱停在茶几西侧空地，Emiliano常服向西门离开。
-【镜头结尾·站位收束】银箱停在茶几西侧空地，Emiliano常服向西门离开。
+【变化】银箱停在茶几西侧空地，Emiliano常服向入口门离开。
+【镜头结尾·站位收束】银箱停在茶几西侧空地，Emiliano常服向入口门离开。
 画面硬切到分镜五。
 分镜五：【景别/视角：门口至衣凳侧面中景 | 运镜：镜头留在客厅，随Vera常服向北轻摇】
 【时长】3.0s
 【构图】Emiliano常服退出并带上门；Vera常服到沙发旁衣凳拿起深绿色薄大衣，双手提住肩部。
 【音效】门扇与门锁随实际开合发声；台词期间压低动作声。
 【台词】无台词。
-【变化】西门关闭，薄大衣在Vera常服双手。
-【镜头结尾·站位收束】西门关闭，薄大衣在Vera常服双手。
+【变化】入口门关闭，薄大衣在Vera常服双手。
+【镜头结尾·站位收束】入口门关闭，薄大衣在Vera常服双手。
 画面硬切到分镜六。
 分镜六：【景别/视角：姐妹关系近景/沙发西侧 | 运镜：缓慢靠近，落在披衣后两人的视线高度】
 【时长】3.5s
@@ -1891,7 +1891,7 @@
 道具：黄色牛皮纸线索信封（文字设定）；@泛黄法律文件；线索信件（文字设定）
 未带@的本段场景或物件按已授权的文字设计执行，保持下述位置、数量和状态。
 [空间布局总览]
-公寓室内为文字确定的连续空间：入口门在西墙，向室内开启；入口向东进入客厅，茶几在中部、沙发在其北侧；东侧为临街落地窗，东北转角窄玻璃面朝相邻楼；阳台移门在南侧。本文方位为世界参照，不随反打改变。Vera常服坐茶几西侧地毯上，Renata常服在北侧沙发睡着，身上盖薄毯；信封在茶几西沿，文件起初在信封内。Vera常服的米色风衣此刻暂搭在沙发旁衣凳上，外套仍属原人物资产，未新增第二件。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+公寓室内为文字确定的连续空间：入口门在南墙西端，向室内开启；入口向东进入客厅，茶几在中部、沙发在其北侧；东侧为临街落地窗，东北转角窄玻璃面朝相邻楼；阳台移门在南墙东端。本文方位为世界参照，不随反打改变。Vera常服坐茶几西侧地毯上，Renata常服在北侧沙发睡着，身上盖薄毯；信封在茶几西沿，文件起初在信封内。Vera常服的米色风衣此刻暂搭在沙发旁衣凳上，外套仍属原人物资产，未新增第二件。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
 [运镜时间线（6个硬切分镜）]
 分镜一：【景别/视角：公寓中全景/西南角 | 运镜：沿沙发前空道向东轻移，建立主次层】
 【时长】3.0s
@@ -1999,8 +1999,8 @@
 角色：@Vera常服；@Renata常服
 道具：@iPhone手机；@米色风衣
 [空间布局总览]
-公寓室内为文字确定的连续空间：入口门在西墙，向室内开启；入口向东进入客厅，茶几在中部、沙发在其北侧；东侧为临街落地窗，东北转角窄玻璃面朝相邻楼；阳台移门在南侧。本文方位为世界参照，不随反打改变。Vera常服从茶几西侧地毯起身，Renata常服仍在北侧沙发熟睡。手机在茶几西南角，风衣在衣凳上；南侧移门通阳台。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
-[运镜时间线（4个硬切分镜）]
+公寓室内为文字确定的连续空间：入口门在南墙西端，向室内开启；入口向东进入客厅，茶几在中部、沙发在其北侧；东侧为临街落地窗，东北转角窄玻璃面朝相邻楼；阳台移门在南墙东端。本文方位为世界参照，不随反打改变。Vera常服从茶几西侧地毯起身，Renata常服仍在北侧沙发熟睡。手机在茶几西南角，风衣在衣凳上；南侧移门通阳台。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（6个硬切分镜）]
 分镜一：【景别/视角：桌面手机近景/南侧 | 运镜：固定，屏幕斜背镜头】
 【时长】3.0s
 【构图】iPhone在茶几上振动，光面只露无字反光；Vera常服右手伸向手机。
@@ -2017,15 +2017,31 @@
 【变化】手机在右手，左手撑地。
 【镜头结尾·站位收束】手机在右手，左手撑地。
 画面硬切到分镜三。
-分镜三：【景别/视角：客厅至阳台关系中景 | 运镜：沿茶几南侧向南伴随，路径始终在室内】
-【时长】3.5s
-【构图】Vera常服借左手支撑起身，拿起米色风衣披好，走到南侧玻璃移门；手机仍在右手。
+分镜三：【景别/视角：Vera常服全身侧面中景 | 运镜：随她起身轻抬，保留左手支撑与双脚】
+【时长】3.0s
+【构图】Vera常服左手撑地、双脚收稳后起身，右手握手机；站直后沿茶几南侧通道走到衣凳旁。
+【音效】鞋底接触地面声、脚步随起停出现；台词期间压低动作声。
+【台词】无台词。
+【变化】Vera常服站衣凳旁，手机仍在右手。
+【镜头结尾·站位收束】Vera常服站衣凳旁，手机仍在右手。
+画面硬切到分镜四。
+分镜四：【景别/视角：衣凳与双手中近景 | 运镜：固定在衣凳南侧，让手部动作可读】
+【时长】3.0s
+【构图】Vera常服先把手机放在衣凳空处，双手拿起原有米色风衣并披好；手机在衣凳上，不占用披衣的手。
+【音效】手指与机身接触的低弱摩擦声；台词期间压低动作声。
+【台词】无台词。
+【变化】风衣披好，手机留衣凳空处。
+【镜头结尾·站位收束】风衣披好，手机留衣凳空处。
+画面硬切到分镜五。
+分镜五：【景别/视角：客厅至阳台关系中景 | 运镜：沿南侧通道伴随，停在玻璃移门前】
+【时长】3.0s
+【构图】Vera常服右手拿回手机，沿空道走到南墙东端的阳台移门；左手空出准备开门。
 【音效】门扇与门锁随实际开合发声、脚步随起停出现；台词期间压低动作声。
 【台词】无台词。
-【变化】Vera常服在移门内，左手空出。
-【镜头结尾·站位收束】Vera常服在移门内，左手空出。
-画面硬切到分镜四。
-分镜四：【景别/视角：移门侧面全身中景 | 运镜：在门内侧固定，让门扇边界清楚】
+【变化】Vera常服到移门内侧，右手持手机，左手空着。
+【镜头结尾·站位收束】Vera常服到移门内侧，右手持手机，左手空着。
+画面硬切到分镜六。
+分镜六：【景别/视角：移门侧面全身中景 | 运镜：在门内侧固定，让门扇边界清楚】
 【时长】3.5s
 【构图】她左手滑开玻璃门，跨过门槛，转身用左手合上移门；相机始终停在室内。
 【音效】门扇与门锁随实际开合发声；台词期间压低动作声。
@@ -2039,7 +2055,7 @@
 - 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
 - 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
-时长：13s</x:v>
+时长：18.5s</x:v>
       </x:c>
       <x:c r="G17" s="2" t="str"/>
       <x:c r="H17" s="2" t="str">
@@ -2053,7 +2069,7 @@
 △ 镜头跟随：Vera 推开通往阳台的玻璃移门，身后的书架排满书籍。她走出去后，反手将门拉上，发出一声轻微的咔哒声。</x:v>
       </x:c>
       <x:c r="I17" s="2" t="str">
-        <x:v>13s</x:v>
+        <x:v>18.5s</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="200" customHeight="1">
@@ -2089,7 +2105,7 @@
 角色：@Vera常服；@Don Ernesto常服
 道具：@iPhone手机
 [空间布局总览]
-公寓室内为文字确定的连续空间：入口门在西墙，向室内开启；入口向东进入客厅，茶几在中部、沙发在其北侧；东侧为临街落地窗，东北转角窄玻璃面朝相邻楼；阳台移门在南侧。本文方位为世界参照，不随反打改变。Vera常服在南侧阳台栏杆内侧，面向城市；Don Ernesto常服只作为电话VO，不入画、不设计其地点。右手持手机，左手可扶栏杆。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+公寓室内为文字确定的连续空间：入口门在南墙西端，向室内开启；入口向东进入客厅，茶几在中部、沙发在其北侧；东侧为临街落地窗，东北转角窄玻璃面朝相邻楼；阳台移门在南墙东端。本文方位为世界参照，不随反打改变。Vera常服在南侧阳台栏杆内侧，面向城市；Don Ernesto常服只作为电话VO，不入画、不设计其地点。右手持手机，左手可扶栏杆。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
 [运镜时间线（7个硬切分镜）]
 分镜一：【景别/视角：阳台侧后中景 | 运镜：沿阳台门外合法步道短移，停在Vera常服侧后】
 【时长】3.0s
@@ -2210,7 +2226,7 @@
 [运镜时间线（5个硬切分镜）]
 分镜一：【景别/视角：Vera常服侧后中景/玄关 | 运镜：沿客厅入口向西跟两步，停在门内】
 【时长】3.0s
-【构图】Vera常服走到西门内，先把目光凑近猫眼，右手还未碰门把。
+【构图】Vera常服走到入口门内，先把目光凑近猫眼，右手还未碰门把。
 【音效】门扇与门锁随实际开合发声、脚步随起停出现；台词期间压低动作声。
 【台词】无台词。
 【变化】Vera常服在门内，门关闭。
@@ -2726,8 +2742,8 @@
 角色：@Vera常服；@Ramón常服；@Carmen常服
 道具：@银色金属球棒
 [空间布局总览]
-公寓门在走廊北墙，向公寓内开启；走廊东西向，电梯在东端。Vera常服起初在门内北侧，Ramón常服在门外正前，Carmen常服在其西侧，Escolta A在其东后侧。Escolta A已向东逃走。Vera常服在门外中央，右手持棒；Ramón常服在她西前方，Carmen常服在Ramón常服西侧；东端电梯门关闭。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
-[运镜时间线（7个硬切分镜）]
+公寓门在走廊北墙，向公寓内开启；走廊东西向，电梯在东端。Escolta A已向东逃走。Vera常服在门外中央，右手持棒；Ramón常服在她西前方，Carmen常服在Ramón常服西侧；东端电梯门关闭。本场可见电梯在入口外东侧约两步处，两人沿这段短距离离场。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（9个硬切分镜）]
 分镜一：【景别/视角：双人腰部中近景/走廊南侧 | 运镜：向西短移，落在Vera常服左手与Ramón常服右腕】
 【时长】3.0s
 【构图】Ramón常服后退，Vera常服先以左手扣住他的右腕，将右手球棒放低倚在门外北墙，确认棒底落地后右手离开球棒。
@@ -2776,13 +2792,29 @@
 【变化】供述说完，Vera常服准备松开。
 【镜头结尾·站位收束】供述说完，Vera常服准备松开。
 画面硬切到分镜七。
-分镜七：【景别/视角：电梯厅纵深全景 | 运镜：镜头向东轻摇，落在电梯门前】
-【时长】3.5s
-【构图】Vera常服先松开腕部再松开前臂，Ramón常服捧住受伤右腕，Carmen常服从西侧上前搀扶其左臂，两人沿走廊东行进入已开启的电梯，门合上。
-【音效】门扇与门锁随实际开合发声、脚步随起停出现；台词期间压低动作声。
-【台词】无台词。
-【变化】两人已入电梯，Vera常服留门口，球棒仍靠门边北墙。
-【镜头结尾·站位收束】两人已入电梯，Vera常服留门口，球棒仍靠门边北墙。
+分镜七：【景别/视角：三人全身关系中景/门外南侧 | 运镜：固定，手腕松开与搀扶接触完整可见】
+【时长】3.0s
+【构图】Vera常服先松开腕部再离开前臂；Ramón常服左手捧住受伤右腕，Carmen常服移到其左侧搀住上臂，扶他站稳。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】Ramón常服站稳，Carmen常服扶左臂，Vera常服已无接触。
+【镜头结尾·站位收束】Ramón常服站稳，Carmen常服扶左臂，Vera常服已无接触。
+画面硬切到分镜八。
+分镜八：【景别/视角：电梯门前中景 | 运镜：沿走廊北侧向东短移，跟到电梯口】
+【时长】2.5s
+【构图】电梯门已打开，Carmen常服扶Ramón常服向东慢行两步，先后跨过电梯门槛，Vera常服留在公寓门外。
+【音效】门扇与门锁随实际开合发声；台词期间压低动作声。
+【台词】无台词。
+【变化】两人都在电梯内，未跨门时提前关门。
+【镜头结尾·站位收束】两人都在电梯内，未跨门时提前关门。
+画面硬切到分镜九。
+分镜九：【景别/视角：电梯与公寓入口关系中景 | 运镜：固定，保持Vera常服与门外北墙球棒同框】
+【时长】2.5s
+【构图】电梯门在两人进入后合拢，Vera常服停在公寓门口，球棒仍靠北墙；不在关门过程中继续拉人入内。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】电梯关闭，两人已离场，Vera常服留门外。
+【镜头结尾·站位收束】电梯关闭，两人已离场，Vera常服留门外。
 [关键约束铁律]
 - 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
 - 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
@@ -2790,7 +2822,7 @@
 - 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
 - 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
-时长：24.5s</x:v>
+时长：29s</x:v>
       </x:c>
       <x:c r="G24" s="2" t="str">
         <x:v>Ramón：「¡Ahhh! ¡Alto!」
@@ -2814,7 +2846,7 @@
 △ 镜头全景：Ramón 捧着折断的手腕，在 Carmen 的搀扶下，连滚带爬地逃进电梯。电梯门缓缓合上。</x:v>
       </x:c>
       <x:c r="I24" s="2" t="str">
-        <x:v>24.5s</x:v>
+        <x:v>29s</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="200" customHeight="1">
@@ -2846,8 +2878,8 @@
 角色：@Vera常服
 道具：@银色金属球棒
 [空间布局总览]
-公寓门在走廊北墙，向公寓内开启；走廊东西向，电梯在东端。Vera常服起初在门内北侧，Ramón常服在门外正前，Carmen常服在其西侧，Escolta A在其东后侧。电梯已关闭，Escolta A已逃离。Vera常服站公寓门外，门仍向内打开，球棒倚门外北墙。室内客厅通道在她身后。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
-[运镜时间线（4个硬切分镜）]
+公寓门在走廊北墙，向公寓内开启；走廊东西向，电梯在东端。电梯已关闭，Escolta A已逃离。Vera常服站公寓门外，门仍向内打开，球棒倚门外北墙。室内客厅通道在她身后。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（5个硬切分镜）]
 分镜一：【景别/视角：走廊关系全景 | 运镜：由东端电梯方向缓拉向门口】
 【时长】3.0s
 【构图】电梯门已经合拢，Vera常服独站门口；右手捡起靠墙球棒，转身退入玄关。
@@ -2856,23 +2888,31 @@
 【变化】Vera常服进入门内，右手持棒。
 【镜头结尾·站位收束】Vera常服进入门内，右手持棒。
 画面硬切到分镜二。
-分镜二：【景别/视角：玄关侧面中景 | 运镜：相机在门内固定，让身体下降过程完整可见】
-【时长】3.0s
-【构图】Vera常服将球棒平放在门内地面，右手离开；背靠门板慢慢屈膝坐下，左手扶地支撑。
+分镜二：【景别/视角：玄关侧面中景 | 运镜：固定，完整显示门扇合拢路径】
+【时长】2.5s
+【构图】Vera常服已退进玄关，右手持球棒向下，左手握门内把手把门合上，确认门锁扣合后松手。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】入口门已关闭，Vera常服站门内，球棒仍在右手。
+【镜头结尾·站位收束】入口门已关闭，Vera常服站门内，球棒仍在右手。
+画面硬切到分镜三。
+分镜三：【景别/视角：玄关侧面中景 | 运镜：相机在门内固定，让身体下降过程完整可见】
+【时长】3.0s
+【构图】Vera常服将球棒平放在门内地面，右手离开；背靠已关闭的门板慢慢屈膝坐下，左手扶地支撑。
 【音效】门扇与门锁随实际开合发声、棒身与接触物的短促撞击声；台词期间压低动作声。
 【台词】无台词。
-【变化】球棒横放门内地面；Vera常服坐在门内，门未凭空改变开向。
-【镜头结尾·站位收束】球棒横放门内地面；Vera常服坐在门内，门未凭空改变开向。
-画面硬切到分镜三。
-分镜三：【景别/视角：Vera常服近景/玄关侧面 | 运镜：缓慢靠近，落在她低垂的眼睑】
+【变化】球棒横放门内地面；Vera常服坐在已关闭的门内侧，左手扶地。
+【镜头结尾·站位收束】球棒横放门内地面；Vera常服坐在已关闭的门内侧，左手扶地。
+画面硬切到分镜四。
+分镜四：【景别/视角：Vera常服近景/玄关侧面 | 运镜：缓慢靠近，落在她低垂的眼睑】
 【时长】3.5s
 【构图】Vera常服短暂低头，呼吸由偏快逐渐变匀；已有紧张留在下颌，肩部只略松。
 【音效】保留本场环境底噪与自然呼吸，不添加强调音。
 【台词】无台词。
 【变化】Vera常服仍坐地，没有新增哭喊。
 【镜头结尾·站位收束】Vera常服仍坐地，没有新增哭喊。
-画面硬切到分镜四。
-分镜四：【景别/视角：低位全身中景 | 运镜：随她起身平缓上抬，保持脚与手的支撑关系】
+画面硬切到分镜五。
+分镜五：【景别/视角：低位全身中景 | 运镜：随她起身平缓上抬，保持脚与手的支撑关系】
 【时长】3.5s
 【构图】Vera常服左掌撑地，右手扶门框，先收脚再起身；站定后视线回到室内，球棒留在地面。
 【音效】保留本场环境底噪与自然呼吸，不添加强调音。
@@ -2886,7 +2926,7 @@
 - 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
 - 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
-时长：13s</x:v>
+时长：15.5s</x:v>
       </x:c>
       <x:c r="G25" s="2" t="str"/>
       <x:c r="H25" s="2" t="str">
@@ -2897,7 +2937,7 @@
 △ 镜头收尾：Vera 抬起头，眼神重新变得坚定，她单手撑地，摇摇晃晃地站了起来。</x:v>
       </x:c>
       <x:c r="I25" s="2" t="str">
-        <x:v>13s</x:v>
+        <x:v>15.5s</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="200" customHeight="1">
@@ -2932,7 +2972,7 @@
 道具：医用纱布；牛皮纸线索信封
 未带@的物件仅作剧本所需普通文字描述，不冒充已完成资产或新增绑定。
 [空间布局总览]
-公寓入口在西墙，茶几位于客厅中部、沙发在北侧，东墙落地窗可见城市，书桌工作区位于窗侧；南侧移门通阳台，桌椅之间保留南侧通道。世界方位不随反打改变。Vera常服坐茶几东侧，Emiliano常服坐茶几西侧，两人面对面。Vera常服左前臂横放茶几；纱布已绕过腕部，卷筒在Emiliano常服右手，左手托其腕。信封在Vera常服右手边。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+公寓入口在南墙西端，茶几位于客厅中部、沙发在北侧，东墙落地窗可见城市，书桌工作区位于窗侧；南墙东端移门通阳台，桌椅之间保留南侧通道。世界方位不随反打改变。Vera常服坐茶几东侧，Emiliano常服坐茶几西侧，两人面对面。Vera常服左前臂横放茶几；纱布已绕过腕部，卷筒在Emiliano常服右手，左手托其腕。信封在Vera常服右手边。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
 [运镜时间线（5个硬切分镜）]
 分镜一：【景别/视角：双手近景/茶几南侧 | 运镜：沿桌沿缓移，落在最后一圈纱布】
 【时长】3.0s
@@ -3837,7 +3877,7 @@
 道具：香槟杯
 未带@的物件仅作剧本所需普通文字描述，不冒充已完成资产或新增绑定。
 [空间布局总览]
-游艇艉部甲板中央是双人餐桌，Víctor常服坐桌西侧朝东，Don Ernesto常服坐桌东侧朝西；Escolta A在北侧通往船舱的入口旁站岗。南侧栏杆外为湖面，餐桌南侧留相机通道。两人的右手酒杯放在各自靠身前桌沿，文件起初收在Don Ernesto常服衣内。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+游艇艉部甲板中央是双人餐桌，Víctor常服坐桌西侧朝东，Don Ernesto常服坐桌东侧朝西；Escolta A在北侧通往船舱的入口旁站岗。南侧栏杆外为湖面，餐桌南侧留相机通道。两只酒杯起初放在各自靠身前桌沿，文件起初收在Don Ernesto常服衣内。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
 [运镜时间线（6个硬切分镜）]
 分镜一：【景别/视角：甲板关系全景/南侧栏杆内 | 运镜：沿桌南侧短移，展示两人相对位置与船舱入口】
 【时长】3.0s
@@ -3952,7 +3992,7 @@
 道具：联合声明文件；香槟杯
 未带@的物件仅作剧本所需普通文字描述，不冒充已完成资产或新增绑定。
 [空间布局总览]
-游艇艉部甲板中央是双人餐桌，Víctor常服坐桌西侧朝东，Don Ernesto常服坐桌东侧朝西；Escolta A在北侧通往船舱的入口旁站岗。南侧栏杆外为湖面，餐桌南侧留相机通道。两人的右手酒杯放在各自靠身前桌沿，文件起初收在Don Ernesto常服衣内。上段举杯后，两人先将杯底落回各自身前杯垫；右手松开后再取文件。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+游艇艉部甲板中央是双人餐桌，Víctor常服坐桌西侧朝东，Don Ernesto常服坐桌东侧朝西；Escolta A在北侧通往船舱的入口旁站岗。南侧栏杆外为湖面，餐桌南侧留相机通道。两人各以右手持一杯，杯底在各自桌沿上方，文件起初收在Don Ernesto常服衣内。上段举杯后，两人先将杯底落回各自身前杯垫；右手松开后再取文件。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
 [运镜时间线（6个硬切分镜）]
 分镜一：【景别/视角：酒杯与Don Ernesto常服中景 | 运镜：从杯底轻抬到衣内取物的手】
 【时长】3.0s
@@ -4062,7 +4102,7 @@
 角色：@Vera常服
 道具：@黑色信封
 [空间布局总览]
-公寓入口在西墙，茶几位于客厅中部、沙发在北侧，东墙落地窗可见城市，书桌工作区位于窗侧；南侧移门通阳台，桌椅之间保留南侧通道。世界方位不随反打改变。黑色信封在西侧入口内地面；Vera常服从客厅南侧通道经过，右手起初空着。她全程使用Vera常服，沿用现有服装与鞋履，不派生赤脚新造型。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+公寓入口在南墙西端，茶几位于客厅中部、沙发在北侧，东墙落地窗可见城市，书桌工作区位于窗侧；南墙东端移门通阳台，桌椅之间保留南侧通道。世界方位不随反打改变。黑色信封在南墙西端入口内地面；Vera常服从客厅南侧通道经过，右手起初空着。她全程使用Vera常服，沿用现有服装与鞋履，不派生赤脚新造型。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
 [运镜时间线（5个硬切分镜）]
 分镜一：【景别/视角：脚步与信封低位近景 | 运镜：沿入口地面向东短移，落在停步位置】
 【时长】3.0s
@@ -4388,7 +4428,7 @@
 角色：@Vera常服；@Damián常服
 道具：@红玫瑰花束
 [空间布局总览]
-高层公寓入口玻璃门位于大楼北侧立面、向大厅内开启；大楼室内在南，室外广场向北展开。Vera常服在半开门内南侧，Damián常服在门外北侧，面向Vera常服，双手托着红玫瑰束；门外东侧空地可供一步接近。Vera常服刚跨到门外半步，Damián常服站门外面对她，双手持花。门向大厅内半开，Vera常服可沿原路回去。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+高层公寓入口玻璃门位于大楼北侧立面、向大厅内开启；大楼室内在南，室外广场向北展开。Damián常服在门外北侧，面向Vera常服，双手托着红玫瑰束；门外东侧空地可供一步接近。Vera常服刚跨到门外半步，Damián常服站门外面对她，双手持花。门向大厅内半开，Vera常服可沿原路回去。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
 [运镜时间线（5个硬切分镜）]
 分镜一：【景别/视角：花束与双人中景 | 运镜：固定，Vera常服手掌、花束、Damián常服持握点均清楚】
 【时长】3.0s
@@ -4580,7 +4620,7 @@
 道具：@金色蝴蝶结礼盒；手电筒
 未带@的物件仅作剧本所需普通文字描述，不冒充已完成资产或新增绑定。
 [空间布局总览]
-庄园铁门沿东西向，庄园内部在北，街道在南，货车停在门外南侧，后车斗朝门口；Guardia常服在门内东侧岗亭，手电在右手。银色礼盒固定在后车斗中央，金色缎带与吊坠保持为同一套配件。Guardia常服已在门内，礼盒仍在车斗。Damián常服从北侧主楼方向走向铁门，两名普通背景保镖随在其后，不复制Escolta A身份。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+庄园铁门沿东西向，庄园内部在北，街道在南，货车停在门外南侧，后车斗朝门口；Guardia常服在门内东侧门边，手电在右手。银色礼盒固定在后车斗中央，金色缎带与吊坠保持为同一套配件。Guardia常服已在门内，礼盒仍在车斗。Damián常服从北侧主楼方向走向铁门，两名普通背景保镖随在其后，不复制Escolta A身份。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
 [运镜时间线（4个硬切分镜）]
 分镜一：【景别/视角：车斗与Guardia常服中景 | 运镜：在门内东侧固定，保持前后位置一致】
 【时长】3.0s
@@ -4928,7 +4968,7 @@
 道具：@iPhone手机；@黑色皮手套；旧发票
 未带@的物件仅作剧本所需普通文字描述，不冒充已完成资产或新增绑定。
 [空间布局总览]
-公寓入口在西墙，茶几位于客厅中部、沙发在北侧，东墙落地窗可见城市，书桌工作区位于窗侧；南侧移门通阳台，桌椅之间保留南侧通道。世界方位不随反打改变。按本场实际动作与落地窗描述取既有公寓的窗侧书桌工作区，不新增独立密室结构。Vera常服坐书桌西侧面向东窗，已有米色风衣暂搭在南侧衣凳，旧发票和黑色皮手套平放桌上，手机在其右手边。El Zorro Blanco只作为电话VO，不入画。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+公寓入口在南墙西端，茶几位于客厅中部、沙发在北侧，东墙落地窗可见城市，书桌工作区位于窗侧；南墙东端移门通阳台，桌椅之间保留南侧通道。世界方位不随反打改变。按本场实际动作与落地窗描述取既有公寓的窗侧书桌工作区，不新增独立密室结构。Vera常服坐书桌西侧面向东窗，已有米色风衣暂搭在南侧衣凳，旧发票和黑色皮手套平放桌上，手机在其右手边。El Zorro Blanco只作为电话VO，不入画。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
 [运镜时间线（6个硬切分镜）]
 分镜一：【景别/视角：桌面与右手近景 | 运镜：沿桌沿向东短移，落在手套与发票边缘】
 【时长】3.0s
@@ -5037,7 +5077,7 @@
 角色：@Vera常服
 道具：@iPhone手机；@米色风衣；@黑色皮手套
 [空间布局总览]
-公寓入口在西墙，茶几位于客厅中部、沙发在北侧，东墙落地窗可见城市，书桌工作区位于窗侧；南侧移门通阳台，桌椅之间保留南侧通道。世界方位不随反打改变。Vera常服在窗侧书桌西侧，手机在右手，手套和旧发票留桌面；外套为Vera常服已有米色风衣，不派生黑风衣。衣凳在她南侧，客厅向西通入口。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+公寓入口在南墙西端，茶几位于客厅中部、沙发在北侧，东墙落地窗可见城市，书桌工作区位于窗侧；南墙东端移门通阳台，桌椅之间保留南侧通道。世界方位不随反打改变。Vera常服在窗侧书桌西侧，手机在右手，手套和旧发票留桌面；外套为Vera常服已有米色风衣，不派生黑风衣。衣凳在她南侧，客厅向西绕茶几后通南墙西端入口。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
 [运镜时间线（4个硬切分镜）]
 分镜一：【景别/视角：Vera常服全身中景/书桌南侧 | 运镜：顺她起身轻抬，保留支撑手与双脚】
 【时长】3.0s
@@ -5068,8 +5108,8 @@
 【构图】Vera常服从书桌西侧沿客厅南侧通道走入较暗处；远处楼体红色光面只提供无字反射，手套留桌上。
 【音效】脚步随起停出现；台词期间压低动作声。
 【台词】无台词。
-【变化】Vera常服走向西侧入口方向，桌面手套与发票未随她移动。
-【镜头结尾·站位收束】Vera常服走向西侧入口方向，桌面手套与发票未随她移动。
+【变化】Vera常服走向南墙西端入口方向，桌面手套与发票未随她移动。
+【镜头结尾·站位收束】Vera常服走向南墙西端入口方向，桌面手套与发票未随她移动。
 [关键约束铁律]
 - 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
 - 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
@@ -5385,7 +5425,7 @@
 道具：单反相机；麦克风
 普通物件及用户另行确认的文字设计项不带@，不冒充已完成资产或新增绑定。
 [空间布局总览]
-会场设于既有晚宴酒店大厅：讲台在北侧矮台，座席面向北；中央通道南北向，主入口在南墙向厅内开，东侧有台阶通矮台。Vera黑色晚宴装在前排西侧靠中央通道座位，Damián常服在前排东侧；Reportero C常服在西侧边道拍摄。Víctor常服在讲台后，Don Ernesto常服站台上东侧，Carmen常服站台上西侧。三名功能性员工在后排西侧，其中一名负责传递文件，不冒充人物表Empleada A。讲台只有一支无线手持麦克风，起初固定于支架；谁拿到它谁发声扩声，其他现场对白保持真实空间声源，不复制麦克风。此时Vera黑色晚宴装尚未进场；Mujer为台下未具名年轻女子的现场OS，只作普通群众和声源描述，不新增身份资产。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+会场设于既有晚宴酒店大厅：讲台在北侧矮台，座席面向北；中央通道南北向，主入口在南墙向厅内开，东侧有台阶通矮台。前排西侧靠中央通道为Vera黑色晚宴装的座位，前排东侧为Damián常服的座位；西侧边道是摄影位。讲台东、西两侧各有站人空处；人物是否在座或已经上台，依本段起始状态与动作描述，不据座位名复位。三名功能性员工在后排西侧，其中一名负责传递文件，不冒充人物表Empleada A。讲台只有一支无线手持麦克风，本段起始归属以下述手部状态为准；在支架上时靠近它的人发声扩声，被取下时由持有者发声扩声，其他现场对白保持真实空间声源，不复制麦克风。此时Vera黑色晚宴装尚未进场；Mujer为台下未具名年轻女子的现场OS，只作普通群众和声源描述，不新增身份资产。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
 [运镜时间线（7个硬切分镜）]
 分镜一：【景别/视角：会场全景/南端中央通道 | 运镜：从入口向北短推，前排座位框出舞台】
 【时长】3.0s
@@ -5499,7 +5539,7 @@
 道具：单反相机；麦克风
 普通物件及用户另行确认的文字设计项不带@，不冒充已完成资产或新增绑定。
 [空间布局总览]
-会场设于既有晚宴酒店大厅：讲台在北侧矮台，座席面向北；中央通道南北向，主入口在南墙向厅内开，东侧有台阶通矮台。Vera黑色晚宴装在前排西侧靠中央通道座位，Damián常服在前排东侧；Reportero C常服在西侧边道拍摄。Víctor常服在讲台后，Don Ernesto常服站台上东侧，Carmen常服站台上西侧。三名功能性员工在后排西侧，其中一名负责传递文件，不冒充人物表Empleada A。讲台只有一支无线手持麦克风，起初固定于支架；谁拿到它谁发声扩声，其他现场对白保持真实空间声源，不复制麦克风。Vera黑色晚宴装从南门进入，前排西侧靠中央通道的座位空着。Emiliano常服尚未走入本段镜头。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+会场设于既有晚宴酒店大厅：讲台在北侧矮台，座席面向北；中央通道南北向，主入口在南墙向厅内开，东侧有台阶通矮台。前排西侧靠中央通道为Vera黑色晚宴装的座位，前排东侧为Damián常服的座位；西侧边道是摄影位。讲台东、西两侧各有站人空处；人物是否在座或已经上台，依本段起始状态与动作描述，不据座位名复位。三名功能性员工在后排西侧，其中一名负责传递文件，不冒充人物表Empleada A。讲台只有一支无线手持麦克风，本段起始归属以下述手部状态为准；在支架上时靠近它的人发声扩声，被取下时由持有者发声扩声，其他现场对白保持真实空间声源，不复制麦克风。Vera黑色晚宴装从南门进入，前排西侧靠中央通道的座位空着。Emiliano常服尚未走入本段镜头。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
 [运镜时间线（5个硬切分镜）]
 分镜一：【景别/视角：鞋与门槛低位近景 | 运镜：从门内西侧侧向伴随，落在完整跨门后的支撑脚】
 【时长】3.0s
@@ -5593,7 +5633,7 @@
 道具：麦克风；单反相机
 普通物件及用户另行确认的文字设计项不带@，不冒充已完成资产或新增绑定。
 [空间布局总览]
-会场设于既有晚宴酒店大厅：讲台在北侧矮台，座席面向北；中央通道南北向，主入口在南墙向厅内开，东侧有台阶通矮台。Vera黑色晚宴装在前排西侧靠中央通道座位，Damián常服在前排东侧；Reportero C常服在西侧边道拍摄。Víctor常服在讲台后，Don Ernesto常服站台上东侧，Carmen常服站台上西侧。三名功能性员工在后排西侧，其中一名负责传递文件，不冒充人物表Empleada A。讲台只有一支无线手持麦克风，起初固定于支架；谁拿到它谁发声扩声，其他现场对白保持真实空间声源，不复制麦克风。Escolta A常服在南门东侧边道，Carmen常服在上一场间隔已到台上西侧；Emiliano常服在南端中央通道外，尚未到前排。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+会场设于既有晚宴酒店大厅：讲台在北侧矮台，座席面向北；中央通道南北向，主入口在南墙向厅内开，东侧有台阶通矮台。前排西侧靠中央通道为Vera黑色晚宴装的座位，前排东侧为Damián常服的座位；西侧边道是摄影位。讲台东、西两侧各有站人空处；人物是否在座或已经上台，依本段起始状态与动作描述，不据座位名复位。三名功能性员工在后排西侧，其中一名负责传递文件，不冒充人物表Empleada A。讲台只有一支无线手持麦克风，本段起始归属以下述手部状态为准；在支架上时靠近它的人发声扩声，被取下时由持有者发声扩声，其他现场对白保持真实空间声源，不复制麦克风。Escolta A常服在南门东侧边道，Carmen常服在上一场间隔已到台上西侧；Emiliano常服在南端中央通道外，尚未到前排。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
 [运镜时间线（7个硬切分镜）]
 分镜一：【景别/视角：Vera黑色晚宴装侧面近景/前排东南侧 | 运镜：缓推，北侧讲台留画外视线目标】
 【时长】3.0s
@@ -5719,7 +5759,7 @@
 道具：麦克风；公证文件
 普通物件及用户另行确认的文字设计项不带@，不冒充已完成资产或新增绑定。
 [空间布局总览]
-会场设于既有晚宴酒店大厅：讲台在北侧矮台，座席面向北；中央通道南北向，主入口在南墙向厅内开，东侧有台阶通矮台。Vera黑色晚宴装在前排西侧靠中央通道座位，Damián常服在前排东侧；Reportero C常服在西侧边道拍摄。Víctor常服在讲台后，Don Ernesto常服站台上东侧，Carmen常服站台上西侧。三名功能性员工在后排西侧，其中一名负责传递文件，不冒充人物表Empleada A。讲台只有一支无线手持麦克风，起初固定于支架；谁拿到它谁发声扩声，其他现场对白保持真实空间声源，不复制麦克风。Emiliano常服从中央通道南端向前排走，左手持厚文件靠身侧；Vera黑色晚宴装仍坐前排西侧。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+会场设于既有晚宴酒店大厅：讲台在北侧矮台，座席面向北；中央通道南北向，主入口在南墙向厅内开，东侧有台阶通矮台。前排西侧靠中央通道为Vera黑色晚宴装的座位，前排东侧为Damián常服的座位；西侧边道是摄影位。讲台东、西两侧各有站人空处；人物是否在座或已经上台，依本段起始状态与动作描述，不据座位名复位。三名功能性员工在后排西侧，其中一名负责传递文件，不冒充人物表Empleada A。讲台只有一支无线手持麦克风，本段起始归属以下述手部状态为准；在支架上时靠近它的人发声扩声，被取下时由持有者发声扩声，其他现场对白保持真实空间声源，不复制麦克风。Emiliano常服从中央通道南端向前排走，左手持厚文件靠身侧；Vera黑色晚宴装仍坐前排西侧。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
 [运镜时间线（7个硬切分镜）]
 分镜一：【景别/视角：Emiliano常服侧后中景/中央通道 | 运镜：沿通道向北跟随，保持空位和讲台可见】
 【时长】3.5s
@@ -5838,7 +5878,7 @@
 道具：公证文件；麦克风；单反相机
 普通物件及用户另行确认的文字设计项不带@，不冒充已完成资产或新增绑定。
 [空间布局总览]
-会场设于既有晚宴酒店大厅：讲台在北侧矮台，座席面向北；中央通道南北向，主入口在南墙向厅内开，东侧有台阶通矮台。Vera黑色晚宴装在前排西侧靠中央通道座位，Damián常服在前排东侧；Reportero C常服在西侧边道拍摄。Víctor常服在讲台后，Don Ernesto常服站台上东侧，Carmen常服站台上西侧。三名功能性员工在后排西侧，其中一名负责传递文件，不冒充人物表Empleada A。讲台只有一支无线手持麦克风，起初固定于支架；谁拿到它谁发声扩声，其他现场对白保持真实空间声源，不复制麦克风。Vera黑色晚宴装站讲台南侧，Víctor常服在讲台后东侧，Carmen常服在后西侧。Emiliano常服已由座后走到台前西侧，左手持成套文件副本；一名功能性员工在其西侧准备接件。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+会场设于既有晚宴酒店大厅：讲台在北侧矮台，座席面向北；中央通道南北向，主入口在南墙向厅内开，东侧有台阶通矮台。前排西侧靠中央通道为Vera黑色晚宴装的座位，前排东侧为Damián常服的座位；西侧边道是摄影位。讲台东、西两侧各有站人空处；人物是否在座或已经上台，依本段起始状态与动作描述，不据座位名复位。三名功能性员工在后排西侧，其中一名负责传递文件，不冒充人物表Empleada A。讲台只有一支无线手持麦克风，本段起始归属以下述手部状态为准；在支架上时靠近它的人发声扩声，被取下时由持有者发声扩声，其他现场对白保持真实空间声源，不复制麦克风。Vera黑色晚宴装站讲台南侧，Víctor常服在讲台后东侧，Carmen常服在后西侧。Emiliano常服已由座后走到台前西侧，左手持成套文件副本；一名功能性员工在其西侧准备接件。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
 [运镜时间线（7个硬切分镜）]
 分镜一：【景别/视角：文件交接侧面近景/台前西侧 | 运镜：固定，双方接触和松手都在画内】
 【时长】3.0s
@@ -5957,7 +5997,7 @@
 道具：麦克风；单反相机
 普通物件及用户另行确认的文字设计项不带@，不冒充已完成资产或新增绑定。
 [空间布局总览]
-会场设于既有晚宴酒店大厅：讲台在北侧矮台，座席面向北；中央通道南北向，主入口在南墙向厅内开，东侧有台阶通矮台。Vera黑色晚宴装在前排西侧靠中央通道座位，Damián常服在前排东侧；Reportero C常服在西侧边道拍摄。Víctor常服在讲台后，Don Ernesto常服站台上东侧，Carmen常服站台上西侧。三名功能性员工在后排西侧，其中一名负责传递文件，不冒充人物表Empleada A。讲台只有一支无线手持麦克风，起初固定于支架；谁拿到它谁发声扩声，其他现场对白保持真实空间声源，不复制麦克风。Vera黑色晚宴装在讲台南侧，Víctor常服在东后半步，Carmen常服在后西侧。Tiburcio常服在南门外，Escolta A常服与一名普通安保各扶其一侧上臂；不复制Escolta A常服身份。Emiliano常服在台前西侧。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+会场设于既有晚宴酒店大厅：讲台在北侧矮台，座席面向北；中央通道南北向，主入口在南墙向厅内开，东侧有台阶通矮台。前排西侧靠中央通道为Vera黑色晚宴装的座位，前排东侧为Damián常服的座位；西侧边道是摄影位。讲台东、西两侧各有站人空处；人物是否在座或已经上台，依本段起始状态与动作描述，不据座位名复位。三名功能性员工在后排西侧，其中一名负责传递文件，不冒充人物表Empleada A。讲台只有一支无线手持麦克风，本段起始归属以下述手部状态为准；在支架上时靠近它的人发声扩声，被取下时由持有者发声扩声，其他现场对白保持真实空间声源，不复制麦克风。Vera黑色晚宴装在讲台南侧，Víctor常服在东后半步，Carmen常服在后西侧。Tiburcio常服在南门外，Escolta A常服与一名普通安保各扶其一侧上臂；不复制Escolta A常服身份。Emiliano常服在台前西侧。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
 [运镜时间线（8个硬切分镜）]
 分镜一：【景别/视角：麦克风与两人中近景/台前东南侧 | 运镜：固定，手掌与支架接触清楚】
 【时长】3.0s
@@ -6084,7 +6124,7 @@
 道具：麦克风；单反相机
 普通物件及用户另行确认的文字设计项不带@，不冒充已完成资产或新增绑定。
 [空间布局总览]
-会场设于既有晚宴酒店大厅：讲台在北侧矮台，座席面向北；中央通道南北向，主入口在南墙向厅内开，东侧有台阶通矮台。Vera黑色晚宴装在前排西侧靠中央通道座位，Damián常服在前排东侧；Reportero C常服在西侧边道拍摄。Víctor常服在讲台后，Don Ernesto常服站台上东侧，Carmen常服站台上西侧。三名功能性员工在后排西侧，其中一名负责传递文件，不冒充人物表Empleada A。讲台只有一支无线手持麦克风，起初固定于支架；谁拿到它谁发声扩声，其他现场对白保持真实空间声源，不复制麦克风。Tiburcio常服站台下中央，两名看管者在两侧，Escolta A常服在东侧。Víctor常服站讲台后东侧，右手持话筒；Vera黑色晚宴装站讲台南侧偏西，Carmen常服在后西侧；Damián常服在前排东侧座旁。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+会场设于既有晚宴酒店大厅：讲台在北侧矮台，座席面向北；中央通道南北向，主入口在南墙向厅内开，东侧有台阶通矮台。前排西侧靠中央通道为Vera黑色晚宴装的座位，前排东侧为Damián常服的座位；西侧边道是摄影位。讲台东、西两侧各有站人空处；人物是否在座或已经上台，依本段起始状态与动作描述，不据座位名复位。三名功能性员工在后排西侧，其中一名负责传递文件，不冒充人物表Empleada A。讲台只有一支无线手持麦克风，本段起始归属以下述手部状态为准；在支架上时靠近它的人发声扩声，被取下时由持有者发声扩声，其他现场对白保持真实空间声源，不复制麦克风。Tiburcio常服站台下中央，两名看管者在两侧，Escolta A常服在东侧。Víctor常服站讲台后东侧，右手持话筒；Vera黑色晚宴装站讲台南侧偏西，Carmen常服在后西侧；Damián常服在前排东侧座旁。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
 [运镜时间线（5个硬切分镜）]
 分镜一：【景别/视角：证人与舞台关系中全景/西边道 | 运镜：侧移绕过已存在的相机前景，落在证人被看管的关系】
 【时长】3.0s
@@ -6186,7 +6226,7 @@
 道具：麦克风
 普通物件及用户另行确认的文字设计项不带@，不冒充已完成资产或新增绑定。
 [空间布局总览]
-会场设于既有晚宴酒店大厅：讲台在北侧矮台，座席面向北；中央通道南北向，主入口在南墙向厅内开，东侧有台阶通矮台。Vera黑色晚宴装在前排西侧靠中央通道座位，Damián常服在前排东侧；Reportero C常服在西侧边道拍摄。Víctor常服在讲台后，Don Ernesto常服站台上东侧，Carmen常服站台上西侧。三名功能性员工在后排西侧，其中一名负责传递文件，不冒充人物表Empleada A。讲台只有一支无线手持麦克风，起初固定于支架；谁拿到它谁发声扩声，其他现场对白保持真实空间声源，不复制麦克风。话筒已回讲台支架，Vera黑色晚宴装在南侧偏西，Víctor常服在讲台后东侧；Tiburcio常服站台下中央，Escolta A常服与普通安保各扶一侧上臂。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+会场设于既有晚宴酒店大厅：讲台在北侧矮台，座席面向北；中央通道南北向，主入口在南墙向厅内开，东侧有台阶通矮台。前排西侧靠中央通道为Vera黑色晚宴装的座位，前排东侧为Damián常服的座位；西侧边道是摄影位。讲台东、西两侧各有站人空处；人物是否在座或已经上台，依本段起始状态与动作描述，不据座位名复位。三名功能性员工在后排西侧，其中一名负责传递文件，不冒充人物表Empleada A。讲台只有一支无线手持麦克风，本段起始归属以下述手部状态为准；在支架上时靠近它的人发声扩声，被取下时由持有者发声扩声，其他现场对白保持真实空间声源，不复制麦克风。话筒已回讲台支架，Vera黑色晚宴装在南侧偏西，Víctor常服在讲台后东侧；Tiburcio常服站台下中央，Escolta A常服与普通安保各扶一侧上臂。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
 [运镜时间线（6个硬切分镜）]
 分镜一：【景别/视角：Vera黑色晚宴装近景/台前东南侧 | 运镜：轻推，停在她与台下证人的视线关系】
 【时长】3.0s
@@ -6300,7 +6340,7 @@
 道具：麦克风；单反相机
 普通物件及用户另行确认的文字设计项不带@，不冒充已完成资产或新增绑定。
 [空间布局总览]
-会场设于既有晚宴酒店大厅：讲台在北侧矮台，座席面向北；中央通道南北向，主入口在南墙向厅内开，东侧有台阶通矮台。Vera黑色晚宴装在前排西侧靠中央通道座位，Damián常服在前排东侧；Reportero C常服在西侧边道拍摄。Víctor常服在讲台后，Don Ernesto常服站台上东侧，Carmen常服站台上西侧。三名功能性员工在后排西侧，其中一名负责传递文件，不冒充人物表Empleada A。讲台只有一支无线手持麦克风，起初固定于支架；谁拿到它谁发声扩声，其他现场对白保持真实空间声源，不复制麦克风。Vera黑色晚宴装在台上讲台南侧，Tiburcio常服在台下中央，两名看管者仍在其两侧；Víctor常服在讲台后东侧，麦克风固定支架。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+会场设于既有晚宴酒店大厅：讲台在北侧矮台，座席面向北；中央通道南北向，主入口在南墙向厅内开，东侧有台阶通矮台。前排西侧靠中央通道为Vera黑色晚宴装的座位，前排东侧为Damián常服的座位；西侧边道是摄影位。讲台东、西两侧各有站人空处；人物是否在座或已经上台，依本段起始状态与动作描述，不据座位名复位。三名功能性员工在后排西侧，其中一名负责传递文件，不冒充人物表Empleada A。讲台只有一支无线手持麦克风，本段起始归属以下述手部状态为准；在支架上时靠近它的人发声扩声，被取下时由持有者发声扩声，其他现场对白保持真实空间声源，不复制麦克风。Vera黑色晚宴装在台上讲台南侧，Tiburcio常服在台下中央，两名看管者仍在其两侧；Víctor常服在讲台后东侧，麦克风固定支架。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
 [运镜时间线（5个硬切分镜）]
 分镜一：【景别/视角：Vera黑色晚宴装近景/台前东南侧 | 运镜：短推后稳住，留出她问完后的停顿】
 【时长】3.5s
@@ -6401,7 +6441,7 @@
 道具：麦克风；单反相机
 普通物件及用户另行确认的文字设计项不带@，不冒充已完成资产或新增绑定。
 [空间布局总览]
-会场设于既有晚宴酒店大厅：讲台在北侧矮台，座席面向北；中央通道南北向，主入口在南墙向厅内开，东侧有台阶通矮台。Vera黑色晚宴装在前排西侧靠中央通道座位，Damián常服在前排东侧；Reportero C常服在西侧边道拍摄。Víctor常服在讲台后，Don Ernesto常服站台上东侧，Carmen常服站台上西侧。三名功能性员工在后排西侧，其中一名负责传递文件，不冒充人物表Empleada A。讲台只有一支无线手持麦克风，起初固定于支架；谁拿到它谁发声扩声，其他现场对白保持真实空间声源，不复制麦克风。Renata常服一直坐后排东侧靠边道位置，本段起身发声；Vera黑色晚宴装在台上讲台南侧，Víctor常服在后东侧，话筒固定支架。Tiburcio常服在台下中央，Escolta A常服与普通安保仍在两侧，Damián常服在前排东侧座旁。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+会场设于既有晚宴酒店大厅：讲台在北侧矮台，座席面向北；中央通道南北向，主入口在南墙向厅内开，东侧有台阶通矮台。前排西侧靠中央通道为Vera黑色晚宴装的座位，前排东侧为Damián常服的座位；西侧边道是摄影位。讲台东、西两侧各有站人空处；人物是否在座或已经上台，依本段起始状态与动作描述，不据座位名复位。三名功能性员工在后排西侧，其中一名负责传递文件，不冒充人物表Empleada A。讲台只有一支无线手持麦克风，本段起始归属以下述手部状态为准；在支架上时靠近它的人发声扩声，被取下时由持有者发声扩声，其他现场对白保持真实空间声源，不复制麦克风。Renata常服一直坐后排东侧靠边道位置，本段起身发声；Vera黑色晚宴装在台上讲台南侧，Víctor常服在后东侧，话筒固定支架。Tiburcio常服在台下中央，Escolta A常服与普通安保仍在两侧，Damián常服在前排东侧座旁。全部人物位置以上述实际空间参照控制；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
 [运镜时间线（8个硬切分镜）]
 分镜一：【景别/视角：Renata常服侧后全身中景/东边道 | 运镜：由后排空座间向上轻抬，跟到她站稳】
 【时长】3.0s

</xml_diff>